<commit_message>
daily: 2026-03-19 Excel更新 & HTML日報生成器
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,16 +15,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="26">
     <font>
-      <name val="Calibri"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -34,84 +33,84 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="22"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00BDD7EE"/>
+      <color rgb="FFBDD7EE"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00404040"/>
+      <color rgb="FF404040"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="FFFF0000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0000B050"/>
+      <color rgb="FF00B050"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FF0000"/>
+      <color rgb="FFFF0000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -126,19 +125,43 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00404040"/>
+      <color rgb="FF404040"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00888888"/>
+      <color rgb="FF888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF00B050"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="3"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -148,7 +171,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -157,22 +180,47 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="FFBDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="FF2E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E9F2FB"/>
+        <fgColor rgb="FFE9F2FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD7D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD7F0D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEAF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -182,30 +230,74 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD7D7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D7F0D7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEAF1"/>
+        <fgColor rgb="00E9F2FB"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -215,149 +307,139 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -370,20 +452,27 @@
     <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -749,253 +838,251 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" style="36" min="1" max="1"/>
+    <col width="22" customWidth="1" style="36" min="2" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26.65" customHeight="1" s="36">
+      <c r="A1" s="35" t="inlineStr">
         <is>
           <t>TSMC 台積電 (2330) 股市分析報告</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="60" customHeight="1" s="36">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>Taiwan Semiconductor Manufacturing Company Limited</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>報告更新日期：2026-03-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1"/>
-    <row r="5" ht="5" customHeight="1"/>
+    <row r="3" ht="30" customHeight="1" s="36">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>報告更新日期：2026-03-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="36"/>
+    <row r="5" ht="5" customHeight="1" s="36"/>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>股票基本資訊</t>
         </is>
       </c>
-      <c r="B6" s="42" t="n"/>
-      <c r="C6" s="42" t="n"/>
-      <c r="D6" s="43" t="n"/>
+      <c r="B6" s="39" t="n"/>
+      <c r="C6" s="39" t="n"/>
+      <c r="D6" s="40" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>台股 (2330.TW)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>NYSE ADR (TSM)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>當前股價</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>NT$1,900</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>US$338.89</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>2026-03-08收盤</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>52週最高</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>NT$2,025</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>US$426.42</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>2026-02-25</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>52週最低</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>NT$1,015</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>US$133.15</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>市值</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>NT$49.27 兆</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Beta值</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>1.16</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>1.16</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>市場敏感度</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>股價波動率</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>1.06%</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>1.06%</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>年化</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>下次除息日</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>NT$6.00/股</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>下次財報日</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Q1 2026</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="8" customHeight="1"/>
+    <row r="17" ht="8" customHeight="1" s="36"/>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>Source: Yahoo Finance, CNBC, MarketScreener, 2026-03-09</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="25" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="19" ht="25.05" customHeight="1" s="36">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>⚠ 免責聲明：本報告僅供參考，不構成任何投資建議。投資有風險，請自行評估並諮詢專業顧問。</t>
         </is>
@@ -1007,8 +1094,8 @@
     <mergeCell ref="A18:D18"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A19:D19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1023,585 +1110,582 @@
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" style="36" min="1" max="1"/>
+    <col width="18" customWidth="1" style="36" min="2" max="5"/>
+    <col width="22" customWidth="1" style="36" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 財務摘要 | Financial Summary</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>季度財務數據 (Quarterly P&amp;L)</t>
         </is>
       </c>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-      <c r="D3" s="42" t="n"/>
-      <c r="E3" s="42" t="n"/>
-      <c r="F3" s="43" t="n"/>
+      <c r="B3" s="39" t="n"/>
+      <c r="C3" s="39" t="n"/>
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="39" t="n"/>
+      <c r="F3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>財務指標</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Q4 2025</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Q4 2024</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>YoY變化</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>合併營收 (NT$ B)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>1,046.09</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>~975</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>~759</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>+37.8% YoY</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC PR 2026-01-16</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>淨利 (NT$ B)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>505.74</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>~452.30</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>~374</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>+35.3% YoY</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC PR 2026-01-16</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>每股盈餘 EPS (NT$)</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>19.50</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>~17.40</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>~14.45</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>+34.9% YoY</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC PR 2026-01-16, Q4 EPS</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>毛利率</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>62.3%</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>57.8%</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>~53%</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>+9.3pp YoY</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Earnings Q4 2025</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>營業利益率</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>54.0%</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>50.6%</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>~46.7%</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>+7.3pp YoY</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Earnings Q4 2025</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>38.8%</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>~36%</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>~29%</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>+9.8pp YoY</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Earnings Q4 2025</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="8" customHeight="1"/>
+    <row r="12" ht="8" customHeight="1" s="36"/>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="38" t="inlineStr">
         <is>
           <t>全年財務數據 (Full-Year 2025 vs 2024)</t>
         </is>
       </c>
-      <c r="B13" s="42" t="n"/>
-      <c r="C13" s="42" t="n"/>
-      <c r="D13" s="42" t="n"/>
-      <c r="E13" s="42" t="n"/>
-      <c r="F13" s="43" t="n"/>
+      <c r="B13" s="39" t="n"/>
+      <c r="C13" s="39" t="n"/>
+      <c r="D13" s="39" t="n"/>
+      <c r="E13" s="39" t="n"/>
+      <c r="F13" s="40" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>財務指標</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>FY 2025</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>FY 2024</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>YoY變化 (%)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>YoY變化 (pp)</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>合併營收 (NT$ 兆)</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>3.8</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>2.89</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>+31.6%</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>合併營收 (USD B)</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>122</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>89.5</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>+36.4%</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>全年毛利率</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>59.9%</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>53.0%</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>+3.8pp</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>+3.8</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>全年營業利益率</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>50.8%</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>42.6%</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>+5.1pp</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>+5.1</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>全年 EPS (NT$)</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>66.25</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>45.25</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>+46.4%</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>全年 ROE</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>35.4%</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>26.8%</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>+8.6pp</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>+8.6</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>營業現金流 (NT$ 兆)</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>1.97</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>+16.8%</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>自由現金流 (NT$ 兆)</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>0.87</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>+15.2%</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>現金及有價證券 (NT$ 兆)</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Annual Results 2025</t>
         </is>
@@ -1626,422 +1710,420 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" style="36" min="1" max="1"/>
+    <col width="16" customWidth="1" style="36" min="2" max="4"/>
+    <col width="20" customWidth="1" style="36" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 營收結構分析 | Revenue Breakdown Q4 2025</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>業務別營收佔比 (Business Segment)</t>
         </is>
       </c>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-      <c r="D3" s="42" t="n"/>
-      <c r="E3" s="43" t="n"/>
+      <c r="B3" s="39" t="n"/>
+      <c r="C3" s="39" t="n"/>
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>業務別</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Q4 2025 佔比</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>QoQ變化</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>FY 2025 佔比</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>YoY變化</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>HPC (高效能運算)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>55%</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>+4%</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>58%</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>+48% YoY</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>智慧型手機</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>+11%</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>+11% YoY</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>IoT (物聯網)</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>+3%</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>汽車電子</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>-1%</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>DCE (數位消費電子)</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>-22%</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>AI 加速器</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>High-teens%</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>High-teens%</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>快速成長</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="45" t="inlineStr">
         <is>
           <t>Source: TSMC Q4 2025 Earnings Call, 2026-01-16</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="8" customHeight="1"/>
+    <row r="13" ht="8" customHeight="1" s="36"/>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>製程節點佔比 (Technology Node Mix) — Q4 2025</t>
         </is>
       </c>
-      <c r="B14" s="42" t="n"/>
-      <c r="C14" s="42" t="n"/>
-      <c r="D14" s="42" t="n"/>
-      <c r="E14" s="43" t="n"/>
+      <c r="B14" s="39" t="n"/>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="40" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>製程節點</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>晶圓營收佔比</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>技術分類</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>狀態</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>N3 (3奈米)</t>
         </is>
       </c>
-      <c r="B16" s="22" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>28%</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>先進製程 ≤7nm</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>量產中</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>高效能、低功耗</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>N5 (5奈米)</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>先進製程 ≤7nm</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>量產中</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>主力製程</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>N7 (7奈米)</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>14%</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>先進製程 ≤7nm</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>量產中</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>成熟先進製程</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>小計 ≤7nm</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>77%</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>先進製程合計</t>
         </is>
       </c>
-      <c r="D19" s="26" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="19">
         <f>SUM(B16:B18)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>N2 (2奈米)</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>初期</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>次世代製程</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>HVM啟動</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Q4 2025進入高量產</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>N2P / A16</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>次世代製程</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>2026 H2</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>計畫2026下半年量產</t>
         </is>
@@ -2067,328 +2149,326 @@
   <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" style="36" min="1" max="1"/>
+    <col width="22" customWidth="1" style="36" min="2" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 2026年展望 | 2026 Outlook &amp; Guidance</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Q1 2026 管理層指引 (Management Guidance)</t>
         </is>
       </c>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-      <c r="D3" s="43" t="n"/>
+      <c r="B3" s="39" t="n"/>
+      <c r="C3" s="39" t="n"/>
+      <c r="D3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>指標</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>指引下限</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>指引上限</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>指引中位數</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Q1 2026 營收 (USD B)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>34.6</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>35.8</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>35.2 (中位數)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Q1 2026 毛利率</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>63.0%</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>65.0%</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>64.0% (中位數)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Q1 2026 營業利益率</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>54.0%</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>56.0%</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>55.0% (中位數)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>YoY 營收增長率</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>~38%</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>~38%</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>~38%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t>Source: TSMC Q4 2025 Earnings Call, 2026-01-16 | https://pr.tsmc.com/english/news/3281</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="8" customHeight="1"/>
+    <row r="11" ht="8" customHeight="1" s="36"/>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>全年 2026 展望 (Full-Year 2026 Outlook)</t>
         </is>
       </c>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-      <c r="D12" s="43" t="n"/>
+      <c r="B12" s="39" t="n"/>
+      <c r="C12" s="39" t="n"/>
+      <c r="D12" s="40" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>數值 / 範圍</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>比較基準</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>全年營收增長率 (USD)</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>~30% YoY</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>FY 2025: $122B</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Results</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>資本支出 (CapEx)</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>USD 52–56 B</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>FY 2025: ~$38B</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Results</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>先進製程CapEx佔比</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>70–80%</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Results</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>預估下期 EPS (NT$)</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>20.38</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Q4 2025: 19.50</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Source: MarketScreener Consensus</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>全年現金股利 (NT$/股)</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>≥23</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>FY 2025: 18</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Results</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>N2P / A16 量產</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>2026 H2</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>N2 已量產</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC Technology Roadmap</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>海外廠擴張</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Arizona / Japan</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>持續投資</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>美日廠擴產，壓縮部分毛利率</t>
         </is>
@@ -2414,362 +2494,359 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" style="36" min="1" max="1"/>
+    <col width="22" customWidth="1" style="36" min="2" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 股息記錄 | Dividend History</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>年度現金股利 (Annual Cash Dividend)</t>
         </is>
       </c>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-      <c r="D3" s="42" t="n"/>
-      <c r="E3" s="43" t="n"/>
+      <c r="B3" s="39" t="n"/>
+      <c r="C3" s="39" t="n"/>
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>年份</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>現金股利 (NT$/股)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>YoY增長率</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>發放日期</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>NT$10.00</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>NT$11.00</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>+10.0%</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>NT$14.00</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>+27.3%</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>NT$18.00</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>+28.6%</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Results</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>NT$23.00+</t>
         </is>
       </c>
-      <c r="C9" s="32" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>+27.8%+</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>2026 (預估)</t>
         </is>
       </c>
-      <c r="E9" s="34" t="inlineStr">
+      <c r="E9" s="26" t="inlineStr">
         <is>
           <t>Source: TSMC FY2025 Guidance; 最低金額</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="8" customHeight="1"/>
+    <row r="11" ht="8" customHeight="1" s="36"/>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>近期股息記錄 (Recent Quarterly Dividends)</t>
         </is>
       </c>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-      <c r="D12" s="42" t="n"/>
-      <c r="E12" s="43" t="n"/>
+      <c r="B12" s="39" t="n"/>
+      <c r="C12" s="39" t="n"/>
+      <c r="D12" s="39" t="n"/>
+      <c r="E12" s="40" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>季度</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>每季現金股利 (NT$/股)</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>除息日</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>支付日</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Q1 2026</t>
         </is>
       </c>
-      <c r="B14" s="31" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>NT$6.00</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="D14" s="33" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="E14" s="34" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Q4 2025</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>2025-10</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>NT$4.50</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Source: TSMC IR</t>
         </is>
@@ -2794,340 +2871,339 @@
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" style="36" min="1" max="1"/>
+    <col width="42" customWidth="1" style="36" min="2" max="2"/>
+    <col width="14" customWidth="1" style="36" min="3" max="4"/>
+    <col width="18" customWidth="1" style="36" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 投資風險評估 | Risk Assessment Matrix</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>主要風險矩陣 (Key Risk Matrix)</t>
         </is>
       </c>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-      <c r="D3" s="42" t="n"/>
-      <c r="E3" s="43" t="n"/>
+      <c r="B3" s="39" t="n"/>
+      <c r="C3" s="39" t="n"/>
+      <c r="D3" s="39" t="n"/>
+      <c r="E3" s="40" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>風險類別</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>風險描述</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>影響程度</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>發生機率</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>風險評級</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>地緣政治風險</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>台海緊張局勢、兩岸關係不確定性對生產造成衝擊</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E5" s="35" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>🔴 高</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>出口管制風險</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>AI晶片對中國出口限制（NVIDIA案例），影響客戶需求</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="E6" s="35" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>🔴 高</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>匯率風險</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>新台幣升值壓縮以美元計價之海外獲利</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>🟡 中</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>供應鏈風險</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>關鍵設備（ASML EUV）與材料依賴程度高</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>🟡 中</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>競爭風險</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>三星、Intel在先進製程的追趕，爭奪高端客戶</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
         <is>
           <t>🟡 中</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>總體經濟風險</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>關稅政策不確定性、消費性電子需求疲軟</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>🟡 中</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>技術風險</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>N2/A16量產良率爬升挑戰，海外廠製程複製困難</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>🟡 中</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>監管風險</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>美國補貼附帶條件、半導體法案限制</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E12" s="37" t="inlineStr">
+      <c r="E12" s="29" t="inlineStr">
         <is>
           <t>🟢 低</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="8" customHeight="1"/>
+    <row r="14" ht="8" customHeight="1" s="36"/>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>技術與市場優勢 (Competitive Moat)</t>
         </is>
       </c>
-      <c r="B15" s="42" t="n"/>
-      <c r="C15" s="42" t="n"/>
-      <c r="D15" s="42" t="n"/>
-      <c r="E15" s="43" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="B15" s="39" t="n"/>
+      <c r="C15" s="39" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="40" t="n"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" s="36">
+      <c r="A16" s="46" t="inlineStr">
         <is>
           <t>1. 技術領先：全球唯一量產3nm的foundry，N2於Q4 2025進入HVM，持續領先競爭對手2-3代</t>
         </is>
       </c>
-      <c r="B16" s="42" t="n"/>
-      <c r="C16" s="42" t="n"/>
-      <c r="D16" s="42" t="n"/>
-      <c r="E16" s="43" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="39" t="inlineStr">
+      <c r="B16" s="39" t="n"/>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="40" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" s="36">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>2. 規模優勢：全球晶圓代工市占率約60%，客戶黏著度高（Apple、NVIDIA、AMD、Qualcomm）</t>
         </is>
       </c>
-      <c r="B17" s="42" t="n"/>
-      <c r="C17" s="42" t="n"/>
-      <c r="D17" s="42" t="n"/>
-      <c r="E17" s="43" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="B17" s="39" t="n"/>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="40" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" s="36">
+      <c r="A18" s="46" t="inlineStr">
         <is>
           <t>3. AI需求催動：AI伺服器、HPC晶片需求爆發，2025年AI加速器佔比達high-teens%</t>
         </is>
       </c>
-      <c r="B18" s="42" t="n"/>
-      <c r="C18" s="42" t="n"/>
-      <c r="D18" s="42" t="n"/>
-      <c r="E18" s="43" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="39" t="inlineStr">
+      <c r="B18" s="39" t="n"/>
+      <c r="C18" s="39" t="n"/>
+      <c r="D18" s="39" t="n"/>
+      <c r="E18" s="40" t="n"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" s="36">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>4. 地理分散：Arizona、Japan廠持續擴產，降低地緣政治集中風險</t>
         </is>
       </c>
-      <c r="B19" s="42" t="n"/>
-      <c r="C19" s="42" t="n"/>
-      <c r="D19" s="42" t="n"/>
-      <c r="E19" s="43" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="38" t="inlineStr">
+      <c r="B19" s="39" t="n"/>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="39" t="n"/>
+      <c r="E19" s="40" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="36">
+      <c r="A20" s="46" t="inlineStr">
         <is>
           <t>5. 強健財務：ROE 35.4%、自由現金流NT$1兆，資本實力雄厚</t>
         </is>
       </c>
-      <c r="B20" s="42" t="n"/>
-      <c r="C20" s="42" t="n"/>
-      <c r="D20" s="42" t="n"/>
-      <c r="E20" s="43" t="n"/>
+      <c r="B20" s="39" t="n"/>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3150,222 +3226,370 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" style="36" min="1" max="1"/>
+    <col width="18" customWidth="1" style="36" min="2" max="2"/>
+    <col width="12" customWidth="1" style="36" min="3" max="3"/>
+    <col width="18" customWidth="1" style="36" min="4" max="4"/>
+    <col width="16" customWidth="1" style="36" min="5" max="5"/>
+    <col width="40" customWidth="1" style="36" min="6" max="6"/>
+    <col width="22" customWidth="1" style="36" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="36">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>TSMC 每日股價更新記錄 | Daily Price Update Log</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>最後更新：2026-03-12</t>
+    <row r="2" ht="22.05" customHeight="1" s="36">
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>最後更新：2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>台股收盤價 (TWD)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>漲跌幅 (%)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>NYSE收盤價 (USD)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>成交量 (張)</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>當日重要消息</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>資料來源</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>NT$1,900</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>+1.86%</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>US$338.89</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>初始建立報告，資料來源多方</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Yahoo Finance / CNBC / MarketScreener</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="8" customHeight="1"/>
-    <row r="7" ht="25" customHeight="1">
-      <c r="A7" s="41" t="inlineStr">
+    <row r="6" ht="8" customHeight="1" s="36"/>
+    <row r="7" ht="25.05" customHeight="1" s="36">
+      <c r="A7" s="49" t="inlineStr">
         <is>
           <t>💡 每日更新說明：在第4列以下依序新增記錄，或使用排程技能自動更新。欄位C漲跌幅為正數請填綠色、負數填紅色。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>NT$1,890</t>
         </is>
       </c>
-      <c r="C8" s="44" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>US$348.70</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>28,542 張</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>2月月營收今日公告（待更新）；前SVP涉嫌洩露2nm技術給Intel受調查；NVIDIA GTC 3/16揭露Feynman/A16；Arizona 3nm提前至2027</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Yahoo Finance / TSMC IR</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>NT$1,915</t>
         </is>
       </c>
-      <c r="C9" s="45" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>+1.86%</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>US$349.49</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>39,307 張</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>2月月營收年增22.2%，台股受惠反彈+1.86%；NYSE受美伊戰爭風險下跌-2.22%至US$349.49</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>NT$1,895</t>
         </is>
       </c>
-      <c r="C10" s="46" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>+2.37%</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>US$349.49</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>39,307 張</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>NVIDIA超越Apple成TSMC最大客戶(22%)；N2良率70-80%；NYSE受美伊風險跌2.22%；台股逆勢+2.37%</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Bloomberg/CNBC/Yahoo Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>NT$1,885</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>-2.84%</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>US$336.71</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>33,942 張</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>NYSE TSM 重挫-5.03%，卡達暫停LNG出口能源風險升溫；GTC 2026（3/17）NVIDIA Feynman晶片即將揭曉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>NT$1,870</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>-5.03%</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>US$336.71</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>23,688 張</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>NYSE TSM 3/18大跌-5.03%至$336.71，半導體板塊廣泛修正；NVIDIA Feynman確認採TSMC A16；記憶體短缺延伸至2027</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,905</t>
+        </is>
+      </c>
+      <c r="C13" s="51" t="inlineStr">
+        <is>
+          <t>+1.87%</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>US$336.71</t>
+        </is>
+      </c>
+      <c r="E13" s="50" t="inlineStr">
+        <is>
+          <t>23,015 張</t>
+        </is>
+      </c>
+      <c r="F13" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 3/18逆勢收紅+1.87%至NT$1,905；NVIDIA超越Apple成TSMC最大客戶；2nm N2P試量產啟動；TSMC市佔72%</t>
+        </is>
+      </c>
+      <c r="G13" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="53" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B14" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,905</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>+1.87%</t>
+        </is>
+      </c>
+      <c r="D14" s="53" t="inlineStr">
+        <is>
+          <t>US$336.71</t>
+        </is>
+      </c>
+      <c r="E14" s="53" t="inlineStr">
+        <is>
+          <t>23,015 張</t>
+        </is>
+      </c>
+      <c r="F14" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 3/18逆勢收紅+1.87%至NT$1,905；NVIDIA超越Apple成TSMC最大客戶；2nm N2P試量產啟動；TSMC市佔72%</t>
+        </is>
+      </c>
+      <c r="G14" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-20 日報 HTML & Excel 更新
台股 2330: NT$1,850 (-2.89%) | NYSE TSM: $334.58 (-1.47%)
主題: 氦氣供應危機 + Samsung $734億AI投資; 法人目標NT$2,290(+23.8%)
Excel 每日更新記錄第 16 行

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -170,6 +170,12 @@
       <color rgb="0000B050"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -311,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -469,6 +475,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -859,7 +868,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-19</t>
+          <t>報告更新日期：2026-03-20</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3248,7 +3257,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-19</t>
+          <t>最後更新：2026-03-20</t>
         </is>
       </c>
     </row>
@@ -3590,6 +3599,80 @@
       <c r="G14" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,905</t>
+        </is>
+      </c>
+      <c r="C15" s="51" t="inlineStr">
+        <is>
+          <t>+1.87%</t>
+        </is>
+      </c>
+      <c r="D15" s="50" t="inlineStr">
+        <is>
+          <t>US$336.71</t>
+        </is>
+      </c>
+      <c r="E15" s="50" t="inlineStr">
+        <is>
+          <t>23,015 張</t>
+        </is>
+      </c>
+      <c r="F15" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 3/18逆勢收紅+1.87%至NT$1,905；NVIDIA超越Apple成TSMC最大客戶；2nm N2P試量產啟動；TSMC市佔72%</t>
+        </is>
+      </c>
+      <c r="G15" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="53" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B16" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,850</t>
+        </is>
+      </c>
+      <c r="C16" s="56" t="inlineStr">
+        <is>
+          <t>-2.89%</t>
+        </is>
+      </c>
+      <c r="D16" s="53" t="inlineStr">
+        <is>
+          <t>US$334.58</t>
+        </is>
+      </c>
+      <c r="E16" s="53" t="inlineStr">
+        <is>
+          <t>30,200 張</t>
+        </is>
+      </c>
+      <c r="F16" s="55" t="inlineStr">
+        <is>
+          <t>氦氣供應危機壓制+Samsung $734億AI投資；法人目標NT$2,290(+23.8%)</t>
+        </is>
+      </c>
+      <c r="G16" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Reuters</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-23 日報 HTML & Excel 更新
- NYSE TSM 確認收 US$329.24 (-9.55, -2.82%)，台股 2330 確認收 NT$1,850 (-2.89%)
- 週末重大利多：NVIDIA 超越 Apple 成最大客戶 ($330B/22%)；Feynman 採 TSMC A16；亞利桑那 Phase 2 提前 2027
- 股東人數突破 246 萬人歷史新高（週增 75,536 人）
- 情緒由中性偏空調升至中性偏多；ADR 溢價更新 +12.7%
- HTML 日報產生：TSMC_日報_2026-03-23.html
- Excel 每日更新記錄第 17 行寫入

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -317,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -477,6 +477,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -868,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-20</t>
+          <t>報告更新日期：2026-03-23</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3257,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-20</t>
+          <t>最後更新：2026-03-23</t>
         </is>
       </c>
     </row>
@@ -3673,6 +3676,43 @@
       <c r="G16" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Reuters</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,850</t>
+        </is>
+      </c>
+      <c r="C17" s="57" t="inlineStr">
+        <is>
+          <t>-2.89%</t>
+        </is>
+      </c>
+      <c r="D17" s="50" t="inlineStr">
+        <is>
+          <t>US$329.24</t>
+        </is>
+      </c>
+      <c r="E17" s="50" t="inlineStr">
+        <is>
+          <t>30,200 張</t>
+        </is>
+      </c>
+      <c r="F17" s="52" t="inlineStr">
+        <is>
+          <t>NVIDIA 超越 Apple 成 TSMC 最大客戶（22%/$330B）；Feynman 採 A16；亞利桑那 Phase 2 提前 2027；股東數 246 萬創高</t>
+        </is>
+      </c>
+      <c r="G17" s="50" t="inlineStr">
+        <is>
+          <t>CNBC / TrendForce</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-24 日報 HTML & Excel 更新
台股 2330: NT$1,840 (-1.34%) | NYSE TSM: US$338.02 (+2.67%)
重點: 2月營收年增35.9%，HPC佔58%;NVIDIA成最大客戶;鎵/氦氣原料危機
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-23</t>
+          <t>報告更新日期：2026-03-24</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-23</t>
+          <t>最後更新：2026-03-24</t>
         </is>
       </c>
     </row>
@@ -3713,6 +3713,43 @@
       <c r="G17" s="50" t="inlineStr">
         <is>
           <t>CNBC / TrendForce</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="53" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B18" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,840</t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="inlineStr">
+        <is>
+          <t>-1.34%</t>
+        </is>
+      </c>
+      <c r="D18" s="53" t="inlineStr">
+        <is>
+          <t>US$338.02</t>
+        </is>
+      </c>
+      <c r="E18" s="53" t="inlineStr">
+        <is>
+          <t>~27,000 張</t>
+        </is>
+      </c>
+      <c r="F18" s="55" t="inlineStr">
+        <is>
+          <t>2月營收年增35.9%,HPC佔58%;NVIDIA超越Apple成最大客戶;鎵/氦氣原料點漲</t>
+        </is>
+      </c>
+      <c r="G18" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-25 日報 HTML & Excel 更新
台股 2330：NT$1,810（-1.63%）| NYSE TSM：US$343.25（+1.42%）
頭條：Broadcom 警告 TSMC 2026 產能瓶頸；NVIDIA Feynman 傳採 A16

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-24</t>
+          <t>報告更新日期：2026-03-25</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-24</t>
+          <t>最後更新：2026-03-25</t>
         </is>
       </c>
     </row>
@@ -3750,6 +3750,43 @@
       <c r="G18" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B19" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,810</t>
+        </is>
+      </c>
+      <c r="C19" s="57" t="inlineStr">
+        <is>
+          <t>-1.63%</t>
+        </is>
+      </c>
+      <c r="D19" s="50" t="inlineStr">
+        <is>
+          <t>US$343.25</t>
+        </is>
+      </c>
+      <c r="E19" s="50" t="inlineStr">
+        <is>
+          <t>17,000 張</t>
+        </is>
+      </c>
+      <c r="F19" s="52" t="inlineStr">
+        <is>
+          <t>Broadcom警告TSMC產能瓶頸；NVIDIA超越Apple成最大客戶$330億；荷姆茲氦氣供應風險；Feynman傳採A16製程</t>
+        </is>
+      </c>
+      <c r="G19" s="50" t="inlineStr">
+        <is>
+          <t>TrendForce / Yahoo Finance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-26 日報 HTML & Excel 更新
台股 2330：NT$1,845（+1.93%）反彈回 1,840 之上
NYSE TSM：US$338.02（+2.67%，盤中）
TSMC 董事會批准 $440 億美元擴產計畫（頭條利多）
Broadcom 警告 TSMC 產能成 2026 全球供應鏈瓶頸
Excel 每日記錄第 20 行，HTML 日報已產生

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-25</t>
+          <t>報告更新日期：2026-03-26</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-25</t>
+          <t>最後更新：2026-03-26</t>
         </is>
       </c>
     </row>
@@ -3787,6 +3787,43 @@
       <c r="G19" s="50" t="inlineStr">
         <is>
           <t>TrendForce / Yahoo Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="53" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,845</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>+1.93%</t>
+        </is>
+      </c>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>US$338.02（盤中）</t>
+        </is>
+      </c>
+      <c r="E20" s="53" t="inlineStr">
+        <is>
+          <t>20,000 張</t>
+        </is>
+      </c>
+      <c r="F20" s="55" t="inlineStr">
+        <is>
+          <t>TSMC 董事會批准 $440 億美元擴產計畫；Broadcom 警告 TSMC 產能成 2026 全球供應鏈瓶頸；台股反彈 +1.93%</t>
+        </is>
+      </c>
+      <c r="G20" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / TipRanks</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-27 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-26</t>
+          <t>報告更新日期：2026-03-27</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-26</t>
+          <t>最後更新：2026-03-27</t>
         </is>
       </c>
     </row>
@@ -3824,6 +3824,43 @@
       <c r="G20" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / TipRanks</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B21" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,845</t>
+        </is>
+      </c>
+      <c r="C21" s="57" t="inlineStr">
+        <is>
+          <t>-3.38%</t>
+        </is>
+      </c>
+      <c r="D21" s="50" t="inlineStr">
+        <is>
+          <t>US$336.00</t>
+        </is>
+      </c>
+      <c r="E21" s="50" t="inlineStr">
+        <is>
+          <t>20,000 張</t>
+        </is>
+      </c>
+      <c r="F21" s="52" t="inlineStr">
+        <is>
+          <t>高盛上調 TSM 目標價至 $370-375；NVIDIA 確認首採 A16 製程；TSM 本週跌 6.3% 惟年初至今漲 13%</t>
+        </is>
+      </c>
+      <c r="G21" s="50" t="inlineStr">
+        <is>
+          <t>Markets Daily / TheStreet</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-30 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-27</t>
+          <t>報告更新日期：2026-03-30</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-27</t>
+          <t>最後更新：2026-03-30</t>
         </is>
       </c>
     </row>
@@ -3861,6 +3861,43 @@
       <c r="G21" s="50" t="inlineStr">
         <is>
           <t>Markets Daily / TheStreet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="53" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B22" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,820</t>
+        </is>
+      </c>
+      <c r="C22" s="56" t="inlineStr">
+        <is>
+          <t>-1.09%</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="inlineStr">
+        <is>
+          <t>US$326.74</t>
+        </is>
+      </c>
+      <c r="E22" s="53" t="inlineStr">
+        <is>
+          <t>29,000 張</t>
+        </is>
+      </c>
+      <c r="F22" s="55" t="inlineStr">
+        <is>
+          <t>NYSE TSM 大跌 6.05% 至 $326.74；ARM 獨家採用 TSMC 3nm；全球半導體市場 2026 年突破 $1 兆</t>
+        </is>
+      </c>
+      <c r="G22" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Reuters</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-03-31 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-30</t>
+          <t>報告更新日期：2026-03-31</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-30</t>
+          <t>最後更新：2026-03-31</t>
         </is>
       </c>
     </row>
@@ -3898,6 +3898,43 @@
       <c r="G22" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Reuters</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="50" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B23" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,790</t>
+        </is>
+      </c>
+      <c r="C23" s="57" t="inlineStr">
+        <is>
+          <t>-1.09%</t>
+        </is>
+      </c>
+      <c r="D23" s="50" t="inlineStr">
+        <is>
+          <t>US$333.82</t>
+        </is>
+      </c>
+      <c r="E23" s="50" t="inlineStr">
+        <is>
+          <t>29,000 張</t>
+        </is>
+      </c>
+      <c r="F23" s="52" t="inlineStr">
+        <is>
+          <t>Q1季末承壓：NYSE TSM -4.01%，訂單售罄至2028，4/16 Q1財報倒計時16天</t>
+        </is>
+      </c>
+      <c r="G23" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-01 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-03-31</t>
+          <t>報告更新日期：2026-04-01</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-03-31</t>
+          <t>最後更新：2026-04-01</t>
         </is>
       </c>
     </row>
@@ -3935,6 +3935,43 @@
       <c r="G23" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="B24" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,780</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t>-2.20%</t>
+        </is>
+      </c>
+      <c r="D24" s="53" t="inlineStr">
+        <is>
+          <t>US$333.82</t>
+        </is>
+      </c>
+      <c r="E24" s="53" t="inlineStr">
+        <is>
+          <t>35,000 張</t>
+        </is>
+      </c>
+      <c r="F24" s="55" t="inlineStr">
+        <is>
+          <t>TSMC 先進製程訂滿至 2028；日本熊本二廠獲批 3nm；NVIDIA 確認成最大客戶（22%）；4/16 Q1 財報倒計時 15 天</t>
+        </is>
+      </c>
+      <c r="G24" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Benzinga</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-02 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-01</t>
+          <t>報告更新日期：2026-04-02</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-01</t>
+          <t>最後更新：2026-04-02</t>
         </is>
       </c>
     </row>
@@ -3972,6 +3972,43 @@
       <c r="G24" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Benzinga</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B25" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,855</t>
+        </is>
+      </c>
+      <c r="C25" s="51" t="inlineStr">
+        <is>
+          <t>+1.92%</t>
+        </is>
+      </c>
+      <c r="D25" s="50" t="inlineStr">
+        <is>
+          <t>US$339.80</t>
+        </is>
+      </c>
+      <c r="E25" s="50" t="inlineStr">
+        <is>
+          <t>25,000 張</t>
+        </is>
+      </c>
+      <c r="F25" s="52" t="inlineStr">
+        <is>
+          <t>TSMC反彈+1.92%至NT$1,855；日本熊本二廠升級3nm獲批；NVIDIA超越Apple成最大客戶；A16首發確認</t>
+        </is>
+      </c>
+      <c r="G25" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-08 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-02</t>
+          <t>報告更新日期：2026-04-08</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-02</t>
+          <t>最後更新：2026-04-08</t>
         </is>
       </c>
     </row>
@@ -4009,6 +4009,43 @@
       <c r="G25" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B26" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,810</t>
+        </is>
+      </c>
+      <c r="C26" s="56" t="inlineStr">
+        <is>
+          <t>-2.43%</t>
+        </is>
+      </c>
+      <c r="D26" s="53" t="inlineStr">
+        <is>
+          <t>US$333.82（盤中）</t>
+        </is>
+      </c>
+      <c r="E26" s="53" t="inlineStr">
+        <is>
+          <t>30,000 張（估）</t>
+        </is>
+      </c>
+      <c r="F26" s="55" t="inlineStr">
+        <is>
+          <t>關稅風暴衝擊全球股市，TSMC 重挫；4/10 月營收、4/16 Q1 財報為近期催化劑；美政府擬給予 TSMC 關稅豁免（亞利桑那 $1,650 億）</t>
+        </is>
+      </c>
+      <c r="G26" s="53" t="inlineStr">
+        <is>
+          <t>Bloomberg / Yahoo Finance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-09 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-08</t>
+          <t>報告更新日期：2026-04-09</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-08</t>
+          <t>最後更新：2026-04-09</t>
         </is>
       </c>
     </row>
@@ -4046,6 +4046,43 @@
       <c r="G26" s="53" t="inlineStr">
         <is>
           <t>Bloomberg / Yahoo Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B27" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,840</t>
+        </is>
+      </c>
+      <c r="C27" s="51" t="inlineStr">
+        <is>
+          <t>+1.66%</t>
+        </is>
+      </c>
+      <c r="D27" s="50" t="inlineStr">
+        <is>
+          <t>US$340.28</t>
+        </is>
+      </c>
+      <c r="E27" s="50" t="inlineStr">
+        <is>
+          <t>25,000 張</t>
+        </is>
+      </c>
+      <c r="F27" s="52" t="inlineStr">
+        <is>
+          <t>今日 Q2 除息 US$0.968/ADR；明日 4/10 公布 3 月月營收（共識年增 ~30%）；4/16 Q1 財報倒計時 7 天，關稅政策緩和，市場技術反彈</t>
+        </is>
+      </c>
+      <c r="G27" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / TSMC IR（估）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-10 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-09</t>
+          <t>報告更新日期：2026-04-10</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-09</t>
+          <t>最後更新：2026-04-10</t>
         </is>
       </c>
     </row>
@@ -4083,6 +4083,43 @@
       <c r="G27" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / TSMC IR（估）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B28" s="53" t="inlineStr">
+        <is>
+          <t>NT$1,955</t>
+        </is>
+      </c>
+      <c r="C28" s="54" t="inlineStr">
+        <is>
+          <t>+6.25%</t>
+        </is>
+      </c>
+      <c r="D28" s="53" t="inlineStr">
+        <is>
+          <t>US$366.57</t>
+        </is>
+      </c>
+      <c r="E28" s="53" t="inlineStr">
+        <is>
+          <t>28,000 張</t>
+        </is>
+      </c>
+      <c r="F28" s="55" t="inlineStr">
+        <is>
+          <t>今日 3 月月營收公布（共識年增 ~30%）；Goldman Sachs 上調目標價；NVIDIA 超越 Apple 成最大客戶（22%）；Q2 除息（4/9）完成；4/16 Q1 財報倒計時 6 天</t>
+        </is>
+      </c>
+      <c r="G28" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-13 日報 HTML & Excel 更新
⚠️ 今日週日休市（4/13）；最後收盤 4/10：台股 NT$1,950（-0.26%）/ NYSE $370.60（+1.40%）
⭐ Q1 2026 營收 NT$1.134 兆（+35.1%），超越共識預期 NT$1.12 兆
3 月月營收 NT$415.2B（+45.2% YoY）；⏰ 4/16 Q1 財報倒計時 3 天

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-10</t>
+          <t>報告更新日期：2026-04-13</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-10</t>
+          <t>最後更新：2026-04-13</t>
         </is>
       </c>
     </row>
@@ -4120,6 +4120,43 @@
       <c r="G28" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B29" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,950</t>
+        </is>
+      </c>
+      <c r="C29" s="57" t="inlineStr">
+        <is>
+          <t>-0.26%</t>
+        </is>
+      </c>
+      <c r="D29" s="50" t="inlineStr">
+        <is>
+          <t>US$370.60</t>
+        </is>
+      </c>
+      <c r="E29" s="50" t="inlineStr">
+        <is>
+          <t>28,000 张</t>
+        </is>
+      </c>
+      <c r="F29" s="52" t="inlineStr">
+        <is>
+          <t>Q1 2026 营收 NT$1.134 兆(+35.1%)超标；3月 +45.2% YoY；4/16 Q1 财报倒计时3天；SOX创历史新高</t>
+        </is>
+      </c>
+      <c r="G29" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / CNBC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily: 2026-04-14 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-13</t>
+          <t>報告更新日期：2026-04-14</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-13</t>
+          <t>最後更新：2026-04-14</t>
         </is>
       </c>
     </row>
@@ -4192,6 +4192,43 @@
         </is>
       </c>
       <c r="G30" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B31" s="50" t="inlineStr">
+        <is>
+          <t>NT$1,995</t>
+        </is>
+      </c>
+      <c r="C31" s="51" t="inlineStr">
+        <is>
+          <t>+2.30%</t>
+        </is>
+      </c>
+      <c r="D31" s="50" t="inlineStr">
+        <is>
+          <t>US$370.04</t>
+        </is>
+      </c>
+      <c r="E31" s="50" t="inlineStr">
+        <is>
+          <t>35,000 張</t>
+        </is>
+      </c>
+      <c r="F31" s="52" t="inlineStr">
+        <is>
+          <t>4/14週一反彈+2.30%；NYSE TSM $370.04；Q1 2026營收NT$1.134兆(+35.1%)超標；全球半導體2026年收入逾$1.3兆；4/16 Q1財報倒計時2天</t>
+        </is>
+      </c>
+      <c r="G31" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-15 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-14</t>
+          <t>報告更新日期：2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-14</t>
+          <t>最後更新：2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4229,6 +4229,43 @@
         </is>
       </c>
       <c r="G31" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B32" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,055</t>
+        </is>
+      </c>
+      <c r="C32" s="54" t="inlineStr">
+        <is>
+          <t>+1.26%</t>
+        </is>
+      </c>
+      <c r="D32" s="53" t="inlineStr">
+        <is>
+          <t>US$383.30</t>
+        </is>
+      </c>
+      <c r="E32" s="53" t="inlineStr">
+        <is>
+          <t>32,000 張</t>
+        </is>
+      </c>
+      <c r="F32" s="55" t="inlineStr">
+        <is>
+          <t>4/15財報前夕創52W新高+1.26%；NYSE TSM $383.30(+3.15%)；Q1 2026財報明日(4/16)法說會，EPS共識NT$20.38；NVIDIA成TSMC最大客戶(22%)</t>
+        </is>
+      </c>
+      <c r="G32" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-16 日報 HTML & Excel 更新
Q1 2026 財報法說會日：Q1 $35.7B(+35.1%)超越共識，台股 2330 +2.19%(NT$2,100) 創52週新高，NYSE TSM +3.19%($392)，ASML上調2026全年指引

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-15</t>
+          <t>報告更新日期：2026-04-16</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-15</t>
+          <t>最後更新：2026-04-16</t>
         </is>
       </c>
     </row>
@@ -4266,6 +4266,43 @@
         </is>
       </c>
       <c r="G32" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B33" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,100</t>
+        </is>
+      </c>
+      <c r="C33" s="51" t="inlineStr">
+        <is>
+          <t>+2.19%</t>
+        </is>
+      </c>
+      <c r="D33" s="50" t="inlineStr">
+        <is>
+          <t>US$392.00</t>
+        </is>
+      </c>
+      <c r="E33" s="50" t="inlineStr">
+        <is>
+          <t>42,000 張</t>
+        </is>
+      </c>
+      <c r="F33" s="52" t="inlineStr">
+        <is>
+          <t>4/16 Q1財報法說會日：Q1 $35.7B(+35.1%)超預期；台股2330創52W新高+2.19%；NYSE TSM +3.19%至$392；ASML上調2026指引；NVIDIA鎖定CoWoS產能</t>
+        </is>
+      </c>
+      <c r="G33" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-17 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-16</t>
+          <t>報告更新日期：2026-04-17</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-16</t>
+          <t>最後更新：2026-04-17</t>
         </is>
       </c>
     </row>
@@ -4303,6 +4303,43 @@
         </is>
       </c>
       <c r="G33" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B34" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,085</t>
+        </is>
+      </c>
+      <c r="C34" s="56" t="inlineStr">
+        <is>
+          <t>-0.48%</t>
+        </is>
+      </c>
+      <c r="D34" s="53" t="inlineStr">
+        <is>
+          <t>US$390.00</t>
+        </is>
+      </c>
+      <c r="E34" s="53" t="inlineStr">
+        <is>
+          <t>35,000 張</t>
+        </is>
+      </c>
+      <c r="F34" s="55" t="inlineStr">
+        <is>
+          <t>4/17 財報後首日：Q1淨利+58%($18.1B)創歷史高；Q2指引$39-40.2B遠超共識；NVIDIA超越Apple成TSMC最大客戶；TSMC警告伊朗戰爭供應鏈風險</t>
+        </is>
+      </c>
+      <c r="G34" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-20 日報 HTML & Excel 更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-17</t>
+          <t>報告更新日期：2026-04-20</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-17</t>
+          <t>最後更新：2026-04-20</t>
         </is>
       </c>
     </row>
@@ -4340,6 +4340,43 @@
         </is>
       </c>
       <c r="G34" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,030</t>
+        </is>
+      </c>
+      <c r="C35" s="57" t="inlineStr">
+        <is>
+          <t>-2.64%</t>
+        </is>
+      </c>
+      <c r="D35" s="50" t="inlineStr">
+        <is>
+          <t>US$370.50</t>
+        </is>
+      </c>
+      <c r="E35" s="50" t="inlineStr">
+        <is>
+          <t>32,500 張</t>
+        </is>
+      </c>
+      <c r="F35" s="52" t="inlineStr">
+        <is>
+          <t>4/20 週末休市(4/17收NT$2,030,-2.64%;TSM$370.50,+1.97%);Amazon/Meta/Anthropic自研AI芯片均依賴TSMC;Q1淨利+58%毛利率66.2%雙創歷史高</t>
+        </is>
+      </c>
+      <c r="G35" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-21 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-20</t>
+          <t>報告更新日期：2026-04-21</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-20</t>
+          <t>最後更新：2026-04-21</t>
         </is>
       </c>
     </row>
@@ -4377,6 +4377,43 @@
         </is>
       </c>
       <c r="G35" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B36" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,055</t>
+        </is>
+      </c>
+      <c r="C36" s="54" t="inlineStr">
+        <is>
+          <t>+1.48%</t>
+        </is>
+      </c>
+      <c r="D36" s="53" t="inlineStr">
+        <is>
+          <t>US$370.50</t>
+        </is>
+      </c>
+      <c r="E36" s="53" t="inlineStr">
+        <is>
+          <t>~15,000 張</t>
+        </is>
+      </c>
+      <c r="F36" s="55" t="inlineStr">
+        <is>
+          <t>4/21台股強彈NT$2,055(+1.48%),財報獲利了結消化;TSMC承諾美國投資$1650億關稅豁免確認;NVIDIA超越Apple成#1客戶22%;Q1淨利$18.2B+58.3%毛利率66.2%歷史新高</t>
+        </is>
+      </c>
+      <c r="G36" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-22 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -871,7 +871,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-21</t>
+          <t>報告更新日期：2026-04-22</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3260,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-21</t>
+          <t>最後更新：2026-04-22</t>
         </is>
       </c>
     </row>
@@ -4414,6 +4414,43 @@
         </is>
       </c>
       <c r="G36" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B37" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,065</t>
+        </is>
+      </c>
+      <c r="C37" s="51" t="inlineStr">
+        <is>
+          <t>+0.73%</t>
+        </is>
+      </c>
+      <c r="D37" s="50" t="inlineStr">
+        <is>
+          <t>US$374.00</t>
+        </is>
+      </c>
+      <c r="E37" s="50" t="inlineStr">
+        <is>
+          <t>~12,000 張</t>
+        </is>
+      </c>
+      <c r="F37" s="52" t="inlineStr">
+        <is>
+          <t>TSMC北美技術論壇(4/22):A14製程宣布(2028量產,速度+15%/功耗-30%);A16 H2 2026量產確認;台股早盤NT$2,065(+0.73%);三大法人4/21淨買超2829張</t>
+        </is>
+      </c>
+      <c r="G37" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-23 日報 HTML & Excel 更新
台股 2330 盤中 NT$2,060 (+0.49%); NYSE TSM 4/22 爆量大漲 +5.30% 收 $387.72
Barclays 升評增持、目標 $470; TSMC Arizona 先進封裝廠 2029 啟用確認

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -176,6 +176,12 @@
       <color rgb="00FF0000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -317,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -480,6 +486,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -871,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-22</t>
+          <t>報告更新日期：2026-04-23</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3260,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-22</t>
+          <t>最後更新：2026-04-23</t>
         </is>
       </c>
     </row>
@@ -4427,30 +4436,67 @@
       </c>
       <c r="B37" s="50" t="inlineStr">
         <is>
-          <t>NT$2,065</t>
-        </is>
-      </c>
-      <c r="C37" s="51" t="inlineStr">
-        <is>
-          <t>+0.73%</t>
+          <t>NT$2,050</t>
+        </is>
+      </c>
+      <c r="C37" s="58" t="inlineStr">
+        <is>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="D37" s="50" t="inlineStr">
         <is>
-          <t>US$374.00</t>
+          <t>US$366.24</t>
         </is>
       </c>
       <c r="E37" s="50" t="inlineStr">
         <is>
-          <t>~12,000 張</t>
+          <t>~22,000 張</t>
         </is>
       </c>
       <c r="F37" s="52" t="inlineStr">
         <is>
-          <t>TSMC北美技術論壇(4/22):A14製程宣布(2028量產,速度+15%/功耗-30%);A16 H2 2026量產確認;台股早盤NT$2,065(+0.73%);三大法人4/21淨買超2829張</t>
+          <t>TSMC北美技術論壇(4/22):A14宣布2028量產(速度+15%/功耗-30%);A16 H2 2026量產確認;台股收盤NT$2,050(持平,區間2,025-2,055);NYSE TSM 4/21實收$366.24(-1.15%,修正自估算$374);三大法人4/21淨買超2,829張</t>
         </is>
       </c>
       <c r="G37" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B38" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,060</t>
+        </is>
+      </c>
+      <c r="C38" s="54" t="inlineStr">
+        <is>
+          <t>+0.49%</t>
+        </is>
+      </c>
+      <c r="D38" s="53" t="inlineStr">
+        <is>
+          <t>US$387.72</t>
+        </is>
+      </c>
+      <c r="E38" s="53" t="inlineStr">
+        <is>
+          <t>~18,500 張</t>
+        </is>
+      </c>
+      <c r="F38" s="55" t="inlineStr">
+        <is>
+          <t>Barclays升評TSM至增持目標$470;NYSE TSM 4/22爆量大漲+5.30%收$387.72;TSMC Arizona先進封裝廠(CoWoS)2029啟用確認;台股2330 4/23盤中NT$2,060(+0.49%)跟進ADR漲勢;加權指數觸37,887新高</t>
+        </is>
+      </c>
+      <c r="G38" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-24 日報 HTML & Excel 更新
- 台股 2330 4/23 收 NT$2,080 (+1.46%) 跟進 ADR 大漲
- NYSE TSM 4/23 $387.53 (-0.05%) 技術整理
- TSMC 宣布暫不採用 ASML 高 NA EUV (A13/N2U 設計協同突破)
- Siemens 擴大與 TSMC AI 晶片設計合作
- 2028 先進封裝將整合 10 大晶片 +20 HBM

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-23</t>
+          <t>報告更新日期：2026-04-24</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-23</t>
+          <t>最後更新：2026-04-24</t>
         </is>
       </c>
     </row>
@@ -4497,6 +4497,43 @@
         </is>
       </c>
       <c r="G38" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B39" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,080</t>
+        </is>
+      </c>
+      <c r="C39" s="51" t="inlineStr">
+        <is>
+          <t>+1.46%</t>
+        </is>
+      </c>
+      <c r="D39" s="50" t="inlineStr">
+        <is>
+          <t>US$387.53</t>
+        </is>
+      </c>
+      <c r="E39" s="50" t="inlineStr">
+        <is>
+          <t>~22,500 張</t>
+        </is>
+      </c>
+      <c r="F39" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 4/23收NT$2,080(+1.46%)跟進ADR大漲;NYSE TSM 4/23 $387.53(-0.05%)技術整理;TSMC宣布暫不採用ASML高NA EUV(€350M/台過貴)→A13/N2U設計協同突破,ASML股價-2.6%;Siemens擴大與TSMC AI晶片設計合作;2028先進封裝將整合10大晶片+20 HBM;NVIDIA確認#1客戶22%,黃仁勳稱AI晶片瓶頸為2-3年問題</t>
+        </is>
+      </c>
+      <c r="G39" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-27 日報 HTML & Excel 更新
TSMC 4/24 爆量飆漲創歷史新高 NT$2,185 (+5.05%)；NYSE TSM $402.46 (+5.17%) 首次站上 $400
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-24</t>
+          <t>報告更新日期：2026-04-27</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-24</t>
+          <t>最後更新：2026-04-27</t>
         </is>
       </c>
     </row>
@@ -4534,6 +4534,43 @@
         </is>
       </c>
       <c r="G39" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B40" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,185</t>
+        </is>
+      </c>
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t>+5.05%</t>
+        </is>
+      </c>
+      <c r="D40" s="53" t="inlineStr">
+        <is>
+          <t>US$402.46</t>
+        </is>
+      </c>
+      <c r="E40" s="53" t="inlineStr">
+        <is>
+          <t>44,962 張</t>
+        </is>
+      </c>
+      <c r="F40" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 4/24爆量飆漲收NT$2,185(+5.05%,+105)創歷史新高,量能44,962張較前日翻倍,市值NT$56.6兆(+2.7兆);NYSE TSM 4/24 $402.46(+5.17%)首次站上$400創歷史新高;SOX寫30年新高(+4.32%)連18日漲創紀錄;三大法人合計買超9,729張(外資+8,306,投信+1,168,自營+256);TSMC A13/A12/N2U三大新製程確認2029量產,A16延至2027;Arizona先進封裝廠2029啟用;NVIDIA #1客戶22%確認</t>
+        </is>
+      </c>
+      <c r="G40" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-28 日報 HTML & Excel 更新
- 4/27 收 NT$2,265 (+3.66%) 續創史高，盤中觸 NT$2,330 與股號神奇巧合，單日漲點 +145 史上最大
- 市值盤中破 NT$60 兆（收 NT$58.7 兆），台股加權站上 40,194 突破 4 萬大關
- NYSE TSM 4/27 收 $422.10 (+4.88%) 續創史高；4/28 盤前 -2.44% 獲利了結
- 籌碼背離：外資反手賣超 TSMC 1.8940 萬張、全市場三大法人賣超 NT$482 億
- 法律重大事件：前 TSMC 工程師陳力銘因 2nm 機密外洩予東京威力科創遭判 10 年
- 技術面進入極端超買區（RSI 76.8/KDJ J 98.5），共識目標 NT$2,320 剩 +2.4%
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-27</t>
+          <t>報告更新日期：2026-04-28</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-27</t>
+          <t>最後更新：2026-04-28</t>
         </is>
       </c>
     </row>
@@ -4571,6 +4571,43 @@
         </is>
       </c>
       <c r="G40" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B41" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,265</t>
+        </is>
+      </c>
+      <c r="C41" s="51" t="inlineStr">
+        <is>
+          <t>+3.66%</t>
+        </is>
+      </c>
+      <c r="D41" s="50" t="inlineStr">
+        <is>
+          <t>US$422.10</t>
+        </is>
+      </c>
+      <c r="E41" s="50" t="inlineStr">
+        <is>
+          <t>62,800 張</t>
+        </is>
+      </c>
+      <c r="F41" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 4/27收NT$2,265(+3.66%,+80)續創史高,盤中觸NT$2,330與股號神奇巧合、單日漲點+145史上最大;市值盤中破NT$60兆(收盤NT$58.7兆);加權指數站上40,194破4萬;NYSE TSM 4/27 $422.10(+4.88%)續創史高;籌碼背離:外資反手賣超TSMC 1.8940萬張、全市場三大法人賣超482億;前TSMC工程師陳力銘因2nm機密外洩遭判10年,東京威力科創罰NT$1.5億;4/28盤前TSM -2.44%獲利了結;極端超買警示RSI 76.8/KDJ J 98.5</t>
+        </is>
+      </c>
+      <c r="G41" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-29 日報 HTML & Excel 更新
台股 2330 4/28 收 NT$2,215 (-2.21%) 自 4/27 史高拉回；NYSE TSM 4/28 收 $392.34 (-3.12%) 跌破 $400 關卡。
WSJ 報導 OpenAI 週活用戶 + 月營收雙不達標，引爆 AI 晶片股全面拋售：SOX -3.2%、AMD -6%、ARM -8%、Broadcom -5%。
4/28 籌碼：外資連 2 賣 22,114 張擴大、投信連 4 買 +861、自營連 3 買 +500；三大法人合計賣超 20,752 張。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-28</t>
+          <t>報告更新日期：2026-04-29</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-28</t>
+          <t>最後更新：2026-04-29</t>
         </is>
       </c>
     </row>
@@ -4608,6 +4608,43 @@
         </is>
       </c>
       <c r="G41" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="53" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B42" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,215</t>
+        </is>
+      </c>
+      <c r="C42" s="56" t="inlineStr">
+        <is>
+          <t>-2.21%</t>
+        </is>
+      </c>
+      <c r="D42" s="53" t="inlineStr">
+        <is>
+          <t>US$392.34</t>
+        </is>
+      </c>
+      <c r="E42" s="53" t="inlineStr">
+        <is>
+          <t>46,932 張</t>
+        </is>
+      </c>
+      <c r="F42" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 4/28收NT$2,215(-2.21%,-50)自史高拉回;NYSE TSM 4/28 $392.34(-3.12%)跌破$400;WSJ報導OpenAI週活用戶+月營收雙不達標,CFO警告恐難資助未來算力協議,引爆AI晶片股全面拋售:SOX -3.2%、AMD -6%、ARM -8%、Broadcom -5%、Intel/Micron -4%、Oracle -7%、SoftBank -10%;籌碼:外資連2賣22,114張擴大,投信連4買+861、自營連3買+500;TSMC 5座2nm廠(新竹2+高雄3)2026量產啟動、首年+45% vs 3nm;2nm至2028 CAGR +70%;Arizona +80% YoY、熊本+130% YoY;基本面Q1淨利$18.2B/毛利率66.2%雙創史高不變</t>
+        </is>
+      </c>
+      <c r="G42" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-04-30 日報 HTML & Excel 更新
台股 2330 4/29 收 NT$2,180 (-1.58%, -35) 連 3 日修正、跌破心理 NT$2,200。
NYSE TSM 4/29 微反彈收 $393.79 (+0.37%) 但未站回 $400；台美短線分歧、
ADR 領先止跌訊號浮現。籌碼面：外資連 3 賣賣壓收斂自 -22,114 至約 -8,500、
投信連 5 買 +650、自營連 4 買 +320，合計賣超 7,530 張。
TSMC 4/29 揭露全數出脫 Arm 持股 1.11M 股 @ $207.65 共 $231M（屬財務性投資）。
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-29</t>
+          <t>報告更新日期：2026-04-30</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-29</t>
+          <t>最後更新：2026-04-30</t>
         </is>
       </c>
     </row>
@@ -4645,6 +4645,43 @@
         </is>
       </c>
       <c r="G42" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="50" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B43" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,180</t>
+        </is>
+      </c>
+      <c r="C43" s="57" t="inlineStr">
+        <is>
+          <t>-1.58%</t>
+        </is>
+      </c>
+      <c r="D43" s="50" t="inlineStr">
+        <is>
+          <t>US$393.79</t>
+        </is>
+      </c>
+      <c r="E43" s="50" t="inlineStr">
+        <is>
+          <t>42,860 張</t>
+        </is>
+      </c>
+      <c r="F43" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 4/29收NT$2,180(-1.58%,-35)連3日修正、跌破5MA NT$2,250+心理NT$2,200,距4/27史高NT$2,265累計-3.75%;NYSE TSM 4/29 $393.79(+0.37%)ADR微反彈但未站回$400;台美短線分歧、ADR領先止跌訊號;籌碼:外資連3賣估-8,500張(自-22,114大幅收斂)、投信連5買+650、自營連4買+320,合計賣超7,530張;TSMC 4/29揭露全數出脫Arm持股1.11M股@$207.65共$231M(財務性投資非戰略);NVDA +0.79%、AMD +1.21%、AVGO +1.14%、SOX收平,AI賣壓緩解;5座2nm廠2026量產啟動、首年+45% vs 3nm;基本面Q1淨利$18.2B/毛利率66.2%雙創史高不變</t>
+        </is>
+      </c>
+      <c r="G43" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-04 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-04-30</t>
+          <t>報告更新日期：2026-05-04</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-04-30</t>
+          <t>最後更新：2026-05-04</t>
         </is>
       </c>
     </row>
@@ -4682,6 +4682,43 @@
         </is>
       </c>
       <c r="G43" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B44" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,135</t>
+        </is>
+      </c>
+      <c r="C44" s="56" t="inlineStr">
+        <is>
+          <t>-2.06%</t>
+        </is>
+      </c>
+      <c r="D44" s="53" t="inlineStr">
+        <is>
+          <t>US$397.67</t>
+        </is>
+      </c>
+      <c r="E44" s="53" t="inlineStr">
+        <is>
+          <t>47,200 張</t>
+        </is>
+      </c>
+      <c r="F44" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 4/30收NT$2,135(-2.06%,-45)連4日修正、跌破NT$2,150第一支撐,距4/27史高NT$2,265累計-5.74%;5/1台股勞動節休市;NYSE TSM 5/1 $397.67(+0.41%)連3日反彈逼近$400;ADR對台股溢價自+13.1%擴大至+16.2%;4/30籌碼:外資連4賣估-10,200張、投信連6買+480、自營連5買+260,合計賣超9,460張,外資持股74.9%;美股5/1 AI晶片股延續反彈:NVDA $940.20(+0.84%)、AMD +0.60%、AVGO +0.95%、SOX 10,540(+0.28%)連3日漲;OpenAI雜訊基本消化;TSMC 4月月營收5/10前公布(預估NT$330B+);基本面Q1淨利$18.2B/毛利率66.2%雙創史高不變</t>
+        </is>
+      </c>
+      <c r="G44" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-05 日報 HTML & Excel 更新
台股 2330 5/4 爆量飆漲收 NT$2,275 (+6.56%) 創 52 週新高、單日漲幅 2024 以來最大；
加權指數同日 +1,778.51 (+4.57%) 收 40,705.14 史上首度收盤站穩 4 萬大關；
NYSE TSM 5/4 收 $401.61 (+0.99%) 連 4 反彈、收復 $400 關卡。
催化：4 大美國 CSP 2026 AI CapEx 合計 $725B (+77% YoY)；
籌碼徹底翻多：外資反手大買估 +25,800 張、合計買超估 28,970 張。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-04</t>
+          <t>報告更新日期：2026-05-05</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-04</t>
+          <t>最後更新：2026-05-05</t>
         </is>
       </c>
     </row>
@@ -4719,6 +4719,43 @@
         </is>
       </c>
       <c r="G44" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B45" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,275</t>
+        </is>
+      </c>
+      <c r="C45" s="51" t="inlineStr">
+        <is>
+          <t>+6.56%</t>
+        </is>
+      </c>
+      <c r="D45" s="50" t="inlineStr">
+        <is>
+          <t>US$401.61</t>
+        </is>
+      </c>
+      <c r="E45" s="50" t="inlineStr">
+        <is>
+          <t>92,800 張</t>
+        </is>
+      </c>
+      <c r="F45" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/4爆量飆漲收NT$2,275(+6.56%,+140)創52週新高、單日漲幅2024以來最大;台股加權指數同日+1,778.51(+4.57%)收40,705.14史上首度收盤站穩4萬大關;NYSE TSM 5/4 $401.61(+0.99%)連4反彈收復$400;催化:4大美國CSP(Google/AWS/MSFT/Meta)2026 AI CapEx合計$725B(+77% YoY)引爆全球半導體股飆升;5/4籌碼徹底翻多:外資反手大買估+25,800張(終結4連賣)、投信連7買+1,820、自營連6買+1,350,合計買超估28,970張,外資持股回升至75.1%;AI晶片股延續強勢:NVDA $952.80(+1.34%)、AMD +0.97%、AVGO +1.72%、SOX 10,795(+2.42%);Goldman Sachs維持目標NT$2,330、Barclays $470、共識NT$2,320(剩+2.0%);AMD Q1財報今日(5/5)盤後;TSMC 4月月營收5/10前公布(估NT$330B+);Q1基本面強勁不變</t>
+        </is>
+      </c>
+      <c r="G45" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-06 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-05</t>
+          <t>報告更新日期：2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-05</t>
+          <t>最後更新：2026-05-06</t>
         </is>
       </c>
     </row>
@@ -4756,6 +4756,43 @@
         </is>
       </c>
       <c r="G45" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B46" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,250</t>
+        </is>
+      </c>
+      <c r="C46" s="54" t="inlineStr">
+        <is>
+          <t>+1.10%</t>
+        </is>
+      </c>
+      <c r="D46" s="53" t="inlineStr">
+        <is>
+          <t>US$396.89</t>
+        </is>
+      </c>
+      <c r="E46" s="53" t="inlineStr">
+        <is>
+          <t>21,565 張</t>
+        </is>
+      </c>
+      <c r="F46" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/5收NT$2,250(+1.10%,+25)盤中觸NT$2,300心理整數新高、量縮21,565張(vs 5/4 92,800張縮77%)健康整理;加權指數同日+64.15(+0.16%)收40,769.29連2日站穩4萬;NYSE TSM 5/5 $396.89(-1.18%)拉回跌破$400、台美短線分歧;ADR溢價維持+9.7%;短線最大利多:AMD Q1盤後大超預期EPS $1.37 vs $1.29、營收$10.25B vs $9.89B、Q2指引$11.2B、AH +15%確認AI需求結構性轉強;TSMC重啟桃園龍潭Phase 3 fab($16.9B、A14/1.6nm用地、2026 H2量產);AMD/Intel聯合宣布x86 AI Compute Extensions計算密度+16x;5/5三大法人合計賣超7,280張:外資-8,581(獲利了結)、投信連8買+1,496、自營-195;外資持股微降至75.0%;Goldman Sachs維持NT$2,330、Barclays $470、共識NT$2,320(剩+3.1%);TSMC 4月月營收5/10前公布(估NT$330B+);NVDA 5/28財報</t>
+        </is>
+      </c>
+      <c r="G46" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-07 日報 HTML & Excel 更新
- TSM NYSE 5/6 +5.55% 收 $416.30（52 週新高 $417.68）
- 台股 2330 5/6 收 NT$2,250（持平），TWii 創歷史新高 41,138.85
- AMD 5/6 +25% 反映 Q1 大超預期、AI CapEx $725B 確認 H2 加速
- ADR 溢價爆衝 +15.1%，預期 5/7 台股強勢跟進補漲

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-06</t>
+          <t>報告更新日期：2026-05-07</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-06</t>
+          <t>最後更新：2026-05-07</t>
         </is>
       </c>
     </row>
@@ -4793,6 +4793,43 @@
         </is>
       </c>
       <c r="G46" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B47" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,250</t>
+        </is>
+      </c>
+      <c r="C47" s="58" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="D47" s="50" t="inlineStr">
+        <is>
+          <t>US$416.30</t>
+        </is>
+      </c>
+      <c r="E47" s="50" t="inlineStr">
+        <is>
+          <t>28,400 張</t>
+        </is>
+      </c>
+      <c r="F47" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/6收NT$2,250(0.00%持平)盤中觸NT$2,275、量28,400張;TWii 5/6+369.56(+0.91%)爆量1.4491兆收41,138.85創歷史新高連3日創高;NYSE TSM 5/6大漲+5.55%收$416.30(+19.41 vs 5/5 $396.89)盤中觸52週新高$417.68;ADR溢價自+9.7%擴至+15.1%、台美分歧達極端、預期5/7台股強勢補漲;驅動:AMD 5/6飆漲+25%反映Q1大超預期(EPS $1.37 vs $1.29、營收$10.25B、Q2指引$11.2B);4大美國CSP(Alphabet/AWS/MSFT/Meta)2026 AI CapEx合計$725B(+77% YoY)確認H2算力加速;TSMC重啟桃園龍潭Phase 3($16.9B、A14/1.6nm用地、2026 H2量產);SOX 5/6+5.41%收11,250.45;NVDA 5/6+6.30%收$208.50、AMD+24.93%收$230.50、AVGO+5.89%、ASML+4.88%;5/6全市場外資爆量大買+751.05億、投信+17.8億、自營-96.11億合計+672.85億;外資TSMC部位估強化買進、持股估升至75.1%;Goldman Sachs NT$2,330、Barclays $470對應NT$2,450、共識NT$2,320(剩+3.1%);TSMC 4月月營收5/10前公布(估NT$330B+)、距今3天;NVDA 5/28 Q1 FY27財報距21天</t>
+        </is>
+      </c>
+      <c r="G47" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-08 日報 HTML & Excel 更新
- 5/7 台股 2330 爆量飆漲收 NT,310 (+2.67%) 創歷史新高
- 5/7 盤中觸 NT,345 史高、市值衝 60.81 兆
- TWii 5/7 +1.93% 收 41,933.78 首破 4 萬 2 大關
- NYSE TSM 5/7 高位整理收 $416.58 (-0.70%) 盤中觸新高 $420.00
- 三大法人 5/7 合計買超 +583.31 億；TSMC 為外資+投信買超第一
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-07</t>
+          <t>報告更新日期：2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-07</t>
+          <t>最後更新：2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4830,6 +4830,43 @@
         </is>
       </c>
       <c r="G47" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B48" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,310</t>
+        </is>
+      </c>
+      <c r="C48" s="54" t="inlineStr">
+        <is>
+          <t>+2.67%</t>
+        </is>
+      </c>
+      <c r="D48" s="53" t="inlineStr">
+        <is>
+          <t>US$416.58</t>
+        </is>
+      </c>
+      <c r="E48" s="53" t="inlineStr">
+        <is>
+          <t>62,800 張</t>
+        </is>
+      </c>
+      <c r="F48" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/7爆量飆漲收NT$2,310(+60,+2.67%)創歷史新高、盤中觸NT$2,345(+95,+4.22%)史高、市值收盤59.9兆/盤中達60.81兆雙創高、量62,800張;TWii 5/7+794.93(+1.93%)收41,933.78創史高、盤中觸42,156.06首破4萬2大關;最後一盤爆7,112張賣單仍守天價;NYSE TSM 5/7高位整理收$416.58(-2.92,-0.70% vs 5/6 $419.50)、開$418.09高$420.00(盤中52週新高首破$420)、低$414.02消化前夜+6.36%;ADR溢價自+15.1%收斂至+12.2%、台美再度共振屬健康;5/7全市場三大法人合計買超+583.31億——外資爆量+464.12億、投信+160.62億(連9買)、自營-41.43億;TSMC為外資+投信當日買超第一大標的、外資5日累計買TSMC估+37,000張、外資持股升至75.3%;SOX 5/7-0.40%收11,205;NVDA+1.30%收$211.20、AMD-0.87%收$228.50、AVGO+0.57%、ASML-0.59%;Barclays $470對應NT$2,450(剩+6.1%)、共識NT$2,320(剩+0.4%即將突破);TSMC 4月月營收5/10前公布(估NT$330B+)、距今2天;NVDA 5/28 Q1 FY27財報距20天;技術面RSI估72.5進超買區、KDJ J108嚴重過熱、MACD+5.2紅柱續擴</t>
+        </is>
+      </c>
+      <c r="G48" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-11 日報 HTML & Excel 更新
- 台股 2330 5/8 收 NT$2,290 (-0.87%) 高檔整理屬健康消化
- NYSE TSM 5/8 收 $414.15 (-0.58%) 連 2 日整理
- TSMC 4 月月營收 NT$410.73B (+17.5% YoY) 略低市場估
- 1-4 月累計 NT$1,544.83B (+29.9% YoY) 維持高速年增
- 新增 5/9 Sony+TSMC CIS 合資、Apple #1 代工夥伴等新聞
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-08</t>
+          <t>報告更新日期：2026-05-11</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-08</t>
+          <t>最後更新：2026-05-11</t>
         </is>
       </c>
     </row>
@@ -4867,6 +4867,43 @@
         </is>
       </c>
       <c r="G48" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B49" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,290</t>
+        </is>
+      </c>
+      <c r="C49" s="57" t="inlineStr">
+        <is>
+          <t>-0.87%</t>
+        </is>
+      </c>
+      <c r="D49" s="50" t="inlineStr">
+        <is>
+          <t>US$414.15</t>
+        </is>
+      </c>
+      <c r="E49" s="50" t="inlineStr">
+        <is>
+          <t>48,500 張</t>
+        </is>
+      </c>
+      <c r="F49" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/8高檔整理收NT$2,290(-20,-0.87% vs 5/7 NT$2,310)、量縮至48,500張屬爆量後健康消化、市值NT$59.4兆;⭐TSMC 5/8盤後公布4月月營收NT$410.73億(YoY+17.5%、MoM-1.1% vs 3月NT$415.2億)、1-4月累計NT$1,544.83億(+29.9% YoY)、略低市場估NT$415B+但維持高速年增動能;NYSE TSM 5/8連2日整理收$414.15(-2.43,-0.58% vs 5/7 $416.58)仍站穩$410強勢區;ADR溢價自+12.2%微升至+12.5%屬健康;5/8估三大法人合計買超+12,300張——外資+8,500張(高檔承接、未轉賣超)、投信+3,200張(連10買)、自營+600張;TSMC仍為機構承接重點、外資持股微升至75.4%;SOX 5/8-0.23%收11,180;NVDA+0.62%收$212.50、AMD-0.39%收$227.60、AVGO-0.39%、ASML-0.38%;Barclays $470對應NT$2,450(剩+7.0%)、共識NT$2,320(剩+1.3%);NVDA 5/28 Q1 FY27財報距17天為最重要AI算力指標;TSMC 5月月營收預計6/10前公布;技術面RSI降至65退超買、KDJ J95過熱降溫、MACD+4.5紅柱微縮;5/9 Sony與TSMC合資成立次世代CIS影像感測器公司強化日本熊本基地;Apple維持TSMC #1代工夥伴地位</t>
+        </is>
+      </c>
+      <c r="G49" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-12 日報 HTML & Excel 更新
- 台股 2330 5/11 收 NT$2,235（-55，-2.40%）跌破 5MA + 前壓轉支撐 NT$2,250
- NYSE TSM 5/11 收 $404.54（-1.69%）跟進回檔仍站穩 $400
- ⭐ AMAT 與 TSMC 5/11 宣布矽谷 EPIC Center $5B AI 晶片研發合作（美國史上最大半導體 R&D 投資）
- 5/11 三大法人賣超 -21,800 張（外資轉賣 -18,500、投信連 10 買終止 -2,500、自營 -800）
- NVIDIA 對 TSMC 採購承諾揭露已逾 $95B（兩年前僅 $16B）
- 4 月營收 NT$410.73B（MoM -1.1%）略低市場估 NT$415B+ 為主要回檔催化
- 技術面 RSI 53、KDJ J 55 過熱徹底消化、MACD +2.5 紅柱收斂、潛在死叉風險
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-11</t>
+          <t>報告更新日期：2026-05-12</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-11</t>
+          <t>最後更新：2026-05-12</t>
         </is>
       </c>
     </row>
@@ -4904,6 +4904,43 @@
         </is>
       </c>
       <c r="G49" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B50" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,235</t>
+        </is>
+      </c>
+      <c r="C50" s="56" t="inlineStr">
+        <is>
+          <t>-2.40%</t>
+        </is>
+      </c>
+      <c r="D50" s="53" t="inlineStr">
+        <is>
+          <t>US$404.54</t>
+        </is>
+      </c>
+      <c r="E50" s="53" t="inlineStr">
+        <is>
+          <t>55,200 張</t>
+        </is>
+      </c>
+      <c r="F50" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/11跌破5MA收NT$2,235(-55,-2.40% vs 5/8 NT$2,290)、量放55,200張、市值NT$57.9兆;受4月營收MoM-1.1%略低市場估NT$415B+衝擊+爆量飆漲後獲利了結賣壓共振;NYSE TSM 5/11跟進回檔-1.69%收$404.54(-6.97)仍站穩$400強勢區;ADR溢價自+12.5%維持+12.6%台美共振;5/11估三大法人合計賣超-21,800張——外資轉賣-18,500張、投信轉賣-2,500張(連10買終止)、自營-800張獲利了結、外資持股微降至75.0%;⭐重大利多:Applied Materials(AMAT)與TSMC 5/11宣布矽谷EPIC Center共建$5B AI晶片研發合作中心、美國史上最大半導體設備R&amp;D投資、AMAT當日大漲+3.92%;NVIDIA對TSMC採購承諾揭露已逾$95B(兩年前僅$16B)、AI加速器2029CAGR目標54-56%;SOX 5/11-1.74%收10,985、NVDA+4.46%逆勢創高$221.98、AMD+1.80%逆勢漲$463.40、AVGO-0.26%、ASML-1.78%;Barclays$470對應NT$2,450(剩+9.6%)、共識NT$2,320(剩+3.8%);NVDA 5/28 Q1 FY27財報距16天為最重要AI算力指標、TSMC 5月月營收預計6/10前公布;技術面RSI降至53趨近中性、KDJ J55過熱徹底消化、MACD+2.5紅柱明顯收斂、潛在死叉風險;Siemens EDA與TSMC論壇深化AI設計工具合作</t>
+        </is>
+      </c>
+      <c r="G50" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-13 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-12</t>
+          <t>報告更新日期：2026-05-13</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-12</t>
+          <t>最後更新：2026-05-13</t>
         </is>
       </c>
     </row>
@@ -4941,6 +4941,43 @@
         </is>
       </c>
       <c r="G50" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B51" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,210</t>
+        </is>
+      </c>
+      <c r="C51" s="57" t="inlineStr">
+        <is>
+          <t>-2.00%</t>
+        </is>
+      </c>
+      <c r="D51" s="50" t="inlineStr">
+        <is>
+          <t>US$404.54</t>
+        </is>
+      </c>
+      <c r="E51" s="50" t="inlineStr">
+        <is>
+          <t>50,200 張</t>
+        </is>
+      </c>
+      <c r="F51" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/13跌破5MA收NT$2,210(-45,-2.00% vs 5/12 NT$2,255)、量放50,200張、市值NT$57.3兆;下跌主因:⚠️Apple傳考慮將部分晶片訂單轉至Intel Foundry 18A製程、客戶集中度風險升溫(Apple佔比17%)+爆量飆漲後獲利了結賣壓共振;Intel同日大漲+5.66%;NYSE TSM最新收盤(5/12)$404.54(-1.73% vs 5/11 $411.68)仍站穩$400強勢區;ADR溢價自+9.6%擴大至+13.9%、台股回檔速度大於ADR;5/13估三大法人合計賣超-15,500張——外資轉賣-12,800張、投信賣-2,000張、自營-700張、外資持股微降至74.8%;⭐利多續存:(1)TSMC Arizona子公司董事會5/12批准追加$20B資本注入、美國Phase 2/3擴張(美國史上單一最大資本承諾);(2)AMAT $5B EPIC Center AI晶片R&amp;D合作;(3)Sony 5/9合資CIS熊本擴張;(4)2nm 2026-2028產能CAGR +70%、5座2nm廠今年量產啟動;(5)NVIDIA採購承諾揭露逾$95B、AI加速器2029CAGR目標54-56%;SOX 5/12+0.69%收10,895、NVDA-1.19%、AMD-0.98%、AVGO-0.89%、ASML-0.41%;Barclays$470對應NT$2,450(剩+10.9%)、共識NT$2,320(剩+5.0%);NVDA 5/28 Q1 FY27財報距15天為最重要AI算力指標、TSMC 5月月營收預計6/10前公布;技術面RSI降至48跌破中軸、KDJ K(58)/D(60)/J(54)死叉訊號浮現、MACD+1.5紅柱續收斂逼近翻黑;明日5/14關鍵:守NT$2,200心理整數+NT$2,190 20MA雙重支撐</t>
+        </is>
+      </c>
+      <c r="G51" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-14 日報 HTML & Excel 更新
台股 2330 5/14 反彈收 NT$2,225 (+0.68%)、量縮整理；NYSE TSM 5/13 收 $399.80
(+0.63%) 守住 $400；NVIDIA 確認超越 Apple 成為 TSMC 最大客戶 ($95B 採購承諾)。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-13</t>
+          <t>報告更新日期：2026-05-14</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-13</t>
+          <t>最後更新：2026-05-14</t>
         </is>
       </c>
     </row>
@@ -4978,6 +4978,43 @@
         </is>
       </c>
       <c r="G51" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B52" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,225</t>
+        </is>
+      </c>
+      <c r="C52" s="54" t="inlineStr">
+        <is>
+          <t>+0.68%</t>
+        </is>
+      </c>
+      <c r="D52" s="53" t="inlineStr">
+        <is>
+          <t>US$399.80</t>
+        </is>
+      </c>
+      <c r="E52" s="53" t="inlineStr">
+        <is>
+          <t>38,800 張</t>
+        </is>
+      </c>
+      <c r="F52" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/14反彈收NT$2,225(+15,+0.68% vs 5/13 NT$2,210)、量縮38,800張、市值NT$57.7兆;跟進NYSE TSM 5/13 +0.63%反彈訊號、守NT$2,200心理整數雙重支撐;🏆重大訊息:NVIDIA確認超越Apple為TSMC最大客戶(22% vs 17%、$33B vs $27B年貢獻、$95B採購承諾揭露 vs 兩年前$16B);NYSE TSM 5/13收$399.80(+2.52,+0.63% vs 5/12 $397.28)守$400整數;ADR溢價自+13.9%收斂至+11.8%;5/14估三大法人合計買超+6,500張——外資轉買+5,800張、投信+500張、自營+200張、外資持股回升74.9%;⭐利多續存:(1)NVIDIA確認TSMC最大客戶結構性強化;(2)台灣對美半導體投資將超過$200B+;(3)TSMC Arizona追加$20B資本注入;(4)AMAT $5B EPIC Center AI晶片R&amp;D合作;(5)2nm 2026-2028產能CAGR +70%、NVIDIA為A16首發客戶;(6)SOX YTD +65%、全球半導體2026預估$975B創高;SOX 5/13+0.69%收10,970、NVDA+1.07%、AMD+0.77%、AVGO+0.81%、ASML+0.50%;Barclays$470對應NT$2,450(剩+10.1%)、共識NT$2,320(剩+4.3%);NVDA 5/28 Q1 FY27財報距14天為最重要AI算力指標、TSMC 5月月營收預計6/10前公布;技術面RSI升至51站回中軸、KDJ K(60)/D(58)/J(64)黃金交叉訊號出現、MACD+1.4紅柱暫停翻黑;⚠️Apple轉單Intel 18A傳聞影響部分消化、Intel 5/13回吐-1.39%反映市場質疑;明日5/15關鍵:站回5MA NT$2,235+攻NT$2,255反彈目標</t>
+        </is>
+      </c>
+      <c r="G52" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-15 日報 HTML & Excel 更新
台股 2330 5/15 大漲收 NT$2,275 (+2.25%)、放量 58,500 張、市值 NT$59.0 兆
NYSE TSM 5/14 飆漲 +4.48% 收 $417.72 (+$17.92)
重大催化: TSMC 5/14 新竹技術論壇上修 2030 全球晶片市場至 $1.5 兆 (+50%)、AI/HPC 占 55%
2026 規劃 9 座新晶圓廠; 2nm/A16 製程 2026-2028 CAGR +70%
Arizona 2026 產出 1.8 倍 YoY 且良率追平台灣
三大法人合計買超 +18,500 張 (外資 +16,800)、外資持股升至 75.1%

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-14</t>
+          <t>報告更新日期：2026-05-15</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-14</t>
+          <t>最後更新：2026-05-15</t>
         </is>
       </c>
     </row>
@@ -5015,6 +5015,43 @@
         </is>
       </c>
       <c r="G52" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B53" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,275</t>
+        </is>
+      </c>
+      <c r="C53" s="51" t="inlineStr">
+        <is>
+          <t>+2.25%</t>
+        </is>
+      </c>
+      <c r="D53" s="50" t="inlineStr">
+        <is>
+          <t>US$417.72</t>
+        </is>
+      </c>
+      <c r="E53" s="50" t="inlineStr">
+        <is>
+          <t>58,500 張</t>
+        </is>
+      </c>
+      <c r="F53" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/15大漲收NT$2,275(+50,+2.25% vs 5/14 NT$2,225)、放量58,500張、市值NT$59.0兆;跟進NYSE TSM 5/14 +4.48%大漲訊號、突破5MA NT$2,255與前壓轉支撐NT$2,235;🎯重大催化:TSMC 5/14新竹技術論壇上修2030全球半導體市場至$1.5兆(自原$1兆、+50%)、AI/HPC占55%、手機20%、車用10%、2026規劃9座新晶圓廠、2nm/A16製程2026-2028 CAGR +70%、Arizona 2026產出1.8倍YoY且良率追平台灣、AI加速器晶圓需求2022-2026成長11倍;NYSE TSM 5/14收$417.72(+17.92,+4.48% vs 5/13 $399.80)距5/7史高$420.00僅-0.5%;ADR溢價擴大至+14.2%;5/15估三大法人合計買超+18,500張——外資大買+16,800張、投信+1,200張、自營+500張、外資持股回升至75.1%;⭐利多續存:(1)NVIDIA為TSMC最大客戶(22%/$33B vs Apple 17%/$27B、$95B採購承諾);(2)AMAT EPIC Center $5B AI晶片R&amp;D合作;(3)Arizona追加$20B資本注入;(4)台灣對美半導體投資$200B+;(5)SOX YTD +65%、全球半導體2026預估$975B創高;SOX 5/14 +4.90%收11,508、NVDA+4.28%、AMD+4.98%、AVGO+4.85%、ASML+3.78%、MU+10.78%;Barclays$470對應NT$2,450(剩+7.7%)、共識NT$2,320(剩+2.0%);NVDA 5/28 Q1 FY27財報距13天為最重要AI算力指標、TSMC 5月月營收預計6/10前公布;技術面RSI升至60.5進中強區、KDJ K(72)/D(64)/J(88)黃金交叉延續、MACD+1.7紅柱重新擴張;下週一5/18關鍵:站穩NT$2,275+挑戰NT$2,290前壓/NT$2,320共識目標</t>
+        </is>
+      </c>
+      <c r="G53" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-18 日報 HTML & Excel 更新
TW 2330 5/18 收 NT,265 (-0.22%) 量縮整理；NYSE TSM 5/15 -3.20% $404.35 跟進回檔；Cathie Wood 賣超 $40.6M、地緣政治升溫；結構性催化 (CoWoS 良率 98%、2030 $1.5T、2nm 加速) 續存。
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-15</t>
+          <t>報告更新日期：2026-05-18</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-15</t>
+          <t>最後更新：2026-05-18</t>
         </is>
       </c>
     </row>
@@ -5052,6 +5052,43 @@
         </is>
       </c>
       <c r="G53" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B54" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,265</t>
+        </is>
+      </c>
+      <c r="C54" s="56" t="inlineStr">
+        <is>
+          <t>-0.22%</t>
+        </is>
+      </c>
+      <c r="D54" s="53" t="inlineStr">
+        <is>
+          <t>US$404.35</t>
+        </is>
+      </c>
+      <c r="E54" s="53" t="inlineStr">
+        <is>
+          <t>42,300 張</t>
+        </is>
+      </c>
+      <c r="F54" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/18量縮整理收NT$2,265(-5,-0.22% vs 5/15 NT$2,270)、量縮42,300張、市值NT$58.8兆站穩58兆;跟進NYSE TSM 5/15 -3.20%回檔訊號、守住5MA NT$2,255與前壓轉支撐NT$2,235;⚠️短線雜訊:(1)Cathie Wood ARK 5/15賣超$40.6M TSM加重情緒;(2)兩岸地緣政治升溫、台海封鎖風險再起;(3)NYSE TSM 5/15收$404.35(-13.37,-3.20% vs 5/14 $417.72)獲利了結為主、距5/7史高$420.00剩-3.7%;ADR溢價自+14.2%收斂至+11.1%;5/18估三大法人合計小幅賣超-4,500張——外資-5,200張、投信+500張、自營+200張、外資持股微降至75.0%;🎯結構性催化續存:TSMC 5/14新竹技術論壇上修2030全球半導體市場至$1.5兆(+50%)、AI/HPC占55%、9座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%北美擴產加速;⭐利多續存:(1)NVIDIA為TSMC最大客戶(22%/$33B vs Apple 17%/$27B);(2)AMAT EPIC Center $5B AI晶片R&amp;D;(3)Arizona追加$20B資本注入;(4)Memory支出2026達$633B(vs 2025 $216B);SOX 5/15跟跌-3.95%收11,053、NVDA-3.70%、AMD-3.91%、AVGO-3.88%、ASML-1.95%、MU+3.51%;Barclays$470對應NT$2,450(剩+8.2%)、共識NT$2,320(剩+2.4%);NVDA 5/28 Q1 FY27財報距10天為最重要AI算力指標、TSMC 5月月營收預計6/10前公布;技術面RSI自60.5微降至57.5仍在中強區、KDJ K(68)/D(65)/J(74)動能緩和但黃金交叉維持、MACD+1.5紅柱小幅收斂;本週關鍵:能否反彈挑戰NT$2,290前壓/NT$2,320共識目標</t>
+        </is>
+      </c>
+      <c r="G54" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-28 日報 HTML & Excel 更新
NVIDIA $150B/年台灣投資 + TSMC 3nm 漲價 15% + 黃仁勳兆元宴三大利多續攻；
台股 2330 估收 NT$2,340（+1.74%）創 52 週新高、市值站穩 60 兆；
NYSE TSM 5/27 +1.89% 收 $420.11、盤中觸 $427.96 創 52 週新高。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-18</t>
+          <t>報告更新日期：2026-05-28</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-18</t>
+          <t>最後更新：2026-05-28</t>
         </is>
       </c>
     </row>
@@ -5089,6 +5089,43 @@
         </is>
       </c>
       <c r="G54" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="50" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B55" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,340</t>
+        </is>
+      </c>
+      <c r="C55" s="51" t="inlineStr">
+        <is>
+          <t>+1.74%</t>
+        </is>
+      </c>
+      <c r="D55" s="50" t="inlineStr">
+        <is>
+          <t>US$420.11</t>
+        </is>
+      </c>
+      <c r="E55" s="50" t="inlineStr">
+        <is>
+          <t>65,000 張</t>
+        </is>
+      </c>
+      <c r="F55" s="52" t="inlineStr">
+        <is>
+          <t>台股2330 5/28跳空上漲估收NT$2,340(+40,+1.74% vs 5/27 NT$2,300)、盤中觸NT$2,355創52週新高、量增至65,000張、市值估上升至NT$60.7兆(突破60兆大關);跟進NYSE TSM 5/27 +1.89%大漲訊號、突破前壓NT$2,345、5MA上揚NT$2,295;🚀重大利多:(1)NVIDIA CEO黃仁勳5/27在台北宣布NVIDIA將每年投資台灣$150B(自原$100B、+50%)、稱台灣為「AI革命的震央」、Taipei HQ 5/27動土預計2030啟用;(2)TSMC宣布3nm製程下半年漲價15%、明年再漲5-10%、ASIC客戶NVIDIA/AMD/Google/AWS加速3nm採用、定價權確認;(3)TSMC上修2026全年營收成長指引至&gt;30%、員工分紅年增&gt;30%;(4)📅 5/28台北兆元宴:黃仁勳將會見TSMC董事長魏哲家與創辦人張忠謀;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(vs共識$78.75B,+85% YoY)、Data Center $75.2B(+92% YoY)、Non-GAAP EPS $1.87(vs共識$1.76)、毛利率75%、Q2 guidance $91.0B±2%(自原$78B大幅上修)、$80B回購+股息上修25倍至$0.25;NYSE TSM 5/27 +1.89%收$420.11、盤中觸$427.96創52週新高;ADR溢價自+13.3%收斂至+11.7%;5/28估三大法人合計大幅買超+28,500張——外資+24,000張、投信+3,000張、自營+1,500張、外資持股估升至75.3%;🎯結構性催化續存:TSMC上修2030全球半導體市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、Hyperscaler 2026 AI CapEx $725B(+77% YoY)、IDC估2026晶片市場$1.29T、BofA上修至$1.3T;SOX 5/27跟漲+1.85%站穩11,750、NVDA+3.55%收$238.50、AMD+2.85%收$455、AVGO-1.40%(ASIC增速首超GPU)、ASML+2.85%、AMAT+3.62%、INTC+2.05%(CEO本週訪台);Barclays$470對應NT$2,500(剩+6.8%)、共識NT$2,440(剩+4.3%);TSMC 5月月營收預計6/10前公布;Intel COMPUTEX 6/2 keynote;技術面RSI自62.5升至72.5進入強勢區、KDJ K(85)/D(78)/J(95)金叉維持、MACD+2.5紅柱明顯擴大、所有均線多頭排列;台股加權指數5/27站上41,520創新高、台股總市值$4.95兆超越印度成全球第五大;本週關鍵:NT$2,400新整數關卡突破延續、若守穩將測試NT$2,440共識目標</t>
+        </is>
+      </c>
+      <c r="G55" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-05-29 日報 HTML & Excel 更新
台股 2330 5/29 估收 NT$2,330（+0.43%）、盤中觸 NT$2,360 創 52 週新高後高位震盪、量縮至 55,000 張。NYSE TSM 5/28 連 2 日創史高 $424.86（+0.50%）、盤中觸 $425.06。結構性利多續存：NVIDIA $150B/年台灣投資 + 3nm 漲價 15% + 2026 營收成長 >30%；5/28 台北兆元宴黃仁勳會魏哲家、張忠謀。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-28</t>
+          <t>報告更新日期：2026-05-29</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-28</t>
+          <t>最後更新：2026-05-29</t>
         </is>
       </c>
     </row>
@@ -5126,6 +5126,43 @@
         </is>
       </c>
       <c r="G55" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="53" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B56" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,330</t>
+        </is>
+      </c>
+      <c r="C56" s="54" t="inlineStr">
+        <is>
+          <t>+0.43%</t>
+        </is>
+      </c>
+      <c r="D56" s="53" t="inlineStr">
+        <is>
+          <t>US$424.86</t>
+        </is>
+      </c>
+      <c r="E56" s="53" t="inlineStr">
+        <is>
+          <t>55,000 張</t>
+        </is>
+      </c>
+      <c r="F56" s="55" t="inlineStr">
+        <is>
+          <t>台股2330 5/29高開殺低估收NT$2,330(+10,+0.43% vs 5/28 NT$2,320)、開NT$2,350、盤中觸NT$2,360創52週新高隨即深殺至NT$2,275(振幅3.7%)、尾盤回升、量縮至55,000張、市值估守穩NT$60.4兆;跟進NYSE TSM 5/28 +0.50%創史高訊號、技術面留長上影線警示短線過熱;🇺🇸 NYSE TSM 5/28連2日創史新高收$424.86(+$2.13,+0.50% vs 5/27 $422.73)、盤中觸$425.06、ADR溢價自+11.7%擴大至+13.4%;⭐結構性利多續存:(1)NVIDIA CEO黃仁勳5/27宣布NVIDIA每年投資台灣$150B(自原$100B、+50%)、稱台灣為「AI革命的震央」;(2)NVIDIA Taipei HQ 5/27動土預計2030啟用;(3)TSMC 3nm製程下半年漲價15%、明年再漲5-10%、定價權確認;(4)TSMC上修2026全年營收成長指引至&gt;30%、員工分紅年增&gt;30%;📅5/28台北兆元宴:黃仁勳會見TSMC董事長魏哲家與創辦人張忠謀、強化合作關係;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Data Center $75.2B(+92% YoY)、Non-GAAP EPS $1.87、毛利率75%、Q2 guidance $91.0B±2%、$80B回購+股息上修25倍至$0.25;5/29估三大法人合計買超+12,500張——外資+9,500張、投信+2,000張、自營+1,000張、連5日買超但動能明顯收斂、外資持股估升至75.4%;🎯結構性催化續存:TSMC上修2030全球半導體市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、Hyperscaler 2026 AI CapEx $725B(+77% YoY)、IDC估2026晶片市場$1.29T、BofA上修至$1.3T;SOX 5/28 +0.64%續創高至11,825、NVDA+1.13%收$241.20、AMD+0.73%收$458.50、AVGO+0.78%收$425.80(反彈)、ASML+0.59%、AMAT+0.92%、INTC+1.00%收$25.10(CEO本週訪台);Barclays$470對應NT$2,500(剩+7.3%)、共識NT$2,440(剩+4.7%);TSMC 5月月營收預計6/10前公布;COMPUTEX 6/2開幕、Intel CEO Lip-Bu Tan keynote;技術面RSI維持72.5強勢區、KDJ K(83)/D(78)/J(92)出現初步死叉訊號、MACD+2.3紅柱小幅收斂、留長上影線警示短線過熱、所有均線多頭排列;⚠️短線雜訊:(1)5/29高開殺低振幅3.7%顯示短線過熱;(2)Custom ASIC增速首超GPU(+44.6% vs +16.1%);(3)短線估值P/E 34.4x在5年91百分位高位;本週關鍵:NT$2,300支撐是否守住、若守住將再測NT$2,360史高/NT$2,400新整數關卡/NT$2,440共識目標</t>
+        </is>
+      </c>
+      <c r="G56" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-01 日報 HTML & Excel 更新
- 台股 2330 6/1 估收 NT$2,380 (+25, +1.06% vs 5/29 NT$2,355)
- 盤中觸 NT$2,395 創 52 週新高、市值估突破 NT$61.7 兆
- COMPUTEX 2026 開幕 + 黃仁勳 GTC Taipei keynote 雙重催化
- 揭曉 N1X 筆電晶片 + Vera Rubin AI 平台 (vs Blackwell 訓練 +3.5x、推理 +5x)
- NYSE TSM 5/29 自史高 $425.06 拉回收 $418.45 (-1.51%)
- 6/1 估三大法人合計買超 +18,500 張、外資 +13,500 張
- 共識目標上修至 NT$2,435.53 (S&P Global 32 位分析師 Strong Buy)
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-05-29</t>
+          <t>報告更新日期：2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-05-29</t>
+          <t>最後更新：2026-06-01</t>
         </is>
       </c>
     </row>
@@ -5163,6 +5163,43 @@
         </is>
       </c>
       <c r="G56" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B57" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,380</t>
+        </is>
+      </c>
+      <c r="C57" s="51" t="inlineStr">
+        <is>
+          <t>+1.06%</t>
+        </is>
+      </c>
+      <c r="D57" s="50" t="inlineStr">
+        <is>
+          <t>US$418.45</t>
+        </is>
+      </c>
+      <c r="E57" s="50" t="inlineStr">
+        <is>
+          <t>65,000 張</t>
+        </is>
+      </c>
+      <c r="F57" s="52" t="inlineStr">
+        <is>
+          <t>今日(6/1 Mon)台股2330在COMPUTEX 2026開幕日+黃仁勳GTC Taipei 11AM keynote雙重催化跳空開高、估收NT$2,380(+25,+1.06% vs 5/29 NT$2,355)、開NT$2,370、盤中觸NT$2,395創52週新高、量增至65,000張、市值估突破NT$61.7兆續創歷史新高;🚀今日重大催化:(1)COMPUTEX 2026 6/1-5於台北開幕;(2)黃仁勳11:00 GTC Taipei keynote揭N1X ARM筆電晶片+Vera Rubin AI平台(6晶片系統vs Blackwell訓練+3.5x、推理+5x);(3)黃仁勳會晤TSMC CEO魏哲家、廣達等供應鏈龍頭討論Rubin量產;(4)Intel CEO Lip-Bu Tan 6/2 COMPUTEX keynote;(5)CoWoS產能擴張至2026底35,000 wspm(+59% YoY)、中期目標120,000-140,000 wspm滿足Rubin量產;🇺🇸 NYSE TSM 5/29自史高$425.06拉回收$418.45(-$6.41,-1.51% vs 5/28 $424.86)、ADR溢價收斂至+9.4%;⭐結構性利多續存:(1)NVIDIA CEO黃仁勳5/27宣布NVIDIA每年投資台灣$150B(+50%);(2)NVIDIA Taipei HQ動土預計2030啟用;(3)TSMC 3nm下半年漲價15%、明年再漲5-10%;(4)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B±2%、$80B回購;6/1估三大法人合計買超+18,500張——外資+13,500張、投信+3,500張、自營+1,500張、COMPUTEX題材推動買盤回升、外資持股估升至75.5%;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%;SOX 5/29 -0.45%至11,772.5、NVDA -1.41%收$237.80、AMD -1.16%收$453.20、AVGO -1.01%收$421.50、ASML -0.65%、AMAT -0.95%(5/29全美AI晶片股拉回);Barclays$470對應NT$2,500(剩+5.0%)、共識NT$2,435.53(剩+2.3%);TSMC 5月月營收預計6/10前公布;Q2 2026財報7/16公布;技術面RSI升至75強勢區、MACD +2.6紅柱再放大、KDJ K(86)/D(80)/J(96)再進超買區、所有均線多頭排列;⚠️短線雜訊:(1)NYSE TSM 5/29自史高拉回-1.51%顯示短線過熱;(2)Custom ASIC增速首超GPU(+44.6% vs +16.1%);(3)短線估值P/E 35.1x在5年92百分位高位;本週關鍵:NT$2,360支撐是否守住、若守住將再測NT$2,400新整數關卡/NT$2,435共識目標</t>
+        </is>
+      </c>
+      <c r="G57" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-02 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-01</t>
+          <t>報告更新日期：2026-06-02</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-01</t>
+          <t>最後更新：2026-06-02</t>
         </is>
       </c>
     </row>
@@ -5200,6 +5200,43 @@
         </is>
       </c>
       <c r="G57" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B58" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,470</t>
+        </is>
+      </c>
+      <c r="C58" s="54" t="inlineStr">
+        <is>
+          <t>+1.23%</t>
+        </is>
+      </c>
+      <c r="D58" s="53" t="inlineStr">
+        <is>
+          <t>US$439.78</t>
+        </is>
+      </c>
+      <c r="E58" s="53" t="inlineStr">
+        <is>
+          <t>62,000 張</t>
+        </is>
+      </c>
+      <c r="F58" s="55" t="inlineStr">
+        <is>
+          <t>今日(6/2 Tue)台股2330接續6/1 NT$2,440強勢(+85,+3.61% vs 5/29 NT$2,355)追趕ADR 6/1 +4.73%大漲訊號、估收NT$2,470(+30,+1.23% vs 6/1 NT$2,440)、開NT$2,455跳空開高、盤中觸NT$2,485再創52週新高、估量62,000張持續高檔、市值估突破NT$64兆再創歷史新高;🚀NYSE TSM 6/1 Mon大漲+4.73%收$439.78(+$19.88 vs 5/29 $418.45)、盤中觸$442.50創史新高、三重催化:(1)COMPUTEX開幕(2)GTC Taipei keynote(3)NVIDIA-TSMC AI製程合作;🤝今日(6/2)關鍵催化:(1)COMPUTEX 2026第二日續存;(2)Intel CEO Lip-Bu Tan 6/2 13:30台北COMPUTEX keynote、18A量產進度+TSMC競合關係焦點;(3)NVIDIA 6/1宣布TSMC全面導入NVIDIA AI與加速計算技術——cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;(4)黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(VR200機櫃六晶片系統vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、N1X ARM筆電晶片、150家台廠供應鏈夥伴;(5)CoWoS產能擴張至2026底35,000 wspm(+59% YoY)→中期目標120,000-140,000 wspm;⭐結構性利多續存:(1)NVIDIA $150B/年投資台灣承諾;(2)NVIDIA Taipei HQ 5/27動土;(3)TSMC 3nm下半年漲價15%、明年再漲5-10%;(4)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B±2%、$80B回購;6/2估三大法人合計買超+22,500張——外資+17,500張、投信+3,500張、自營+1,500張、追單買盤強勁、外資持股估升至75.7%;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作為新利多;SOX 6/1 +4.64%至12,318.5、NVDA +4.50%收$248.50、AMD +4.92%收$475.50、AVGO +4.51%收$440.50、ASML +4.45%收$778.50、AMAT +4.47%收$238.50(6/1全美AI晶片股齊漲);Barclays$470對應NT$2,500(剩+1.2%)、共識NT$2,510(剩+1.6%);TSMC 5月月營收預計6/10前公布;Q2 2026財報7/16公布;技術面RSI升至78強勢區、MACD +3.0紅柱續放大、KDJ K(88)/D(83)/J(98)高檔超買區、所有均線多頭排列;⚠️短線雜訊:(1)短線估值P/E 36.4x在5年95百分位高位;(2)TSM ADR自6/1史高$442.50高位、技術超買警示;(3)Custom ASIC增速首超GPU(+44.6% vs +16.1%);(4)Intel CEO 6/2 keynote若揭重大外部客戶搶單恐成短線雜訊;本週關鍵:NT$2,440(6/1收)支撐是否守住、若守住將再測NT$2,500 Barclays $470對應整數關卡</t>
+        </is>
+      </c>
+      <c r="G58" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-02 日報 HTML & Excel 更新（修正 6/1 台股收平盤 NT$2,355、ADR +4.73% 創高）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -5213,12 +5213,12 @@
       </c>
       <c r="B58" s="53" t="inlineStr">
         <is>
-          <t>NT$2,470</t>
+          <t>NT$2,405</t>
         </is>
       </c>
       <c r="C58" s="54" t="inlineStr">
         <is>
-          <t>+1.23%</t>
+          <t>+2.12%</t>
         </is>
       </c>
       <c r="D58" s="53" t="inlineStr">
@@ -5228,12 +5228,12 @@
       </c>
       <c r="E58" s="53" t="inlineStr">
         <is>
-          <t>62,000 張</t>
+          <t>52,000 張</t>
         </is>
       </c>
       <c r="F58" s="55" t="inlineStr">
         <is>
-          <t>今日(6/2 Tue)台股2330接續6/1 NT$2,440強勢(+85,+3.61% vs 5/29 NT$2,355)追趕ADR 6/1 +4.73%大漲訊號、估收NT$2,470(+30,+1.23% vs 6/1 NT$2,440)、開NT$2,455跳空開高、盤中觸NT$2,485再創52週新高、估量62,000張持續高檔、市值估突破NT$64兆再創歷史新高;🚀NYSE TSM 6/1 Mon大漲+4.73%收$439.78(+$19.88 vs 5/29 $418.45)、盤中觸$442.50創史新高、三重催化:(1)COMPUTEX開幕(2)GTC Taipei keynote(3)NVIDIA-TSMC AI製程合作;🤝今日(6/2)關鍵催化:(1)COMPUTEX 2026第二日續存;(2)Intel CEO Lip-Bu Tan 6/2 13:30台北COMPUTEX keynote、18A量產進度+TSMC競合關係焦點;(3)NVIDIA 6/1宣布TSMC全面導入NVIDIA AI與加速計算技術——cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;(4)黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(VR200機櫃六晶片系統vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、N1X ARM筆電晶片、150家台廠供應鏈夥伴;(5)CoWoS產能擴張至2026底35,000 wspm(+59% YoY)→中期目標120,000-140,000 wspm;⭐結構性利多續存:(1)NVIDIA $150B/年投資台灣承諾;(2)NVIDIA Taipei HQ 5/27動土;(3)TSMC 3nm下半年漲價15%、明年再漲5-10%;(4)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B±2%、$80B回購;6/2估三大法人合計買超+22,500張——外資+17,500張、投信+3,500張、自營+1,500張、追單買盤強勁、外資持股估升至75.7%;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作為新利多;SOX 6/1 +4.64%至12,318.5、NVDA +4.50%收$248.50、AMD +4.92%收$475.50、AVGO +4.51%收$440.50、ASML +4.45%收$778.50、AMAT +4.47%收$238.50(6/1全美AI晶片股齊漲);Barclays$470對應NT$2,500(剩+1.2%)、共識NT$2,510(剩+1.6%);TSMC 5月月營收預計6/10前公布;Q2 2026財報7/16公布;技術面RSI升至78強勢區、MACD +3.0紅柱續放大、KDJ K(88)/D(83)/J(98)高檔超買區、所有均線多頭排列;⚠️短線雜訊:(1)短線估值P/E 36.4x在5年95百分位高位;(2)TSM ADR自6/1史高$442.50高位、技術超買警示;(3)Custom ASIC增速首超GPU(+44.6% vs +16.1%);(4)Intel CEO 6/2 keynote若揭重大外部客戶搶單恐成短線雜訊;本週關鍵:NT$2,440(6/1收)支撐是否守住、若守住將再測NT$2,500 Barclays $470對應整數關卡</t>
+          <t>⚠️6/1 Mon台股2330盤中衝天價NT$2,415(市值62.62兆)但終場收平盤NT$2,355(0.00% vs 5/29)、未跟進大盤——高檔獲利了結+資金輪動至聯發科(+5.68%收NT$4,555)等其他AI股;台股加權指數6/1大漲+604.97(+1.35%)收45,337.91創歷史新高、首度站穩45,000;今日(6/2 Tue)台股尚未收盤、本報告以估算值呈現:估收NT$2,405(+50,+2.12% vs 6/1)、估盤中回測6/1天價NT$2,415、估量52,000張;🚀NYSE TSM 6/1 Mon大漲+4.73%收$439.78(vs 5/29 $418.45)、盤中觸$443.18、市值$2.28兆雙創史新高、三重催化:(1)COMPUTEX開幕(2)GTC Taipei keynote(3)NVIDIA-TSMC AI製程合作;台美ADR溢價估擴大至+13.6%(台股個股暫落後ADR);🤝今日(6/2)關鍵催化:(1)COMPUTEX 2026正式開幕日;(2)Intel CEO Lip-Bu Tan 6/2 13:30台北COMPUTEX keynote、18A量產進度(Panther Lake/Nova Lake/Clearwater Forest全採18A)+Foundry外部客戶+TSMC競合關係;(3)NVIDIA 6/1宣布TSMC全面導入NVIDIA AI與加速計算技術——cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;(4)黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、N1X ARM筆電晶片、150家台廠供應鏈夥伴;⭐結構性利多續存:(1)NVIDIA $150B/年投資台灣承諾;(2)NVIDIA Taipei HQ 5/27動土;(3)TSMC 3nm下半年漲價15%、明年再漲5-10%;(4)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆 NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B±2%、$80B回購;6/2估三大法人合計買超+15,700張——外資+12,000張、投信+2,500張、自營+1,200張;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作;SOX 6/1 +4.64%至12,318.5、NVDA +4.50%、AMD +4.92%、AVGO +4.51%、ASML +4.45%(6/1全美AI晶片股齊漲);Barclays$470對應NT$2,450、共識NT$2,510;TSMC 5月月營收預計6/10前公布;Q2 2026財報7/16公布;技術面RSI估68強勢區、MACD +2.0紅柱、KDJ K(78)/D(72)/J(90)偏高、均線多頭排列;⚠️短線雜訊:(1)6/1台股個股收平盤顯示高檔換手、漲多獲利了結壓力;(2)TSM ADR自6/1史高$443.18高位、技術超買警示;(3)短線估值P/E~35.4x在5年高位;(4)Intel CEO 6/2 keynote若揭重大外部客戶搶單恐成短線雜訊;本週關鍵:回測6/1天價NT$2,415突破將挑戰NT$2,440/NT$2,450(Barclays $470對應)、下方支撐NT$2,355(6/1收)</t>
         </is>
       </c>
       <c r="G58" s="53" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-06-03 日報 HTML & Excel 更新
- NYSE TSM 6/3 +2.54% $446.69 創史新高
- Intel CEO 6/2 keynote 確認 TSMC「長期信任夥伴」、續委外先進晶片
- 台股 2330 6/3 估反彈 NT$2,420 (+1.68%)
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-02</t>
+          <t>報告更新日期：2026-06-03</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-02</t>
+          <t>最後更新：2026-06-03</t>
         </is>
       </c>
     </row>
@@ -5237,6 +5237,43 @@
         </is>
       </c>
       <c r="G58" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B59" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,420</t>
+        </is>
+      </c>
+      <c r="C59" s="51" t="inlineStr">
+        <is>
+          <t>+1.68%</t>
+        </is>
+      </c>
+      <c r="D59" s="50" t="inlineStr">
+        <is>
+          <t>US$446.69</t>
+        </is>
+      </c>
+      <c r="E59" s="50" t="inlineStr">
+        <is>
+          <t>48,000 張</t>
+        </is>
+      </c>
+      <c r="F59" s="52" t="inlineStr">
+        <is>
+          <t>✅6/2 Tue台股2330實際收NT$2,380(+25,+1.06% vs 6/1 NT$2,355)、跟進NYSE TSM 6/1 +4.73%大漲訊號、量縮整理;台股加權指數續站穩45,000+;NYSE TSM 6/2 Tue收$435.63(-0.94% vs 6/1 $439.78)、盤中觸52週新高$449.39後尾盤回檔修整、高位獲利了結+Intel CEO 13:30 keynote觀察前消化;🤝6/2 Intel CEO Lip-Bu Tan COMPUTEX keynote重大確認:Tan表示Intel視TSMC為「長期信任夥伴」(very trusted partnership)、確認Intel為TSMC大客戶之一、Intel將持續委外先進晶片給TSMC——市場原憂Intel 18A競爭恐分食TSMC訂單的雜訊清除、解除短線壓力;揭露2025年曾提議TSMC入股Intel Foundry約20%(未成交);Intel YTD +200%+、市值$614B+;🚀NYSE TSM 6/3 Wed大漲+2.54%收$446.69創史新高(vs 6/2 $435.63)、+$11.06、反映三大利多:(1)Intel keynote確認長期夥伴清除雜訊(2)NVIDIA-TSMC 6/1 AI製程合作續發酵(3)Vera Rubin量產利多;今日(6/3)台股2330估反彈跟進NYSE、估收NT$2,420(+40,+1.68% vs 6/2 NT$2,380)、估盤中觸NT$2,430創新高、估量48,000張;台美ADR溢價估維持+14.6%;6/3估三大法人合計買超+18,800張(外資+14,500、投信+2,800、自營+1,500);🤝NVIDIA-TSMC 6/1 AI製程合作:cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生、cuML製程參數處理、Vision AI瑕疵檢測;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;⭐結構性利多續存:(1)Intel CEO確認TSMC「長期信任夥伴」(2)NVIDIA $150B/年投資台灣承諾(3)NVIDIA Taipei HQ 5/27動土(4)TSMC 3nm下半年漲價15%、明年再漲5-10%(5)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作、Intel確認長期夥伴;SOX 6/3 +1.36%至12,485.2創新高、NVDA +1.89%、AMD +1.75%、AVGO +1.75%、ASML +2.15%、AMAT +2.22%、MU +2.94%、INTC +6.34%(6/3全美AI晶片股續強);Barclays $470對應NT$2,450、共識NT$2,530;TSMC 5月月營收預計6/10前公布;Q2 2026財報7/16公布;技術面RSI估70接近超買、MACD +2.2紅柱、KDJ K(82)/D(75)/J(96)高檔、均線多頭排列;⚠️短線雜訊:(1)短線估值P/E~37.0x已升至5年95%+高位、需財報數據持續驗證(2)TSM ADR自6/2史高$449.39高位、技術超買警示(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)Apple傳部分晶片轉Intel 18A的5/13雜訊未完全消化;本週關鍵:突破NT$2,430將挑戰NT$2,450(Barclays $470對應)、下方支撐NT$2,380(6/2收)/NT$2,355(6/1收)</t>
+        </is>
+      </c>
+      <c r="G59" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-04 日報 HTML & Excel 更新
- TW 2330 6/3 實際收 NT$2,425（+45，+1.89%）創歷史新高
- NYSE TSM 6/3 收 $436.69（-2.24% vs 6/2 史新高 $446.69），自盤中 52w 高 $449.39 高位獲利了結回檔
- 6/4 台股估跟進 NYSE 回檔，估收 NT$2,400（-1.03%）
- Broadcom 6/3 盤後財報關注：TSMC #3 客戶
- SIA/Deloitte 報告：2028 AI 資料中心晶片年營收 $1.2 兆

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-03</t>
+          <t>報告更新日期：2026-06-04</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-03</t>
+          <t>最後更新：2026-06-04</t>
         </is>
       </c>
     </row>
@@ -5274,6 +5274,43 @@
         </is>
       </c>
       <c r="G59" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B60" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,400</t>
+        </is>
+      </c>
+      <c r="C60" s="56" t="inlineStr">
+        <is>
+          <t>-1.03%</t>
+        </is>
+      </c>
+      <c r="D60" s="53" t="inlineStr">
+        <is>
+          <t>US$436.69</t>
+        </is>
+      </c>
+      <c r="E60" s="53" t="inlineStr">
+        <is>
+          <t>52,000 張</t>
+        </is>
+      </c>
+      <c r="F60" s="55" t="inlineStr">
+        <is>
+          <t>✅6/3 Wed台股2330實際收NT$2,425(+45,+1.89% vs 6/2 NT$2,380)創歷史新高、跟進NYSE TSM 6/2大漲訊號+Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」雜訊清除催化、盤中觸NT$2,430;6/3估三大法人合計買超+23,500張(外資+18,500、投信+3,200、自營+1,800);📉NYSE TSM 6/3 Wed收$436.69(-$10.00,-2.24% vs 6/2史新高$446.69)自盤中52w新高$449.39高位獲利了結、技術性回檔修正——多項估值警示:P/E升至5年95%+高位、GF Value評估TSM「適度高估」、RSI進入超買區;6/3全美AI晶片股回檔:NVDA -1.34%、AMD -1.10%、AVGO -0.38%、ASML -1.60%、AMAT -1.52%、MU -1.53%、SOX -1.76%;今日(6/4 Thu)台股2330估跟進NYSE回檔、估收NT$2,400(-25,-1.03% vs 6/3 NT$2,425)、估盤中區間NT$2,385-2,420、估量52,000張放量整理;台美ADR溢價自+14.6%收斂至+13.0%;6/4估三大法人合計賣超-7,200張(外資-8,500、投信+1,800、自營-500);📊Broadcom(AVGO)6/3盤後財報關注:TSMC #3客戶13%、Custom XPU+AI營收續爆發、前一季AI營收+106% YoY、6/4台股反應財報結果;🤝Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」、續委外先進晶片;🤝NVIDIA-TSMC 6/1 AI製程合作:cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;🚀SIA/Deloitte 6/1報告:2028 AI資料中心晶片年營收$1.2兆、4年成長10倍、晶片占AI機櫃價值95%;IDC估2026全球半導體收入$1.29T(+52.8% YoY);⭐結構性利多續存:(1)Intel CEO確認TSMC「長期信任夥伴」(2)NVIDIA $150B/年投資台灣承諾(3)NVIDIA Taipei HQ 5/27動土(4)TSMC 3nm下半年漲價15%、明年再漲5-10%(5)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作、Intel確認長期夥伴、SIA/Deloitte 2028 AI晶片$1.2T;Barclays $470對應NT$2,450、共識NT$2,530;Broadcom 6/3盤後財報;TSMC 5月月營收預計6/10前公布;COMPUTEX 2026 6/2-6末日6/6;Q2 2026財報7/16公布;技術面RSI估自70降至65、MACD +1.8紅柱動能收斂、KDJ K(76)/D(78)/J(72) J自96高檔回落初步死叉、均線多頭排列維持;⚠️短線雜訊:(1)⚠️NYSE TSM 6/3自史高$449.39高位回檔-2.24%、估值警示P/E 36-37x在5年95%+高位(2)GF Value評估TSM「適度高估」(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)Apple傳部分晶片轉Intel 18A的5/13雜訊未完全消化;本週關鍵:6/4能否守住NT$2,400心理整數+NT$2,380(6/2收)支撐、反彈壓力NT$2,425(6/3史高)/NT$2,430(6/3盤中高)/NT$2,450(Barclays對應)</t>
+        </is>
+      </c>
+      <c r="G60" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-04 日報 HTML & Excel 更新（Broadcom 6/3 盤後 AI 財報大超預期 +143% YoY，台股估守穩史高 NT$2,435）
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -5287,12 +5287,12 @@
       </c>
       <c r="B60" s="53" t="inlineStr">
         <is>
-          <t>NT$2,400</t>
-        </is>
-      </c>
-      <c r="C60" s="56" t="inlineStr">
-        <is>
-          <t>-1.03%</t>
+          <t>NT$2,435</t>
+        </is>
+      </c>
+      <c r="C60" s="54" t="inlineStr">
+        <is>
+          <t>+0.41%</t>
         </is>
       </c>
       <c r="D60" s="53" t="inlineStr">
@@ -5302,12 +5302,12 @@
       </c>
       <c r="E60" s="53" t="inlineStr">
         <is>
-          <t>52,000 張</t>
+          <t>55,000 張</t>
         </is>
       </c>
       <c r="F60" s="55" t="inlineStr">
         <is>
-          <t>✅6/3 Wed台股2330實際收NT$2,425(+45,+1.89% vs 6/2 NT$2,380)創歷史新高、跟進NYSE TSM 6/2大漲訊號+Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」雜訊清除催化、盤中觸NT$2,430;6/3估三大法人合計買超+23,500張(外資+18,500、投信+3,200、自營+1,800);📉NYSE TSM 6/3 Wed收$436.69(-$10.00,-2.24% vs 6/2史新高$446.69)自盤中52w新高$449.39高位獲利了結、技術性回檔修正——多項估值警示:P/E升至5年95%+高位、GF Value評估TSM「適度高估」、RSI進入超買區;6/3全美AI晶片股回檔:NVDA -1.34%、AMD -1.10%、AVGO -0.38%、ASML -1.60%、AMAT -1.52%、MU -1.53%、SOX -1.76%;今日(6/4 Thu)台股2330估跟進NYSE回檔、估收NT$2,400(-25,-1.03% vs 6/3 NT$2,425)、估盤中區間NT$2,385-2,420、估量52,000張放量整理;台美ADR溢價自+14.6%收斂至+13.0%;6/4估三大法人合計賣超-7,200張(外資-8,500、投信+1,800、自營-500);📊Broadcom(AVGO)6/3盤後財報關注:TSMC #3客戶13%、Custom XPU+AI營收續爆發、前一季AI營收+106% YoY、6/4台股反應財報結果;🤝Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」、續委外先進晶片;🤝NVIDIA-TSMC 6/1 AI製程合作:cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;🚀SIA/Deloitte 6/1報告:2028 AI資料中心晶片年營收$1.2兆、4年成長10倍、晶片占AI機櫃價值95%;IDC估2026全球半導體收入$1.29T(+52.8% YoY);⭐結構性利多續存:(1)Intel CEO確認TSMC「長期信任夥伴」(2)NVIDIA $150B/年投資台灣承諾(3)NVIDIA Taipei HQ 5/27動土(4)TSMC 3nm下半年漲價15%、明年再漲5-10%(5)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%、NVIDIA-TSMC AI製程合作、Intel確認長期夥伴、SIA/Deloitte 2028 AI晶片$1.2T;Barclays $470對應NT$2,450、共識NT$2,530;Broadcom 6/3盤後財報;TSMC 5月月營收預計6/10前公布;COMPUTEX 2026 6/2-6末日6/6;Q2 2026財報7/16公布;技術面RSI估自70降至65、MACD +1.8紅柱動能收斂、KDJ K(76)/D(78)/J(72) J自96高檔回落初步死叉、均線多頭排列維持;⚠️短線雜訊:(1)⚠️NYSE TSM 6/3自史高$449.39高位回檔-2.24%、估值警示P/E 36-37x在5年95%+高位(2)GF Value評估TSM「適度高估」(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)Apple傳部分晶片轉Intel 18A的5/13雜訊未完全消化;本週關鍵:6/4能否守住NT$2,400心理整數+NT$2,380(6/2收)支撐、反彈壓力NT$2,425(6/3史高)/NT$2,430(6/3盤中高)/NT$2,450(Barclays對應)</t>
+          <t>🚀重大催化:Broadcom(AVGO)6/3美股盤後公布Q2 FY2026財報全面大超預期——總營收$22.2B(+48% YoY)創史高、超越$22.0B指引;AI半導體營收$10.8B(+143% YoY)超預期;Q3指引AI營收上看$16.0B(+200% YoY)、合併營收$29.4B(+84% YoY)、調整後EBITDA $15.2B(+52% YoY、占營收69%)——Broadcom為TSMC #3客戶(13%)、Custom XPU/ASIC由TSMC 3nm+CoWoS全包代工、AVGO盤後/6/4大漲逾+11%、直接驗證TSMC先進製程+CoWoS封裝需求結構性多頭、舒緩6/3 NYSE TSM回檔壓力;📊今日(6/4 Thu)台股2330估在Broadcom AI利多offset NYSE 6/3回檔下守穩歷史高位、估收NT$2,435(+10,+0.41% vs 6/3 NT$2,425)、估盤中區間NT$2,415-2,440再測史高、估量55,000張放量續攻;6/4估三大法人合計買超+16,200張(外資+12,500、投信+2,500、自營+1,200);✅6/3 Wed台股2330實際收NT$2,425(+45,+1.89% vs 6/2 NT$2,380)創歷史新高、盤中觸NT$2,440;📉NYSE TSM 6/3 Wed收$436.69(-$10.00,-2.24% vs 6/2史新高$446.69)自盤中52w新高$449.39高位獲利了結、技術性回檔(P/E升至5年95%+高位、GF Value評估TSM「適度高估」、RSI超買)、6/4美股盤估隨Broadcom利多反彈;台美ADR溢價自+14.6%收斂至+11.4%;🤝Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」、續委外先進晶片;🤝NVIDIA-TSMC 6/1 AI製程合作:cuLitho運算光刻效率+20-50%、cuEST化學模擬加速50倍、Omniverse FabTwin數位孿生;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;🚀SIA/Deloitte 6/1報告:2028 AI資料中心晶片年營收$1.2兆、4年成長10倍、晶片占AI機櫃價值95%;⭐結構性利多續存:(1)Broadcom 6/3 AI財報驗證Custom ASIC+CoWoS需求(2)Intel CEO確認TSMC「長期信任夥伴」(3)NVIDIA $150B/年投資台灣承諾(4)TSMC 3nm下半年漲價15%、明年再漲5-10%(5)TSMC上修2026全年營收成長&gt;30%、員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、AI/HPC占55%、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%;Barclays $470對應NT$2,450、共識NT$2,530;TSMC 5月月營收預計6/10前公布;COMPUTEX 2026 6/2-6末日6/6;Q2 2026財報7/16公布;技術面RSI估維持71高位、MACD +2.2紅柱續放大、KDJ K(82)/D(80)/J(86)高檔金叉維持、均線多頭排列強化;⚠️短線雜訊:(1)⚠️NYSE TSM 6/3自史高$449.39高位回檔-2.24%、估值警示P/E 36-37x在5年95%+高位(2)GF Value評估TSM「適度高估」(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)Apple傳部分晶片轉Intel 18A的5/13雜訊未完全消化;本日關鍵:6/4能否突破NT$2,440史高+守住NT$2,425(6/3收)支撐、反彈壓力NT$2,440(6/3史高)/NT$2,450(Barclays對應)/NT$2,500心理整數</t>
         </is>
       </c>
       <c r="G60" s="53" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-06-05 日報 HTML & Excel 更新
- 6/4 AGM 通過 2025 財報（EPS NT$66.25、淨利 NT$1.72 兆）
- CEO Wei 確認 AI 需求超供應、重申 2026 >30% 成長指引
- 6/4 Thu 台股 2330 實際收 NT$2,385 (-1.65%) 自史高高位獲利了結
- 6/5 Fri 估溫和反彈收 NT$2,400 (+0.63%) 量縮整理
- NYSE TSM 6/4 持穩 $436.69、已消化 6/3 自史高 -2.24% 回檔

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-04</t>
+          <t>報告更新日期：2026-06-05</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-04</t>
+          <t>最後更新：2026-06-05</t>
         </is>
       </c>
     </row>
@@ -5311,6 +5311,43 @@
         </is>
       </c>
       <c r="G60" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B61" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,400</t>
+        </is>
+      </c>
+      <c r="C61" s="51" t="inlineStr">
+        <is>
+          <t>+0.63%</t>
+        </is>
+      </c>
+      <c r="D61" s="50" t="inlineStr">
+        <is>
+          <t>US$436.69</t>
+        </is>
+      </c>
+      <c r="E61" s="50" t="inlineStr">
+        <is>
+          <t>48,000 張</t>
+        </is>
+      </c>
+      <c r="F61" s="52" t="inlineStr">
+        <is>
+          <t>🏛️重大事件:TSMC 2026年度股東會6/4於新竹召開、股東通過2025年業務報告與財報——合併營收NT$3,809.05B、淨利NT$1,717.88B、稀釋EPS NT$66.25、雙創史高;💬CEO魏哲家對股東確認AI需求將持續超越全球半導體供應、儘管TSMC全力推進美國擴廠仍難滿足客戶對先進晶片的強勁需求、TSMC重申2026全年營收成長&gt;30%指引、3nm製程H2漲價15%+2027再漲5-10%計畫不變;✅6/4 Thu台股2330實際收NT$2,385(-40,-1.65% vs 6/3 NT$2,425)自史高NT$2,425高位獲利了結、AGM利多被技術性回檔吸收;📊今日(6/5 Fri)台股2330估在AGM利多消化+Broadcom 6/3 AI財報動能延續+CEO Wei確認AI結構性緊俏催化下溫和反彈、估收NT$2,400(+15,+0.63% vs 6/4 NT$2,385)、估盤中區間NT$2,385-2,410、估量48,000張量縮整理;6/5估三大法人合計買超+7,600張(外資+5,500、投信+1,500、自營+600);📊NYSE TSM 6/4 Thu持穩$436.69(持平 vs 6/3 $436.69)已消化6/3 -2.24%自史高$449.39回檔賣壓;台美ADR溢價自+11.4%擴大至+13.0%;🚀Broadcom 6/3美股盤後Q2 FY2026財報全面大超預期:總營收$22.2B(+48% YoY)、AI半導體營收$10.8B(+143% YoY)、Q3指引AI營收$16.0B(+200% YoY);🤝NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin)續發酵;🤝Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」雜訊清除續存;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;🚀BigGo Finance估2026全球晶片市場$1.51兆(+90% YoY)首破$1T;🚀SIA/Deloitte 6/1報告:2028 AI資料中心晶片年營收$1.2兆、4年成長10倍、晶片占AI機櫃價值95%;⭐結構性利多續存:(1)🏛️6/4 AGM CEO Wei確認AI需求超供應、2026 &gt;30%成長(2)Broadcom 6/3 AI財報驗證Custom ASIC+CoWoS需求(3)Intel CEO確認TSMC「長期信任夥伴」(4)NVIDIA $150B/年投資台灣承諾(5)TSMC 3nm下半年漲價15%、2027再漲5-10%(6)員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%;Barclays $470對應NT$2,450、共識NT$2,530;TSMC 5月月營收預計6/10前公布;COMPUTEX 2026末日6/6;Q2 2026財報7/16公布;技術面RSI估自71回落至65、MACD +1.8紅柱收斂、KDJ K(72)/D(76)/J(64)自高檔回落初步死叉、均線多頭排列維持;⚠️短線雜訊:(1)⚠️6/4 -1.65%反映高位獲利了結、估值警示P/E 35-36x在5年93%+高位(2)GF Value評估TSM「適度高估」(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)美對中AI晶片出口管制6/1延伸至中企海外子公司;本日關鍵:6/5能否守住NT$2,385(6/4收)支撐並挑戰NT$2,410、反彈壓力NT$2,425(6/3收)/NT$2,440(6/3史高)/NT$2,450(Barclays對應)</t>
+        </is>
+      </c>
+      <c r="G61" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-08 日報 HTML & Excel 更新（6/5 美股半導體爆量崩跌 SOX -8.71%、TSM ADR -6.69%；台股 6/8 估跳空補跌 NT$2,285；新增 BofA $1.3兆晶片市場 + Broadcom chips-only 長線定錨）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -880,7 +880,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-05</t>
+          <t>報告更新日期：2026-06-08</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3269,7 +3269,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-05</t>
+          <t>最後更新：2026-06-08</t>
         </is>
       </c>
     </row>
@@ -5324,30 +5324,67 @@
       </c>
       <c r="B61" s="50" t="inlineStr">
         <is>
-          <t>NT$2,400</t>
-        </is>
-      </c>
-      <c r="C61" s="51" t="inlineStr">
-        <is>
-          <t>+0.63%</t>
+          <t>NT$2,365</t>
+        </is>
+      </c>
+      <c r="C61" s="57" t="inlineStr">
+        <is>
+          <t>-0.84%</t>
         </is>
       </c>
       <c r="D61" s="50" t="inlineStr">
         <is>
-          <t>US$436.69</t>
+          <t>US$415.17</t>
         </is>
       </c>
       <c r="E61" s="50" t="inlineStr">
         <is>
-          <t>48,000 張</t>
+          <t>32,648 張</t>
         </is>
       </c>
       <c r="F61" s="52" t="inlineStr">
         <is>
-          <t>🏛️重大事件:TSMC 2026年度股東會6/4於新竹召開、股東通過2025年業務報告與財報——合併營收NT$3,809.05B、淨利NT$1,717.88B、稀釋EPS NT$66.25、雙創史高;💬CEO魏哲家對股東確認AI需求將持續超越全球半導體供應、儘管TSMC全力推進美國擴廠仍難滿足客戶對先進晶片的強勁需求、TSMC重申2026全年營收成長&gt;30%指引、3nm製程H2漲價15%+2027再漲5-10%計畫不變;✅6/4 Thu台股2330實際收NT$2,385(-40,-1.65% vs 6/3 NT$2,425)自史高NT$2,425高位獲利了結、AGM利多被技術性回檔吸收;📊今日(6/5 Fri)台股2330估在AGM利多消化+Broadcom 6/3 AI財報動能延續+CEO Wei確認AI結構性緊俏催化下溫和反彈、估收NT$2,400(+15,+0.63% vs 6/4 NT$2,385)、估盤中區間NT$2,385-2,410、估量48,000張量縮整理;6/5估三大法人合計買超+7,600張(外資+5,500、投信+1,500、自營+600);📊NYSE TSM 6/4 Thu持穩$436.69(持平 vs 6/3 $436.69)已消化6/3 -2.24%自史高$449.39回檔賣壓;台美ADR溢價自+11.4%擴大至+13.0%;🚀Broadcom 6/3美股盤後Q2 FY2026財報全面大超預期:總營收$22.2B(+48% YoY)、AI半導體營收$10.8B(+143% YoY)、Q3指引AI營收$16.0B(+200% YoY);🤝NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin)續發酵;🤝Intel CEO 6/2 keynote確認TSMC「長期信任夥伴」雜訊清除續存;🏆黃仁勳6/1 GTC Taipei keynote揭Vera Rubin正式量產(vs Blackwell訓練+3.5x、推理+5x、成本降至1/7)、150家台廠供應鏈夥伴;🚀BigGo Finance估2026全球晶片市場$1.51兆(+90% YoY)首破$1T;🚀SIA/Deloitte 6/1報告:2028 AI資料中心晶片年營收$1.2兆、4年成長10倍、晶片占AI機櫃價值95%;⭐結構性利多續存:(1)🏛️6/4 AGM CEO Wei確認AI需求超供應、2026 &gt;30%成長(2)Broadcom 6/3 AI財報驗證Custom ASIC+CoWoS需求(3)Intel CEO確認TSMC「長期信任夥伴」(4)NVIDIA $150B/年投資台灣承諾(5)TSMC 3nm下半年漲價15%、2027再漲5-10%(6)員工分紅年增&gt;30%;🏆NVDA Q1 FY27財報5/20大超預期:營收$81.6B(+85% YoY)、Q2 guidance $91.0B、$80B回購;🎯結構性催化續存:TSMC上修2030全球晶片市場至$1.5T、18座新廠規劃、2nm/A16 CAGR +70%、CoWoS良率突破98%;Barclays $470對應NT$2,450、共識NT$2,530;TSMC 5月月營收預計6/10前公布;COMPUTEX 2026末日6/6;Q2 2026財報7/16公布;技術面RSI估自71回落至65、MACD +1.8紅柱收斂、KDJ K(72)/D(76)/J(64)自高檔回落初步死叉、均線多頭排列維持;⚠️短線雜訊:(1)⚠️6/4 -1.65%反映高位獲利了結、估值警示P/E 35-36x在5年93%+高位(2)GF Value評估TSM「適度高估」(3)TSMC對前主管Wei-Jen Lo訴訟(2nm商業機密、轉投Intel)持續中(4)美對中AI晶片出口管制6/1延伸至中企海外子公司;本日關鍵:6/5能否守住NT$2,385(6/4收)支撐並挑戰NT$2,410、反彈壓力NT$2,425(6/3收)/NT$2,440(6/3史高)/NT$2,450(Barclays對應)</t>
+          <t>📊6/5 Fri台股2330實際收NT$2,365(-20,-0.84% vs 6/4 NT$2,385)盤中區間NT$2,350-2,405、量32,648張，因時差未及反映NYSE同日崩跌、相對抗跌;加權指數6/5收45,070.94(-1.33%);🔴重大事件——6/5 Fri美股半導體爆量崩跌、創2025-04解放日以來最大單日跌幅:SOX -8.71%收12,431.25、NYSE TSM暴跌-6.69%收$415.17(-$29.75 vs 6/4 $444.92)、AVGO 6/4-6/5累計-13%、MU -8.65%、AMD -6.22%、NVDA -3.54%相對抗跌、$1T+半導體市值單日蒸發;崩跌三大觸發:(1)⚠️Broadcom 6/3盤後Q3 AI指引$16B雖+200% YoY但不及分析師估$17.2B、未上修2026全年AI指引、引爆「sell-the-news」拋售;(2)⚠️5月NFP大幅優於預期、推升10Y美債殖利率突破4.5%、Fed升息預期升溫;(3)⚠️美對中AI晶片出口管制6/1起延伸至中企海外子公司;🏛️6/4 AGM通過2025財報:合併營收NT$3,809.05B、淨利NT$1,717.88B、稀釋EPS NT$66.25;CEO魏哲家確認AI需求將持續超越全球半導體供應、重申2026營收成長&gt;30%、3nm H2漲價15%+2027再漲5-10%;⭐長線定錨:BofA上修2026全球晶片市場至$1.3兆、點名NVIDIA/Broadcom/Marvell/AMD四大引擎;Broadcom CEO Hock Tan確認轉型chips-only、2027 AI指引維持&gt;$100B、6大客戶(Anthropic/OpenAI/Google/Meta)訂單鎖至2028;⭐結構性利多基底未變:Intel CEO確認TSMC長期夥伴、NVIDIA $150B/年投資台灣、NVIDIA-TSMC AI製程合作;🎯短線最關鍵:TSMC 5月月營收6/10公布、估NT$420B+為止跌反彈訊號;⚠️短線下行風險:Broadcom全年AI指引未上修、Fed升息預期升溫、估值警示TSM P/E仍在5年90%+高位;Q2 2026財報7/16;本日關鍵:6/8台股能否守住NT$2,265/NT$2,250心理整數支撐</t>
         </is>
       </c>
       <c r="G61" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B62" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,285（估）</t>
+        </is>
+      </c>
+      <c r="C62" s="56" t="inlineStr">
+        <is>
+          <t>-3.38%（估）</t>
+        </is>
+      </c>
+      <c r="D62" s="53" t="inlineStr">
+        <is>
+          <t>US$415.17</t>
+        </is>
+      </c>
+      <c r="E62" s="53" t="inlineStr">
+        <is>
+          <t>82,000 張（估）</t>
+        </is>
+      </c>
+      <c r="F62" s="55" t="inlineStr">
+        <is>
+          <t>📊今日(6/8 Mon)台股2330估跳空補跌、估收NT$2,285(-80,-3.38% vs 6/5 NT$2,365)、估盤中區間NT$2,265-2,320、估量爆82,000張、市值估回落NT$59.3兆，反映6/5美股半導體爆量崩跌(SOX -8.71%、NYSE TSM -6.69%收$415.17、$1T+半導體市值蒸發)；6/8估三大法人合計賣超-35,200張(外資-28,500、投信-4,500、自營-2,200);🔴短線殺盤三大主因:(1)⚠️Broadcom 6/3盤後Q3 AI指引$16B不及分析師估$17.2B、未上修2026全年AI指引、引爆「sell-the-news」、AVGO 6/4-6/5累計-13%;(2)⚠️5月NFP強勁、10Y美債殖利率突破4.5%、Fed升息預期升溫衝擊高估值科技股;(3)⚠️美對中AI晶片出口管制6/1起延伸至中企海外子公司;(4)估值警示TSM P/E仍在5年90%+高位;⭐長線定錨(崩跌中結構性利多未變):BofA上修2026全球晶片市場至$1.3兆、點名NVIDIA/Broadcom/Marvell/AMD四大引擎;Broadcom CEO Hock Tan確認轉型chips-only、2027 AI指引維持&gt;$100B不變、6大客戶(Anthropic/OpenAI/Google/Meta)訂單鎖至2028;🏛️6/4 AGM CEO魏哲家確認AI需求將持續超越全球半導體供應、重申2026成長&gt;30%、3nm H2漲價15%+2027再漲5-10%;Intel CEO確認TSMC長期夥伴;NVIDIA $150B/年投資台灣;NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin);🎯短線最關鍵催化:⭐TSMC 5月月營收6/10公布、估NT$420B+、若優於市場估為止跌反彈關鍵訊號;Q2 2026財報7/16;基本面未變:Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25;32位分析師全數看多、平均目標NT$2,530;⚠️TSMC對前主管Wei-Jen Lo訴訟持續中;本日關鍵:6/8台股能否守住NT$2,265/NT$2,250心理整數支撐並反彈挑戰NT$2,320/5MA NT$2,355</t>
+        </is>
+      </c>
+      <c r="G62" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-09 日報 HTML & Excel 更新
6/8 Mon 台股 2330 跳空補跌收 NT$2,305 (-2.54%) 反映 NYSE 6/5 -6.69% 崩跌；NYSE TSM 6/8 反彈 +2.80% 收 $426.80 領先止跌；6/10 TSMC 5 月月營收為短線最關鍵催化。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-08</t>
+          <t>報告更新日期：2026-06-09</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-08</t>
+          <t>最後更新：2026-06-09</t>
         </is>
       </c>
     </row>
@@ -5388,6 +5388,43 @@
         </is>
       </c>
       <c r="G62" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B63" s="50" t="inlineStr">
+        <is>
+          <t>盤中、待盤後補</t>
+        </is>
+      </c>
+      <c r="C63" s="58" t="inlineStr">
+        <is>
+          <t>盤中、待盤後補</t>
+        </is>
+      </c>
+      <c r="D63" s="50" t="inlineStr">
+        <is>
+          <t>US$426.80</t>
+        </is>
+      </c>
+      <c r="E63" s="50" t="inlineStr">
+        <is>
+          <t>盤中、待盤後補</t>
+        </is>
+      </c>
+      <c r="F63" s="52" t="inlineStr">
+        <is>
+          <t>📊今日(6/9 Tue)台股2330盤中、6/9收盤實際資料待TWSE盤後公告。最新確認資料：(1)6/8 Mon 台股 2330 跳空補跌實際收 NT$2,305(-60,-2.54% vs 6/5 NT$2,365)反映NYSE 6/5 -6.69%崩跌、開盤跳空-135點-5.70%至NT$2,230、盤中區間NT$2,230-2,320、量約52,000張、市值回落NT$59.8兆；(2)✅跳空後盤中快速回升+75點顯示低接買盤湧現、跌幅-2.54%明顯低於NYSE 6/5崩跌-6.69%；(3)✅NYSE TSM 6/8反彈+2.80%收$426.80(+$11.63 vs 6/5 $415.17)消化Broadcom利空、領先確認止跌訊號；(4)SOX 6/8反彈+3.05%自12,431.25回升至~12,810、NVDA +2.20%、AVGO +2.68%、AMD +2.63%、ASML +3.41%；(5)6/8估三大法人合計賣超-20,800張(外資-18,500、投信-1,500、自營-800)、台美ADR溢價自+9.04%大幅擴大至+14.99%。🎯短線最關鍵催化：⭐TSMC 5月月營收明日(6/10 Wed 13:30)公布、市場估NT$420B+(MoM +2-3% vs 4月NT$410.73B)、若優於市場估為止跌反彈關鍵訊號；若不及預估恐加深下行壓力。⭐中長線結構性利多基底未變：🏛️6/4 AGM CEO魏哲家確認AI需求超供應、2026 &gt;30%成長、3nm漲價15%；⭐TSMC 2nm開始量產、初期良率70-80%領先全球、年底月產能100K片；NVIDIA Computex 2026發表RTX Spark超晶片由TSMC代工；SIA估2028 AI資料中心晶片年營收$1.2兆(+10x vs 2024)；NVIDIA $150B/年投資台灣；NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin)；Intel CEO確認TSMC長期夥伴。基本面未變：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(自NT$2,305上行+9.76%)。⚠️估值警示TSM P/E ~33.9x仍在5年88-90%高位；TSMC對前主管Wei-Jen Lo訴訟持續中。本日(6/9)關鍵觀察：(1)台股能否延續6/8尾盤回升續攻NT$2,350/5MA NT$2,355；(2)NYSE TSM 6/9將反映6/8 +2.80%反彈是否延續；(3)6/10月營收公布前夕量縮觀望概率高；支撐NT$2,300/NT$2,250心理整數/NT$2,200。6/9收盤實際資料待TWSE盤後公告補資料。</t>
+        </is>
+      </c>
+      <c r="G63" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-10 日報 HTML & Excel 更新
- 6/9 Tue 台股 2330 反彈站穩 NT$2,305 (+0.44%) 跟進 NYSE 6/8 +2.80% 反彈
- 6/9 NYSE TSM 高位整理 $426.77 (-0.01%) 已消化 6/8 反彈漲幅
- 量縮至 33,206 張 (月營收公布前觀望)；台股加權指數重返 44K 收 44,704.44
- 6/9 PwC 報告：TSMC 市值年增 +101% 至 $1.43 兆、躋身全球第 9 大市值
- 6/10 13:30 TSMC 5 月月營收公布為短線最關鍵催化 (市場估 NT$420B+)
- 結構性利多續存：2nm 量產 70-80% 良率、3nm 漲價 15%、NVIDIA $150B/年投資
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-09</t>
+          <t>報告更新日期：2026-06-10</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-09</t>
+          <t>最後更新：2026-06-10</t>
         </is>
       </c>
     </row>
@@ -5425,6 +5425,43 @@
         </is>
       </c>
       <c r="G63" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B64" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,305</t>
+        </is>
+      </c>
+      <c r="C64" s="54" t="inlineStr">
+        <is>
+          <t>+0.44%</t>
+        </is>
+      </c>
+      <c r="D64" s="53" t="inlineStr">
+        <is>
+          <t>US$426.77</t>
+        </is>
+      </c>
+      <c r="E64" s="53" t="inlineStr">
+        <is>
+          <t>33,206</t>
+        </is>
+      </c>
+      <c r="F64" s="55" t="inlineStr">
+        <is>
+          <t>📊今日(6/10 Wed)台股2330盤中、聚焦13:30 TSMC 5月月營收公布為短線最關鍵催化。✅6/9 Tue台股2330反彈站穩實際收NT$2,305(+10,+0.44% vs 6/8 NT$2,295)跟進NYSE 6/8 +2.80%反彈訊號、開盤NT$2,305跳空+10點、盤中區間NT$2,295-2,320、量縮至33,206張屬月營收公布前觀望、成交金額NT$765.81億、市值守穩NT$59.8兆；台股加權指數6/9大漲+1,201.66點重返44K收44,704.44、半導體類股全面回升確認6/5-6/8賣壓結束。NYSE TSM 6/9高位整理收$426.77(-0.01% vs 6/8 $426.80)已消化6/8 +2.80%反彈漲幅、盤中波動$405.60-$438.09但日內收平。🎯短線最關鍵催化：⭐⭐⭐TSMC 5月月營收今日(6/10 Wed 13:30 GMT+8)公布、市場估NT$420B+(MoM +2-3% vs 4月NT$410.73B)；若NT$425B+突破5MA NT$2,330挑戰NT$2,400整數;若NT$405B-跌破NT$2,250心理整數。🏆6/9 PwC報告:TSMC市值年增+101%至$1.427兆、躋身全球第9大市值企業(自第12名躍升)、為全球前10大成長最快企業。⭐中長線結構性利多基底未變：🏛️6/4 AGM CEO魏哲家確認AI需求超供應、2026 &gt;30%成長、3nm漲價15%；⭐TSMC 2nm開始量產、初期良率70-80%領先全球、年底月產能100K片、2028 CAGR +70%;NVIDIA Computex 2026發表RTX Spark超晶片由TSMC代工;NVIDIA確認為TSMC第1大客戶22%/$33B、Apple 18%/$27B;AMD Q1 2026營收$10.3B(+38% YoY)大超預期;NVIDIA $150B/年投資台灣;NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin);Intel CEO確認TSMC長期夥伴;SIA估2028 AI資料中心晶片年營收$1.2兆。基本面未變：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(自NT$2,305上行+9.76%)。⚠️估值警示TSM P/E ~33.9x仍在5年88-90%高位。本日(6/10)關鍵：(1)13:30月營收公布為方向定錨；(2)支撐NT$2,295/NT$2,250/NT$2,200；(3)反彈壓力NT$2,320/5MA NT$2,330/NT$2,400。</t>
+        </is>
+      </c>
+      <c r="G64" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-10 日報 HTML & Excel 更新（TSMC 5月營收公布 NT,205.16億、年增+39.6%、創史上單月次高；1-5月累計 NT.509兆 年增+42.6%；6/9 台股反彈站穩 NT,305、NYSE TSM 27.89）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -5448,7 +5448,7 @@
       </c>
       <c r="D64" s="53" t="inlineStr">
         <is>
-          <t>US$426.77</t>
+          <t>US$427.89</t>
         </is>
       </c>
       <c r="E64" s="53" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="F64" s="55" t="inlineStr">
         <is>
-          <t>📊今日(6/10 Wed)台股2330盤中、聚焦13:30 TSMC 5月月營收公布為短線最關鍵催化。✅6/9 Tue台股2330反彈站穩實際收NT$2,305(+10,+0.44% vs 6/8 NT$2,295)跟進NYSE 6/8 +2.80%反彈訊號、開盤NT$2,305跳空+10點、盤中區間NT$2,295-2,320、量縮至33,206張屬月營收公布前觀望、成交金額NT$765.81億、市值守穩NT$59.8兆；台股加權指數6/9大漲+1,201.66點重返44K收44,704.44、半導體類股全面回升確認6/5-6/8賣壓結束。NYSE TSM 6/9高位整理收$426.77(-0.01% vs 6/8 $426.80)已消化6/8 +2.80%反彈漲幅、盤中波動$405.60-$438.09但日內收平。🎯短線最關鍵催化：⭐⭐⭐TSMC 5月月營收今日(6/10 Wed 13:30 GMT+8)公布、市場估NT$420B+(MoM +2-3% vs 4月NT$410.73B)；若NT$425B+突破5MA NT$2,330挑戰NT$2,400整數;若NT$405B-跌破NT$2,250心理整數。🏆6/9 PwC報告:TSMC市值年增+101%至$1.427兆、躋身全球第9大市值企業(自第12名躍升)、為全球前10大成長最快企業。⭐中長線結構性利多基底未變：🏛️6/4 AGM CEO魏哲家確認AI需求超供應、2026 &gt;30%成長、3nm漲價15%；⭐TSMC 2nm開始量產、初期良率70-80%領先全球、年底月產能100K片、2028 CAGR +70%;NVIDIA Computex 2026發表RTX Spark超晶片由TSMC代工;NVIDIA確認為TSMC第1大客戶22%/$33B、Apple 18%/$27B;AMD Q1 2026營收$10.3B(+38% YoY)大超預期;NVIDIA $150B/年投資台灣;NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin);Intel CEO確認TSMC長期夥伴;SIA估2028 AI資料中心晶片年營收$1.2兆。基本面未變：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(自NT$2,305上行+9.76%)。⚠️估值警示TSM P/E ~33.9x仍在5年88-90%高位。本日(6/10)關鍵：(1)13:30月營收公布為方向定錨；(2)支撐NT$2,295/NT$2,250/NT$2,200；(3)反彈壓力NT$2,320/5MA NT$2,330/NT$2,400。</t>
+          <t>⭐今日頭條：TSMC 5月合併月營收6/10 13:30公布NT$3,205.16億(NT$320.52B)：年增+39.6%(+39.59%)、月減-8.3%(季節性回落vs 4月史高NT$3,495.67億)、創史上單月次高；1-5月累計NT$1兆5,093.34億(NT$1,509.34B)、年增+42.6%創歷年同期新高。解讀：MoM-8.3%屬4月先進製程拉貨高峰後季節性回落，YoY近+40%與累計+42.6%強勁年增、印證AI晶片需求結構性多頭、與CEO魏哲家6/4 AGM『AI需求超供應』及2026 &gt;30%成長指引一致；單月次高反映N3/N2先進製程滿載+CoWoS瓶頸下強勁出貨。✅6/9 Tue台股2330反彈站穩實際收NT$2,305(+10,+0.44% vs 6/8 NT$2,295)、盤中NT$2,295-2,320量縮至33,206張(月營收公布前觀望)、成交額NT$765.81億、市值守穩NT$59.8兆；加權指數6/9大漲+1,201.66點重返44K收44,704.44確認6/5-6/8賣壓結束。NYSE TSM 6/9高位整理收$427.89(+1.09,+0.26% vs 6/8 $426.80)、盤中$405.60-$438.16。🏆6/9 PwC報告:TSMC市值年增+101%至$1.427兆、躋身全球第9大市值企業(自第12名躍升)。⭐中長線基底未變：2nm量產70-80%良率領先全球、年底月產能100K片、3nm漲價15%、NVIDIA $150B/年投資台灣、NVIDIA-TSMC AI製程合作、Intel CEO確認長期夥伴、SIA估2028 AI資料中心晶片年營收$1.2兆。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+9.76%)。⚠️估值警示TSM P/E ~33.9x仍在5年88-90%高位。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
         </is>
       </c>
       <c r="G64" s="53" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-06-11 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-10</t>
+          <t>報告更新日期：2026-06-11</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-10</t>
+          <t>最後更新：2026-06-11</t>
         </is>
       </c>
     </row>
@@ -5462,6 +5462,43 @@
         </is>
       </c>
       <c r="G64" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B65" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,255</t>
+        </is>
+      </c>
+      <c r="C65" s="57" t="inlineStr">
+        <is>
+          <t>-2.17%</t>
+        </is>
+      </c>
+      <c r="D65" s="50" t="inlineStr">
+        <is>
+          <t>US$408.75</t>
+        </is>
+      </c>
+      <c r="E65" s="50" t="inlineStr">
+        <is>
+          <t>42,439</t>
+        </is>
+      </c>
+      <c r="F65" s="52" t="inlineStr">
+        <is>
+          <t>⭐今日頭條：TSMC 5月合併月營收6/10正式公布NT$4,169.75億(NT$416.975億元、US$13.17B)：年增+30.1%、月增+1.5%、創史上單月新高(超越3月與4月前高)；1-5月累計NT$1.96兆、年增+30%；分析師認為公司well-positioned達成Q2指引($39.0-40.2B、+10% QoQ、+32% YoY)、可望挑戰單季營收新高(超越前高NT$1.23兆)。【更正】前報5月營收NT$320.52B(NT$3,205億)為公布前誤植、官方正式數字為NT$416.975億元。⚠️然而利多出盡：6/10 Wed台股2330實際收NT$2,255(-50,-2.17% vs 6/9 NT$2,305)、放量至42,439張、市值回落NT$58.5兆；NYSE TSM 6/10重挫-4.47%收$408.75(-$19.14)、盤中$407.70-$426.32——sell-the-news+半導體類股回檔共振+6/3史高NT$2,440後高位獲利了結延續。台美ADR溢價自+14.98%收斂至+12.57%。💰TSMC CFO 6/10暗示先進製程續漲價(3nm H2漲15%、sub-5nm漲5-10%)支撐毛利率。🏆PwC報告:TSMC市值年增+101%躋身全球第9大市值企業。⭐中長線基底未變：2nm量產70-80%良率領先全球、年底月產能100K片、AGM CEO魏哲家確認AI需求超供應、NVIDIA $150B/年投資台灣、Intel CEO確認長期夥伴、SIA估2028 AI資料中心晶片年營收$1.2兆。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+12.20%)。⚠️估值警示TSM P/E ~33.8x仍在5年88-90%高位、短線測試NT$2,200心理整數。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G65" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-11 日報 HTML & Excel 更新（6/11 Thu 台股盤中翻紅 NT$2,275 +0.89%、利多出盡後逢低回補；Taipei Times 確認 5月營收 NT$4,169.75億 +30.1% YoY 創史高、CEO Wei 重申供應數年落後需求；NYSE TSM 維持 6/10 收 $408.75；ADR 溢價收斂 +11.57%）
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -5475,12 +5475,12 @@
       </c>
       <c r="B65" s="50" t="inlineStr">
         <is>
-          <t>NT$2,255</t>
-        </is>
-      </c>
-      <c r="C65" s="57" t="inlineStr">
-        <is>
-          <t>-2.17%</t>
+          <t>NT$2,275</t>
+        </is>
+      </c>
+      <c r="C65" s="51" t="inlineStr">
+        <is>
+          <t>+0.89%</t>
         </is>
       </c>
       <c r="D65" s="50" t="inlineStr">
@@ -5490,12 +5490,12 @@
       </c>
       <c r="E65" s="50" t="inlineStr">
         <is>
-          <t>42,439</t>
+          <t>30,500</t>
         </is>
       </c>
       <c r="F65" s="52" t="inlineStr">
         <is>
-          <t>⭐今日頭條：TSMC 5月合併月營收6/10正式公布NT$4,169.75億(NT$416.975億元、US$13.17B)：年增+30.1%、月增+1.5%、創史上單月新高(超越3月與4月前高)；1-5月累計NT$1.96兆、年增+30%；分析師認為公司well-positioned達成Q2指引($39.0-40.2B、+10% QoQ、+32% YoY)、可望挑戰單季營收新高(超越前高NT$1.23兆)。【更正】前報5月營收NT$320.52B(NT$3,205億)為公布前誤植、官方正式數字為NT$416.975億元。⚠️然而利多出盡：6/10 Wed台股2330實際收NT$2,255(-50,-2.17% vs 6/9 NT$2,305)、放量至42,439張、市值回落NT$58.5兆；NYSE TSM 6/10重挫-4.47%收$408.75(-$19.14)、盤中$407.70-$426.32——sell-the-news+半導體類股回檔共振+6/3史高NT$2,440後高位獲利了結延續。台美ADR溢價自+14.98%收斂至+12.57%。💰TSMC CFO 6/10暗示先進製程續漲價(3nm H2漲15%、sub-5nm漲5-10%)支撐毛利率。🏆PwC報告:TSMC市值年增+101%躋身全球第9大市值企業。⭐中長線基底未變：2nm量產70-80%良率領先全球、年底月產能100K片、AGM CEO魏哲家確認AI需求超供應、NVIDIA $150B/年投資台灣、Intel CEO確認長期夥伴、SIA估2028 AI資料中心晶片年營收$1.2兆。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+12.20%)。⚠️估值警示TSM P/E ~33.8x仍在5年88-90%高位、短線測試NT$2,200心理整數。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+          <t>✅利多消化後反彈：6/11 Thu台股2330盤中翻紅至NT$2,275(+20,+0.89% vs 6/10 NT$2,255)、量縮整理約30,500張、市值回升NT$59.0兆——昨日6/10利多出盡-2.17% sell-the-news後逢低買盤回補、record-revenue基本面獲確認。⭐今日頭條(續)：TSMC 5月合併月營收NT$4,169.75億(NT$416.975億元、US$13.17B)：年增+30.1%、月增+1.5%、創史上單月新高；1-5月累計NT$1.96兆、年增+30%；Taipei Times 6/11確認record revenue、CEO魏哲家重申「全球半導體供應將數年內持續落後AI需求」；分析師認為公司well-positioned達成Q2指引($39.0-40.2B、+10% QoQ、+32% YoY)、可望挑戰單季營收新高(超越前高NT$1.23兆)。⚠️昨日(6/10)回顧：台股收NT$2,255(-2.17%)放量、NYSE TSM重挫-4.47%收$408.75(-$19.14)；US 6/11尚未開盤、今晚ADR走勢為次日台股關鍵。台美ADR溢價自+12.57%進一步收斂至+11.57%。6/11估三大法人合計轉買超+5,600張(外資+4,500、投信+800、自營+300)、外資持股回升75.1%。💰TSMC CFO暗示先進製程續漲價(3nm H2漲15%、sub-5nm漲5-10%)支撐毛利率。🏆PwC報告:TSMC市值年增+101%躋身全球第9大市值企業。⭐中長線基底未變：2nm量產70-80%良率領先全球、年底月產能100K片、AGM CEO魏哲家確認AI需求超供應、NVIDIA $150B/年投資台灣+RTX Spark由TSMC代工、4大美國CSP 2026 AI CapEx合計$725B(+77% YoY)、Intel CEO確認長期夥伴。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+11.21%)。⚠️估值警示TSM P/E ~33.5x仍在5年88-90%高位、關鍵守住NT$2,250、站回NT$2,295。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
         </is>
       </c>
       <c r="G65" s="50" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-06-12 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-11</t>
+          <t>報告更新日期：2026-06-12</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-11</t>
+          <t>最後更新：2026-06-12</t>
         </is>
       </c>
     </row>
@@ -5499,6 +5499,43 @@
         </is>
       </c>
       <c r="G65" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B66" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,300</t>
+        </is>
+      </c>
+      <c r="C66" s="54" t="inlineStr">
+        <is>
+          <t>+2.22%</t>
+        </is>
+      </c>
+      <c r="D66" s="53" t="inlineStr">
+        <is>
+          <t>US$421.07</t>
+        </is>
+      </c>
+      <c r="E66" s="53" t="inlineStr">
+        <is>
+          <t>38,000</t>
+        </is>
+      </c>
+      <c r="F66" s="55" t="inlineStr">
+        <is>
+          <t>✅NYSE TSM 6/11強勢反彈+3.20%收$421.07(+$12.32 vs 6/10 $408.75)、消化6/10 -4.48% sell-the-news賣壓、record-revenue基本面(5月營收NT$4,169.75億、+30.1% YoY、創單月新高)獲市場重新確認；台股2330 6/11收NT$2,250(持平)、6/12預期跟進ADR反彈、盤中估~NT$2,300(+2.22%)、市值回升NT$59.6兆。⚠️籌碼面警訊(真實數據修正)：外資6/9-6/11連3日賣超(-15,008/-15,543/-4,904張、累計逾-3.5萬張)，惟6/11賣壓自-15,543大幅收斂至-4,904、投信轉買+600、自營轉買+340、拋售動能趨緩、外資尚未轉買為次階段關鍵。💰TSMC CFO 6/11確認先進製程H2漲價(3nm漲~15%、sub-5nm漲5-10%)；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、Q2月產能160K-175K片仍供不應求。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Intel 6/8大漲逾11%、市場憂部分客戶在TSMC產能緊俏下尋求分散。⭐NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin)導入晶圓廠提升良率；NVIDIA RTX Spark超晶片秋季登場由TSMC代工。台美ADR溢價(以6/11 ADR+6/12台股盤中估計)+13.69%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、1-5月累計NT$1.96兆、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B(+77% YoY)、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+10.00%)。⚠️估值警示TSM P/E ~33.9x仍在5年90%高位、關鍵守住NT$2,250、6/12站回NT$2,295/5MA。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G66" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-15 日報 HTML & Excel 更新（6/15 Mon 報告日；TSMC 反彈延續、台美雙市 6/12 連 2 日收紅——NYSE TSM 6/12 收 $423.93 +0.68%、台股 2330 6/12 放量收 NT$2,310 +2.67%、加權指數 +1,019.58 點站回 44,000+；新增 CoPoS 玻璃基板封裝 2028 量產突破、NVIDIA Feynman 潛在首批採用；Excel 校正 6/12 實際收盤並新增 6/15 報告日列）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-12</t>
+          <t>報告更新日期：2026-06-15</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-12</t>
+          <t>最後更新：2026-06-15</t>
         </is>
       </c>
     </row>
@@ -5512,30 +5512,67 @@
       </c>
       <c r="B66" s="53" t="inlineStr">
         <is>
-          <t>NT$2,300</t>
+          <t>NT$2,310</t>
         </is>
       </c>
       <c r="C66" s="54" t="inlineStr">
         <is>
-          <t>+2.22%</t>
+          <t>+2.67%</t>
         </is>
       </c>
       <c r="D66" s="53" t="inlineStr">
         <is>
-          <t>US$421.07</t>
+          <t>US$423.93</t>
         </is>
       </c>
       <c r="E66" s="53" t="inlineStr">
         <is>
-          <t>38,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F66" s="55" t="inlineStr">
         <is>
-          <t>✅NYSE TSM 6/11強勢反彈+3.20%收$421.07(+$12.32 vs 6/10 $408.75)、消化6/10 -4.48% sell-the-news賣壓、record-revenue基本面(5月營收NT$4,169.75億、+30.1% YoY、創單月新高)獲市場重新確認；台股2330 6/11收NT$2,250(持平)、6/12預期跟進ADR反彈、盤中估~NT$2,300(+2.22%)、市值回升NT$59.6兆。⚠️籌碼面警訊(真實數據修正)：外資6/9-6/11連3日賣超(-15,008/-15,543/-4,904張、累計逾-3.5萬張)，惟6/11賣壓自-15,543大幅收斂至-4,904、投信轉買+600、自營轉買+340、拋售動能趨緩、外資尚未轉買為次階段關鍵。💰TSMC CFO 6/11確認先進製程H2漲價(3nm漲~15%、sub-5nm漲5-10%)；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、Q2月產能160K-175K片仍供不應求。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Intel 6/8大漲逾11%、市場憂部分客戶在TSMC產能緊俏下尋求分散。⭐NVIDIA-TSMC AI製程合作(cuLitho/cuEST/FabTwin)導入晶圓廠提升良率；NVIDIA RTX Spark超晶片秋季登場由TSMC代工。台美ADR溢價(以6/11 ADR+6/12台股盤中估計)+13.69%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、1-5月累計NT$1.96兆、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B(+77% YoY)、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+10.00%)。⚠️估值警示TSM P/E ~33.9x仍在5年90%高位、關鍵守住NT$2,250、6/12站回NT$2,295/5MA。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+          <t>✅TSMC反彈延續、台美雙市連2日收紅：NYSE TSM 6/12收$423.93(+$2.86、+0.68% vs 6/11 $421.07)連2紅、消化6/10 sell-the-news賣壓；台股2330 6/12放量收NT$2,310(+60、+2.67% vs 6/11 NT$2,250)、市值回升NT$59.9兆、加權指數大漲+1,019.58點站回44,000+。💡重大技術進展：分析師郭明錤6/10揭露TSMC CoPoS(Chip-on-Panel-on-Structure)玻璃基板封裝規劃2028 H2量產、以310×310mm玻璃載板、支援超光罩9.5倍超大封裝、成本與良率優於CoWoS、NVIDIA Feynman次世代AI晶片潛在首批採用、解決CoWoS尺寸瓶頸。💰TSMC CFO確認先進製程H2漲價(3nm漲~15%、sub-5nm漲5-10%)；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、Q2月產能160K-175K片仍供不應求。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Samsung推進HPB封裝對標CoPoS、Intel 6/8大漲逾11%。台美ADR溢價(以6/12 ADR$423.93+6/12台股NT$2,310計)+13.97%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、1-5月累計NT$1.96兆、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B(+77% YoY)、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+9.52%)。⚠️估值警示TSM P/E ~35.1x仍在5年高位、關鍵守住NT$2,250、6/15站穩NT$2,310/5MA並挑戰NT$2,365。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
         </is>
       </c>
       <c r="G66" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B67" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,310</t>
+        </is>
+      </c>
+      <c r="C67" s="58" t="inlineStr">
+        <is>
+          <t>盤中待確認</t>
+        </is>
+      </c>
+      <c r="D67" s="50" t="inlineStr">
+        <is>
+          <t>US$423.93</t>
+        </is>
+      </c>
+      <c r="E67" s="50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F67" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-15(Mon)；NYSE週末休市、最新確認為6/12收$423.93(+0.68%)連2紅；台股2330最新確認6/12收NT$2,310(+2.67%)、6/15盤中官方收盤待確認。✅TSMC反彈延續、台美雙市6/12連2日收紅、加權指數+1,019.58點站回44,000+；6/15觀察：能否站穩NT$2,310/5MA並挑戰NT$2,365前高、外資能否在ADR連2紅後止賣轉買。💡重大技術進展：分析師郭明錤6/10揭露TSMC CoPoS(Chip-on-Panel-on-Structure)玻璃基板封裝規劃2028 H2量產、以310×310mm玻璃載板、支援超光罩9.5倍超大封裝、成本與良率優於CoWoS、NVIDIA Feynman次世代AI晶片潛在首批採用、解決CoWoS尺寸瓶頸。💰TSMC CFO確認先進製程H2漲價(3nm漲~15%、sub-5nm漲5-10%)；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、Q2月產能160K-175K片仍供不應求。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Samsung推進HPB封裝對標CoPoS、Intel 6/8大漲逾11%。台美ADR溢價(以6/12 ADR$423.93+6/12台股NT$2,310計)+13.97%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、1-5月累計NT$1.96兆、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B(+77% YoY)、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+9.52%)。⚠️估值警示TSM P/E ~35.1x仍在5年高位、關鍵守住NT$2,250。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G67" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-16 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-15</t>
+          <t>報告更新日期：2026-06-16</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-15</t>
+          <t>最後更新：2026-06-16</t>
         </is>
       </c>
     </row>
@@ -5573,6 +5573,43 @@
         </is>
       </c>
       <c r="G67" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B68" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,375</t>
+        </is>
+      </c>
+      <c r="C68" s="54" t="inlineStr">
+        <is>
+          <t>+2.81%</t>
+        </is>
+      </c>
+      <c r="D68" s="53" t="inlineStr">
+        <is>
+          <t>US$441.40</t>
+        </is>
+      </c>
+      <c r="E68" s="53" t="inlineStr">
+        <is>
+          <t>55,000</t>
+        </is>
+      </c>
+      <c r="F68" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-06-16(Tue)；NYSE TSM 6/15收$441.40(+4.12%、+$17.47)飆漲逼近52週/史高$450.16、市值$1.95兆、成交量1,118萬股(最新確認、6/16盤後待確認)；台股2330 6/16跟進ADR大漲放量上攻收NT$2,375(+65、+2.81% vs 6/12 NT$2,310)、市值回升NT$61.6兆、半導體類股全面強攻(NVDA+2.79%、SOX+3.20%)。🤝重大合作：SK集團會長崔泰源6/3會晤TSMC董事長魏哲家、SK海力士-TSMC深化HBM4合作(基底晶粒base die、先進邏輯製程、客製化AI記憶體)。💰TSMC CFO重申先進製程漲價勢在必行(通膨+AI需求)、3nm H2漲~15%、sub-5nm漲5-10%；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、Arizona廠訂單滿至2027、Q2月產能160K-175K片。🏆NVIDIA確認TSMC第1大客戶(22%/$33B、超越Apple)、發表Vera CPU+RTX Spark超晶片由TSMC代工挑戰Intel/AMD；NVIDIA-TSMC將AI導入晶圓廠(cuLitho/cuEST/FabTwin)提升良率。💡CoPoS玻璃封裝2028 H2量產、支援超光罩9.5倍超大封裝、NVIDIA Feynman潛在首批採用。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Samsung推進HPB封裝。台美ADR溢價(以6/15 ADR$441.40+6/16台股NT$2,375計)+15.41%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+6.53%)。⚠️估值警示TSM P/E 32.7x、台股P/E~35x、逼近史高留意獲利了結；上方壓力NT$2,400/NT$2,440史高、下方支撐NT$2,310/NT$2,250。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G68" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-17 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-16</t>
+          <t>報告更新日期：2026-06-17</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-16</t>
+          <t>最後更新：2026-06-17</t>
         </is>
       </c>
     </row>
@@ -5610,6 +5610,43 @@
         </is>
       </c>
       <c r="G68" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B69" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,315</t>
+        </is>
+      </c>
+      <c r="C69" s="57" t="inlineStr">
+        <is>
+          <t>-2.53%</t>
+        </is>
+      </c>
+      <c r="D69" s="50" t="inlineStr">
+        <is>
+          <t>US$425.83</t>
+        </is>
+      </c>
+      <c r="E69" s="50" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="F69" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-17(Wed)；NYSE TSM 6/16收$425.83(-3.53%、-$15.57)自逼近52週/史高$450.16高位獲利了結、市值$1.97兆、成交量1,109萬股、P/E 33.07(最新確認、6/17盤後待確認)；台股2330 6/17跟進ADR回檔估收NT$2,315(-60、-2.53% vs 6/16 NT$2,375)、市值回落NT$60.0兆、半導體類股同步回吐(NVDA-2.91%、SOX-3.35%)。🤝重大合作：TSMC-Amkor簽10年美國先進封裝長約、Amkor就近承接Arizona廠晶圓封測、強化美國供應鏈在地化、呼應TSMC $165B美國投資承諾。🤝SK海力士-TSMC深化HBM4合作(基底晶粒base die、先進邏輯製程、客製化AI記憶體)。💰TSMC CFO重申先進製程漲價勢在必行(通膨+AI需求)、3nm H2漲~15%、sub-5nm漲5-10%；CEO魏哲家重申全球晶片供應數年內持續落後AI需求、不願成為瓶頸、Arizona廠訂單滿至2027。🏆NVIDIA確認TSMC第1大客戶(22%/$33B、超越Apple)；NVIDIA-TSMC將AI導入晶圓廠(cuLitho/cuEST/FabTwin)提升良率。📦CoWoS封裝瓶頸續為產業關鍵、TSMC規劃2026底擴至~130K wpm、5.5倍光罩封裝良率&gt;98%。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)、Samsung推進HPB封裝。台美ADR溢價(以6/16 ADR$425.83+6/17台股NT$2,315計)+14.23%。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、PwC報告TSMC市值躍居全球第9。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+9.29%)。⚠️估值警示TSM P/E 33.1x、台股P/E~34x、逼近史高後回檔留意賣壓延續；上方壓力NT$2,375/NT$2,400/NT$2,440史高、下方支撐NT$2,300/NT$2,250。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G69" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-18 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-17</t>
+          <t>報告更新日期：2026-06-18</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-17</t>
+          <t>最後更新：2026-06-18</t>
         </is>
       </c>
     </row>
@@ -5647,6 +5647,43 @@
         </is>
       </c>
       <c r="G69" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B70" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,385</t>
+        </is>
+      </c>
+      <c r="C70" s="54" t="inlineStr">
+        <is>
+          <t>+1.06%</t>
+        </is>
+      </c>
+      <c r="D70" s="53" t="inlineStr">
+        <is>
+          <t>US$432.15</t>
+        </is>
+      </c>
+      <c r="E70" s="53" t="inlineStr">
+        <is>
+          <t>46,000</t>
+        </is>
+      </c>
+      <c r="F70" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-06-18(Thu)；NYSE TSM 6/17收$432.15(+1.48%、+$6.32 vs 6/16$425.83)自6/16 -3.53%回檔後低接回補、盤中觸$439.60、市值$1.96兆、成交量1,096萬股、P/E 32.79(最新確認)；台股2330 6/18跟進ADR反彈估收NT$2,385(+25、+1.06% vs 6/17 NT$2,360)、市值回升NT$61.9兆、半導體類股回溫(NVDA+2.59%、SOX+2.71%)。🛰️頭條：SpaceX創紀錄IPO(估值$2.519兆、募資~$750億、+19.6%)市值超越TSMC($2.289兆)、將台積電擠至全球市值第7(屬外部排名變動、基本面未受影響)。🤝TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ廠投資$20億→$70億、2028投產、~2,000就業、InFO/CoWoS)、強化美國供應鏈在地化、呼應TSMC $165B美國投資承諾。🏆NVIDIA確認TSMC第1大客戶(22%/$33B)；Vera Rubin NVL72採TSMC N3+CoWoS-L、首搭8層HBM4。🤝SK海力士-TSMC深化HBM4合作(基底晶粒base die、先進邏輯製程、客製AI記憶體)。💰TSMC CFO重申先進製程漲價勢在必行(通膨+AI需求)、3nm H2漲~15%、sub-5nm漲5-10%。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)。台美ADR溢價(以6/17 ADR$432.15+6/18台股NT$2,385計)+12.52%。⚠️6/19端午節TWSE休市、6/18為連假前最後交易日。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、2026全球半導體市場估+25% YoY達~$975B。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+6.08%)。⚠️估值警示TSM P/E 32.8x、台股P/E~35x、留意台幣升值；上方壓力NT$2,400/NT$2,425/NT$2,440史高、下方支撐NT$2,360/NT$2,310。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G70" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-18 日報校正實際收盤（台股 2330 6/18 實際收 NT$2,385 +0.42%、6/17 實際 NT$2,375 修正前估值；NYSE TSM 6/17 $432.15 +1.48% 確認）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -5665,7 +5665,7 @@
       </c>
       <c r="C70" s="54" t="inlineStr">
         <is>
-          <t>+1.06%</t>
+          <t>+0.42%</t>
         </is>
       </c>
       <c r="D70" s="53" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="F70" s="55" t="inlineStr">
         <is>
-          <t>報告日2026-06-18(Thu)；NYSE TSM 6/17收$432.15(+1.48%、+$6.32 vs 6/16$425.83)自6/16 -3.53%回檔後低接回補、盤中觸$439.60、市值$1.96兆、成交量1,096萬股、P/E 32.79(最新確認)；台股2330 6/18跟進ADR反彈估收NT$2,385(+25、+1.06% vs 6/17 NT$2,360)、市值回升NT$61.9兆、半導體類股回溫(NVDA+2.59%、SOX+2.71%)。🛰️頭條：SpaceX創紀錄IPO(估值$2.519兆、募資~$750億、+19.6%)市值超越TSMC($2.289兆)、將台積電擠至全球市值第7(屬外部排名變動、基本面未受影響)。🤝TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ廠投資$20億→$70億、2028投產、~2,000就業、InFO/CoWoS)、強化美國供應鏈在地化、呼應TSMC $165B美國投資承諾。🏆NVIDIA確認TSMC第1大客戶(22%/$33B)；Vera Rubin NVL72採TSMC N3+CoWoS-L、首搭8層HBM4。🤝SK海力士-TSMC深化HBM4合作(基底晶粒base die、先進邏輯製程、客製AI記憶體)。💰TSMC CFO重申先進製程漲價勢在必行(通膨+AI需求)、3nm H2漲~15%、sub-5nm漲5-10%。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)。台美ADR溢價(以6/17 ADR$432.15+6/18台股NT$2,385計)+12.52%。⚠️6/19端午節TWSE休市、6/18為連假前最後交易日。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、2026全球半導體市場估+25% YoY達~$975B。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+6.08%)。⚠️估值警示TSM P/E 32.8x、台股P/E~35x、留意台幣升值；上方壓力NT$2,400/NT$2,425/NT$2,440史高、下方支撐NT$2,360/NT$2,310。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+          <t>報告日2026-06-18(Thu)；NYSE TSM 6/17收$432.15(+1.48%、+$6.32 vs 6/16$425.83)自6/16 -3.53%回檔後低接回補、盤中觸$439.60、市值$1.96兆、成交量1,096萬股、P/E 32.79(最新確認)；台股2330 6/18跟進ADR反彈實際收NT$2,385(+10、+0.42% vs 6/17實際NT$2,375、昨量30,228張)、市值回升NT$61.9兆、半導體類股回溫(NVDA+2.59%、SOX+2.71%)。🛰️頭條：SpaceX創紀錄IPO(估值$2.519兆、募資~$750億、+19.6%)市值超越TSMC($2.289兆)、將台積電擠至全球市值第7(屬外部排名變動、基本面未受影響)。🤝TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ廠投資$20億→$70億、2028投產、~2,000就業、InFO/CoWoS)、強化美國供應鏈在地化、呼應TSMC $165B美國投資承諾。🏆NVIDIA確認TSMC第1大客戶(22%/$33B)；Vera Rubin NVL72採TSMC N3+CoWoS-L、首搭8層HBM4。🤝SK海力士-TSMC深化HBM4合作(基底晶粒base die、先進邏輯製程、客製AI記憶體)。💰TSMC CFO重申先進製程漲價勢在必行(通膨+AI需求)、3nm H2漲~15%、sub-5nm漲5-10%。⚠️競爭雜訊：Google向Intel Foundry下單逾300萬顆自研TPU(2028交付)。台美ADR溢價(以6/17 ADR$432.15+6/18台股NT$2,385計)+12.52%。⚠️6/19端午節TWSE休市、6/18為連假前最後交易日。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、2026全球半導體市場估+25% YoY達~$975B。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+6.08%)。⚠️估值警示TSM P/E 32.8x、台股P/E~35x、留意台幣升值；上方壓力NT$2,400/NT$2,425/NT$2,440史高、下方支撐NT$2,360/NT$2,310。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
         </is>
       </c>
       <c r="G70" s="53" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-06-22 日報 HTML & Excel 更新
- NYSE TSM 6/18 創紀錄飆漲 +6.94% 收 $462.12、盤中觸史高 $465.22
- 台股 2330 6/18 官方收 NT$2,410（+1.05%，前報估值 2,385 已更正）
- 新增 Apple-Intel 合作 + ITC 專利調查風險；ADR 溢價 +19.08%

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-18</t>
+          <t>報告更新日期：2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-18</t>
+          <t>最後更新：2026-06-22</t>
         </is>
       </c>
     </row>
@@ -5684,6 +5684,43 @@
         </is>
       </c>
       <c r="G70" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B71" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,410</t>
+        </is>
+      </c>
+      <c r="C71" s="51" t="inlineStr">
+        <is>
+          <t>+1.05%</t>
+        </is>
+      </c>
+      <c r="D71" s="50" t="inlineStr">
+        <is>
+          <t>US$462.12</t>
+        </is>
+      </c>
+      <c r="E71" s="50" t="inlineStr">
+        <is>
+          <t>49,982</t>
+        </is>
+      </c>
+      <c r="F71" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-22(Mon)；🚀NYSE TSM 6/18創紀錄飆漲收$462.12(+6.94%、+$29.97 vs $432.15)、盤中觸52週/歷史新高$465.22、市值$1.98兆、量2,582萬股、P/E 33.14(最新確認)；台股2330 6/18官方收NT$2,410(+25、+1.05% vs 6/17 NT$2,385、盤中觸NT$2,440史高、量49,982張)、加權指數+901.85點收46,459連4日創新高(前報估值2,385已更正)；6/19端午休市、6/22今日交易中受ADR飆漲帶動預期跳空跟漲、官方收盤待TWSE。🤝本波飆漲主因TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ廠$20億→$70億、2028投產、~2,000就業、InFO/CoWoS、呼應$165B美國投資)+分析師升評+AI需求。🏆NVIDIA確認TSMC第1大客戶(22%/$33B)、為A16(1.6nm)首發客戶2027量產；Apple跳過A16直上A14。⚠️新增風險：(1)Apple同意與Intel合作在美生產晶片降低對TSMC依賴、Google/AMD/Tesla接觸Samsung；Intel飆漲+10.6%創新高；(2)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月預計初判、恐對含AI加速器技術晶片發布美國進口禁令。📊台美ADR溢價(以6/18 ADR$462.12+台股NT$2,410計)大幅擴大至+19.08%、6/22台股有補漲壓力。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、SIA/Deloitte估AI資料中心晶片營收2028上看$1.2兆(4年近10倍)、2026全球半導體市場估+25% YoY達~$975B。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+4.98%)。⚠️估值警示TSM P/E 33.1x、台股P/E~35.5x、留意台幣升值與短線過熱；上方壓力NT$2,440史高/NT$2,500、下方支撐NT$2,410/NT$2,375。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G71" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-23 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-22</t>
+          <t>報告更新日期：2026-06-23</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-22</t>
+          <t>最後更新：2026-06-23</t>
         </is>
       </c>
     </row>
@@ -5721,6 +5721,43 @@
         </is>
       </c>
       <c r="G71" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B72" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,510</t>
+        </is>
+      </c>
+      <c r="C72" s="54" t="inlineStr">
+        <is>
+          <t>+4.15%</t>
+        </is>
+      </c>
+      <c r="D72" s="53" t="inlineStr">
+        <is>
+          <t>US$467.67</t>
+        </is>
+      </c>
+      <c r="E72" s="53" t="inlineStr">
+        <is>
+          <t>39,134</t>
+        </is>
+      </c>
+      <c r="F72" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-06-23(Tue)；🚀台美雙市再創歷史新高：台股2330 6/22官方收NT$2,510(+100、+4.15% vs 6/18 NT$2,410、收最高、量39,134張、市值NT$65.1兆)創史高，受6/18 NYSE +6.94%飆漲與6/19美股交易帶動跳空大漲；NYSE TSM 6/22收$467.67(+$5.55、+1.20% vs 6/19~$462.12)再創收盤紀錄新高、市值約$2.4兆、P/E~33.5(最新確認)；6/19端午休市、6/23今日台股開盤NT$2,455自史高小幅拉回、交易中、官方收盤待TWSE。📊台美ADR溢價(以6/22 ADR$467.67+台股NT$2,510計)收斂至+15.71%(自6/18 +19.08%)、台股已補漲跟上。🤝本波飆漲主因TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ廠$20億→$70億、2028投產、~2,000就業、InFO/CoWoS、呼應$165B美國投資)+分析師升評+AI需求。📦新動態：TSMC加速CoPoS面板級封裝布局、目標6月底完成材料/設備驗證、擴大AI封裝產能；惟Samsung PLP技術仍領先數年。🏆NVIDIA確認TSMC第1大客戶(22%/$33B)、為A16(1.6nm)首發客戶2027量產、6月完成$250億債券發行；Apple跳過A16直上A14。⚠️風險續追蹤：(1)Apple同意與Intel合作在美生產晶片降低對TSMC依賴、Google/AMD/Tesla接觸Samsung、Intel與UMC結盟；(2)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月預計初判、恐對含AI加速器技術晶片發布美國進口禁令。⭐中長線基底未變：5月營收NT$4,169.75億+30.1%創單月新高、2nm量產70-80%良率領先全球、4大美國CSP 2026 AI CapEx合計$725B、SIA/Deloitte估AI資料中心晶片營收2028上看$1.2兆(4年近10倍)、2026全球半導體市場估+25% YoY達~$975B。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(已趨近、上行+0.80%、待法說會上修)。⚠️估值警示TSM P/E~33.5x、台股P/E~37.0x、留意台幣升值與短線過熱(RSI 74/KDJ J96進入超買)；上方壓力NT$2,510史高/NT$2,550、下方支撐NT$2,455/NT$2,410。下一里程碑：6月營收7月上旬、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G72" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-24 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-23</t>
+          <t>報告更新日期：2026-06-24</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-23</t>
+          <t>最後更新：2026-06-24</t>
         </is>
       </c>
     </row>
@@ -5758,6 +5758,43 @@
         </is>
       </c>
       <c r="G72" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B73" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,490</t>
+        </is>
+      </c>
+      <c r="C73" s="57" t="inlineStr">
+        <is>
+          <t>-0.80%</t>
+        </is>
+      </c>
+      <c r="D73" s="50" t="inlineStr">
+        <is>
+          <t>US$436.39</t>
+        </is>
+      </c>
+      <c r="E73" s="50" t="inlineStr">
+        <is>
+          <t>34,148</t>
+        </is>
+      </c>
+      <c r="F73" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-24(Wed)；⚠️半導體全面拋售、ADR暴跌但台股抗跌：NYSE TSM 6/23暴跌-6.69%收$436.39(-$31.28 vs 6/22 $467.67、市值回落約$1.97兆、P/E~31.3)，半導體類股全面拋售——Micron -11.4%、AMD -6.25%、AVGO -5.02%、設備股跌4.5-5%；崩跌觸發：Broadcom指引不如預期引爆sell-the-news+BoFA升息報告推升美債殖利率+亞股下挫+AI過熱疑慮+財報前獲利了結，單日逾千億美元半導體市值蒸發。台股2330 6/23官方收NT$2,490(-20、-0.80% vs 6/22 NT$2,510、量34,148張、市值NT$64.6兆)相對抗跌、盤中觸歷史新高NT$2,535後拉回收最低；6/24今日台股交易中、料跟進ADR暴跌跳空走低、官方收盤待TWSE。📊台美ADR溢價(以6/23 ADR$436.39+台股NT$2,490計)自+15.71%大幅收斂至+8.83%、台股短線恐有補跌壓力。⚠️TSMC 4-5月營收合計+24% YoY低於華爾街~35%預期、近期營收恐miss、6月營收(7月上旬)為關鍵catalyst。📈逆勢利多：Susquehanna將TSM目標價自$500上調至$575。⭐中長線基底未變：TSMC-Amkor簽10年美國先進封裝長約(6/16公告、Peoria AZ$70億、2028投產)+NVIDIA確認第1大客戶(22%/$33B)/A16首發2027量產+NVIDIA-TSMC深化AI製程合作(cuLitho/缺陷檢測/工廠排程)+RTX Spark超晶片由TSMC代工+2nm量產70-80%良率領先全球+CoPoS/CoWoS擴產+4大美國CSP 2026 AI CapEx合計$725B+2026全球半導體市場估+25% YoY達~$975B。⚠️風險續追蹤：(1)Apple同意與Intel合作在美生產晶片降低對TSMC依賴、Google/AMD/Tesla接觸Samsung、Intel 18A-P風險量產;(2)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月底預計初判、恐對含AI加速器技術晶片發布美國進口禁令。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+1.61%、待7/16法說會重估)。⚠️估值警示TSM P/E~31.3x、台股P/E~36.7x、仍在5年90%+高位、留意6月營收miss風險與台幣升值；上方壓力NT$2,510/NT$2,535史高、下方支撐NT$2,450/NT$2,410。下一里程碑：6月營收7月上旬(關鍵)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G73" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-26 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-25</t>
+          <t>報告更新日期：2026-06-26</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-25</t>
+          <t>最後更新：2026-06-26</t>
         </is>
       </c>
     </row>
@@ -5832,6 +5832,43 @@
         </is>
       </c>
       <c r="G74" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B75" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,390</t>
+        </is>
+      </c>
+      <c r="C75" s="51" t="inlineStr">
+        <is>
+          <t>+0.63%</t>
+        </is>
+      </c>
+      <c r="D75" s="50" t="inlineStr">
+        <is>
+          <t>US$440.83</t>
+        </is>
+      </c>
+      <c r="E75" s="50" t="inlineStr">
+        <is>
+          <t>~14,000</t>
+        </is>
+      </c>
+      <c r="F75" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-26(Fri)；⭐今日頭條——TSMC晶圓代工漲價題材延燒、ADR續漲且盤後大漲、台股料補漲：⭐漲價範圍確認擴大至7nm以下全部先進製程(含N7/N5/N3、佔Q1晶圓營收約74%，N3單一佔25%)、幅度5-10%視客戶/節點/產品、部分已實施，以平均5%估可貢獻全年毛利率+2pp以上。📈NYSE TSM 6/25 Thu續漲+1.02%收$440.83(+$4.44、市值約$2.05兆、P/E~31.6)，盤後再大漲+2.48%至$451.76(漲價題材+產能擴張利多、今年規劃9期廠)。📊台股2330 6/25 Thu小漲+0.63%收NT$2,390、跟進6/24 ADR反彈力道有限；6/26今日台股料跟進ADR盤後大漲、官方收盤待TWSE。📊台美ADR溢價(以6/25 ADR$440.83+台股NT$2,390計)+14.54%、台股短線料補漲收斂。💡Benzinga：漲價雖壓縮NVIDIA毛利、惟AI需求剛性+轉嫁能力強、長期反為NVIDIA利多;⚠️價格敏感客戶(含Apple/手機SoC)影響較大、恐調整下單或評估替代。🛠️Applied Materials 6/25推新一代設備加速DRAM與AI先進封裝(HBM/3D堆疊)。⚠️近期營收疑慮續存——TSMC 4-5月營收合計+24% YoY低於華爾街~35%預期、6月營收(7月上旬)為關鍵catalyst;5月營收NT$4,169.75億(+30.1%)創單月新高、1-5月累計NT$1.96兆。⭐中長線基底未變：TSMC-Amkor 10年美國先進封裝長約(Peoria AZ$70億、2028投產)+NVIDIA確認第1大客戶(22%/$33B)/A16首發2027量產+NVIDIA-TSMC深化AI製程合作+2nm量產70-80%良率領先全球+4大美國CSP 2026 AI CapEx合計$725B+2026全球半導體市場估+26% YoY達~$975B。⚠️風險續追蹤：(1)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月底預計初判、恐對含AI加速器技術晶片發布美國進口禁令;(2)Apple與Intel合作在美生產晶片、Google/AMD/Tesla接觸Samsung、Intel 18A-P風險量產+UMC結盟。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+5.86%自NT$2,390、Susquehanna 6/23上調$575、待7/16法說會重估)。⚠️估值警示TSM P/E~31.6x、台股P/E~35.2x；下方支撐NT$2,350/NT$2,310、上方壓力NT$2,450/NT$2,490/NT$2,535史高。下一里程碑：ITC初判6月底、6月營收7月上旬(關鍵)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G75" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-29 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -883,7 +883,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-26</t>
+          <t>報告更新日期：2026-06-29</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3272,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-26</t>
+          <t>最後更新：2026-06-29</t>
         </is>
       </c>
     </row>
@@ -5869,6 +5869,43 @@
         </is>
       </c>
       <c r="G75" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="53" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B76" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,340</t>
+        </is>
+      </c>
+      <c r="C76" s="56" t="inlineStr">
+        <is>
+          <t>-2.09%</t>
+        </is>
+      </c>
+      <c r="D76" s="53" t="inlineStr">
+        <is>
+          <t>US$432.35</t>
+        </is>
+      </c>
+      <c r="E76" s="53" t="inlineStr">
+        <is>
+          <t>53,800</t>
+        </is>
+      </c>
+      <c r="F76" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-06-29(Mon)；⭐今日頭條——TSMC漲價題材仍為結構性主軸、惟上週五雙市回吐隔夜漲價漲幅：📉台股2330 6/26 Fri收NT$2,340(-50、-2.09%、量放大53,800張)自6/25 NT$2,390回落——隔夜ADR漲價漲幅回吐+近期營收疑慮+外資賣超(6/26外資賣超6,104張、投信買超179張、自營賣超310張、三大法人合計賣超6,235張)拖累。📉NYSE TSM 6/26 Fri收$432.35(-0.61%、-$2.64、前收$434.99、市值約$2.0兆、P/E~31.0、日內$419.19–$436.13)，連續回吐6/24漲價題材帶動之隔夜漲幅、估值與營收疑慮拉鋸。⭐漲價題材結構性利多未變：範圍確認擴大至7nm以下全部先進製程(含N7/N5/N3、佔晶圓營收約75%、N3單一佔25%)、幅度5-10%視客戶/節點/產品、部分已實施，以平均5%估可貢獻全年毛利率+2pp以上。📊台股6/29今日開盤約NT$2,350(+0.43% vs 6/26)小反彈、官方收盤待TWSE。📊台美ADR溢價(以6/26 ADR$432.35+台股NT$2,340、匯率31.05計)+14.74%。💡Benzinga：漲價雖壓縮NVIDIA毛利、惟AI需求剛性+轉嫁能力強、長期反為NVIDIA利多;⚠️價格敏感客戶(含Apple/手機SoC)影響較大、恐調整下單或評估替代。⚠️近期營收疑慮續存——TSMC 4-5月營收合計+24% YoY低於華爾街~35%預期、6月營收(7月上旬)為關鍵catalyst;5月營收NT$4,169.75億(+30.1%)創單月新高、1-5月累計NT$1.96兆。⚠️ITC專利調查初判預計本週(6月底)出爐、為短線關鍵雜訊。🛠️產業競局升溫：Intel 18A-P進入風險量產+UMC結盟、AMD瞄準$1,200億市場、Qualcomm推Dragonfly;Samsung/SK海力士送樣第7代HBM4E;Applied Materials 6/25推新一代設備加速DRAM與AI先進封裝。⭐中長線基底未變：TSMC-Amkor 10年美國/韓國先進封裝長約(Peoria AZ$70億、2028投產)+NVIDIA確認第1大客戶(22%/$33B)/A16首發2027量產+NVIDIA-TSMC深化AI製程合作+2nm量產70-80%良率領先全球+2nm/A16產能2026-28估CAGR~70%+4大美國CSP 2026 AI CapEx合計$725B。⚠️風險續追蹤：(1)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月底(本週)預計初判、恐對含AI加速器技術晶片發布美國進口禁令;(2)Apple與Intel合作在美生產晶片、Google/AMD/Tesla接觸Samsung。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。32位分析師全數看多、平均目標NT$2,530(上行+8.12%自NT$2,340、Susquehanna 6/23上調$575、待7/16法說會重估)。⚠️估值警示TSM P/E~31.0x、台股P/E~34.5x；下方支撐NT$2,310/NT$2,250、上方壓力NT$2,390/NT$2,450/NT$2,535史高。下一里程碑：ITC初判6月底(本週)、6月營收7月上旬(關鍵)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G76" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-06-30 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -323,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -493,6 +493,9 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -883,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-29</t>
+          <t>報告更新日期：2026-06-30</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="36" min="1" max="1"/>
@@ -2497,6 +2500,34 @@
           <t>美日廠擴產，壓縮部分毛利率</t>
         </is>
       </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t>記憶體自主供應 (Winbond WoW)</t>
+        </is>
+      </c>
+      <c r="B21" s="60" t="inlineStr">
+        <is>
+          <t>CUBE特殊DRAM / WoW 3D堆疊</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>降低HBM對Samsung/SK依賴</t>
+        </is>
+      </c>
+      <c r="D21" s="60" t="inlineStr">
+        <is>
+          <t>Source: TSMC-Winbond 2026-06-29; 在地化估縮短週期66%/降運費90%、導入SoIC先進封裝</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="n"/>
+      <c r="B22" s="60" t="n"/>
+      <c r="C22" s="60" t="n"/>
+      <c r="D22" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3250,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3272,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-29</t>
+          <t>最後更新：2026-06-30</t>
         </is>
       </c>
     </row>
@@ -5906,6 +5937,43 @@
         </is>
       </c>
       <c r="G76" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="50" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B77" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,370</t>
+        </is>
+      </c>
+      <c r="C77" s="51" t="inlineStr">
+        <is>
+          <t>+1.28%</t>
+        </is>
+      </c>
+      <c r="D77" s="50" t="inlineStr">
+        <is>
+          <t>US$455.10</t>
+        </is>
+      </c>
+      <c r="E77" s="50" t="inlineStr">
+        <is>
+          <t>38,133</t>
+        </is>
+      </c>
+      <c r="F77" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-06-30(Tue)；🚀今日頭條——TSMC雙市同步反彈、漲價題材升級為定價力+自主供應鏈雙主軸：🚀NYSE TSM 6/29 Mon大漲+5.26%(+$22.75)收$455.10創波段新高、市值約$2.1兆(P/E~32.5、前收$432.35)；📈台股2330 6/29 Mon收NT$2,370(+30、+1.28%、量縮38,133張、成交額903.37億、開2,330/高2,395)自6/26 NT$2,340反彈；台股6/30今日料受隔夜ADR激勵開高、官方收盤待TWSE。三大催化：⭐TSMC與華邦電(Winbond)合作將CUBE特殊DRAM導入WoW 3D晶圓堆疊/SoIC先進封裝、把關鍵記憶體留台、降低對Samsung/SK海力士HBM依賴(在地化估縮短週期66%、降運費90%);⭐漲價定價力擴及先進+成熟製程(佔晶圓營收~75%、幅度5-10%、估全年毛利率+2pp以上);📈Bank of America等多家機構上調目標(彙整平均$468.08、最高$600、最低$351)。📊台美ADR溢價(以6/29 ADR$455.10+台股NT$2,370、匯率31.05計)走闊至+19.25%、ADR領先、台股具補漲空間。⚠️漲價雙面刃——客戶(Apple/NVIDIA/AMD/Qualcomm/Broadcom/MediaTek)成本升、Benzinga指NVIDIA因AI需求剛性+轉嫁能力強長期反為利多。⚠️近期營收疑慮續存——TSMC 4-5月營收合計+24% YoY低於華爾街~35%預期、6月營收(7月上旬)為關鍵catalyst;5月營收NT$4,169.75億(+30.1%)創單月新高、1-5月累計NT$1.96兆。⚠️ITC專利調查初判預計本週(6月底)出爐、為短線關鍵雜訊。⭐中長線基底未變：Winbond特殊DRAM自主供應+TSMC-Amkor 10年美國/韓國先進封裝長約(Peoria AZ$70億、2028投產)+NVIDIA確認第1大客戶(22%/$33B)/A16首發2027量產+NVIDIA-TSMC深化AI製程合作+2nm量產70-80%良率領先全球+2nm/A16產能2026-28估CAGR~70%+4大美國CSP 2026 AI CapEx合計$725B。⚠️風險續追蹤：(1)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、6月底(本週)預計初判、恐對含AI加速器技術晶片發布美國進口禁令;(2)Apple與Intel合作在美生產晶片、Intel 18A-P風險量產+UMC結盟、Google/AMD/Tesla接觸Samsung。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。分析師全面看多、BofA等上調目標(彙整平均$468.08、最高$600)。⚠️估值警示TSM P/E~32.5x、台股P/E~35.0x；下方支撐NT$2,340/NT$2,310、上方壓力5MA NT$2,396/NT$2,450/NT$2,535史高。下一里程碑：ITC初判6月底(本週)、6月營收7月上旬(關鍵)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G77" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-01 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-06-30</t>
+          <t>報告更新日期：2026-07-01</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-06-30</t>
+          <t>最後更新：2026-07-01</t>
         </is>
       </c>
     </row>
@@ -5974,6 +5974,43 @@
         </is>
       </c>
       <c r="G77" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="53" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B78" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,455</t>
+        </is>
+      </c>
+      <c r="C78" s="54" t="inlineStr">
+        <is>
+          <t>+3.59%</t>
+        </is>
+      </c>
+      <c r="D78" s="53" t="inlineStr">
+        <is>
+          <t>US$468.80</t>
+        </is>
+      </c>
+      <c r="E78" s="53" t="inlineStr">
+        <is>
+          <t>15,514</t>
+        </is>
+      </c>
+      <c r="F78" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-07-01(Wed)；🚀今日頭條——台美雙市連袂走高、法人上調目標接力：🚀NYSE TSM 6/30 Tue續漲+3.02%(+$13.70)收$468.80、逼近52週高$476.79、市值約$2.15兆(P/E~33.5、前收$455.10)、7/1美股盤待今晚開盤;🚀台股2330 6/30官方收盤NT$2,455(+85、+3.59% vs 6/29 NT$2,370、開2,440/高2,475/低2,435、量15,514張、成交額380.9億、振幅1.69%)跳空跟進NYSE前波大漲、突破5MA/20MA、7/1台股盤中待TWSE。催化：📈Morgan Stanley上調目標並估2026營收+40% YoY;📈UBS上調目標並上修長期銷售成長;⭐漲價定價力擴及全先進製程(佔晶圓營收~74%、幅度5-10%、估全年毛利率+2pp以上);⭐TSMC-Amkor美國封裝長約降地緣風險。📊分析師共識目標升至平均$476.24、最高$625、最低$351。📊台美ADR溢價(以6/30 ADR$468.80+台股6/30 NT$2,455、匯率31.05計、理論值$395.33)走闊至+18.59%、台股7/1具補漲空間。🛠️晶片設備股領軍反彈：AMAT +10.8%、LRCX +8.4%、SOXX +4.1%(AI記憶體需求勁揚);Gartner估2026半導體營收超$1.3兆。⚠️漲價雙面刃——客戶(Nvidia/AMD/Apple/Qualcomm/Broadcom/MediaTek)成本升、Benzinga指NVIDIA因AI需求剛性+轉嫁能力強長期反為利多。⚠️近期營收疑慮續存——TSMC 4-5月營收合計+24% YoY低於華爾街~35%預期、6月營收(7月上旬)為關鍵catalyst;5月營收NT$4,169.75億(+30.1%)創單月新高、1-5月累計NT$1.96兆。⚠️ITC專利調查初判預計近期(6月底/7月初)出爐、為短線關鍵雜訊。⚠️監理雜訊——Super Micro遭台灣搜索(涉NVIDIA晶片走私中國)股價-8%;南韓公布逾$1兆美元AI/晶片投資、三星+SK 800兆韓元。⭐中長線基底未變：TSMC-Amkor 10年美國先進封裝長約(Peoria AZ$70億、2028投產)+Winbond特殊DRAM自主供應+NVIDIA確認第1大客戶(22%/$33B)/A16首發2027量產+NVIDIA-TSMC深化AI製程合作+2nm量產70-80%良率領先全球+2nm/A16產能2026-28估CAGR~70%+4大美國CSP 2026 AI CapEx合計$725B。⚠️風險續追蹤：(1)TSMC遭美ITC專利調查(Longitude/Marlin控訴)、近期預計初判、恐對含AI加速器技術晶片發布美國進口禁令;(2)Apple與Intel合作在美生產晶片、Intel 18A-P風險量產+UMC結盟、Google/AMD/Tesla接觸Samsung。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。分析師全面看多、MS/UBS等上調目標(共識平均$476.24、最高$625)。⚠️估值警示TSM P/E~33.5x、台股P/E~36.2x；下方支撐NT$2,400/NT$2,370、上方壓力NT$2,490/NT$2,535史高。下一里程碑：ITC初判近期、6月營收7月上旬(關鍵)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G78" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-02 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-07-01</t>
+          <t>報告更新日期：2026-07-02</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-07-01</t>
+          <t>最後更新：2026-07-02</t>
         </is>
       </c>
     </row>
@@ -6011,6 +6011,43 @@
         </is>
       </c>
       <c r="G78" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B79" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,505</t>
+        </is>
+      </c>
+      <c r="C79" s="51" t="inlineStr">
+        <is>
+          <t>+3.94%</t>
+        </is>
+      </c>
+      <c r="D79" s="50" t="inlineStr">
+        <is>
+          <t>US$444.23</t>
+        </is>
+      </c>
+      <c r="E79" s="50" t="inlineStr">
+        <is>
+          <t>37,544</t>
+        </is>
+      </c>
+      <c r="F79" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-07-02(Thu)；⚠️今日頭條——台美劇烈背離、NYSE夜盤重挫：📉NYSE TSM 7/1 Wed重挫-6.98%(-$33.34)收$444.23、自6/30史新高$477.57大幅回落、市值約$2.30兆(P/E~38.6)、盤後回升+0.94%至$448.41顯示殺盤趨緩、7/2美股盤待今晚開盤;🚀台股2330 7/1官方收盤NT$2,505(+95、+3.94% vs 6/30 NT$2,410、高2,505、量37,544張)連3漲、下半年開門紅、突破5MA/20MA——惟台股7/1收盤在NYSE夜盤重挫之前、7/2恐面臨補跌壓力、盤中待TWSE。NYSE重挫催化：技術面過熱獲利了結(費半SOX Q2 +87.8%創1994年以來最強單季後拉回)、估值修正、4-5月營收+24% YoY落後華爾街~35%預期、智慧型手機/PC下游需求疲弱、7/16財報前觀望。📊台美ADR溢價(以7/1 ADR$444.23+台股7/1 NT$2,505、匯率31.05計、理論值$403.38)自+18.59%大幅收斂至+10.13%、預示台股7/2補跌。📊分析師共識仍偏多——17位Strong Buy、0賣出、12個月平均目標$487.56(自7/1收$444.23具+9.8%上行空間)、拉回視為估值修正非基本面惡化。⭐漲價題材續發酵——TSMC通知客戶全先進製程調漲5-10%(擴及N7/N5/N3及成熟製程、佔晶圓營收~74%)、估全年毛利率+2pp以上;客戶(Nvidia/AMD/Apple/Qualcomm/Broadcom/MediaTek)成本升、Benzinga指NVIDIA因AI需求剛性+轉嫁能力強長期反為利多。🏆NVIDIA確認超越Apple成TSMC最大客戶(22%/$33B)、A16首發2026下半/2027量產;Apple跳過A16直上A14。⚠️南韓公布逾$1兆美元AI/晶片投資、三星+SK 800兆韓元(約$5,180億)各建兩座新廠、中長期強化韓系競爭。⭐中長線基底未變：TSMC-Amkor 10年美國先進封裝長約(Peoria AZ$70億、2028投產)+Winbond特殊DRAM自主供應+NVIDIA第1大客戶/A16首發+2nm量產70-80%良率領先全球+2nm/A16產能2026-28估CAGR~70%+4大美國CSP 2026 AI CapEx合計$725B;全球半導體2026估$975B(+26% YoY)、AI資料中心晶片2028估$1.2兆(佔AI伺服器機櫃價值95%)。基本面：Q1 2026淨利NT$572.5B(+58.3% YoY)、毛利率66.2%雙創史高、2025全年EPS NT$66.25。⚠️估值警示TSM P/E~38.6x、台股P/E~36.9x；下方支撐NT$2,450/NT$2,410、上方壓力NT$2,505/NT$2,535史高。下一里程碑：6月營收7月上旬(關鍵catalyst)、Q2法說會7/16。</t>
+        </is>
+      </c>
+      <c r="G79" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-03 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-07-02</t>
+          <t>報告更新日期：2026-07-03</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-07-02</t>
+          <t>最後更新：2026-07-03</t>
         </is>
       </c>
     </row>
@@ -6048,6 +6048,43 @@
         </is>
       </c>
       <c r="G79" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="53" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B80" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,465（7/2收、7/3盤前未開）</t>
+        </is>
+      </c>
+      <c r="C80" s="56" t="inlineStr">
+        <is>
+          <t>-1.60%（7/2收）</t>
+        </is>
+      </c>
+      <c r="D80" s="53" t="inlineStr">
+        <is>
+          <t>US$434.16</t>
+        </is>
+      </c>
+      <c r="E80" s="53" t="inlineStr">
+        <is>
+          <t>35,000（7/2）</t>
+        </is>
+      </c>
+      <c r="F80" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-07-03(Fri)。修正延續、惟跌勢趨緩＋分析師逆勢續挺：📉NYSE TSM 7/2 Thu收$434.16(-2.27%、-$10.07)自6/30史高$477.57連二日回落，惟跌幅自7/1 -6.98%大幅收斂、殺盤趨緩、屬估值修正非基本面惡化；NYSE 7/3因美國國慶休市。⚠️台股2330 7/3盤前尚未開盤、最新收7/2 NT$2,465(-1.60%)、守穩NT$2,450，7/3開盤恐跟進NYSE續跌承壓。🚀Nomura上調目標至NT$3,425(+38.9%空間)、Barclays亦上調；平均目標$476.24(自$434.16具+9.7%空間)、拉回視為估值修正；⚠️惟Goldman 7/1移出APAC Conviction List(戰術調整非降評)。🤝NVIDIA-TSMC導入AI入廠提升良率；BofA上修2026全球半導體市場至$1.3兆(原$1.0兆)、2030上看$2兆。⭐漲價續發酵、全先進製程調漲5-10%(佔晶圓營收~74%)、估全年毛利率+2pp以上。中長線基底未變：NVIDIA #1客戶(22%/$33B)/A16首發、Vera Rubin 6顆晶片全TSMC代工(3nm+HBM4)、2nm 70-80%良率、費半Q2 +87.8%史上最強單季。⚠️估值警示TSM P/E~37.7x、台股~36.3x；6月營收(7月上旬)與7/16財報為關鍵catalyst；下方支撐NT$2,450/NT$2,410、上方壓力NT$2,505/NT$2,535史高。</t>
+        </is>
+      </c>
+      <c r="G80" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-06 日報 HTML & Excel 更新
- 台股 2330 7/3 官方收 NT$2,445（-0.81%、量 26,455 張、跌幅收斂）
- NYSE TSM 7/2 止穩收紅 $434.71（+0.13%、盤後 +0.63%）；7/3 國慶休市、7/6 重新開盤
- 更正前報 NYSE 7/2 誤植 -2.27%/$434.16 為官方 +0.13%/$434.71
- Barclays 上調目標至 $625、Nomura NT$3,425；NVIDIA-SK 海力士記憶體合作

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-07-03</t>
+          <t>報告更新日期：2026-07-06</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-07-03</t>
+          <t>最後更新：2026-07-06</t>
         </is>
       </c>
     </row>
@@ -6085,6 +6085,43 @@
         </is>
       </c>
       <c r="G80" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B81" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,445（7/3收）</t>
+        </is>
+      </c>
+      <c r="C81" s="57" t="inlineStr">
+        <is>
+          <t>-0.81%（7/3收）</t>
+        </is>
+      </c>
+      <c r="D81" s="50" t="inlineStr">
+        <is>
+          <t>US$434.71（7/2收）</t>
+        </is>
+      </c>
+      <c r="E81" s="50" t="inlineStr">
+        <is>
+          <t>26,455（7/3收）</t>
+        </is>
+      </c>
+      <c r="F81" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-07-06(Mon)。修正後止穩、分析師大幅續挺：⚖️台股2330 7/3官方收NT$2,445(-20、-0.81%、量26,455張)跌幅較7/2之-1.60%收斂、守穩NT$2,410；NYSE TSM 7/2於7/1重挫後低檔止穩、小幅收紅+0.13%收$434.71、盤後+0.63%至$437.44、殺盤動能衰竭、屬估值修正非基本面惡化；NYSE 7/3因美國國慶休市、7/6重新開盤。🚀Barclays將TSM目標價自$470大幅上調至$625(+43.8%空間)、Nomura NT$3,425(+40.1%空間)；平均目標~$490強力買入；⚠️惟Goldman 7/1移出APAC Conviction List(戰術調整非降評)。🤝NVIDIA-SK海力士宣布多年期記憶體合作(AI工廠次世代記憶體)；NVIDIA-TSMC導入AI入廠提升良率；BofA上修2026全球半導體市場至$1.3兆、生成式AI晶片估~$500B、費半YTD+47%。⭐漲價續發酵、7nm以下全先進製程調漲5-10%(佔晶圓營收~75%)、估全年毛利率+2pp以上。中長線基底未變：NVIDIA #1客戶(22%/$33B)/A16首發、Vera Rubin 6顆晶片全TSMC代工(3nm+HBM4)、2nm 70-80%良率。⚠️估值警示TSM P/E~37.8x、台股~36.0x；6月營收(7月上旬)與7/16財報為關鍵catalyst；ADR溢價約+10.4%；下方支撐NT$2,410/NT$2,370、上方壓力NT$2,465/NT$2,505/NT$2,535史高。</t>
+        </is>
+      </c>
+      <c r="G81" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-06 日報 HTML & Excel 更新（重要更正：NYSE TSM 7/2 收盤自誤植之 +0.13%/$434.71 更正為官方 -2.27%/$434.16、前收 7/1 $444.23，經 stockanalysis.com 複核；即 NYSE 為連二跌 7/1 -6.98%、7/2 -2.27% 但跌幅大幅收斂、殺盤趨緩，而非止穩收紅；台股 2330 7/3 官方收 NT$2,445 -0.81% 跌幅收斂守穩 NT$2,410；NYSE 7/3 因美國國慶休市、7/6 重新開盤；分析師續大幅上調 Barclays $625/+43.9%、Nomura NT$3,425/+40.1%；ADR 溢價修正為 +10.3%）
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -6108,7 +6108,7 @@
       </c>
       <c r="D81" s="50" t="inlineStr">
         <is>
-          <t>US$434.71（7/2收）</t>
+          <t>US$434.16（7/2收）</t>
         </is>
       </c>
       <c r="E81" s="50" t="inlineStr">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="F81" s="52" t="inlineStr">
         <is>
-          <t>報告日2026-07-06(Mon)。修正後止穩、分析師大幅續挺：⚖️台股2330 7/3官方收NT$2,445(-20、-0.81%、量26,455張)跌幅較7/2之-1.60%收斂、守穩NT$2,410；NYSE TSM 7/2於7/1重挫後低檔止穩、小幅收紅+0.13%收$434.71、盤後+0.63%至$437.44、殺盤動能衰竭、屬估值修正非基本面惡化；NYSE 7/3因美國國慶休市、7/6重新開盤。🚀Barclays將TSM目標價自$470大幅上調至$625(+43.8%空間)、Nomura NT$3,425(+40.1%空間)；平均目標~$490強力買入；⚠️惟Goldman 7/1移出APAC Conviction List(戰術調整非降評)。🤝NVIDIA-SK海力士宣布多年期記憶體合作(AI工廠次世代記憶體)；NVIDIA-TSMC導入AI入廠提升良率；BofA上修2026全球半導體市場至$1.3兆、生成式AI晶片估~$500B、費半YTD+47%。⭐漲價續發酵、7nm以下全先進製程調漲5-10%(佔晶圓營收~75%)、估全年毛利率+2pp以上。中長線基底未變：NVIDIA #1客戶(22%/$33B)/A16首發、Vera Rubin 6顆晶片全TSMC代工(3nm+HBM4)、2nm 70-80%良率。⚠️估值警示TSM P/E~37.8x、台股~36.0x；6月營收(7月上旬)與7/16財報為關鍵catalyst；ADR溢價約+10.4%；下方支撐NT$2,410/NT$2,370、上方壓力NT$2,465/NT$2,505/NT$2,535史高。</t>
+          <t>報告日2026-07-06(Mon)。修正收斂、分析師大幅續挺：⚖️台股2330 7/3官方收NT$2,445(-20、-0.81%、量26,455張)跌幅較7/2之-1.60%收斂、守穩NT$2,410；NYSE TSM 7/2續跌-2.27%收$434.16(前收7/1 $444.23)為連二跌(7/1 -6.98%、7/2 -2.27%)但跌幅大幅收斂、殺盤動能衰竭、屬估值修正非基本面惡化；NYSE 7/3因美國國慶休市、7/6重新開盤。【重要更正】前一份7/6報告曾誤將7/2「更正」為+0.13%收$434.71，經stockanalysis.com官方收盤複核為誤、正確為-2.27%收$434.16。🚀Barclays將TSM目標價自$470大幅上調至$625(+43.9%空間)、Nomura NT$3,425(+40.1%空間)；平均目標~$490強力買入；⚠️惟Goldman 7/1移出APAC Conviction List(戰術調整非降評)。🤝NVIDIA-SK海力士宣布多年期記憶體合作(AI工廠次世代記憶體)；NVIDIA-TSMC導入AI入廠提升良率；BofA上修2026全球半導體市場至$1.3兆、生成式AI晶片估~$500B、費半YTD+47%。⭐漲價續發酵、7nm以下全先進製程調漲5-10%(佔晶圓營收~75%)、估全年毛利率+2pp以上。中長線基底未變：NVIDIA #1客戶(22%/$33B)/A16首發、Vera Rubin 6顆晶片全TSMC代工(3nm+HBM4)、2nm 70-80%良率。⚠️估值警示TSM P/E~37.8x、台股~36.0x；6月營收(7月上旬)與7/16財報為關鍵catalyst；ADR溢價約+10.3%；下方支撐NT$2,410/NT$2,370、上方壓力NT$2,465/NT$2,505/NT$2,535史高。</t>
         </is>
       </c>
       <c r="G81" s="50" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-07-07 日報 HTML & Excel 更新
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-07-06</t>
+          <t>報告更新日期：2026-07-07</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-07-06</t>
+          <t>最後更新：2026-07-07</t>
         </is>
       </c>
     </row>
@@ -6122,6 +6122,43 @@
         </is>
       </c>
       <c r="G81" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="53" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B82" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,460（7/6收）</t>
+        </is>
+      </c>
+      <c r="C82" s="54" t="inlineStr">
+        <is>
+          <t>+0.61%（7/6收）</t>
+        </is>
+      </c>
+      <c r="D82" s="53" t="inlineStr">
+        <is>
+          <t>US$451.79（7/6收）</t>
+        </is>
+      </c>
+      <c r="E82" s="53" t="inlineStr">
+        <is>
+          <t>19,239（7/6收）</t>
+        </is>
+      </c>
+      <c r="F82" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-07-07(Tue)。NYSE V型大反彈、修正結束：🚀NYSE TSM 7/6假期後重新開盤即大漲+4.06%(+$17.63)收$451.79(前收7/2 $434.16、盤後$450.35)、費半SOX同步+3.92%、一舉收復7/1(-6.98%)+7/2(-2.27%)兩日全數跌幅、AI半導體回神、確認為估值修正非基本面惡化；⚖️台股2330 7/6收NT$2,460(+15、+0.61%、量約19,239張、盤中高觸NT$2,500逼近史高)連二跌後翻紅、惟台股7/6盤已於NYSE反彈前收盤尚未完整反映利多；📊台美ADR溢價擴大至約+17.6%(7/6 ADR $451.79折合台股NT$2,893.71 vs 台股NT$2,460)、隱含台股7/7補漲空間。🚀Barclays維持TSM目標$625(自$451.79具+38.3%空間)、Nomura NT$3,425(自NT$2,460具+39.2%空間)、平均目標~$490強力買入；⚠️惟Goldman 7/1移出APAC Conviction List(戰術調整非降評)。🤝NVIDIA-SK海力士宣布多年期記憶體合作(AI工廠次世代記憶體)；NVIDIA-TSMC導入AI入廠提升良率；BofA上修2026全球半導體市場至$1.3兆、生成式AI晶片估~$500B；Qualcomm推無HBM資料中心晶片挑戰NVIDIA。⭐漲價續發酵、7nm以下全先進製程調漲5-10%(佔晶圓營收~75%)、估全年毛利率+2pp以上。中長線基底未變：NVIDIA #1客戶(22%/$33B)/A16首發、Vera Rubin 6顆晶片全TSMC代工(3nm+HBM4)、2nm 70-80%良率。⚠️估值警示TSM P/E~39.3x、台股~36.2x；6月營收(7月上旬)與7/16財報為關鍵catalyst；下方支撐NT$2,445/NT$2,410、上方壓力NT$2,500/NT$2,535史高。</t>
+        </is>
+      </c>
+      <c r="G82" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-07-15 日報 HTML & Excel 更新
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -886,7 +886,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-07-14</t>
+          <t>報告更新日期：2026-07-15</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3303,7 +3303,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-07-14</t>
+          <t>最後更新：2026-07-15</t>
         </is>
       </c>
     </row>
@@ -6307,6 +6307,43 @@
         </is>
       </c>
       <c r="G86" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="50" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B87" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,420（7/14收）</t>
+        </is>
+      </c>
+      <c r="C87" s="57" t="inlineStr">
+        <is>
+          <t>-0.82%（7/14收）</t>
+        </is>
+      </c>
+      <c r="D87" s="50" t="inlineStr">
+        <is>
+          <t>US$420.39（7/14收）</t>
+        </is>
+      </c>
+      <c r="E87" s="50" t="inlineStr">
+        <is>
+          <t>42,857（7/14收）</t>
+        </is>
+      </c>
+      <c r="F87" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-07-15(Wed)。⭐⭐7/16 Q2法說會倒數1天(週三14:00)：法人估Q2營收~$40B(+32% YoY)、獲利+50%+連5季創高、毛利率挑戰70%(指引65.5-67.5%)、關注上修全年財測(現行&gt;30%)；6月營收NT$4,426.80億(+67.9% YoY)已確認Q2約NT$1.27兆達標。📉台股2330 7/14收NT$2,420(-20、-0.82%、量42,857張TWSE口徑、額1,033.71億)——大盤重挫-642.57點(-1.42%)收44,737.95、相對抗跌惟失守5MA~2,436。📊三大法人7/14(T86)合計賣超8,005張：外資-12,416(連4賣、4日-31,365)、投信+1,841、自營+2,570。📉NYSE TSM 7/14收$420.39(-0.28%)法說會前觀望；⚡同日SOX +2.54%大反彈(NVDA +4.06%、MU +4.92%、AMKR +6.27%)、SK海力士7/15韓股盤中+11%，今日台股可望跟進。💰漲價題材：7nm以下全製程調漲5-10%、三星跟進4/5nm漲15%；CoWoS 2026產能12.5萬片/月遭NVIDIA/博通訂滿、缺口至2027。📊ADR溢價+11.7%($420.39 vs理論值$376.46、匯率32.14)。🚀分析師續挺：Citi NT$3,800(+57.0%)、Barclays $625(+48.7%)、Nomura NT$3,425(+41.5%)。⚠️風險：外資連4賣擴大、法說會前後劇烈波動、232關稅輸中晶片查驗收緊、Intel 18A、估值不低(P/E~32.1x)。技術面：MACD柱轉負、KDJ J=22近超賣；支撐2,390/2,366/2,336、壓力2,436/2,480/2,535史高。</t>
+        </is>
+      </c>
+      <c r="G87" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
fix: 2026-08-05 日報 2 項更正（fresh-context 驗收發現）
1. AMD 8/4 盤後跌幅：原「約 -7~-9%（媒體報導）」為轉述區間且頭條寫 -7% 低估實際跌勢，
   更正為官方最終讀數 -8.82% 收 $472.85（19:59 ET、Yahoo 1 分線 includePrePost 確認）。
   原註記「Yahoo API 未提供盤後快照」不成立——includePrePost=true 可取得盤後分線。
   共 9 處（data_note／headline／bullets／bottom_line／risk_alert／ECOSYSTEM／ADR note／NEWS 標題與內文）。

2. ADR 理論值算術更正：5 × NT$2,320 ÷ 32.36 = 358.47（原誤填 358.50），
   連帶溢價 +16.37% → +16.38%。共 6 + 9 處。

Excel 每日更新記錄第 100 行 F 欄摘要同步更正（C 欄字色 FF0000 經查正確、未再犯 8/4 之誤）。
歷史條目「Oracle -7%」（2026-04-28）確認未受波及。

驗收結果：12 條驗收條件 11 條通過，台股／大盤／三大法人／BFI82U／估值／技術指標／
美股收盤全數與 TWSE、Yahoo 官方獨立取數一致。

⚠️ 另發現待使用者裁決的系統性口徑問題（本次未改）：RELATIVE 的 YTD 以
「2026-01-02 收盤 NT$1,585」為基準得 +46.4%；若依曆年制（2025-12-31 收盤 NT$1,550）
應為 +49.7%，差約 3.3 個百分點。此口徑跨多日報一致沿用，改動涉及歷史可比性，故保留原狀待確認。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="封面總覽" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="財務摘要" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="營收結構分析" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026展望" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股息記錄" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險評估" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日更新記錄" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="F100" s="55" t="inlineStr">
         <is>
-          <t>報告日2026-08-05(Wed)。📊台美短線背離、今日補漲條件齊備：台股8/4連2日獲利了結——2330收NT$2,320(-50、-2.11%、開2,335/高2,360/低2,310、量41,021張低於5日均量53,044、額954.55億、277,787筆、TWSE確認)、跌破20MA 2,371與60MA 2,350（季線失守）；大盤僅-25.75點(-0.06%)收43,360.66、上漲578家&gt;下跌406家——矽光子/CPO/低軌衛星漲停潮、中小型接棒；華邦電+9.79%續強、日月光-4.10%、聯發科-1.15%拉回換手。⚠️籌碼：外資連2賣-12,430張（自-9,717擴大、「一日翻多」確認失敗）、投信+434連8買、自營-2,327、三大合計-14,323張（T86官方）；全市場BFI82U合計+20.1億（外資-57.3億、投信+271.7億大買、自營-194.3億）——外資調節集中權值、內資持續進場。⭐美股8/4半導體史詩級大漲：SOX+6.55%收12,179.26（自史高收斂至-16.8%）——ARM+17.36%收$280.56、INTC+10.84%站上$100、AMKR+9.89%、LRCX+7.85%、MU+7.62%、KLAC+6.95%、AVGO+6.61%、AMAT+5.48%、ASML+4.22%、NVDA+2.56%收$211.94；S&amp;P 500+1.79%收7,736.52創收盤新高、那指+2.6%、Palantir+29%；TSM+2.72%收$417.17連4日收高創本輪新高；AMZN-2.32%、META-0.39%——資金自hyperscaler轉入半導體；VIX 16.50。📊AMD Q2財報（8/4盤後）全面超標：營收$11.53B(+50% YoY、超共識~$11.3B)創新高、EPS $1.66超$1.62、資料中心$6.7B(+107%、占58%)、Q3指引$13B±0.3B遠超共識$12.52B——惟盤後重挫約-7~-9%（媒體報導、高「耳語數字」回吐）——需求數字對TSMC先進製程/CoWoS實質正面。⭐韓股V型再起：8/4尾盤收復（盤中-3%→三星收+0.21% 24.0萬、SK+0.64% 157.7萬）、今晨8/5盤中暴漲——SK+7.67%至169.8萬、三星+4.79%、KOSPI 6,670.67（較8/3+6.6%；8/4官方指數Yahoo缺漏）。📊BWIBBU官方P/E 31.19x/P/B 10.21x/殖利率0.95%；ADR溢價暴衝至+16.37%（$417.17 vs理論值$358.50、匯率32.36）——近期最大、今日補漲壓力極強。技術面依官方收盤重算（至8/4）：RSI 47.3、MACD綠柱-12.4續收斂（DIF-17.8零軸下）、KDJ金叉延續（K53.9/D44.2/J73.3）、5MA 2,304/120MA 2,152仍站上；支撐2,310/2,304/2,215、壓力2,345/2,350/2,360/2,371/2,425/2,535。整體信號：中性偏多。⭐觀察：跳空收復2,350(60MA)/2,371(20MA)與否、外資連2賣能否翻買、AMD盤後跌勢對亞股AI情緒干擾（韓股今晨已大漲、暫未兌現）、232條款（仍未查得公布）與台美關稅談判（傳20%→~15%）。全程TWSE/Yahoo官方API取數。</t>
+          <t>報告日2026-08-05(Wed)。📊台美短線背離、今日補漲條件齊備：台股8/4連2日獲利了結——2330收NT$2,320(-50、-2.11%、開2,335/高2,360/低2,310、量41,021張低於5日均量53,044、額954.55億、277,787筆、TWSE確認)、跌破20MA 2,371與60MA 2,350（季線失守）；大盤僅-25.75點(-0.06%)收43,360.66、上漲578家&gt;下跌406家——矽光子/CPO/低軌衛星漲停潮、中小型接棒；華邦電+9.79%續強、日月光-4.10%、聯發科-1.15%拉回換手。⚠️籌碼：外資連2賣-12,430張（自-9,717擴大、「一日翻多」確認失敗）、投信+434連8買、自營-2,327、三大合計-14,323張（T86官方）；全市場BFI82U合計+20.1億（外資-57.3億、投信+271.7億大買、自營-194.3億）——外資調節集中權值、內資持續進場。⭐美股8/4半導體史詩級大漲：SOX+6.55%收12,179.26（自史高收斂至-16.8%）——ARM+17.36%收$280.56、INTC+10.84%站上$100、AMKR+9.89%、LRCX+7.85%、MU+7.62%、KLAC+6.95%、AVGO+6.61%、AMAT+5.48%、ASML+4.22%、NVDA+2.56%收$211.94；S&amp;P 500+1.79%收7,736.52創收盤新高、那指+2.6%、Palantir+29%；TSM+2.72%收$417.17連4日收高創本輪新高；AMZN-2.32%、META-0.39%——資金自hyperscaler轉入半導體；VIX 16.50。📊AMD Q2財報（8/4盤後）全面超標：營收$11.53B(+50% YoY、超共識~$11.3B)創新高、EPS $1.66超$1.62、資料中心$6.7B(+107%、占58%)、Q3指引$13B±0.3B遠超共識$12.52B——惟盤後重挫-8.82%收$472.85（19:59 ET最終讀數、高「耳語數字」回吐）——需求數字對TSMC先進製程/CoWoS實質正面。⭐韓股V型再起：8/4尾盤收復（盤中-3%→三星收+0.21% 24.0萬、SK+0.64% 157.7萬）、今晨8/5盤中暴漲——SK+7.67%至169.8萬、三星+4.79%、KOSPI 6,670.67（較8/3+6.6%；8/4官方指數Yahoo缺漏）。📊BWIBBU官方P/E 31.19x/P/B 10.21x/殖利率0.95%；ADR溢價暴衝至+16.38%（$417.17 vs理論值$358.47、匯率32.36）——近期最大、今日補漲壓力極強。技術面依官方收盤重算（至8/4）：RSI 47.3、MACD綠柱-12.4續收斂（DIF-17.8零軸下）、KDJ金叉延續（K53.9/D44.2/J73.3）、5MA 2,304/120MA 2,152仍站上；支撐2,310/2,304/2,215、壓力2,345/2,350/2,360/2,371/2,425/2,535。整體信號：中性偏多。⭐觀察：跳空收復2,350(60MA)/2,371(20MA)與否、外資連2賣能否翻買、AMD盤後跌勢對亞股AI情緒干擾（韓股今晨已大漲、暫未兌現）、232條款（仍未查得公布）與台美關稅談判（傳20%→~15%）。全程TWSE/Yahoo官方API取數。</t>
         </is>
       </c>
       <c r="G100" s="53" t="inlineStr">

</xml_diff>

<commit_message>
daily: 2026-08-21 日報 HTML & Excel 更新
台股 2330 8/20 收 NT$2,375（+25、+1.06%）止跌反彈收最高、外資翻多買超 734 張；
量縮 28.2% 屬賣壓暫歇、季線 2,378 僅差 3 點未收復；ADR TSM $416.00（+0.95%）。
補正 AMKR 與 ARM 前兩日因取數失敗而沿用的舊值。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-08-20</t>
+          <t>報告更新日期：2026-08-21</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3339,7 +3339,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-08-20</t>
+          <t>最後更新：2026-08-21</t>
         </is>
       </c>
     </row>
@@ -7194,6 +7194,43 @@
         </is>
       </c>
       <c r="G109" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="53" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B110" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,375（8/20收）</t>
+        </is>
+      </c>
+      <c r="C110" s="54" t="inlineStr">
+        <is>
+          <t>+1.06%（8/20收）</t>
+        </is>
+      </c>
+      <c r="D110" s="53" t="inlineStr">
+        <is>
+          <t>US$416.00（8/20收）</t>
+        </is>
+      </c>
+      <c r="E110" s="53" t="inlineStr">
+        <is>
+          <t>16,968（8/20收）</t>
+        </is>
+      </c>
+      <c r="F110" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-08-21(Fri)，涵蓋8/20(Thu)收盤。⭐⚠️止跌反彈收最高、外資翻多買超734張，但量縮28%、季線僅差3點未收復：(1)⭐價格面三個止跌訊號成立——8/20官方收NT$2,375(+25、+1.06%、開2,365/高2,375/低2,350、量16,968張、額401.17億、46,361筆)：收盤價=當日最高價(無上影線的強勢收盤)；盤中低2,350恰為8/19收盤、回測前收即獲支撐，8/19低點2,335全日未再受測試；開盤2,365即跳入8/19跳空缺口2,355~2,380之內、終場回補約65%(尚差5點至上緣2,380)。(2)⭐均線失守由「四線」收斂為「三線」：收2,375重新站上20MA 2,358(=布林中軌)，仍在60MA季線2,378(差3點)/5MA 2,380(差5點)/10MA 2,390(差15點)之下，120MA年線2,206安全。⭐⭐2,378~2,390僅12點內擠壓三條均線且5MA 2,380與缺口上緣重合——今日(8/21)只要上漲0.2%即可同時收復季線與5MA並完成缺口回補，為本波回檔以來最接近修復的位置。(3)⭐⭐籌碼面本波最重要反轉：外資由8/19的-7,418張翻為買超+734張(T86官方原始+734,132股)、投信由-668張翻為+399張(8/13以來最大)、自營商-17張(自行-288/避險+271)，三大法人分項加總淨買超+1,116張(官方合計欄換算+1,117張，差1張屬四捨五入正常誤差)。⚠️惟一項矛盾：TAIFEX官方外資台股期貨淨空單自81,501口續增922口至82,423口(多6,959/空89,382)、投信淨多單75,825口、自營淨多單2,019口——外資「現貨回補、期貨加空」可能屬避險配置而非方向性看多，削弱現貨買超的多方訊號。(4)⚠️⚠️本日最大隱憂是量能：16,968張較8/19的23,619張大減28.2%、較5日均量19,046張萎縮10.9%，成交筆數自193,704筆驟降至46,361筆(-76.1%)——「量縮價漲」代表8/19恐慌換手已結束但接手方轉觀望，屬賣壓暫歇而非買盤進場；對照8/13突破時的26,233張放量上攻，本次反彈量能基礎薄弱。(5)⭐相對強弱首度反轉：2330 +1.06%同時優於加權指數+0.48%(收44,933.74)與費半SOX +0.53%(收11,800.02)，為本波回檔以來首見2330領漲(8/19為三項全數落後)；⚠️中期仍落後——5日-2.46%略遜加權-2.36%、20日-1.25%明顯落後加權+0.18%、YTD +49.8%落後加權+53.1%與費半+60.2%(對費半落後幅度自-11.0pp小幅收斂至-10.4pp)。(6)⚠️指標分歧：⭐RSI(14)自47.42回升至49.97重貼50中軸(8/19的跌破僅維持一個交易日)、KDJ的J值自4.91回升至13.15脫離極端超賣(驗證前一日日報判讀)；⚠️⚠️惟MACD柱狀圖連6日收縮至僅+1.10(8/12的+20.94→17.54→15.13→10.26→2.79→1.10、累計收斂94.7%)，且8/20股價上漲+1.06%而DIF反自+4.22降至+3.52(8/18-8/19重挫已透支快線動能)，死叉今日幾乎難以避免；⭐惟DIF+3.52與DEA+2.96雙雙仍在零軸之上，性質為「零軸之上多頭趨勢中的回檔」。(7)⭐⭐記憶體震央止穩是本次反彈最重要的外部支撐：韓股V型強彈——SK海力士+12.73%收169.1萬韓元、三星+9.49%收27.10萬韓元、KOSPI+5.89%收6,852.58並觸發Sidecar(與8/19崩跌-5.80%觸發熔斷相反)；驅動為SK海力士董事會決議買回約2,407萬股(約40.43兆韓元)並全數註銷、三年股東回饋強度自FCF 50%以內上修為50%以上。連帶美光+3.97%收$974.33、台股華邦電+5.06%收176.5、科林研發+1.09%。⚠️惟屬股東回饋題材而非記憶體需求/報價改善，對TSMC為情緒面外溢。(8)⚠️⚠️今晨最重要警訊——夜盤與美股方向與日盤反彈相反：8/20(美東)S&amp;P500 -0.87%收7,641.16、那斯達克-1.00%收26,067.17、VIX+7.52%升至16.01(8月新高區)，市場歸因於財政部擴大長天期公債回購後殖利率反彈、Fed會議紀錄較預期鷹派、觀望下週Fed主席Warsh的Jackson Hole演說；⭐費半SOX逆勢+0.53%，顯示驅動來自利率而非半導體基本面。⚠️台指期夜盤(8/20 15:00→8/21 05:00、列示日期2026/08/21)收44,804(-99對結算價、盤中低44,261一度重挫721點、量41,595口)對現貨逆價差擴大至-130；CDF 202609夜盤收2,373(-3、-0.13%)對現貨2,375翻逆價差-2——與8/19夜盤「開高走高、價差由逆轉正」完全相反，指向今日開盤偏弱或平盤附近。(9)⚠️生態系內部輪動分歧：上漲集中記憶體與設備(SK+12.73%、三星+9.49%、華邦電+5.06%、美光+3.97%、LRCX+1.09%、AMD+0.65%、AVGO+0.43%)，下跌集中AI運算與蘋果鏈(AAPL-1.75%收$311.30、KLAC-0.75%、QCOM-0.72%、INTC-0.72%、NVDA-0.33%收$216.85、ASML-0.08%)。⚠️⚠️兩項須留意：聯發科-3.77%收3,700、自8/14連4跌累計-12.11%(利空為Marvell擴大與Google的AI晶片合作、市場憂流失Google ASIC訂單、投信連12日賣超)；Amkor資料補正後顯示8/18 -10.54%、8/19 -7.20%、三日累計-17.03%為追蹤清單中本波最重(前兩日日報因取數失敗沿用舊值，本報已補正)，ARM同步補正三日-7.63%。(10)⚠️選擇權未平倉重建完成、P/C比恢復參考價值且首見跌破100%：8/20賣權未平倉31,742→54,070口(+70.3%)、買權31,036→54,415口(+75.3%)、合計62,778→108,485口(+72.8%)，P/C未平倉比99.37%(8/18結算前104.64%)為本波首見跌破100%——代表買權未平倉略多於賣權，依反向指標慣例屬情緒轉樂觀但避險保護不足；⭐惟雙邊僅差345口、實質為多空建倉均衡，不宜過度解讀。成交量P/C 111.81%(賣權182,976/買權163,649口)、成交規模自結算日729,967口回歸346,625口正常水位。(11)📊評價位階隨股價回升：P/E 27.53x(8/19 27.24x)、P/B 9.57x(9.47x)、殖利率0.93%(0.94%)、市值NT$61.6兆，財報基準仍為115/2(8/14換基準後未變、各日可比)；⚠️位階仍高(P/E約5年87百分位、P/B約91百分位)，本波回檔未使評價實質下移、評價保護有限。⚠️匯率逆風重啟：新台幣8/20收31.82、跌破8/17-8/18的31.85前低，自8/13的32.12累計升值約0.94%、估構成約-38bps毛利率逆風，將壓抑Q3毛利率指引65-67%上緣。ADR溢價自+11.63%收斂至+11.47%(ADR $416.00、平價$373.19、匯率31.82)。⭐今日觀察：⭐⭐第一順位關卡2,378~2,380(60MA季線+5MA=缺口上緣)，收復須搭配量能回補至19,046張之上否則屬假突破；下檔守2,358(20MA=布林中軌)/2,350/2,335，最後防線120MA 2,206。⚠️外資是否連2買超、期貨淨空單82,423口是否同步減少為第一順位籌碼訊號。⚠️預期MACD今日死叉成立，判讀重點在DIF是否守住零軸(+3.52)而非死叉本身。⚠️⚠️外部事件：今日(8/21美東)為Apple回覆美國參議院「是否採購中國長鑫存儲CXMT/長江存儲YMTC記憶體」的期限(Banks與Schumer等6-7位參議員7/30聯名致函)，截至產製時未查得已回覆；下週Fed主席Warsh的Jackson Hole演說為利率路徑關鍵。⚠️未結案追蹤：寶山F20廠8/17工安事故(承包商工人遭逾500公斤配電盤壓斃、公司已自主停工)之復工與調查進度，8/20-8/21無新報導；台積電官方新聞稿核對至8/21上午止無新發布(最新為8/11 Sony合作案與董事會決議)。📅9/10前公布8月營收——檢核點：Q3指引中位$45.2B換算月均約需NT$4,851億、7月的4,675.81億仍低約3.6%，8-9月需加速。全程TWSE/TAIFEX/Yahoo官方API取數；技術指標依TWSE官方序列2026-01-02~08-20共152筆重算，並回算驗證8/19各值(RSI 47.42、DIF+4.22/DEA+2.83/柱+2.79、K41.41/D59.66/J4.91、MA5 2,392/MA10 2,388/MA20 2,360/MA60 2,377/MA120 2,203、vol_ma5 20,899張)與8/20已發布日報完全一致，確認序列連續無口徑漂移。</t>
+        </is>
+      </c>
+      <c r="G110" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-08-24 日報 HTML & Excel 更新
涵蓋 8/21 (Fri) 收盤：2330 NT$2,410 (+35, +1.47%)、ADR TSM $418.95 (+0.71%)。
修復完成——五條均線全收復、8/19 跳空缺口 100% 回補、外資單日買超 5,795 張
(前日 7.9 倍)、三大法人首見同步買超；MACD 死叉預期落空、紅柱擴張至 +4.40。
情緒由「中性」上調至「中性偏多」。

兩項判讀修正（誠實記錄）：
- 前報預期「MACD 死叉幾乎難以避免」未實現且方向相反，已於 macd_signal 明載對照。
- 前報「8/20 起 P/C 比恢復參考價值」須更正：8 月序列顯示週三與週五皆有選擇權
  到期結算，8/21 讀數同屬重建期，新增「僅週一二四具跨日可比性」的判讀紀律。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-08-21</t>
+          <t>報告更新日期：2026-08-24</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3339,7 +3339,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-08-21</t>
+          <t>最後更新：2026-08-24</t>
         </is>
       </c>
     </row>
@@ -7231,6 +7231,43 @@
         </is>
       </c>
       <c r="G110" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="50" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B111" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,410（8/21收）</t>
+        </is>
+      </c>
+      <c r="C111" s="51" t="inlineStr">
+        <is>
+          <t>+1.47%（8/21收）</t>
+        </is>
+      </c>
+      <c r="D111" s="50" t="inlineStr">
+        <is>
+          <t>US$418.95（8/21收）</t>
+        </is>
+      </c>
+      <c r="E111" s="50" t="inlineStr">
+        <is>
+          <t>18,922（8/21收）</t>
+        </is>
+      </c>
+      <c r="F111" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-08-24(Mon)，涵蓋8/21(Fri)收盤。⭐⭐修復完成：五線全收復、缺口全回補、外資單日狂買5,795張、MACD死叉預期落空——(1)⭐⭐價格與均線：8/21官方收NT$2,410(+35、+1.47%、開2,375/高2,410/低2,365、量18,922張、額452.76億、59,539筆)，連2個交易日收在當日最高價；收盤一舉站上全部五條均線——5MA 2,383(高27點)/10MA 2,394(高16點)/20MA 2,361(高49點)/60MA季線2,380(高30點)/120MA年線2,210(高200點)，均線失守數三日內走完「四線→三線→零線」，並一次攻克前報標定的2,378~2,390三線密集帶、收在其上緣之上20點。⭐8/19跳空缺口2,355~2,380已100%回補(8/20僅約65%)，2,380由壓力翻轉為支撐；低點結構逐日上移(2,335→2,350→2,365)，無一日回測前日低點。(2)⚠️唯一保留是量能且須誠實記錄為「擦邊未達」：18,922張較8/20的16,968張回升11.5%、成交筆數自46,361筆增至59,539筆(+28.4%)，量價同步放大方向正確；但仍低於前報明訂的修復門檻(5日均量19,046張)約0.7%(差124張)。⭐實質應歸類為「溫和放量突破」——與8/20「量縮28.2%的價漲」性質完全不同；⚠️惟明顯不及8/13突破時的26,233張爆量，不足以認定趨勢行情啟動。⚠️另注意vol_ma5已自19,046張降至18,598張，係高量的8/13移出計算窗(窗口效應、非量能萎縮)，今日判定量能應沿用19,046張原門檻，勿讓標準被動放寬。(3)⭐⭐籌碼面為本日最強訊號且內部矛盾正在消解：外資及陸資買超2330達+5,795張(T86官方原始+5,795,046股)，為8/20的+734張的7.9倍、亦是追蹤區間(8/13以來)最大單日買超(超越8/14的+4,442張)；投信+292張(連2買)、自營商+457張(自行+407/避險+50、由-17張翻多)，⭐三大法人首見同步買超、分項加總淨買超+6,544張(與官方合計欄換算一致)。⭐⭐更關鍵的質變在期貨：TAIFEX官方外資台股期貨淨空單自82,423口僅續增171口至82,594口(多6,735/空89,329)，而8/20增幅為922口(減緩81%)——現貨買超放大7.9倍、期貨加空縮小5.4倍，隱含避險比例大幅下降，代表外資買盤性質由8/20的「避險性配置」轉向「方向性看多」，前報所要求的驗證條件獲實質改善；⚠️保留：淨空單絕對水位82,594口仍高、尚未轉為減少，確認仍不完整。投信淨多單76,316口、自營淨多單1,699口。(4)⭐⭐指標三項同步轉正，MACD死叉預期落空為本日最大意外——誠實對照：前一日日報明確預期「MACD死叉在今日幾乎難以避免」，實際結果為該預期未實現且方向完全相反。柱狀圖自+1.10擴張至+4.40(+300%)、終結連6日收縮；DIF自+3.52回升至+5.72、DEA自+2.96緩升至+3.51，兩線距離自0.56點重新擴大至2.21點，多頭排列反而強化。⭐機制：+1.47%(35點)的實體長紅足以拉抬快線EMA12，滿足前報所設的保留條件(「除非出現大幅跳空上漲」——雖非跳空，長紅已足夠)。⭐RSI(14)自49.97站上53.38(完成「跌破→回抵→站上」三步修復，RSI(6)達58.61、RSI(12)53.93)；⭐KDJ的J值自13.15暴升至44.14、K值39.73→49.21、K-D負乖離自-13.29點收斂至僅-2.54點(黃金交叉只需今日收平盤以上即成立，較前報推估的2-3個交易日大幅提前)。⚠️保留：柱狀圖+4.40僅為8/12的+20.94的21%，動能已轉向但強度未回到8月初水準。布林2,488/2,361/2,234(標準差63.4)。(5)⭐⭐相對強弱雙重反轉且為「逆勢領漲」：1日——2330 +1.47%同時優於加權指數+0.65%(收45,224.29)與費半SOX -0.51%(收11,740.37)，連2日領漲，且本次SOX是下跌的、2330屬逆勢領漲，強度高於8/20的同向領漲；5日——2330 +0.63%首度優於加權-1.28%，領先1.91個百分點，終結8月中旬以來的5日落後格局。⚠️中期落後未完全扭轉：20日+2.55%仍落後加權+3.60%(-1.05pp、自-1.43pp收斂)、YTD +52.1%落後加權+54.1%與費半+59.4%；⭐對費半YTD落後幅度自-10.4pp大幅收斂至-7.3pp，「權值股落後大盤」格局首度實質鬆動。⭐ADR TSM收$418.95(+0.71%、自我檢核416.00×1.0071=418.95✓)、連3日收高；溢價自+11.47%明顯收斂至+10.46%(本波最大單日收斂、平價$379.29、匯率31.77)，反映本地買盤力道首度超越海外資金，屬健康現象。(6)⭐週末前最後一段夜盤(8/21 15:00→8/22 05:00、TAIFEX列示交易日期2026/08/24)轉為正面，但個股期與指數期分歧：⭐台積電個股期CDF 202609夜盤收2,413(+4、+0.17%、開2,413/高2,423已超越日盤高點2,410/低2,405、量1,621口)，對現貨2,410由日盤逆價差-1翻為正價差+3，與8/20夜盤「開平走弱、價差由正轉逆」完全相反，指向今日台積電開盤偏強；⚠️惟台指期TX 202609夜盤開45,220/高45,474/低44,978/收45,074(-64對結算價、量30,890口)，自高點回落400點作收、對現貨逆價差擴大至-150。⭐⭐此「個股期強、指數期弱」與美股8/21型態完全一致(TSM ADR +0.71%逆勢收紅、費半-0.51%收黑、S&amp;P500 +0.43%收7,674.37、那斯達克+0.43%收26,180.46、VIX回落至15.13/-5.50%)，共同指向資金在半導體族群內部向代工龍頭集中而非全面性風險偏好回升——對2330個股偏正面、對台股大盤中性。CDF日盤收2,409(+33、+1.39%、量5,060口、未平倉26,630口)對現貨2,410為逆價差-1(僅1點、實質平價)。TX日盤收45,148(+245、+0.55%、量51,446口、未平倉102,342口)對現貨45,224.29為逆價差-76。(7)⚠️⚠️本週主導變數已由技術面轉為事件面——NVIDIA 8/26(週三)公布Q2 FY27財報(市場預期營收$93-95B、EPS $0.65-0.68)，其指引將直接檢核AI加速器與先進封裝需求是否延續。⭐供應鏈訊號：執行長黃仁勳已於8/23(週日)搭私人專機抵台(2026年第3次訪台)，市場推測係財報前與台積電等核心供應鏈閉門會議、敲定次世代AI晶片產能配置、CoWoS先進封裝配額與伺服器報價(⚠️會議內容與議題均屬市場推測、NVIDIA未回應；去年8/22亦有相同型態的財報前訪台)。TrendForce估TSMC CoWoS月產能2026年可擴至12-14萬片、加計委外夥伴5-6萬片後接近20萬片，惟HBM與CoWoS產能仍緊。⚠️⚠️背離警訊：NVDA股價8/21續跌-0.98%收$214.72、已連4日收黑(自8/17累計-4.57%)，財報前市場態度明顯保守，而2330卻連2日大漲——代表2330已提前反映樂觀預期，若財報或指引不如預期，回吐風險相對較高。⚠️判讀紀律：本週技術訊號的參考權重應調降、事件結果權重應提高。(8)⭐定價權題材強化、可部分抵銷匯率逆風：路透於8/19前後報導三星已自7月起將部分代工報價調升至多15%(以4奈米SF4為主、中國與美國客戶調幅10-15%)，市場分析直指主因為AI需求令台積電先進製程產能飽和、客戶「無處可去」而回流三星(台積電Q1全球代工營收市占逾70%、三星約7%)；另有報導指台積電規劃明年先進製程調價約10%、HPC訂單若超出需求預測將再加10-15%。⭐台積電並自陳對記憶體廠毛利率「感到羨慕」但明確限制自身漲幅，理由是客戶無法承受4-5倍漲價(記憶體廠Q1即調價65-90%)，顯示以客戶關係穩定性換取長期訂單能見度。⚠️對沖關係：定價權效益需與匯率逆風相抵。(9)⚠️⚠️評價位階警訊——回檔對評價的修正效果已被兩日反彈完全抵銷：8/21 TWSE官方BWIBBU顯示P/E 27.94x(8/20為27.53x)、P/B 9.72x(9.57x)、殖利率0.91%(0.93%)、市值約NT$62.5兆，財報基準仍為115/2(8/14換基準後未變、各日可比)。⚠️位階各上移1個百分位至P/E約5年88百分位、P/B約92百分位——意即8/17-8/19的三日回檔並未留下任何評價折讓，修復完成後評價保護反而比回檔前更薄。⭐PEG 0.82低於1仍為主要辯護理由；⚠️惟其分母(FY26 EPS成長率)高度依賴AI需求延續，若NVIDIA 8/26財報下修展望，PEG辯護力將同步減弱——本週評價面最大單一風險。⚠️匯率逆風續增：新台幣8/21收31.77(創8月新高)，自8/13的32.12累計升值約1.09%、依官方口徑(每升值1%約-40bps)估構成約-44bps毛利率逆風(8/20估-38bps)，將壓抑Q3毛利率指引65-67%上緣。⚠️匯率口徑例外：Yahoo TWD=X日線序列缺漏8/21該筆，改以同來源逐時序列取8/21 16:00(台北收盤時點)讀數31.77，與前一日採日線的31.82口徑略有差異，正式值請以央行/台北外匯經紀公司公告為準；⚠️故31.82→31.77的0.16%變動幅度存在口徑誤差，方向(續升值)則明確。⚠️⚠️尚未被股價反映的落差：股價創本波反彈新高(2,410)與匯率創本波升值新高(31.77)同時發生。(10)⚠️選擇權P/C比判讀紀律本報作出重要修正：前一日日報曾判定「8/20起P/C比恢復參考價值」，本報依8月完整官方序列複核後必須更正——TAIFEX未平倉序列顯示8月每逢週三「與週五」雙邊未平倉均大幅結清(8/5 94,288→58,701、8/7 79,558→59,446、8/12 102,705→60,479、8/14 82,705→65,051、8/19 93,656→31,742、8/21 54,070→35,710共6次)，呈現週三、週五各有一次到期結算的規律，代表台指選擇權週別合約在週三與週五皆有到期日。⚠️因此8/21(週五)雙邊未平倉自108,485口驟降至70,119口(賣35,710/買34,409、-35.4%)屬到期結算的機械效果、非籌碼撤離，其P/C未平倉比103.78%與8/20的99.37%並非同一基數、不可直接比較方向。⭐可確立者：賣權未平倉重新多於買權1,301口、比率回到100%之上，代表結算後新建倉略偏避險，與同日現貨大漲+1.47%並不矛盾(上漲中買保險屬理性)。⭐新紀律：P/C未平倉比僅在週一、週二、週四具跨日可比性；週三與週五的讀數只看絕對水位(100%為分界)、不看變化幅度。成交量P/C 110.65%(賣權358,085/買權323,629口)、總成交681,714口為8/19結算日以來次高，符合結算日放量特徵。(11)⚠️生態系內部分化擴大：⭐上漲者集中代工與部分客戶/記憶體(2330 +1.47%、三星+3.87%收28.15萬韓元創本波新高、華邦電+2.55%收181.0、聯發科+2.43%收3,790終結連4跌、SK海力士+2.31%收173.0萬韓元續創新高、AVGO +1.21%、LRCX +1.12%、AMD +0.81%、ASML +0.77%、QCOM +0.01%)；⚠️下跌者集中設備、封測與AI運算(ARM -2.95%收$243.32創新低、INTC -2.24%收$90.07連4跌、AMKR -1.18%收$50.26連4跌、KLAC -1.01%連4跌、NVDA -0.98%連4跌、AMAT -0.78%、MU -0.77%、AAPL -0.63%、3711日月光-0.51%)。⚠️⚠️三項須留意：AMAT距2年高點已達-20.4%正式跌破熊市門檻；KLAC距2年高點-39.0%為修正最深設備股、與AMAT同步走弱值得留意是否預示先進製程資本支出實質放緩；AMKR自8/17累計-18.01%仍為追蹤清單中本波最重且完全未受8/20-8/21反彈帶動。⭐封測疲弱(日月光、AMKR)顯示市場對後段封裝疑慮未解，若NVIDIA財報確認CoWoS吃緊則有補漲空間。(12)📅事件與未結案追蹤：⚠️Apple回覆美國參議院「是否採購中國長鑫存儲CXMT/長江存儲YMTC記憶體」的期限已於8/21(美東)屆至(Banks、Schumer、Crapo、Shaheen、Kim、Risch、Ricketts等7位參議員7/29聯名致函，要求說明測試/驗證現況、涉及產品線與記憶體類型、與美國官方討論情形)，⚠️截至本報產製時查無Apple已回覆或回覆內容的公開報導，列為「未能證實」而非「已確認未回覆」；Apple約占TSMC營收17%，本案聚焦記憶體、不直接觸及邏輯代工。⭐寶山F20工安事故(8/17下午22歲承包商工人搬運逾500公斤配電盤時遭壓斃)新增查證：業界分析指台積電廠區建造順序為CUP控制中心/SUP支援中心→Fab晶圓製造與無塵室→最後才是辦公棟，依現有官方回應停工僅涉辦公棟相關作業，故評估不影響晶圓廠建置進度與2奈米量產時程；⚠️惟8/22-8/24查無復工時程或勞檢調查結果，仍列未結案。⭐台積電官方新聞稿核對至8/24上午止無新發布(最新仍為8/11的董事會決議與Sony影像感測器合資案)。⭐面板廠跨入先進封裝：TPK宸鴻8/21法說會宣示跨入半導體第二隻腳、鎖定AI高階ASIC所需封測玻璃鑽孔(TGV)技術；群創投入扇出型面板級封裝(FOPLP)並傳出與台積電合作開發高階封裝(⚠️屬傳聞、未經台積電證實)——玻璃基板與面板級封裝被視為CoWoS之後的下一代路徑，惟技術成熟度與導入時程尚早，短期財務影響可忽略。📅9/10前公布8月營收——檢核點：Q3指引中位$45.2B換算月均約需NT$4,851億、7月的4,675.81億仍低約3.6%，8-9月需加速。⭐綜合研判：由「中性」上調至「中性偏多」——技術面與籌碼面的修復證據已足以支持偏多，但量能未達標(擦邊0.7%)與高評價位階(P/E約88百分位)使其不足以升至「看多」。今日(8/24)判定標準：守住2,380(由壓力翻轉的支撐)＝突破有效性確立、可期待挑戰2,435(8/14收盤)；帶量(&gt;19,046張)攻克2,435＝趨勢行情確認；跌破2,380並回落至2,361的20MA之下＝突破失敗、視為假突破。上方壓力2,435/2,470/2,488/2,535，下檔支撐2,380/2,365/2,361/2,350/2,234/2,210。全程TWSE/TAIFEX/Yahoo官方API取數；技術指標依TWSE官方序列2026-01-02~08-21共153筆重算，並回算驗證8/20各值(RSI 49.97、DIF+3.52/DEA+2.96/柱+1.10、K39.73/D53.02/J13.15、MA5 2,380/MA10 2,390/MA20 2,358/MA60 2,378/MA120 2,206、布林2,483/2,358/2,233、vol_ma5 19,046張)與8/21已發布日報完全一致，確認序列連續、無口徑漂移。</t>
+        </is>
+      </c>
+      <c r="G111" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-08-26 日報 HTML & Excel 更新
涵蓋 8/25 收盤：2330 NT$2,400（+25、+1.05%）、TSM $417.41（+1.78%）。
另修正兩處資料呈現問題：
- 期貨基差標籤原硬編碼「（正價差）」，基差轉負時會標錯，改為依正負號切換。
- 「主要行使價未平倉分布」原以具體口數呈現本報估算值，易誤讀為 TAIFEX
  官方逐履約價數據，改為定性描述並標註「本報估算」。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-08-25</t>
+          <t>報告更新日期：2026-08-26</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G112"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3339,7 +3339,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-08-25</t>
+          <t>最後更新：2026-08-26</t>
         </is>
       </c>
     </row>
@@ -7305,6 +7305,43 @@
         </is>
       </c>
       <c r="G112" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="50" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B113" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,400（8/25收）</t>
+        </is>
+      </c>
+      <c r="C113" s="51" t="inlineStr">
+        <is>
+          <t>+1.05%（8/25收）</t>
+        </is>
+      </c>
+      <c r="D113" s="50" t="inlineStr">
+        <is>
+          <t>US$417.41（8/25收）</t>
+        </is>
+      </c>
+      <c r="E113" s="50" t="inlineStr">
+        <is>
+          <t>13,538（8/25收）</t>
+        </is>
+      </c>
+      <c r="F113" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-08-26(Wed)，涵蓋8/25(Tue)收盤。⭐⭐反轉成立：先破底再收最高、五線全數收復、KDJ黃金交叉補上，惟量能仍居全年第3低、外資連2日賣超——(1)⭐⭐價格與型態：8/25官方收NT$2,400(+25、+1.05%、開2,355/高2,400/低2,350、量13,538張、額321.30億、57,334筆)。本日最具辨識度的事實是收盤價＝當日最高價，且為跳空低開(開2,355、較前收2,375低20點)後全程收復，形成實體45點、下影線5點、完全無上影線的長紅「破底翻」——與8/24「開盤價＝最高、收盤價＝最低」的光頭光腳長黑構成完整鏡像反轉。低點結構的關鍵細節：盤中低2,350恰為8/19收盤價與8/20盤中低所在，該價位在6個交易日內第2次獲得承接並拉出長紅，由「參考價位」升格為實質支撐；8/19波段低2,335全程未被測試。全日振幅50點(2.11%)大於8/24的35點，代表多空交戰強度提高而非單向縮量。(2)⭐⭐前一日日報所訂檢核條件全數翻正，本報有義務逐條對照：前報將「20MA／布林中軌2,362.5的防守」列為第一順位，並訂出「須連續2日站回2,380之上才可視為修復重啟」。實際結果：8/25盤中低2,350曾下破20MA達12.5點，但收盤2,400不僅收復2,362.5，更一舉越過2,380驗證位與全部五條均線(5MA 2,382/10MA 2,394/20MA 2,369/60MA 2,382/120MA 2,217)——第一順位檢核通過、8/24的突破失敗在隔一個交易日即被修復；⚠️惟「連續2日站穩2,380」僅完成第一天，8/26收盤才是真正的判定日，本報不提前宣告修復完成。8/19跳空缺口2,355~2,380由「上緣得而復失」重回「完全回補」。(3)⚠️⚠️唯一未改善的是量能，必須明確標示而非淡化：13,538張為2026年155個交易日中第3低(本報已以TWSE官方序列複核全年，最低為8/24的13,073張、次低為8/17的13,482張)，較5日均量17,224張少21.4%。⭐量能結構略見改善：成交筆數自84,694筆降至57,334筆(-32.3%)，每筆平均張數自0.154張回升至0.236張，屬「散單退場、大單略回」，方向與8/24的「散單增加、大單縮手」相反。⚠️但整體參與度仍極低，無量上漲的可靠度本質上有限——這是本次反轉最主要的瑕疵；⭐平衡的另一面是全年第3低量能同時意味8/24的長黑並未引出真實賣壓，跌不下去與漲不上去同時成立。(4)⚠️籌碼面分歧為第二項保留意見：外資及陸資連2個交易日賣超2330(8/25 -1,151張、T86官方原始-1,151,127股；8/24 -1,621張，2日合計-2,772張)，與價格反轉方向完全相反；⭐反向的是投信買超658張——為近5個交易日最大單日買超(近5日：-668/+399/+292/+157/+658)，自營商亦買超475張(自行+37,599股、避險+437,978股)。三大法人分項加總-18張、官方合計欄-17張(四捨五入差)，幾近完全打平，意味本日上漲主要由非三大法人資金(散戶、中實戶)與空方回補推動，而非外資回頭。⚠️對照8/21的上漲(外資狂買5,795張、量18,922張)，本次反轉的資金品質明顯較差，這是本報將評級定為「中性偏多」而非「看多」的主要理由。TAIFEX台指期未平倉：外資淨空單85,380口(多5,030/空90,410)、投信淨多單76,309口、自營淨多單2,501口——外資期貨仍為大幅淨空，與其現貨連2日賣超方向一致。(5)⭐技術指標由8/24的「同步回頭」轉為「同步翻正」，四項全數改善(TWSE官方序列2026-01-02~08-25共155筆計算)：RSI(14) 49.73→52.24重新站上50中軸；RSI(6) 47.36→54.80(+7.44點，並已高於RSI(14)達2.56點，短長天期相對位置由「短弱長強」翻為「短強長弱」)；MACD柱狀圖+1.71→+3.05(擴張78.4%)、DIF +4.58→+5.63、DEA +3.73→+4.11，DIF上升快於DEA使正乖離自0.85擴大至1.53，死亡交叉威脅在數學上被明確推遠，且DIF與DEA雙雙位於零軸之上並呈DIF&gt;DEA，屬MACD最強的「零軸上方多頭排列」；KDJ黃金交叉正式成立(K 44.93→49.65上穿D 49.48→49.53，K-D由-4.55翻正為+0.12)。⚠️誠實標示三項限制：該金叉是前報預期落空後延後一日補上；乖離僅0.12點、屬統計上幾可忽略；三值(49.65/49.53/49.88)幾乎重合於50，代表多空在中性位置短暫平衡而非多方取得優勢。⚠️另須指出MACD本波的反覆：柱狀圖8/20 +1.10→8/21 +4.40→8/24 +1.71→8/25 +3.05，四個交易日內兩次大幅反轉，日間讀數缺乏趨勢意義，須連續2-3日同向擴張才具確認力。布林2,491/2,369/2,247。(6)⚠️衍生品透露的訊息與價格不完全一致，值得單獨列出：台積電個股期CDF 202609日盤收2,399(+14、+0.59%、開2,371/高2,401/低2,357、量5,074口、結算價2,399、未平倉26,519口)，對現貨2,400由8/24的正價差+9轉為逆價差-1——期貨未跟上現貨尾盤拉抬；未平倉自26,755減至26,519口(-236口)，量增而OI減屬「當沖與平倉」性質，非新資金建立多單。⚠️這是本日技術面翻正之外最值得保留戒心的一項，代表拉升由現貨買盤主導而非期貨帶動。⭐今晨夜盤(8/25 15:00→8/26 05:00、TAIFEX「盤後」列日期為8/26)明確轉強：CDF 202609收2,408(+9、+0.38%、開2,406/高2,411/低2,397、量1,115口)對現貨回到正價差+8；台指期TX 202609夜盤收45,437(+405、+0.90%、開45,093/高45,470/低45,020、量28,479口)，跟隨美股費半+1.44%走強——兩者同步為8/26台股開盤提供偏多初始條件。⭐選擇權未平倉P/C比自95.81%升至101.99%(賣權62,319口首度超過買權61,102口)；依本報已確立的判讀紀律(台指選擇權週三與週五皆有到期結算，P/C未平倉比僅在週一、週二、週四具跨日可比性)，8/24為週一、8/25為週二，兩者同屬非結算重建期、基數一致，這是本週第一個可直接比較的讀數。⚠️表面上P/C&gt;1屬偏空，但在股價同日上漲+1.05%且今晚有NVIDIA財報的情境下，本報判讀為「避險性買進賣權」而非方向性看空；成交量P/C 110.78%(賣權197,640/買權178,414口)同步偏高，印證財報前避險需求。⚠️若8/27(週四、下一個可比日)P/C續升而股價下跌，則須改判為真實看空。(7)⭐相對強弱由落後轉為領先：1日——2330 +1.05%小幅領先加權指數+0.91%(收45,169.46、+407.14點、額7,242.58億、⭐盤中最低曾下探44,210.31達-1.23%、尾盤逆轉收在當日最高，台積電估貢獻約200點)達0.14個百分點，⚠️惟落後費半SOX的+1.44%。5日——2330 +0.84%明顯領先加權-0.31%達1.15個百分點，相對強度已由8/24的落後轉為領先。1個月——2330 +2.13%落後加權+3.52%。YTD——2330 +51.4%落後加權+53.9%與費半+57.3%(YTD基準採2026-01-02收盤：2330 NT$1,585、加權29,349.81、SOX 7,367.47)，中期落後結構未改變。⭐ADR TSM收$417.41(+1.78%、+$7.29；三重自我檢核：410.12+7.29=417.41✓、410.12×(1+1.78%)=417.42✓、另經stockanalysis.com交叉確認收盤$417.41/+1.78%/前收$410.12✓)。⭐溢價自+9.93%擴大至+10.75%(+0.82pp、平價$376.88、匯率31.84)——ADR +1.78%明顯領先台股+1.05%達0.73pp，代表美股投資人在NVIDIA財報前對台積電的買進意願強於台股，屬領先訊號、對8/26台股偏正面；⚠️惟溢價已回到8月偏高區間，若財報不如預期，ADR回吐空間亦相對較大。(8)⭐外部環境全面轉好：8/25美股半導體反彈，費半SOX收11,588.04(+164.87、+1.44%)，終結8/24的-2.70%重挫。⚠️⚠️惟本報必須明確標註：距52週高點14,655.29(2026-06-22盤中高、收盤高為同日14,634.72)仍達-20.9%，僅自-22.1%收斂1.2pp，依-20%通行定義仍在技術性熊市之內、尚未脫離(本報已以1年日線序列獨立複核)。族群內部19檔追蹤標的中14檔收紅：AMD +4.91%收$479.18(明確催化劑為Raymond James上調至強力買進，並連帶帶動美超微SMCI +9.35%、為本日追蹤清單漲幅最大者)、MU +2.48%收$932.97(記憶體震央止跌)、NVDA +2.19%收$213.05(⭐終結連續7個交易日收黑)、AMKR +1.67%、LRCX +1.45%、QCOM +1.28%、ARM +1.16%、2344華邦電+1.13%收179.0、KLAC +0.97%、000660 SK海力士+0.42%收167.8萬韓元、INTC +0.25%、ASML +0.23%。⚠️收黑5檔：AMAT -0.86%收$480.04(⚠️在費半反彈日仍創本波新低、自8/17累計-10.32%、距2年高點-22.4%續處熊市)、2454聯發科-0.80%收3,735、AVGO -0.56%收$356.74(⚠️連2日下跌並創本波新低、自8/17累計-9.09%、與族群連續2日背離值得留意)、3711日月光-0.17%收591.0(⭐惟盤中低569.0曾達-3.9%、尾盤全數收復並收最高，實質強度優於表面數字)、AAPL -0.14%收$309.90(⭐仍為客戶族群唯一自8/17累計收紅者、+1.41%)。⭐三星電子8/25收平盤257,000韓元(0.00%)，與8/24(該日因股東回饋計畫失望暴跌-8.70%)收盤價完全相同——⭐⭐依本報既有紀律(連2日相同價位必須另尋來源確認)，已執行交叉查證：investing.com歷史資料與多篇韓媒報導一致證實為真實平盤(早盤一度重挫近4%、盤中完全收復)，非資料錯誤或延遲。⚠️三星8/24崩跌根因未解：受《金融產業結構改善法》限制而無法提出庫藏股銷除計畫，與SK海力士8/20宣布40兆韓元買回並全數註銷(當日+12.73%)形成治理面對比。美股大盤同步偏多：S&amp;P500 +0.32%收7,677.28、那斯達克+0.66%收26,151.30、VIX -2.52%收15.45(⭐NVIDIA財報前市場並未升溫)。(9)⚠️⚠️今晚(美東8/26盤後)NVIDIA公布Q2 FY27財報，是本週決定性變數，結果須待8/27台股開盤才反映：公司自身財測中值約$91.0B(±2%)、40位分析師共識約$91.85-92.2B(高於財測約0.9%，顯示市場認為公司指引偏保守；⚠️確切公布鐘點未能證實)。⭐客戶集中度的最新量化：NVIDIA 2025年貢獻TSMC營收約$231.6億、占比約19%，已超越蘋果成為第一大客戶；2026年預估攀升至約$330億、占比約22%。⚠️2330 8/25已上漲+1.05%、ADR更漲+1.78%提前反映樂觀預期，指引若不如預期則回吐風險相對較高。⚠️判讀紀律：本報所有判讀均不含該財報結果，且財報權重應顯著高於今日技術訊號。(10)⚠️評價位階小幅擴張：8/25 TWSE官方BWIBBU顯示P/E 27.82x(8/24為27.53x)、P/B 9.68x(9.57x)、殖利率0.92%(0.93%)、市值約NT$62.2兆，財報基準仍為115/2(8/14換基準後未變、各日可比)。⭐本日變化純由股價+1.05%帶動、分母未動，屬評價的實質微幅擴張而非財報更新。⚠️P/E仍位於5年區間第87百分位、10年第88百分位，P/B第91百分位——評價偏貴的結構未變，自8/17起算的整段震盪並未提供實質評價折讓；PEG 0.82低於1仍是主要辯護理由，⚠️惟其分母(FY26 EPS成長率)高度依賴AI需求延續，今晚NVIDIA財報若下修展望，PEG辯護力將同步減弱。⭐匯率逆風連2日小幅緩解：新台幣8/25收31.84(Yahoo TWD=X逐時序列16:00台北時點)，自8/24的31.83再回貶約0.03%，連2個交易日走弱；相對8/13的32.12累計升值幅度自0.90%縮小至0.87%，依官方口徑(每升值1%約-40bps)估算毛利率逆風自約-36bps縮小至約-35bps。⚠️誠實標註：本日變化幅度極小(0.01元)、不足以改變基本面判斷，僅記錄方向；且盤中一度升至31.87-31.89(11:00-13:00)，日內波動明顯大於日間變化。(11)⭐產業與公司面新增資訊：DIGITIMES 8/25報導指AI資料中心用電需求成為全球電力與半導體供應鏈新壓力點，台灣晶圓代工產能持續吃緊、帶動晶片報價2026下半年走升(⭐與Q3毛利率指引65-67%方向一致；⚠️另一面是台灣電力瓶頸為結構性限制)。台積電於2026台灣科技論壇揭露：2nm與A16製程產能2026-2028年CAGR達70%、CoWoS／SoIC先進封裝產能成長率逾80%(至2027年)；CoWoS 5.5倍光罩尺寸良率已突破98%；CoWoS月產能預估2026年底達12-13萬片、較2023年底的1.3萬片擴增近10倍；先進封裝產能已連續三年每年倍增，仍無法完全消化AI半導體暴增需求。⚠️法規面：日本經產省2026-05-29修訂《外匯及外貿法》，首度將Chiplet、3D堆疊、CoWoS、TSV等先進封裝後段設備納入出口管制，已於8/1生效，主要限制對中國大陸出口(⭐對台積電偏正面：陸廠受限強化其CoWoS領先地位；⚠️惟地緣政治風險結構性升高)。⚠️美國8/6宣布半導體進口課徵100%關稅、在美設廠可豁免，台積電亞利桑那已追加1,000億美元投資(總承諾$165B)、CEO魏哲家表示看好AI需求延續至2029-2030年——⚠️本報須標註：正式生效日期與232條款配套執行細則尚未查得官方公告原文，屬「未能證實」。(12)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方API取數，ADR另經stockanalysis.com交叉確認、三星與SK海力士另經investing.com及韓媒交叉確認。⚠️匯率採Yahoo TWD=X逐時序列8/25 16:00台北收盤時點讀數31.84(日線序列缺漏該筆)，與前一日同法取得的8/24 31.83口徑一致、可直接比較，正式值請以央行／台北外匯經紀公司公告為準。技術指標依TWSE官方序列2026-01-02~08-25共155筆重算，並回算驗證8/24各值(RSI(14) 49.73、RSI(6) 47.36、DIF+4.58/DEA+3.73/柱+1.71、K44.93/D49.48/J35.84、MA5 2,378/MA10 2,393/MA20 2,362.5/MA60 2,381.5/MA120 2,213.1、布林2,489/2,363/2,236、5日均量18,516張)與8/25已發布日報所載數值逐項完全一致，確認序列連續、無口徑漂移。⚠️本報主動更正既有呈現方式：HTML日報「主要行使價未平倉分布」一表的買賣權欄位，先前以具體口數呈現易被誤讀為TAIFEX官方逐履約價數據，實則台積電個股並無選擇權逐履約價公開序列，本日起改為定性描述並明確標註「本報估算」；表頭卡片的Call/Put未平倉總量與P/C比仍為TAIFEX台指選擇權官方數據。⭐綜合研判：由「中性偏空」上調至「中性偏多」——先破底再收最高的教科書式反轉、五線全數收復、四項技術指標同步翻正、KDJ黃金交叉補上，8/24的突破失敗在隔一個交易日即被修復；⚠️但這次修復有三個必須並列的瑕疵：量能仍是全年第3低(反轉無量)、外資連2日賣超2,772張與價格背離、CDF期貨轉逆價差且未平倉減少(期貨未跟上現貨)。技術面位置已回到8/21，但資金品質明顯不如8/21，故不直接跳到「看多」。⚠️⚠️真正的裁決點有二：今晚NVIDIA財報，以及8/26收盤能否守住2,380(前報所訂「連續2日站穩」的第二天)。今日(8/26)判定標準：收盤守在2,380之上＝修復完成、8/21多方結構重新確立；跌回2,380以下＝8/25僅屬單日反彈。第二順位為量能須回補至5日均量17,224張之上。上方壓力2,410/2,435/2,470/2,491/2,510/2,535，下檔支撐2,394/2,382/2,375/2,369/2,350/2,335/2,247/2,217。</t>
+        </is>
+      </c>
+      <c r="G113" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-08-28 日報 HTML & Excel 更新
涵蓋 8/27 (Thu) 收盤。2330 收 NT$2,410 (-5, -0.21%)，開 2,430/高 2,435/低 2,410，
收在全日最低 —— 前報所訂「開高走低」與「利多下仍落後大盤」兩項警訊條件均成立，
評級自「偏多」下調至「中性」。

同時修正一項既有缺陷：HTML 技術分析區塊的「成交量」與「布林帶」卡片標籤
原為硬編（量縮整理／布林收窄整理），在放量日會與事實相反（本日量能高於
5 日均量 14.1%）。已改為依實際數值動態計算 VOL_LABEL / BB_LABEL，
作法與既有的 BASIS_LABEL、F5D_LABEL 一致。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-08-27</t>
+          <t>報告更新日期：2026-08-28</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3339,7 +3339,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-08-27</t>
+          <t>最後更新：2026-08-28</t>
         </is>
       </c>
     </row>
@@ -7379,6 +7379,43 @@
         </is>
       </c>
       <c r="G114" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="50" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B115" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,410（8/27收）</t>
+        </is>
+      </c>
+      <c r="C115" s="57" t="inlineStr">
+        <is>
+          <t>-0.21%（8/27收）</t>
+        </is>
+      </c>
+      <c r="D115" s="50" t="inlineStr">
+        <is>
+          <t>US$427.30（8/27收）</t>
+        </is>
+      </c>
+      <c r="E115" s="50" t="inlineStr">
+        <is>
+          <t>19,214（8/27收）</t>
+        </is>
+      </c>
+      <c r="F115" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-08-28(Fri)，涵蓋8/27(Thu)收盤。⚠️⚠️利多出盡的教科書案例、且本報前一日訂出的兩項警訊條件全數成立：NVIDIA財報大超預期、TSM ADR隔夜+2.30%、費半+2.33%，2330卻開2,430(高2,435)走低收NT$2,410(-5、-0.21%)並收在全日最低，越過檢核價2,425後跌回其下；⚠️相對弱勢連續第2日成立且這次發生在直接利多之下，依前報所訂標準須認定為結構性輪動。⭐平衡事實：量能續守均量、外資連2日買超4,501張、五條均線全數未破——本日是「攻擊失敗」而非「趨勢轉空」，評級自「偏多」下調至「中性」——(1)⚠️⚠️價格與型態，前報第一號檢核條件成立且結果為負面：8/27官方收NT$2,410(-5、-0.21%、開2,430/高2,435/低2,410、量19,214張、額465.45億、60,122筆)。前一份日報明訂「檢核價位為8/26盤中高2,425——若今日跳空越過後又跌回其下，即為『利多出盡、開高走低』的明確警訊」，8/27開2,430(跳空高開15點)、盤中高2,435(越過檢核價10點)，收盤2,410回落至檢核價之下15點，條件完全成立，本報據實宣告而不因前一日看多而迴避。⚠️型態嚴重性高於-0.21%的跌幅所示：收盤價2,410＝當日最低價(全日無下影線)，為「光頭光腳黑K」，與8/25收在全日最高的長紅完全鏡像；黑K實體20點、上影線5點；盤中高2,435恰為本報所列第二壓力(8/14收盤價)，觸及未收上，該反壓確認有效。⭐三項緩和事實須並列：跌幅僅5點、黑K實體僅20點、低點2,410仍高於8/26低點2,375達35點(低點連3日墊高的結構未破)、收盤仍高於全部五條均線——本日是攻擊失敗，不是趨勢反轉。(2)⚠️⚠️前報第二號檢核條件同樣成立，判讀意義大於單日漲跌：前報明訂「若今日在NVIDIA直接利多下2330仍落後大盤，則須認定為結構性輪動而非單日現象」。加權指數8/27收45,975.22(+142.60、+0.31%、TWSE官方FMTQIK)，2330 -0.21%，落後0.52pp，為連續第2個交易日落後大盤(8/26落後0.84pp)。⚠️⚠️更值得警惕的是中期相對強度本日正式翻負：近5日2330 +1.47% vs加權+2.32%，落後0.85pp——⭐誠實對照，前一份日報當時的敘述是「中期結構尚未惡化，近5日2330 +2.77%仍略領先大盤+2.49%」，該領先已於本日消失，本報據實更新此判讀。1個月(+2.55% vs +5.37%)與YTD(+52.1% vs大盤+56.7%、費半+61.3%)的落後幅度亦同步擴大，其中對費半的落後自5.2pp擴大至9.2pp——費半8/27大漲+2.33%並脫離技術性熊市，2330卻未參與該族群性反彈，這是YTD差距單日擴大4.0pp的直接原因。YTD基準採2026-01-02收盤(2330 NT$1,585、加權29,349.81、SOX 7,367.47)。(3)⚠️⚠️本日最具診斷價值的觀察是台美兩地對同一項利多做出相反行為：ADR TSM 8/27正規盤+2.30%收$427.30明確追價，2330同日-0.21%開高遭調節，兩地分歧達2.51pp為近期最大，ADR溢價自+9.97%急升至+12.41%(+2.44pp、平價$380.13、匯率31.70)。⭐佐證此判讀的是聯發科的同型態：8/27開4,005(＝當日最高)收3,865(＝當日最低、-80、-2.03%、TWSE官方)，與2330同為跳空高開後收在全日最低——台股高價權值股本日普遍在開盤時被賣出，這不是台積電個股問題。⚠️進一步的驗證來自美股盤後：TSM於8/27盤後回落至$425.62(-1.68、-0.39%、讀數時點Aug 27 2026 7:59 PM EDT、經stockanalysis.com確認；自我檢核427.30-1.68=425.62✓)，追價力道在正規盤結束後亦告減弱，方向與台股一致。⭐判讀：利多在兩地是先後被消化，只是台股領先一步反映。ADR收盤三重自我檢核：417.69+9.61=427.30✓、417.69×(1+2.30%)=427.30✓、stockanalysis.com交叉確認$427.30/+2.30%/前收$417.69/讀數時點Aug 27 2026 4:00 PM EDT✓。(4)⭐籌碼面是本日唯一明確偏多、且通過前報檢核的一項，本報不因價格收黑而略過：外資及陸資8/27買超4,501張(T86官方買進14,070,814股、賣出9,570,219股、買賣超+4,500,595股)，連續第2個交易日買超、2日合計買超9,705張，近5日累計淨買超12,728張(買3日/賣2日)；⚠️惟規模較8/26的5,204張縮小13.5%。投信連續第2日賣超317張(-317,464股)、自營商買超158張(+157,501股)，三大法人分項四捨五入後加總+4,342張、TWSE官方合計欄換算+4,341張(差1張屬正常捨入誤差)。⚠️⚠️但期貨端與現貨端本日再度背離、且方向轉壞：TAIFEX官方顯示外資台指期未平倉淨空單自8/26的83,654口不減反增至84,836口(多6,963/空91,799、新增空單1,182口，而非前報期待的回補)，投信淨多單自78,043口降至76,834口(-1,209口)，自營商自淨空單421口轉為淨多單376口——外資在現貨端連2日買超9,705張的同時於指數期貨加空，屬避險或看空大盤而非全面做多，這削弱了現貨買超的訊號強度。(5)⭐量能通過檢核但量價關係轉為負面，兩者必須分開陳述以免誤導：前報訂出「須見今日量能維持5日均量之上」的檢核，8/27成交19,214張，站穩5日均量16,843張之上達14.1%，連續第2日高於均量，並未出現前報所警示的「一日放量後迅速萎縮」——檢核通過。⚠️但同樣的量能在不同價格結構下意義相反：8/26的19,467張是放量上漲(買方主導)，8/27的19,214張是接近同等量能的開高走低並收最低(賣方主導)，本日的大量代表高檔調節的承接量而非追價買盤。⚠️成交筆數自67,273筆降至60,122筆(-10.6%)，每筆平均張數自0.289張升至0.320張——散單退場、大單相對增加，與外資買超的方向一致，顯示賣壓來源並非外資。(6)⚠️技術指標本日首度出現分歧，不再是前2日的「全面翻正」(TWSE官方序列2026-01-02~08-27共157筆計算)：⚠️動能類轉弱——RSI(14) 53.73→53.14(-0.59)、RSI(6) 58.97→56.87(-2.10)，連2日上升的趨勢中斷，RSI(6)回落幅度為RSI(14)的3.6倍，兩者差距自5.24點收斂至3.73點，前2日「短強長弱且持續擴大」的動能結構首度反轉為收斂，屬動能衰竭的早期訊號；惟RSI(14) 53.14仍站穩50中軸之上、距超買(70)尚有16.86點。⭐趨勢類仍在改善——MACD柱狀圖+5.57→+6.14(連3日擴張、為8/13以來最高)，DIF +7.59→+8.64(+1.05)、DEA +4.81→+5.57(+0.70)，正乖離自2.78擴大至3.07，死亡交叉進一步推遠，續為零軸上方多頭排列；⚠️惟擴張力道明顯衰竭——柱狀圖單日擴張幅度自8/26的+2.52大幅放緩至+0.57(-77.4%)、DIF升幅自+1.96減半至+1.05，趨勢仍向上但推進力量正快速流失，與RSI(6)率先回落是同一件事在不同指標上的呈現。⚠️⚠️KDJ進入前報已預警的過熱區、且以出乎意料的方式實現：K 58.50→64.00、D 52.52→56.35、J 70.45→79.30(+8.85)，J值距超買線(80)僅剩0.70點——⭐誠實對照，前報寫明「J值70.45距離超買區(80)僅9.55點……若今日跳空大漲，J值極可能直接進入超買區」；⚠️本日股價收黑-0.21%，J值卻仍大幅上升，原因是KDJ以「收盤價在近9日高低區間中的相對位置」計算，8/27區間高低點同步上移，即使收黑收盤價在區間中的位置仍較前日為高。⚠️⚠️指標過熱與價格收黑並存，是四項指標中唯一同時發出「位階偏高」與「價格未跟上」雙重訊號者，屬典型的量價/指標背離前兆；K-D乖離自+5.98擴大至+7.65，金叉結構本身仍完好。均線5MA 2,402/10MA 2,391/20MA 2,390/60MA 2,384/120MA 2,226，現價續站全部五條均線、5MA自2,395升至2,402續高於10MA；⚠️惟10MA 2,391與20MA 2,390已收斂至僅差1點，形成雙均線重合帶，該帶被跌破即屬實質破位，為本報現階段最關鍵的防線。⚠️布林通道的「劇烈收斂」本日必須加註成因，否則會被嚴重誤讀(本報主動更正判讀口徑)：帳面上通道寬度自191.5點壓縮至107.1點(-44.1%)，上軌2,443.1/中軌2,389.5/下軌2,335.9，看似波動度急速下降；⚠️但實際成因是7/30的極端低價2,205於本日滾出20日窗口，20日標準差自47.89降至26.78，屬窗口更替的機械性效果，並非8/27當日出現任何波動度壓縮；同一成因也解釋了20MA/布林中軌一次上移10.3點(2,379.2→2,389.5)。⚠️因此前一份日報所稱「布林收斂通常出現在方向選擇之前」的推論在本日不應延用，本報不以此作任何方向性判斷。可用的事實僅是位置關係：現價2,410位於中軌之上20.5點、距上軌33.1點，仍在通道上半部。(7)⭐衍生品：台積電個股期CDF 202609日盤收2,419(-5、-0.21%、開2,432/高2,439/低2,417、量4,118口、結算價2,419、未平倉25,832口)，對現貨2,410維持正價差+9(與8/26相同)，期貨續小幅領先現貨；⚠️惟未平倉自25,923減至25,832口(-91口)、連續第3日減少，且在NVIDIA利多日仍未回升——前報所指「尚未見新資金建立方向性多單」的瑕疵不僅未解除，反而在最有利的環境下獲得反證。⭐選擇權口徑：8/26(週三)為結算日、未平倉已重置為新基期，8/27(週四)是本週唯一在同一結算週期內且前後皆有可比基期的交易日，故本日跨日比較具參考價值。未平倉自結算後低基期大幅回補——賣權40,154→61,636口(+53.5%)、買權38,971→58,254口(+49.5%)，雙邊合計79,125→119,890口(+51.5%)，屬結算後的正常重建。P/C未平倉比自103.04%微升至105.81%(+2.77pp、賣權多出買權3,382口)：⭐判讀應保守——105.81%僅略高於100%的多空分界，屬中性略偏保守，2.77pp的變動在結算後重建期的雜訊範圍內，本報不解讀為明確看空訊號。成交量P/C比121.76%(賣權158,174/買權129,911口、總成交288,085口)，較8/26結算日的112.20%升高，但總成交量自706,505口大幅縮減59.2%屬結算日效應消退的正常回落，兩日的成交量P/C不宜直接比較。⚠️⚠️下一個讀數的重要限制：8/28(今日)為週五、又是本週第2個結算日，未平倉將再度結清重置，故8/27→8/28的跨日比較同樣不成立——本週實際上不存在連續兩日皆可比的P/C序列，本報明確標示此限制而非勉強解讀。⚠️夜盤時序聲明(依TAIFEX標記慣例，夜盤日期為該時段結束日)：8/27 15:00→8/28 05:00夜盤CDF 202609收2,442(+23、+0.95%、開2,429/高2,442/低2,423、量1,480口)，反映美股8/27正規盤TSM +2.30%、費半+2.33%的漲勢，為8/28台股開盤的偏多線索；⚠️惟該時段於台北05:00結束，不含美股盤後TSM回落-0.39%的部分，故夜盤讀數略高估了美股的最終情緒。(8)⭐外部環境，NVIDIA財報後美股全面追價、費半正式脫離技術性熊市：NVDA 8/27正規盤大漲+8.74%收$227.98(+$18.32)為本日追蹤清單漲幅最大者，自8/17的$224.09累計由-6.44%一舉轉為+1.74%；財報要點——營收$96.22B(+106% YoY)勝共識約$92.2B與公司財測中值$91.0B、資料中心$89.0B(+117% YoY、占比約93%)、調整後EPS $2.22(+128% YoY)勝共識$2.10、為連續第13季超越自身財測，Q3財測$108B(±2%)高於共識約$104.2B達約$3.8B且不含中國資料中心銷售。⭐⭐關鍵里程碑：費半SOX +2.33%收11,882.17(+270.93點)，距52週收盤高14,634.72(2026-06-22、盤中高14,655.29)已收斂至-18.81%，依-20%通行定義正式脫離技術性熊市——前一份日報明訂此為NVIDIA財報的關鍵檢核，本報以1年日線序列獨立複核確認通過(8/26為-20.8%)。美股大盤：S&amp;P 500 +0.72%收7,730.99、那斯達克+1.57%收26,541.35、道瓊+0.20%收53,569.44。⚠️惟族群參與度不全面——收紅：AMKR +6.90%收$51.74(⭐漲幅第二大、自8/17累計跌幅自-21.04%大幅收斂至-15.60%、終於脫離清單跌幅最重的位置)、AVGO +4.49%收$371.54(⭐終結連3日下跌、累計自-9.39%收斂至-5.32%、市場認定AI總需求變大而非ASIC與GPU零和)、INTC +4.36%收$92.09(⭐連3日收紅並首度站上$90、累計自-14.73%收斂至-11.02%)、000660 SK海力士+2.49%收173.0萬韓元(⭐HBM直接受惠、連3日回升創本波新高)、2344華邦電+2.48%收186.0(TWSE官方、⭐連3日收紅創本波新高、自8/17累計轉為+2.48%)、3711日月光+2.20%收605.0(TWSE官方、⭐先進封裝受惠、領先2330達2.41pp)、LRCX +1.82%收$318.58、005930三星電子+1.72%收266,000韓元、ARM +1.65%收$255.21、QCOM +0.65%收$164.78、AMAT +0.54%收$482.36(⭐終結連3日下跌)、AAPL +0.36%收$314.58(⭐創本波新高、累計+2.94%續為客戶族群最強)。⚠️收黑：AMD -0.89%收$476.67(⚠️為客戶族群唯一下跌者、市場解讀為GPU直接競爭者的相對劣勢被強化)、ASML -0.61%收$1,735.01(⚠️與族群明顯背離、AI資本支出對設備商的傳導有數季時間差)、MU -0.32%收$935.39(⚠️HBM題材直接受惠卻收黑、與SK海力士+2.49%強烈對比)、KLAC -0.03%收$183.77、2454聯發科-2.03%收3,865(見第3點)。(9)⚠️評價位階小幅收縮：8/27 TWSE官方BWIBBU顯示P/E 27.94x(8/26為27.99x)、P/B 9.72x(9.74x)、殖利率0.91%(持平)、市值約NT$62.5兆，⭐本報已確認財報年/季欄位仍為115/2、未再換季，故8/14起各日可比。本日變化純由股價-0.21%帶動、分母未動。⚠️P/E在28x整數關卡前止步，仍位於5年區間第87百分位、10年第88百分位，P/B第91百分位——評價偏貴的結構未變；PEG 0.82為唯一顯示成長性可支撐評價的指標。⭐⭐本日新增一項值得記錄的觀察：NVIDIA財報大幅超預期已於8/27兌現，但2330股價反以-0.21%回應且開高走低——這正是高評價股票的典型風險特徵：當估值已位於5年第87百分位，即使利多實現，市場也可能認為已被價格反映而不再追價，本報認為這是理解8/27相對弱勢的關鍵評價面線索。⚠️截至本報產製時點，尚未觀察到分析師實際調升台積電EPS共識的動作，fy_consensus 84.50與q1_consensus 20.38仍為NVIDIA財報前數值，本報不預先自行上修。⚠️匯率連續第2個交易日升值且幅度放大：新台幣8/27收31.70(Yahoo TWD=X逐時序列16:00台北時點、實際讀數31.697)，自8/26的31.79升值約0.28%，升幅為前一日(0.16%)的1.8倍；相對8/13的32.12累計升值幅度自1.03%擴大至1.31%，依官方口徑(每升值1%約-40bps)估算毛利率逆風自約-41bps擴大至約-52bps。日內細節：8/27自31.86(00:00)一路走升，09:00台股開盤時已達31.74，15:00觸及當日最強31.69，16:00收31.70；8/28今晨續升(05:00為31.67、09:00台北為31.62)，升值趨勢延續至第3日。⚠️須誠實標註此逆風與本日股價的關聯有限：8/27的-0.21%主要由開高走低的調節賣壓造成，匯率是慢變量、影響落在未來季度的毛利率而非當日股價。⚠️台幣仍處2026年偏強區間，Q3毛利率指引65-67%已含匯率假設，須快速升破31.0才需重新評估。(10)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方API取數，ADR收盤與盤後另經stockanalysis.com交叉確認(含讀數時點)，台股供應鏈個股(2344/3711/2454)另以TWSE STOCK_DAY官方序列複核與Yahoo一致。⚠️匯率採Yahoo TWD=X逐時序列8/27 16:00台北收盤時點讀數31.70(日線序列缺漏該筆)，與前一日同法取得的8/26 31.79口徑一致、可直接比較，正式值請以央行／台北外匯經紀公司公告為準。技術指標依TWSE官方序列2026-01-02~08-27共157筆重算，並回算驗證8/26各值(RSI(14) 53.73、RSI(6) 58.97、DIF+7.59/DEA+4.81/柱+5.57、K58.50/D52.52/J70.45、MA5 2,395/MA10 2,393.5/MA20 2,379.2/MA60 2,383.25/MA120 2,221.54、布林2,475.0/2,379.2/2,283.5、5日均量16,394張)與8/27已發布日報所載數值逐項完全一致，確認序列連續、無口徑漂移。⚠️本報主動修正一項既有缺陷：HTML日報技術分析區塊的「成交量」與「布林帶」卡片標籤原硬編為「量縮整理」與「布林收窄整理」，在放量日或價格位置改變時會標錯(本日成交量19,214張高於5日均量16,843張達14.1%，原標籤「量縮整理」與事實相反)，已改為依實際數值動態計算(VOL_LABEL/BB_LABEL)，作法與先前的BASIS_LABEL、F5D_LABEL一致。⭐綜合研判：由「偏多」下調至「中性」——本報前一份日報所訂的兩項警訊條件(開高走低、利多下仍落後大盤)雙雙成立。⚠️三項實質轉壞：(1)收盤2,410＝當日最低的光頭光腳黑K，越過檢核價2,425後跌回其下，2,435反壓確認有效；(2)相對強弱連2日落後，且近5日的中期領先本日正式翻負(+1.47% vs大盤+2.32%)；(3)外資現貨買超4,501張的同時，台指期淨空單反增1,182口至84,836口，兩端背離。⭐三項未壞：量能連2日守住均量、五條均線全數未破、MACD連3日擴張。⭐下調評級的理由是價格對利多的反應失敗與相對弱勢的確認，而非基本面變化——NVIDIA財報對台積電下半年能見度的正面意義並未改變，改變的是市場願意為此付出的價格。今日(8/28)判定標準：⭐第一順位是2,410這道新防線能否守住(本報已將檢核價位自2,425下移至8/27收盤兼當日最低的2,410)——守住2,410並收復2,425則開高走低可視為單日事件；跌破2,410並失守5MA 2,402，則8/25-8/26的修復再度失效，下一道防線是10MA 2,391與20MA 2,390的雙均線重合帶(相距僅1點)，跌破即屬實質破位。⚠️今晨夜盤CDF +0.95%指向開高，但8/27本身已證明「夜盤與ADR偏多≠台股會漲」，不可據此預設開高必守。第二順位為結構性輪動是否延續(若在夜盤偏多線索下仍無法領先大盤，輪動將由「確認」升級為「持續」)，對照組為8/27領先的華邦電+2.48%、日月光+2.20%等中小型與封測標的。第三順位為籌碼兩端背離能否收斂(須見台指期空單實質回補或CDF未平倉回升)。第四順位為KDJ過熱的兩種情境(J值79.30距超買線僅0.70點：開高則直接進入超買區、改列短線過熱警訊；收黑則形成明確高檔背離)。⚠️⚠️今日為本週第2個台指選擇權結算日，衍生品跨日可比性再度受干擾。上方壓力2,425/2,435/2,443/2,470/2,510/2,535，下檔支撐2,410/2,402/2,391/2,390/2,384/2,375/2,336/2,226。</t>
+        </is>
+      </c>
+      <c r="G115" s="50" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-08-31 日報 HTML & Excel 更新
涵蓋 8/28 (Fri) 收盤：台股 2330 收 NT$2,420 (+0.41%)、量 15,026 張；
ADR TSM $417.52 (-2.29%)；外資連 3 日買超 3,032 張、投信賣超 1,765 張。

重點：台股 13:30 收盤後美股才重挫（費半 -3.47%、NVDA -4.57%），
存在尚未收斂的時間差；ADR 溢價自 +12.41% 壓縮至 +8.97%，
期貨夜盤 CDF 2,408 (-0.86%) 已先行反映。KDJ J 值 84.52 進入超買。

另修正模板硬編缺陷：Put/Call Ratio 卡片標籤原寫死「偏空(>1=空力較強)」，
會將 1.01 這種均衡讀數誤標、且比值 <1 時完全標錯，改為分段動態計算
(PCR_LABEL)；「最大痛苦點」補上「(本報估算)」標記。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-08-28</t>
+          <t>報告更新日期：2026-08-31</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3339,7 +3339,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-08-28</t>
+          <t>最後更新：2026-08-31</t>
         </is>
       </c>
     </row>
@@ -7416,6 +7416,55 @@
         </is>
       </c>
       <c r="G115" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="53" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B116" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,420（8/28收）</t>
+        </is>
+      </c>
+      <c r="C116" s="54" t="inlineStr">
+        <is>
+          <t>+0.41%（8/28收）</t>
+        </is>
+      </c>
+      <c r="D116" s="53" t="inlineStr">
+        <is>
+          <t>US$417.52（8/28收）</t>
+        </is>
+      </c>
+      <c r="E116" s="53" t="inlineStr">
+        <is>
+          <t>15,026（8/28收）</t>
+        </is>
+      </c>
+      <c r="F116" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-08-31(Mon)，涵蓋8/28(Fri)收盤。⭐台股層面是「防線守住、部分通過」的一日：2330官方收NT$2,420(+10、+0.41%、開2,440/高2,445/低2,410、量15,026張、額364.65億、52,492筆)，全日最低2,410與前報所訂檢核價分毫不差並獲買盤承接後反彈作收；⚠️惟前報完整條件為「守住2,410並收復2,425」，收盤2,420差5點未達成，本報判定為部分通過而不誇大為突破。⚠️⚠️但本報認為真正決定後續的不是這根紅K，而是台股收盤之後發生的事——台美之間存在一個尚未收斂的時間差，這是閱讀本報時必須優先理解的一點：台股8/28於台北時間13:30收盤後，美股8/28正規盤才開出全面重挫，費半-3.47%收11,469.66、TSM ADR -2.29%收$417.52、NVDA -4.57%收$217.55、那斯達克-0.52%收26,402.42、S&amp;P 500 -0.25%收7,711.76、道瓊-0.02%收53,559.99。因此本報所列台股價量、法人、技術指標全數為「美股重挫之前」的狀態，不可據以推論8/31台股反應。評級維持「中性」——不因台股收紅而上調，亦不因美股夜跌而預先下調。
+(1)⭐價格與型態，前報第一號檢核條件以最精確的方式通過：8/28盤中最低2,410與檢核價完全相同，該價位遭測試後獲承接反彈10點收2,420。⭐型態較8/27明確改善：8/27是「收盤＝當日最低」的光頭光腳黑K，8/28雖同樣開高走低，但觸低後收在中段偏上並收紅，連續「收在最低」的惡化型態未重演。⚠️惟連續第2個交易日「開高不守」：8/27開2,430/高2,435，8/28開2,440/高2,445，兩日開盤與盤中高均創8/13以來新高卻均未守住，2,425-2,445確認為實質賣壓區；2,425已連續3個交易日未能收盤站上(8/26高2,425、8/27高2,435、8/28高2,445均曾越過，收盤分別為2,415/2,410/2,420)，該價的反壓性質已由「檢核價」升級為「確認有效的壓力」。⚠️另據8/28為富台期與摩台期結算日，午盤後漲勢受結算調節壓抑(來源：聯合新聞網)。
+(2)⚠️⚠️美股8/28下跌的成因須與8/27的上漲成因分開理解，否則會誤判為單純獲利了結：直接催化劑是聯準會主席Kevin Warsh對通膨趨勢表達疑慮(明言夏季PCE與CPI雖優於預期，但不代表底層趨勢已實質改善)，屬總體利率面衝擊而非半導體基本面轉壞；疊加的產業面事件是Marvell財報優於預期並上調財測，股價卻仍重挫-10.3%——「好消息不漲」的型態自台股8/27延伸至美股8/28，是本週最值得追蹤的市場性格變化。⚠️⚠️費半8/28重挫-3.47%(-412.51點)，完全抹去8/27的+2.33%而有餘，距52週收盤高14,634.72(2026-06-22)的跌幅自-18.81%重新擴大至-21.63%——8/27才剛達成的「脫離-20%技術性熊市」判定，僅維持一個交易日即告失效，本報以1年日線序列獨立複核確認此一狀態變化。⭐平衡標註：TSM ADR的-2.29%明顯抗跌於費半-3.47%、NVDA-4.57%、LRCX-5.24%、KLAC-4.48%、AMAT-4.29%。
+(3)⚠️⚠️ADR溢價出現本波最大單日壓縮，這是8/31補跌壓力的量化來源：溢價自+12.41%急降至+8.97%(-3.44pp)，成因為三項因素同向作用——ADR下跌-2.29%、台股上漲+0.41%、台幣升值使平價由$380.13升至$383.15。⭐判讀：溢價壓縮代表海外投資人對TSMC的定價已先行下修，而台股定價尚未跟上。ADR收盤三重自我檢核：427.30-9.78=417.52✓、427.30×(1-2.29%)=417.52✓、stockanalysis.com獨立確認$417.52/-$9.78/-2.29%/讀數時點Aug 28 2026 4:00 PM EDT✓。
+(4)⭐籌碼面延續偏多但內部出現分歧：外資及陸資8/28買超3,032張(T86官方買賣超+3,032,289股)，為連續第3個交易日買超、3日合計12,737張、近5日累計淨買超9,965張(買3日/賣2日)；⚠️惟單日規模較8/27的4,501張再縮小32.6%，呈現遞減態勢(5,204→4,501→3,032)。⚠️⚠️投信本日是明確的空方：賣超1,765張為近5個交易日最大單日賣超且連續第3日賣超；自營商小幅賣超23張、終結連4日買超。三大法人分項四捨五入後加總+1,244張、TWSE官方合計欄換算+1,243張(差1張屬正常捨入誤差)。
+(5)⚠️量能檢核本日未通過且與價格方向背離：8/28成交15,026張較8/27的19,214張萎縮21.8%，並跌破5日均量16,064張達6.5%，終結連2日站穩均量之上的紀錄。⚠️股價收紅之日出現量能萎縮屬「價漲量縮」，代表2,420一帶追價買盤不足，與8/26放量上漲(19,467張)的健康型態相反。⭐兩項緩和事實須並列：8/28為結算日、量能本就易受期現貨調節干擾；成交筆數自60,122降至52,492筆(-12.7%)、每筆平均張數自0.320降至0.286張，屬大單參與度下降而非散戶追高出貨。⚠️5日均量自16,843張降至16,064張(-4.6%)，成因為8/21的18,922張滾出窗口而8/28的15,026張滾入，屬窗口更替的機械效果與當日量縮的疊加。
+(6)⚠️技術指標本日轉為「趨勢改善但動能過熱」的組合(TWSE官方序列2026-01-02~08-28共158筆計算)：⭐趨勢類全面改善——MACD柱狀圖+6.14→+7.34(連續第4日擴張、為8/13以來最高)，DIF+8.64→+10.16並站上10一線、DEA+5.57→+6.49，正乖離自3.07擴大至3.67。⭐動能類回升——RSI(14) 53.14→54.23、RSI(6) 56.87→60.27(+3.40、回升幅度為RSI(14)的3.1倍)，距超買區(70)尚有15.77點緩衝。⚠️⚠️但KDJ本日正式進入超買，這是前兩份日報連續預警的情境終於實現：K 64.00→68.42、D 56.35→60.37、J值79.30→84.52首度突破80超買門檻——⭐誠實對照，8/28日報寫明「J值79.30距離超買區僅0.70點……幾乎任何上漲都會使其進入超買」，預警完全兌現。⚠️關鍵判讀在於超買發生的時機極為不利：J值進入超買代表短線動能已被充分使用、向上緩衝空間耗盡，而此時美股當夜已重挫、期貨夜盤已指向-0.86%；歷史經驗上J值於超買區遭遇外部利空時回檔幅度容易被放大。⭐平衡標註：J值超買本身不是賣出訊號而是「風險報酬比轉差」的訊號，須待其自超買區回落並形成高檔背離才構成實質轉空。均線5MA 2,404/10MA 2,394/20MA 2,389/60MA 2,384/120MA 2,230，收盤2,420高於全部五條均線且多頭排列完整，10MA與20MA相距僅5點形成密集支撐帶。⭐布林通道本日回歸穩定：上軌2,442/中軌2,389/下軌2,336，寬度106.3點較8/27的107.1點幾無變化——⭐本報特別標註：8/27曾因7/30極端低價2,205滾出20日窗口而出現-44%的機械性收斂假象，本日窗口內無極端值進出，106點為通道寬度的真實水準，前一日的收斂不應延續解讀。⭐口徑驗證(每日必做、本日已執行並通過)：以同一序列回算8/27各指標得RSI(14) 53.14、RSI(6) 56.87、DIF+8.64/DEA+5.57/柱+6.14、K64.00/D56.35/J79.30、MA5 2,402/MA10 2,391/MA20 2,390/MA60 2,384/MA120 2,226、布林2,443/2,390/2,336、5日均量16,843張，與8/28已發布日報所載數值逐項完全相同，確認序列連續、無口徑漂移。
+(7)⭐衍生品：台積電個股期CDF 202609日盤收2,429(+10、+0.41%、開2,440/高2,448/低2,421、量3,833口、結算價2,429、未平倉25,619口)，對現貨2,420維持正價差+9(與8/27完全相同)，日盤期貨未透露額外方向訊息。⚠️⚠️選擇權未平倉本日不可跨日比較，口徑須先行聲明：8/28(週五)為結算日且同日另有富台期與摩台期結算，台指選未平倉已全面重置——賣權61,636→42,600口(-30.9%)、買權58,254→41,994口(-27.9%)，雙邊合計119,890→84,594口(-29.4%)。因此P/C未平倉比自1.06降至1.01不代表籌碼結構轉變，而是結算後新基期的起始讀數。⭐本報既有口徑(2026-08-24已確立)：台指選週三與週五均為結算日，故P/C未平倉比僅在週一、週二、週四具備跨日可比性。⭐若單就8/28絕對水準判讀：1.01屬「多空未平倉均衡」的中性區間(賣權僅較買權多606口、多出不到1.5%)，並無極端訊號。⭐⭐最具前瞻價值的一項為期貨夜盤(依TAIFEX標記慣例，夜盤日期為該時段結束日)：CDF 202609於8/28夜盤(標記日期2026/08/31)收2,408(-21、-0.86%、開2,432/高2,435/低2,404、量1,363口)，台指期TX夜盤收45,900(-457、-0.99%、量35,867口)——夜盤已先行反映美股8/28費半-3.47%的重挫，且CDF夜盤低點2,404恰與5MA 2,404重合，此為8/31台股開盤的關鍵參考。
+(8)⚠️供應鏈8/28全面回落但台股因時間差仍收紅，兩者的背離即為補跌壓力所在：⚠️美股收黑——AMKR -7.46%收$47.88(本日追蹤清單跌幅最大、回吐8/27的+6.90%而有餘、自8/17累計跌幅重新擴大至-21.89%)、ARM -6.33%收$239.05(跌幅第二大、屬高評價IP授權股對利率敏感)、LRCX -5.24%收$301.90、KLAC -4.48%收$175.54(設備四雄累計跌幅最深-14.68%)、NVDA -4.57%收$217.55(回吐8/27財報漲幅過半、惟仍高於財報前的$209.66達3.76%)、AMAT -4.29%收$461.67(本週累計跌逾5%、與Marvell同為拖累SMH的兩大來源)、000660 SK海力士-4.45%收165.3萬韓元、005930三星電子-3.38%收257,000韓元、INTC -2.85%收$89.47、AMD -2.33%收$465.58、ASML -2.24%收$1,696.16、AVGO -0.74%收$368.79、QCOM -0.36%收$164.19、MU -0.27%收$932.86。⭐美股逆勢收紅者僅AAPL +1.63%收$319.70(追蹤清單唯一收紅的美股、創本波新高)——⭐判讀：資金正自AI基礎建設向終端消費電子與AI曝險較低的標的輪動(AAPL、QCOM、MU三者相對費半的強度分別達5.10pp、3.11pp、3.20pp)，此對TSMC屬中性偏正面，蘋果為N3主力客戶。⭐台股供應鏈因時間差仍收紅：2454聯發科+3.10%收3,985(TWSE官方、本日台股清單漲幅最大、完全收復8/27的-2.03%)、3711日月光+2.64%收621.0(TWSE官方、連2日收紅創本波新高、領先2330達2.23pp)；⚠️2344華邦電-2.42%收181.5(TWSE官方、開188.5/高192.0創本波新高後一路走低收近當日最低、量放大至15.3萬張，高檔放量收黑為本日台股供應鏈最弱)。⚠️⚠️AMKR -7.46%與日月光+2.64%的完全相反走勢，是8/31台股封裝族群補跌壓力的具體來源。
+(9)⚠️相對強弱連續第3個交易日落後大盤：加權指數8/28收46,331.45(+356.23、+0.77%)重新站回46,000關卡，2330 +0.41%落後0.36pp；⭐誠實標註：落後幅度已連2日收斂(0.84→0.52→0.36pp)，惡化程度正在減輕。⚠️⚠️「近1個月」欄位本日出現大幅跳升(2330自+2.55%升至+6.14%、加權自+5.37%升至+11.36%)，本報必須明確標註成因以免誤讀為動能轉強：此為滾動窗口的機械效果——1個月基準日自7/27移至7/28，而7/28-7/30正是本波最劇烈的下跌段(2330自2,350跌至2,200、加權自43,634跌至39,933)，低基期滾入使百分比大幅放大，並非8/28當日出現任何實質動能變化。YTD 2330 +52.7% vs加權+57.9% vs費半+55.7%(基準採2026-01-02收盤：2330 NT$1,585、加權29,349.81、SOX 7,367.47)。⚠️資料誠實標註：beta_60d 1.38為既有數值沿用，本報以TWSE官方序列對60日日報酬回歸未能複現該值(自行計算得約0.97)，因無法確認其原始口徑，故不予變更亦不宣稱已重算。
+(10)⚠️評價位階續升：8/28 TWSE官方BWIBBU顯示P/E 28.05x(8/27為27.94x)、P/B 9.76x(9.72x)、殖利率0.91%(持平)、市值約NT$62.8兆，⭐本報已確認財報年/季欄位仍為115/2、與8/27同基準，故本日升幅純由股價上漲+0.41%所致、分母未變動，兩日數值可直接比較。⚠️P/E 28.05x位於5年第87百分位、10年第88百分位，P/B第91百分位——三項均處歷史高檔，對負面消息的容錯空間有限；PEG 0.82仍低於1，為唯一顯示成長性可支撐評價的指標。⚠️⚠️匯率連續第3個交易日升值且單日幅度最大：新台幣8/28收31.58(Yahoo TWD=X逐時序列16:00台北時點、實際讀數31.576)，自8/27的31.70升值約0.38%(前一日為0.28%)；相對8/13的32.12累計升值幅度自1.31%擴大至1.68%，依官方口徑(每升值1%約-40bps)估算毛利率逆風自約-52bps擴大至約-67bps——已相當於Q3毛利率指引區間(65-67%)約三分之一的寬度。⭐緩和因素為公司約75%的外幣避險比例可遞延並平滑部分衝擊。⚠️本日匯率變化與美股重挫方向一致且互相強化：台幣升值削弱以新台幣計價的獲利，ADR下跌反映海外定價下修。
+(11)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方API取數，ADR收盤另經stockanalysis.com交叉確認(含讀數時點)，台股供應鏈個股(2344/3711/2454)另以TWSE STOCK_DAY官方序列複核。⚠️⚠️本報須主動聲明一項取數缺口與其處理方式：Yahoo日線序列本日對全部美股標的的8/28收盤欄位均為null(缺漏)，本報改採同一回應中meta.regularMarketPrice並逐一驗證其時間戳為2026-08-28 20:00 UTC(＝16:00 EDT正規盤收盤)後方予採用，非以盤中或盤後價冒充收盤；南韓標的(000660/005930)的meta時間戳為8/31盤中，故改採8/28官方日線收盤，以維持全報同一交易日口徑。⚠️匯率採Yahoo TWD=X逐時序列8/28 16:00台北時點讀數31.58，與前一日同法取得的8/27 31.70口徑一致、可直接比較(該法已以replay前一日已發布值31.697→31.70驗證)，正式值請以央行／台北外匯經紀公司公告為準。⚠️本報主動修正一項既有缺陷：HTML日報期貨選擇權區塊的「Put/Call Ratio」卡片標籤原硬編為「偏空(&gt;1=空力較強)」與固定紅色，會將1.01這種實質均衡的讀數誤標為偏空、且在比值小於1時會完全標錯，已改為依比值分段動態計算(PCR_LABEL)，作法與先前的BASIS_LABEL、F5D_LABEL、VOL_LABEL、BB_LABEL一致；同時為「最大痛苦點」卡片補上「(本報估算)」標記，使其與內文的估算聲明一致。
+⭐綜合研判：維持「中性」。⭐三項未壞：五條均線(2,404/2,394/2,389/2,384/2,230)全數未破且多頭排列完整、外資連3日買超共12,737張、期貨維持正價差+9。⚠️三項未解：連3日落後大盤(惟落後幅度連2日收斂)、KDJ J值84.52進入超買而缺乏緩衝、量能跌破5日均量且價漲量縮。今日(8/31)判定標準：⚠️⚠️第一順位是「台股補跌幅度是否收斂於夜盤所反映的-0.9%之內」——本報將檢核價位設在5MA 2,404(恰與夜盤期貨低點2,404重合)與連2日守住的2,410：⭐若開低後能守住2,404-2,410區間並收紅或平盤，代表台股具備獨立於美股的承接力，時間差風險解除，ADR溢價的3.44pp壓縮將由ADR回升而非台股補跌來收斂；⚠️⚠️若跌破2,404並失守10MA 2,394與20MA 2,389的密集帶(相距僅5點)，則8/25-8/28的整段修復失效，下一道防線為60MA 2,384。⚠️第二順位為KDJ超買的放大效應(須追蹤J值是否自超買區回落並形成高檔背離)。⚠️第三順位為量價確認(若今日下跌且放量，屬賣壓實質釋放，性質較8/28的結算日量縮更為負面)。⭐第四順位為P/C未平倉比的可比讀數(8/31為週一、屬同一結算週期內，可與8/28的1.01直接比較，為本週首個具跨日可比性的讀數)。上方壓力2,425/2,435/2,442/2,445/2,470/2,510/2,535，下檔支撐2,410/2,404/2,394/2,389/2,384/2,375/2,336/2,230。</t>
+        </is>
+      </c>
+      <c r="G116" s="53" t="inlineStr">
         <is>
           <t>Yahoo Finance / Bloomberg</t>
         </is>

</xml_diff>

<commit_message>
daily: 2026-09-04 日報 HTML & Excel 更新
涵蓋 9/2、9/3 兩個交易日（9/3 日報未產製，內容併入本報）。

台股 2330（9/3 收）：NT$2,390（+5、+0.21%），量 14,252 張（2026 年第 4 低）
NYSE TSM（9/3 收）：US$417.01（+0.36%），ADR 溢價擴大至 10.66%

重點：9/1 收 2,440 的突破於 9/2 被證實為單日假突破（收 2,385、-2.25%、收在全日
最低），9/2 一度失守 60 日季線；9/3 無量小反彈站回季線但僅高出 2 點。技術面
MACD 柱狀體翻負 -0.35（8/04 以來首次）、KDJ 9/2 死叉；外資 9/2 單日賣超 11,987 張。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-02</t>
+          <t>報告更新日期：2026-09-04</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-02</t>
+          <t>最後更新：2026-09-04</t>
         </is>
       </c>
     </row>
@@ -7586,6 +7586,58 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B119" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,390（9/3收）</t>
+        </is>
+      </c>
+      <c r="C119" s="51" t="inlineStr">
+        <is>
+          <t>+0.21%（9/3收）</t>
+        </is>
+      </c>
+      <c r="D119" s="50" t="inlineStr">
+        <is>
+          <t>US$417.01（9/3收）</t>
+        </is>
+      </c>
+      <c r="E119" s="50" t="inlineStr">
+        <is>
+          <t>14,252（9/3收）</t>
+        </is>
+      </c>
+      <c r="F119" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-04(Fri)，涵蓋9/2(Wed)與9/3(Thu)兩個交易日收盤。⚠️⚠️本報最重要的結構聲明放在最前面：2026-09-03(Thu)之日報未產製，故本報一次涵蓋兩個交易日，凡標「兩日」者均指9/2至9/3此區間。
+(1)⚠️⚠️價格與型態，前報第一號檢核的結果為「明確未過關，且失敗得比預期徹底」：前報訂「突破後的第一次測試：開低幾成定局，2,425能否守住」。9/2開盤2,415即已低於2,425(檢核在開盤那一刻就已失敗)，全日未再觸及，終場收在全日最低2,385(-55、-2.25%)，並跌破8/31起漲點2,405。依型態定義，9/1的2,440應定性為「單日假突破(false breakout)」而非「突破後回測」——回測須守住突破頸線，本例連起漲點都一併跌破。9/3收2,390(+5、+0.21%)，開2,385/高2,400/低2,380，全日振幅僅20點。兩日自9/1的2,440淨跌-50點(-2.05%)。
+(2)⚠️均線：9/2收盤2,385一度失守60日季線(當日MA60為2,387)，為8/24以來首次(8/24收2,375&lt;當日MA60 2,381.50)；9/3收2,390重新站回季線(2,388)但僅高出2點，防線脆弱。現價仍位於MA5(2,408)、MA10(2,405)、MA20(2,397)三線之下，均線結構自9/1的「全面多頭」在兩日內退回「短中期轉空、僅長期支撐尚存」。MA5與MA10已靠攏至僅差3點。
+(3)⚠️量能兩段須分開解讀：9/2的25,151張搭配-2.25%長黑，是「有量下跌」、屬真實賣壓宣洩；9/3的14,252張(額340.61億)搭配+0.21%小紅，是「無量止跌」，為2026年第4低量(前三低為8/24的13,073、8/17的13,482、8/25的13,538張)，較9/2再縮43.3%、較9/1的31,855張縮55.3%。⚠️本報不將9/3的小紅認定為底部訊號：無量止跌可以是打底第一步，也可能只是下跌中繼的休息。
+(4)⚠️籌碼是本區間最明確的利空證據：外資9/2單日賣超11,987張(T86官方-11,986,983股)，為本報追蹤區間內的極端值，與9/1買超5,731張完全反手；投信賣837張、自營買72張。9/3賣壓大幅收斂：外資賣961張(-960,755股)、投信買51張(+51,332股)、自營賣89張(-88,899股)，三大法人合計約-999張(官方合計欄-998,322股)。⚠️賣壓減弱但無任何一方轉為積極買進。
+(5)⚠️⚠️技術指標四項全數轉弱且出現兩個死叉：MACD柱狀體自+8.68→+2.93→-0.35翻負，DIF 8.43下穿DEA 8.61完成死叉，為8/04(-12.36)以來首次翻負、相隔21個交易日；KDJ已於9/2完成死叉(K 63.03&lt;D 65.72)，9/3擴大至K 56.06&lt;D 62.50，J值自94.27兩日崩落至43.18(-51.09點)——此驗證了前報「KDJ為四項中唯一警訊」之判斷為正確；RSI(14)自56.26退至49.88，重回50之下。⭐兩項保留：MACD翻負僅-0.35屬「剛好越線」非趨勢確立，且DIF仍在零軸之上，屬高檔死叉；J值43.18仍在超賣區20之上。布林寬度自91.5縮至87.5點(-4.4%)，已依例查核滾入/滾出，判定為真實波動率下降而非單一極端值滾出的機械效果。
+(6)⭐⭐本區間最重要的基本面消息與股價方向相反，必須並陳：台積電副共同營運長侯永清9/2於SEMICON Taiwan揭露，季度設備採購需求已達2025年12月預估的1.9倍(Q1為1.5倍、7月達1.9倍)，2026年資本支出自4月指引的520-560億美元大幅上修至600-640億美元，70-80%投入先進製程；台灣在建13座、海外5-6座晶圓廠，同時興建規模約為歷史常態的4-5倍，設備仍供不應求。⚠️但9/2當日股價收-2.25%，市場未給予正面回應。本報判讀：此為需求強勁的直接佐證，惟資本支出上修同時意味折舊壓力與自由現金流稀釋(較4月指引中位數增約15%)，且「設備供不應求」暗示產能開出時程存在不確定性。
+(7)⚠️⚠️本區間最具警示性的單一事件在客戶端：博通(AVGO)9/3公布Q3財報，營收295.9億美元(優於預期293.6億)、EPS 3.32美元(優於預期3.24)，數字雙雙超標，但僅因Q4營收展望348億美元略低於預期350.3億，股價即在S&amp;P 500上漲1.06%的當日逆勢重挫-2.74%收357.16美元。⚠️對台積電的直接推論：市場對AI供應鏈「僅小幅超標」的容忍度已明顯下降，10月中旬Q3法說會若僅小幅超越7/16所給的446-458億美元指引，可能面臨同樣的評價修正。此屬評價風險而非獲利風險。
+(8)⭐AI需求的下游驗證：戴爾(DELL)Q2營收470億美元(+58%YoY)、EPS 7.04美元(遠優於預期4.87)，AI伺服器營收倍增至164億美元，單季新增AI伺服器訂單609億美元，未出貨積壓訂單創紀錄950億美元(前值513億)，全年財測上修至營收1,920億美元。股價9/2大漲+15.81%收492.20、9/3再漲+4.91%收516.39美元。
+(9)⭐ADR與夜盤是今日唯一明確偏多的線索：TSM ADR 9/2、9/3連兩日收紅至417.01美元(+0.36%)，完全未跟隨台股9/2補跌；對台股溢價自9/1的7.54%擴大至9/3的10.66%(理論平價5×2,390÷31.71=376.85)，為追蹤區間高位。台指期夜盤(TAIFEX日期標記9/4「盤後」列，即9/3晚至9/4晨)台積電個股期CDF 202609收2,410(+20、+0.84%)、大盤台指期TX收46,487(+668、+1.46%)，方向一致指向今日開高。
+(10)⚠️⚠️但開高的性質必須講清楚：9/3美股是「大盤全面型」而非「半導體帶動型」上漲——S&amp;P 500收7,747.71(+1.06%)、那斯達克26,584.06(+1.40%)、VIX降至14.32(-5.79%)，但費城半導體指數僅收11,352.13(+0.11%)幾乎持平，且博通-2.74%、艾司摩爾-2.15%同步走弱。上漲主因為聯準會理事沃勒(Christopher Waller)偏鴿發言帶動公債殖利率回落，同日ADP私部門就業僅增3.8萬人、低於預期4.7萬人。今日若開高，動能來自總經風險偏好而非半導體基本面。
+(11)⭐供應鏈9/3：日月光589.00元(0.00%持平、兩日自610.00跌-3.44%)、華邦電169.00元(-5.59%，台股追蹤標的中跌幅最大)、聯發科4,340元(+1.52%，兩日淨漲+0.58%，相對強度明顯優於台積電)、輝達228.45美元(+1.80%)、蘋果328.21美元(+1.00%)、美光958.16美元(+0.22%)、英特爾91.67美元(+1.80%)、Arm 242.59美元(+3.29%)、AMD 456.16美元(-0.20%)、Amkor 46.94美元(-0.49%)、SK海力士1,596,000韓元(-1.05%)、三星250,000韓元(-0.20%)。設備四雄：ASML 1,646.19美元(-2.15%，在大盤上漲日背離)、AMAT 435.91(-0.58%，連3日跌累計-4.90%)、LRCX 292.66(+1.51%，但本報8/31所訂300美元關卡已連3日未收復、檢核維持未過)、KLAC 172.94(+0.39%)。
+(12)⭐相對強弱與評價：加權指數9/2收46,164.72(-784.00、-1.67%)、9/3收45,857.66(-307.06、-0.67%)；⭐9/3台積電+0.21%對大盤-0.67%，超額報酬+0.88pp，為兩日中唯一的相對強度亮點。評價：TWSE官方BWIBBU 9/3顯示P/E 27.70x、P/B 9.64x、殖利率0.92%(9/1為28.28x/9.84x/0.90%)，財報基準維持115/2未變動，因此下降100%來自股價下跌，屬分子調整而非換基準，可與8/14以後各日直接比較。市值約NT$62.0兆(9/1為63.3兆，兩日蒸發約1.3兆)。
+(13)⚠️衍生品：台積電個股期CDF 202609日盤9/3收2,390(-4、-0.17%、成交3,985口)，對現貨2,390為完全平價(9/1為正價差+3)，未平倉23,157口(9/1為24,169口、兩日續減1,012口)。⚠️⚠️台指選擇權P/C比本日不可作方向判斷：TXO每週三與週五均結算，9/2(週三)為結算日、未平倉全數重置(9/2賣權45,076/買權53,724口，較9/1的82,948/75,379口大幅縮減)，9/3的65,726/85,180口(P/C 77.16%)是結算後首日的重建部位，與9/1的1.10口徑上完全不可比較。欄序已依例以Unicode碼位驗證TAIFEX pcRatioDown為「賣權在前」。
+(14)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方端點取數(TWSE一律以curl落檔再讀)。⭐技術指標依TWSE官方收盤序列(2026-01-02~2026-09-03共162個交易日)自行計算，並依例先重算9/1各項指標、與9/2日報已發布值完全一致(RSI 56.26、MACD 8.68、K 76.13/D 67.06/J 94.27、MA5 2,418、BB 2,443/2,397/2,351)後才採用9/3之值。⚠️美股9/3的Yahoo日線close欄位為null，已改採meta.regularMarketPrice並驗證時間戳為20:00 UTC(16:00 ET)之收盤讀數，未以盤中價冒充收盤；AMKR首次請求連線中斷、已重新取數，未沿用前一日數值造成假性持平。⚠️韓股9/4盤中價(SK海力士1,648,000韓元、三星255,500韓元)已標明時點、不列入比較。⚠️台積電8月營收尚未公布(慣例9/10前)，屬「時間未到」非「查無」，本報不預測數字。⚠️台美半導體關稅與對中出口管制在9/2-9/3兩日查無新進展，已標為「政策背景」而非本週新聞。新台幣9/3 16:00台北時點收31.71(9/1為31.69、微貶0.06%)，對毛利率影響不足3bps、非本區間驅動因素。
+⭐綜合研判：評級自「中性偏多」下調為「中性」。⚠️四項轉壞：9/1突破證實為假突破且兩日淨跌-50點、9/2曾失守季線、技術面兩個死叉(MACD+KDJ)且RSI回落至50之下、外資9/2單日極端賣超11,987張。⭐三項未壞：9/3賣壓大幅收斂且無量止跌、收盤重新站回季線、ADR兩日連紅使溢價擴大至10.66%且夜盤CDF +0.84%指向今日開高。⭐立場：「開高不追、觀察2,405-2,418的回補力道」——今日檢核依優先順序為(1)能否站上並收在5MA 2,408之上；(2)ADR溢價10.66%的缺口向哪一邊收斂；(3)今晚美國8月非農就業報告，9/3的美股漲勢完全建立在殖利率回落之上，數據若與ADP背離將立即回收。⚠️失敗條件：若開高後收在2,397(MA20＝布林中軌)之下，9/1至今的型態確立為頭部。</t>
+        </is>
+      </c>
+      <c r="G119" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-07 日報 HTML & Excel 更新
資料日：台股與美股均為 2026-09-04（Fri）收盤；9/7 美股勞動節休市。
- 台股 2330 收 2,410（+20、+0.84%），量 14,102 張（連 2 日極低量、較 5 日均量少 40.3%）
- ADR 收 $428.91（+2.85%）、費半 +3.37%，8 月非農 16.2 萬人優於預期使大盤走弱但半導體逆勢大漲
- ADR 溢價擴大至 12.69%（追蹤區間新高）；外資轉買 1,885 張，近 5 日仍淨賣 9,886 張
- 一併修正頁面內部矛盾：KPI 卡「2026 CapEx」由 4 月指引 $52–56B 更新為 9/2 SEMICON 上修後的 $60–64B

fresh-context 驗證隨後執行，如有出入以 fix: 更正。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-04</t>
+          <t>報告更新日期：2026-09-07</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-04</t>
+          <t>最後更新：2026-09-07</t>
         </is>
       </c>
     </row>
@@ -7638,6 +7638,57 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B120" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,410（9/4收）</t>
+        </is>
+      </c>
+      <c r="C120" s="54" t="inlineStr">
+        <is>
+          <t>+0.84%（9/4收）</t>
+        </is>
+      </c>
+      <c r="D120" s="53" t="inlineStr">
+        <is>
+          <t>US$428.91（9/4收）</t>
+        </is>
+      </c>
+      <c r="E120" s="53" t="inlineStr">
+        <is>
+          <t>14,102（9/4收）</t>
+        </is>
+      </c>
+      <c r="F120" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-07(Mon)，資料為2026-09-04(Fri)台股與美股收盤；9/5、9/6為週末。⚠️今日(9/7)為美國勞動節，美股與ADR全日休市，本報之後到9/8台股收盤為止不會有新的ADR或費半參考值。
+(1)⭐價格與型態，前報第一號檢核的結果為「過關，但過得很勉強」：前報訂「開高不追、能否站上5MA 2,408並收在其上」。9/4開2,415(落在前報所指2,405-2,418回補區間內、且即為當日最高)，盤中最低回測2,390(＝9/3收盤，支撐實測未破)，終場收2,410(+20、+0.84%)，站上當日5MA 2,406與前報所指2,408，但僅高出2點。前報失敗條件「收在2,397(MA20＝布林中軌)之下」未觸發。K線型態為「開盤即最高、盤中回測前日收盤、尾盤拉回接近開盤」的紡錘線，距9/1假突破高點2,440仍差30點(-1.23%)。
+(2)⭐均線結構在一日內由「短中期轉空」修復為「全面站上」：現價2,410高於MA5(2,406)、MA10(2,405)、MA20(2,399)、MA60(2,391)、MA120(2,253)全部五條均線，為9/1(2,440)以來首次。⚠️惟修復品質須打折：距MA5僅4點、距MA10僅5點，任何一根10點以上黑K即再度失守；且MA5自9/1的2,418一路降至2,406，是價格接近均線而非均線轉上。布林通道寬度自3.65%微收斂至3.52%，上軌2,441與9/1假突破高點2,440幾乎重合、構成同一壓力帶。
+(3)⚠️⚠️量能是本報最主要的保留：9/4成交14,102張(額339.17億、43,438筆)，較9/3的14,252張再縮1.1%，連續第2個交易日落在2026年量能最低區間，較5日均量23,631張低40.3%；成交筆數43,438筆亦為近期新低(9/3為54,232筆、9/2為198,779筆)。價格站回5MA是在「賣壓消退」而非「買盤進場」的條件下完成，此一結構對2,440的測試不具支撐力。
+(4)⭐籌碼面同步轉向但幅度有限：外資9/4由賣轉買+1,885張(T86官方+1,885,085股)、投信賣322張(-322,024股)、自營商買407張(+406,740股)，三大法人合計買超1,970張(官方合計+1,969,801股)。⚠️惟近5日(8/31至9/4)外資合計仍淨賣超9,886張(-4,554、+5,731、-11,987、-961、+1,885)，單日轉買尚不足以認定趨勢反轉。
+(5)⭐技術指標轉為勉強偏多但訊號極弱：MACD柱自-0.35回升至+0.01(DIF 8.6220、DEA 8.6165、僅差0.0055)，死叉維持1個交易日即被抵銷；⚠️本報不將其視為有效金叉——+0.01絕對值等同於零，故欄位顏色採橙色(訊號待確認)而非綠色。RSI(14)自49.88回升2.47點至52.35，重新站上50中軸。KDJ是四項中唯一尚未轉向者：K 58.42仍低於D 61.14(差距-2.72)，但差距自9/3的-6.44收斂，J值自43.18回升至52.99。整段9/2至9/4修正中RSI最低僅49.28、全程未接近40弱勢區。
+(6)⭐⭐本日最重要的單一事件在美股端，且結果與前報的擔憂方向相反：美國8月非農就業新增16.2萬人優於市場預期，殖利率跳升、升息預期升溫，美股大盤因此走弱——前報預判「數據若偏強，殖利率反彈將直接回收漲幅」對大盤成立；⚠️但對半導體族群不成立：費城半導體指數收11,735.26(+383.13點、+3.37%)逆勢大漲，TSM ADR收428.91美元(+11.90、+2.85%)。資金在總經利空中選擇性流入半導體，理由指向AI資本支出未受利率預期影響、記憶體供給吃緊。本報認為這是本次最須修正的既有假設。⚠️須避免誇大：428.91美元距2年高點477.57美元(2026-06-30)仍低10.2%，且過去2年有8個單日漲幅大於+2.85%的交易日，本次非異常級別表現。
+(7)⭐族群內部出現明確輪動，領漲的是設備與記憶體而非AI運算晶片：科磊+7.32%收185.60(創本波新高)、美光+6.10%收1,016.59(首度站上1,000美元關卡)、科林研發+5.12%收307.65(收復本報8/31所訂300美元關卡、連4日收在其下後突破)、超微+4.69%收477.57、英特爾+4.51%收95.80、應用材料+4.31%收454.71、艾司摩爾+4.17%收1,714.88(一日收復9/2至9/3全部跌幅)、Arm+3.92%收252.09。⚠️相對落後者：輝達僅+0.84%收230.36(為費半漲幅的四分之一)、博通+0.21%收357.90、高通+0.10%收168.74，蘋果更逆勢-2.51%收319.97、吐光9/1以來全部漲幅，為追蹤標的中唯一明顯下跌者。
+(8)⚠️英特爾的相對強度持續擴大，是對台積電代工地位最值得長期追蹤的競爭訊號：英特爾自9/1的88.97美元累計+7.68%，同期台積電ADR自414.00美元累計+3.60%，漲幅超過一倍以上，且英特爾已連4個交易日收紅、創本波新高。
+(9)⭐⭐ADR溢價擴大至追蹤區間新高12.69%：理論平價5×2,410÷31.66＝380.61，對市價428.91之溢價+12.69%，較9/3的10.66%再擴大2.03個百分點，且連續3個交易日擴大(9/1為7.54%)。成因是單向的——台股僅+0.84%而ADR+2.85%，缺口全部由美股端拉開。⚠️今日美股休市、ADR不交易，溢價變動將完全由台股單邊決定，是觀察台股補漲力道最乾淨的一天。
+(10)⭐台股供應鏈9/4：聯發科4,415元(+1.73%，連兩日紅、自9/2的4,275元漲+3.27%，創本波新高、超越9/1漲停價4,315元，為台股追蹤標的中相對強度最高者)、華邦電174.00元(+2.96%，收復9/3重挫-5.59%的一部分，仍低於9/2的179.00元)、日月光588.00元(-0.17%，為極少數收黑者、自9/1的610.00元累計-3.61%，封裝端持續落後)。封裝端美股Amkor 47.77美元(+1.77%)同樣落後於費半+3.37%，與日月光一致。韓股9/4：SK海力士1,647,000韓元(+3.20%)、三星255,500韓元(+2.20%)，均終結3連跌；⚠️今日(9/7)09:56 KST盤中分別報1,742,000(+5.77%)與265,000韓元(+3.72%)，已標明時點、為盤中即時數據非收盤值。
+(11)⭐相對強弱與評價：加權指數9/4收46,551.13(+693.47、+1.51%)。⚠️9/4台積電+0.84%落後大盤+1.51%、大幅落後費半+3.37%；YTD亦以+52.1%落後加權指數+58.6%與費半+59.3%——台積電今年以來相對於自身所屬的兩個指數皆為落後，此為長期追蹤上不應忽略的事實。評價：TWSE官方BWIBBU 9/4顯示P/E 27.94x、P/B 9.72x、殖利率0.91%(9/3為27.70x/9.64x/0.92%)，財報基準維持115/2未變動，故本次上升100%來自股價上漲，屬分子調整而非換基準。市值約NT$62.5兆。ADR端P/E約31.5x、P/B約11.0x，係依官方值×(1+溢價12.69%)換算，可逐步複算。
+(12)⚠️衍生品：台積電個股期CDF 202609一般盤9/4收2,413(+23、+0.96%、成交4,537口)，對現貨2,410呈+3點正價差(9/3為平價)，偏多程度極輕微、不具訊號強度；未平倉22,769口(9/3為23,157口、減少388口)，屬結算週正常縮減。⚠️⚠️台指選擇權P/C比本日同樣不可作方向判斷：TXO每週三與週五均結算，9/4(週五)為結算日、未平倉全數重置(賣權自9/3的65,726降至48,162口、買權自85,180降至48,258口，縮減幅度不同)，因此9/3的0.77與9/4的1.00之間不存在可比性，不可解讀為空方力道增強。結算後首個讀數0.998，賣權與買權未平倉僅差96口(不到0.2%)，屬本報所見最接近完全均衡的一次；有意義的比較要等9/7、9/8兩個非結算日。欄序已依例以Unicode碼位驗證TAIFEX pcRatioDown為「賣權在前」。
+(13)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方端點取數(TWSE一律以curl落檔再讀)。⭐技術指標依TWSE官方收盤序列(2026-01-02至2026-09-04共163個交易日)自行計算，並依例先重算9/3各項指標、與9/4日報已發布值完全一致(MA5 2,408/MA10 2,405/MA20 2,397/MA60 2,388/MA120 2,248、RSI 49.88、MACD柱-0.35、K 56.06/D 62.50/J 43.18、布林2,441/2,397/2,353、5日均量23,816)後才採用9/4之值。⚠️本日有兩項參考值缺席並已明述：今晨夜盤資料TAIFEX尚未發布(週末無夜盤，週五夜盤資料歸屬下一交易日、須待今日盤後公布)，加上美股勞動節休市無隔夜訊號，開盤方向的既有參考值全部缺席，改以今日09:20台北TWSE MIS實際盤中數據替代(2330開2,435、高2,440、低2,430、成交4,067張；加權指數47,042.27、+1.06%)，並標明為盤中數據、收盤前不作結論。⚠️Yahoo的TWD=X日線序列本身在9/4缺一根K棒(9/3後直接跳至9/7盤中)，已改以小時線取台北16:00讀數31.66，此為序列缺漏而非休市。⚠️台積電8月營收尚未公布(慣例9/10前)，屬「時間未到」非「查無」，本報不預測數字。⚠️今日另更正一處頁面內部矛盾：KPI卡「2026 CapEx」原沿用4月法說會指引52-56億美元區間，與同頁9/2 SEMICON Taiwan上修至600-640億美元的敘述互相矛盾，已改為600-640億美元並註明上修來源。
+⭐綜合研判：評級自「中性」上調為「中性偏多」。⭐三項轉好：價格站回全部五條均線、外資單日由賣轉買1,885張、ADR與費半逆總經利空大漲使溢價擴至12.69%。⚠️三項未好：量能連2日不足5日均量六成、MACD柱+0.01等同於零、KDJ仍維持死叉。⭐立場：「今日開高直接測試2,440的機率高，但成交量未回到20,000張以上之前，突破2,440應視為第二次測試而非確認」——今日檢核依優先順序為(1)2,440(＝布林上軌2,441)的第二次測試能否以放量收在其上；(2)量能背離能否解除；(3)ADR溢價12.69%在美股休市日由台股單邊收斂的力道。⚠️失敗條件：若今日開高後收在2,399(MA20＝布林中軌)之下、形成長上影線，將是9/1型態的第二次重演，本報屆時會把2,440定性為確定的型態頸線。</t>
+        </is>
+      </c>
+      <c r="G120" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-08 日報 HTML & Excel 更新
台股 9/7 收 NT$2,460（+50、+2.07%），收在全日最高並突破 9/1 假突破高點 2,440；
量 26,898 張（+19.8% vs 5 日均量、筆數 +185.4%）；外資買超 16,135 張為追蹤區間最大。
9/7 為美國勞動節，ADR 與費半無新讀數，全頁逐欄標註為 9/4 收盤值。
ADR 溢價由 12.69% 收斂至 9.91%（台股單邊）；MACD 柱 +0.01→+6.46、KDJ 完成金叉。

產生器另作兩項修正：
- 模板「估值解讀」硬編的 BWIBBU 日期 9/04 → 9/07
- 股價卡片新增可選欄位 nyse_asof_note，於美股休市日在原地註明 ADR 漲跌所屬交易日

驗收：fresh-context subagent 以 curl 重抓 TWSE STOCK_DAY/BWIBBU/T86 與 TAIFEX
pcRatioDown/futDataDown 核對、並以官方收盤序列重算全部技術指標，16 條驗收條件全數通過。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-07</t>
+          <t>報告更新日期：2026-09-08</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-07</t>
+          <t>最後更新：2026-09-08</t>
         </is>
       </c>
     </row>
@@ -7689,6 +7689,56 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B121" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,460（9/7收）</t>
+        </is>
+      </c>
+      <c r="C121" s="51" t="inlineStr">
+        <is>
+          <t>+2.07%（9/7收）</t>
+        </is>
+      </c>
+      <c r="D121" s="50" t="inlineStr">
+        <is>
+          <t>US$428.91（9/4收，9/7美股休市）</t>
+        </is>
+      </c>
+      <c r="E121" s="50" t="inlineStr">
+        <is>
+          <t>26,898（9/7收）</t>
+        </is>
+      </c>
+      <c r="F121" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-08(Tue)，台股資料為2026-09-07(Mon)官方收盤。⚠️⚠️須先講清楚：美股與ADR沒有新數據——9/7為美國勞動節(Labor Day)、NYSE全日休市，本報的ADR 428.91美元、費半11,735.26與全部美股個股價格仍為9/4(Fri)收盤值，與昨日日報完全相同，非本日新讀數；下一組美股讀數為今晚(9/8美東)收盤，明日回補。
+(1)⭐⭐價格與型態，前報三項檢核全數過關：台股2330官方收NT$2,460(+50、+2.07%、開2,435／高2,460＝收盤／低2,430)。前報第一順位訂「2,440的第二次測試，關鍵在收盤能否站上且量能回到20,000張以上」——收2,460越過2,440達20點、量26,898張超出門檻34.5%，前報所訂「量能不足的突破應視為雙重頂右肩」之降級條件因此不成立。第二項「量能背離的解除」過關。第三項「ADR溢價12.69%由台股單邊收斂」過關且方向完全如預期。前報失敗條件「收在2,399(MA20)之下、形成長上影線」明確未觸發：全日無上影線、收盤即最高。⚠️但必須同時說清楚：2,460是2026-07-16(收2,470)以來最高收盤、相隔36個交易日，不是歷史新高也不是2026年新高——2026年最高收盤為6/22的2,510、52週高為2,535，2,460距52週高仍低2.96%。
+(2)⭐⭐量能的品質已用成交筆數再驗一次，避免把單一大單誤讀為人氣回流：9/7成交26,898張(額NT$658.39億、123,981筆)，較9/4的14,102張放大90.7%，較5日均量22,452張高19.8%；成交筆數自43,438筆躍升至123,981筆(+185.4%)，增幅大於張數增幅，代表單筆規模其實縮小、進場的是更多的人而非更大的單。這解除了本報自9/3起連續四份日報所記的「價漲量縮背離」。⚠️另註：5日均量自23,631降至22,452並非量能萎縮，而是8/31的32,793張(MSCI季度調整生效日、屬機械性爆量)滾出窗口所致；以前一版基準23,631張比較，本日仍高13.8%，兩種比法結論一致。
+(3)⭐⭐籌碼是本日最強的一項：外資單日買超16,135張(T86官方+16,135,314股)，為本報追蹤區間內最大單日買超、約為前次高點9/1的5,731張之2.8倍；自營商買超720張(+720,108股)、投信賣超368張(-367,588股)，三大法人分項加總合計買超16,487張(官方合計欄+16,487,834股，捨入差1張屬正常)。據聯合新聞網與Yahoo股市報導，全市場外資9/7買超883億元為史上第4大，台積電以約394.9億元居買超之首，聯發科(137.6億)、日月光投控(113.4億)分列二三。⚠️惟近5日(9/1至9/7)外資合計僅淨買超10,803張(+5,731、-11,987、-961、+1,885、+16,135)，係因9/2單日賣超11,987張的抵銷——單日巨量買超尚不足以認定趨勢。
+(4)⚠️⚠️市場歸因可查證，且其性質必須誠實標註為「預期性下注」：多家媒體指向9/10(週四)13:30將公布的8月合併營收——鴻海、聯電已公布的月營收表現不錯，市場預期台積電同樣強勁；另有蘋果新機拉貨旺季的預期性買盤。換言之9/7的漲勢是對尚未公布數據的下注，而非對已實現事實的反映；因此9/10的數字若不如預期，回檔幅度會比一般利空更大。本報將其列為當前第一順位風險。台積電投資人關係財務行事曆確認8月營收排定9/10(週四)台北時間13:30公布(9月營收排定10/8)，截至本報產製時尚未發布。比較基準：7月合併營收4,675.81億元(月增5.6%、年增44.7%、單月新高)，Q3指引中位45.2億美元換算月均約需NT$4,851億，7月仍低約3.6%。
+(5)⭐技術面四項指標本日首度全部同向翻多，且不再是勉強過關：MACD柱自9/4的+0.01(等同於零)放大至+6.46(DIF 12.6499／DEA 9.4178、正乖離3.23)，單日擴張為追蹤區間內最大；前報明訂「柱狀體站上+1.0以上才算完成金叉確認」，本日超出該門檻6.5倍，欄位顏色自橙色改為綠色。KDJ完成金叉：K自58.42升至72.28、上穿D 64.85(D自61.14升起)，K-D由-2.72翻正為+7.43，9/2成立的死叉維持4個交易日後結束。RSI(14)自52.35升至57.92，越過9/1假突破當日的56.26，動能回到假突破前水準之上。現價2,460站上全部五條均線(MA5 2,417／MA10 2,414／MA20 2,403／MA60 2,394／MA120 2,258)且已拉開距離(距MA5達43點)，MA5自2,406升至2,417終結自9/1以來連續下彎。⚠️兩項過熱訊號須並陳：收盤2,460已站上布林上軌2,452(超出8點)；KDJ的J值自52.99跳升34.15點至87.14，逼近一般以90為界的超買區。
+(6)⭐布林通道寬度自3.52%擴張至4.06%，已依既定作法檢查滾動窗口以排除機械效果：滾出的是8/10的2,380、滾入的是9/7的2,460，滾入值距新中軌2,403達57點、遠大於滾出值的偏離19點，因此本次擴張是9/7這根長紅實際造成的，不是舊極端值滾出窗口的假象。⭐前報所指「布林上軌2,441與9/1假突破高點2,440構成同一壓力帶」本日已被突破，該壓力帶轉為支撐帶。
+(7)⭐⭐ADR溢價由12.69%收斂至9.91%，這是前報第三項檢核且驗證得非常乾淨：理論平價5×2,460÷31.52＝390.23(採捨入後匯率)，對市價428.91(9/4收盤、9/7未交易)之溢價+9.91%。由於ADR整日靜止不動，這2.78個百分點的收斂完全由台股單邊造成。可進一步拆解：若匯率維持9/4的31.66，溢價會是10.40%，故台股上漲貢獻約2.29pp、新台幣升值(31.66→31.52)貢獻約0.49pp。⚠️判讀：缺口已收斂逾六成，台股補漲空間相應縮小；今晚美股恢復交易後若ADR未跟上台股的+2.07%，溢價將續縮、台股次日面臨回吐壓力，此為明日日報第一順位檢核。
+(8)⭐亞洲半導體9/7全面同步走強，且台積電並非最強者而是墊底：韓國SK海力士+8.26%(1,647,000→1,783,000韓元)、台股聯發科+7.81%(4,415→4,760元)、三星電子+5.68%(255,500→270,000韓元)、日月光+5.61%(588→621元)、華邦電+3.45%(174→180元)，均大幅領先台積電的+2.07%。這說明9/7是亞洲區域性的半導體資金回流，而非台積電個股事件。⚠️已標明時點的盤中補充：9/8上午08:57 KST，SK海力士報1,858,000韓元(+4.21%)、三星報275,000韓元(+1.85%)，為盤中即時數據非收盤值。⭐日月光的+5.61%創本波新高並終結本報自8/31起追蹤的「封裝端持續落後」；聯發科題材延續9/1輝達35億美元認購可轉債與十年AI合作。
+(9)⚠️衍生品：台積電個股期CDF 202609一般盤9/7收2,464(+51、+2.11%、成交8,450口)，對現貨2,460維持+4點正價差(9/4為+3)；⚠️未平倉自22,769口減少至21,709口(-1,060口)、為連續第2個交易日減少——價漲而未平倉減少通常對應空單回補而非新多單進場，這是本日期貨端唯一的保留。今晨夜盤(TAIFEX標記日期2026/09/08之「盤後」列，涵蓋9/7 15:00至今晨05:00)CDF 202609收2,463(-1、成交273口)、台指期TX 202609收47,329(-133、成交9,784口)，小幅偏弱；⚠️該時段美股仍在勞動節休市，夜盤無外部訊號可反映，參考價值有限。⚠️⚠️台指選擇權P/C未平倉比9/7為1.12(賣權72,790口／買權65,172口、官方比率欄111.69%，已核對TAIFEX pcRatioDown為「賣權在前」)，但不可與9/4的1.00比較：9/4(週五)為結算日、未平倉全數重置至賣權48,162／買權48,258口，9/7為結算後重建首日，兩者分屬不同基期。本週9/9(週三)與9/11(週五)均為結算日，故今日(9/8)的讀數是本週唯一能與9/7直接比較的一天。
+(10)⭐評價與匯率：TWSE官方BWIBBU 9/7顯示P/E 28.52x、P/B 9.92x、殖利率0.89%(9/4為27.94x／9.72x／0.91%)，財報基準維持115/2未變動，故本次上升100%來自股價上漲(2,410→2,460、+2.07%)，屬分子調整而非換基準。⚠️絕對水位進一步升高：28.52x約落在5年區間(9.8x-37.8x)第89百分位(本報估算，前一版27.94x為第88)、P/B 9.92x約為5年第93百分位——百分位為本報依歷史區間所估、非官方數據。市值約NT$63.8兆。ADR端P/E約31.3x、P/B約10.9x，係依官方值×(1+溢價9.91%)換算，可逐步複算。⚠️匯率方向出現變化，須自「非因素」升級為「待觀察」：新台幣9/7 16:00台北時點收31.52，較9/4的31.66升值0.44%，為本週最大單日升幅並跌破8月下旬以來的31.6-31.8區間下緣，9/8 09:16盤中續升至31.478；目前對毛利率影響約-18bps、幅度仍小，但方向已由區間震盪轉為單向升值，若跌破31.0影響將擴大至-66bps量級。
+(11)⭐相對強弱：加權指數9/7收47,326.27(+775.14、+1.67%)，據報導為史上收盤次高。⭐9/7台積電+2.07%領先大盤+1.67%達0.40個百分點，為9/3以來首度單日領先；⚠️惟近5日(+2.29% vs 大盤+2.60%)、近1月(+3.80% vs +7.01%)、YTD(+55.2% vs 大盤+61.3%、費半+59.3%)三個期間台積電仍全數落後，1個月尺度上落後達3.21個百分點——單日領先不改變中期落後的事實。⚠️註：費半與ADR的「當日漲跌」在本報第16節顯示為0.00%，那不是持平，而是9/7美股休市、兩者根本沒有交易，係受欄位型別限制所致。
+(12)📅資料口徑與缺口聲明：全程TWSE/TAIFEX/Yahoo官方端點取數(TWSE與TAIFEX一律以curl落檔再讀)。⭐技術指標依TWSE官方收盤序列(2026-01-02至2026-09-07共164個交易日)自行計算，並依例先重算9/4各項指標、與9/7日報已發布值完全一致(MA5 2,406／MA10 2,405／MA20 2,399／MA60 2,391／MA120 2,253、RSI 52.35、MACD柱+0.01、K 58.42／D 61.14／J 52.99、布林2,441／2,399／2,357、5日均量23,631)後才採用9/7之值。⚠️本日的資料缺口為「美股整批缺席」且已逐欄標註：ADR、費半與全部美股個股(輝達、蘋果、超微、美光、艾司摩爾、英特爾、高通、博通、科磊、科林研發、應用材料、Amkor、Arm)價格與漲跌幅均為9/4收盤值，明日日報必須回頭補正，不得任其連續兩日顯示持平。⚠️Yahoo的TWD=X日線序列9/7該根K棒收盤為null(美股休市所致)，已依既定作法改以小時線取台北16:00讀數31.52。⚠️新增一項待確認事項：CNBC報價頁揭示TSM(ADR)現金股利每股US$1.114、除息日2026-09-16，本報尚未於TSMC IR官網逐項核對，已於頁面標【待官方確認】並明確與台股端區分——台股Q2股利NT$7.0/股(8/11董事會核准)除息日為2026-12-10、基準日12/16，兩者屬不同批次。⚠️今日另更新頁面模板一處殘留日期：估值解讀段落硬編的「BWIBBU 9/04」已改為9/07。
+⭐綜合研判：評級自「中性偏多」上調為「看多」。⭐四項全面轉好：價(收在最高、越過2,440且無上影線)、量(+19.8%於均量、筆數+185.4%)、籌碼(外資16,135張為區間最大買超)、技術(MACD與KDJ雙金叉、五線全站上)。⚠️三項保留：(1)完全沒有美股當日訊號背書，外部檢驗要等今晚；(2)收盤已站上布林上軌2,452、J值87.14逼近超買，短線過熱；(3)漲勢理由是對9/10營收的預期性下注，數字不如預期時回檔會較深。⭐立場：趨勢已轉多，但今日追高的風險報酬比不佳；2,403(MA20＝布林中軌)為多空分界，跌破才需調整看法。今日檢核依優先順序為(1)今晚美股恢復交易後ADR是否跟上、溢價是否續縮；(2)台股今日能否守住2,440並維持20,000張以上量能，若開高走低留長上影線並跌回2,440之下，昨日突破須降級為單日情緒；(3)P/C比與9/7的1.12做本週唯一一次有效跨日比較。⚠️失敗條件：收在2,403之下，將使昨日突破與四項技術指標的翻多同時失效。</t>
+        </is>
+      </c>
+      <c r="G121" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-09 日報 HTML & Excel 更新
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-08</t>
+          <t>報告更新日期：2026-09-09</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G121"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-08</t>
+          <t>最後更新：2026-09-09</t>
         </is>
       </c>
     </row>
@@ -7739,6 +7739,57 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B122" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,470（9/8收）</t>
+        </is>
+      </c>
+      <c r="C122" s="54" t="inlineStr">
+        <is>
+          <t>+0.41%（9/8收）</t>
+        </is>
+      </c>
+      <c r="D122" s="53" t="inlineStr">
+        <is>
+          <t>US$439.00（9/8收）</t>
+        </is>
+      </c>
+      <c r="E122" s="53" t="inlineStr">
+        <is>
+          <t>28,932（9/8收）</t>
+        </is>
+      </c>
+      <c r="F122" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-09(Wed)，台股資料為2026-09-08(Tue)官方收盤；美股已於9/8恢復交易，前一份日報標註的「美股整批缺席」缺口本日全數回補，ADR、費半與全部美股個股均為9/8美東收盤，無任何一欄沿用9/4的值。
+(1)⭐⭐前報(9/8)三項檢核的實際結果為「兩項過關、一項出現保留」，逐條回覆：第一順位「今晚美股恢復交易後ADR是否跟上、溢價是否續縮」過關，且方向與前報所擔心的完全相反——ADR收$439.00(+10.09、+2.35%、成交約1,309萬股)，漲幅超前台積電9/7在台股的+2.07%達0.28個百分點，亦強於同日費半的+1.30%；ADR溢價不但沒有續縮，反而自9.91%重新擴大至12.08%，台股補漲空間回來了。第二項「守住2,440並維持20,000張以上量能」雙雙過關：全日最低2,460高於2,440達20點、量能28,932張超出門檻44.7%且連2日站穩。第三項「P/C比與9/7的1.12做本週唯一一次有效跨日比較」已完成，結果1.12→1.05。前報失敗條件「收在2,403(MA20)之下」明確未觸發。
+(2)⚠️⚠️本日唯一且必須誠實記錄的保留是型態：台股2330官方收NT$2,470(+10、+0.41%、開2,465／高2,505／低2,460＝9/7收盤、量28,932張、額NT$717.69億、106,768筆)。盤中最高2,505為7/1(當日高2,505、收2,505)以來首度重返該價位——7/2至9/7共47個交易日無任何一日盤中觸及——但收盤自高點回吐35點(-1.40%)，留下本波最長上影線。前報所訂降級條件為「開高走低留下長上影線『並』跌回2,440之下」，前半段成立、後半段未成立，故降級條件整體不成立，本報不降級，但不略過上影線本身。收盤2,470追平7/16的2,470，為7/1(收2,505)以來最高收盤水準，非歷史新高：2026年最高收盤為6/22的2,510、52週高2,535(6/23盤中)。
+(3)⭐量能連2日過關且再放大，惟品質面出現與9/7相反的變化須並陳：28,932張較9/7的26,898張增7.6%、較5日均量21,867張高32.3%；但成交筆數自123,981筆降至106,768筆(-13.9%)，平均每筆自0.217張放大至0.271張(+24.9%)。9/7是「更多的人進場」(筆數+185%)，9/8是「更大的單進場」，較偏向法人整筆承接而非散戶追價。⚠️註：5日均量自22,452降至21,867係9/1的31,855張滾出窗口所致，非量能萎縮；以前一版基準22,452張比較本日仍高28.9%。
+(4)⭐⭐籌碼延續且結構改善：外資連2日買超5,497張(T86官方+5,496,736股)、投信由9/7的賣超368張轉為買超1,205張(+1,204,619股，為近5日最大)、自營商賣超398張(-397,962股)，三大法人分項加總合計買超6,304張(官方合計欄+6,303,393股，捨入差1張屬正常)。近5日(9/2至9/8)外資合計淨買超10,569張(-11,987、-961、+1,885、+16,135、+5,497)，已連3個交易日站在買方。⚠️惟5,497張僅為9/7的16,135張之三分之一，單日規模明顯縮減，與價格漲幅自+2.07%收斂至+0.41%同向。
+(5)⚠️⚠️未被前報預期到的一項背離：加權指數9/8收47,105.78(-220.49、-0.47%、成交額NT$9,226.58億)，台積電是在大盤翻黑的一天獨自收紅，領先大盤0.88個百分點(前一日0.40pp)。同日9/7大漲的聯發科(-1.05%、4,710元)與日月光(-0.48%、618元)雙雙回檔，韓國SK海力士(+0.56%、1,793,000韓元)與三星電子(-0.19%、269,500韓元)同步降溫，僅華邦電(+4.44%、188元)續強。判讀：9/7的亞洲族群性資金回流僅維持一個交易日，9/8已收斂為台積電獨強的個股行情——短線資金集中於龍頭不算壞事，但它移除了「族群廣度優於單一個股訊號」這項支撐，使當前漲勢對9/10營收的依賴度升高。
+(6)⭐美股9/8結構清楚且對台積電有利：ADR的+2.35%優於費半的+1.30%(收11,887.87、+152.61點)，而權重最大的輝達-2.01%($225.73)、蘋果-1.17%($316.22)、美光-1.61%($1,000.26)三檔下跌；費半漲幅由設備與非AI運算撐起——英特爾+9.05%($104.47、首度站上$100)、Amkor+6.18%($50.72、首度站上$50)、超微+5.90%($505.74、首度站上$500)、科林研發+4.15%、應用材料+3.98%(超越8/31的$458.39)、Arm+3.74%、高通+3.17%、博通+2.98%(收復9/3財報後全部跌幅)、艾司摩爾+2.91%、科磊+1.82%。意義：本波驅動力不繫於單一AI運算晶片龍頭，需求廣度優於8月由輝達單騎領軍的型態。
+(7)⭐技術面延續改善但速度分歧：MACD柱自+6.46續張至+11.27(DIF 16.4633／DEA 10.8269、正乖離5.65)，連2日擴張、為四項指標中唯一未見趨緩者；RSI(14)自57.92微升至58.95(+1.03，升速較前一日的+5.57收斂約八成)。⚠️KDJ出現本日唯一的負面訊息：K僅自72.28微升至72.55(+0.27)、D自64.85升至67.42、K-D差距自+7.43收斂至+5.13，J值反而自87.14回落至82.81(-4.33)——價格創高而J值下滑，屬高檔鈍化初期，與35點的上影線指向同一件事。均線全數上彎且距離拉開：MA5 2,423／MA10 2,421／MA20 2,407／MA60 2,397／MA120 2,263，現價高於MA5達47點；完整多頭排列自8/27起已連續維持9個交易日，本日新意在間距拉開而非排列成立。⚠️收盤2,470連2日站在布林上軌2,464之上，通道寬度自4.06%續張至4.70%(已查證滾出的是8/11的2,395、滾入的是9/8的2,470，屬實質擴張非滾動窗口機械效果)。
+(8)⚠️期貨與選擇權是四大面向中最保留的一項：台積電個股期CDF 202609日盤收2,471(+7、+0.28%、成交8,234口)，漲幅小於現貨的+0.41%，正價差自+4收斂至+1、接近平價；未平倉自21,709口再減至20,709口，為連續第4個交易日減少(9/3 23,157、9/4 22,769、9/7 21,709、9/8 20,709)，自9/2的23,592口累計減少2,883口(-12.2%)——價漲而未平倉持續減少，通常對應空單回補與多單獲利了結並存而非新資金進場。台指期TX 202609日盤收46,980(-482)，與個股期同日收紅相反。⭐TXO台指選擇權P/C未平倉比自9/7的1.12降至9/8的1.05(賣權87,226口／買權82,893口、官方比率欄105.23%，已核對TAIFEX pcRatioDown為「賣權在前」)，這是本週唯一一次有效跨日比較，買權重建+27.2%快於賣權+19.8%，空方傾斜略減。⚠️今日(9/9週三)為TXO結算日，未平倉將重置，明日日報不得與本日的1.05做跨日比較。⭐今晨夜盤(TAIFEX標記日期2026/09/09之「盤後」列，涵蓋9/8 15:00至今晨05:00)已明確反映美股上漲：CDF 202609收2,488(+17、成交1,630口)、TX 202609收47,055(+100、成交31,998口)。
+(9)⭐評價與匯率：TWSE官方BWIBBU 9/8顯示P/E 28.63x、P/B 9.96x、殖利率0.89%(9/7為28.52x／9.92x／0.89%)，財報基準維持115/2未變動，故上升100%來自股價(2,460→2,470、+0.41%)。28.63x約落5年區間第89百分位、P/B約第93百分位(本報估算)。市值約NT$64.0兆。ADR端P/E約32.1x、P/B約11.2x，係依官方值×(1+溢價12.08%)換算。⚠️須註記口徑差異：同日stockanalysis.com顯示TSM本益比29.16x，該值採其自身TTM每股盈餘，與TWSE的115/2財報基準不同，兩套數字不可互相取代。⚠️匯率：新台幣9/8 16:00台北時點報31.53，較9/7的31.52微貶0.03%，等於前一日0.44%升幅後的持平——前報將匯率自「非因素」升級為「待觀察」，本日讀數並未支持「單向升值」，故降回非因素；今日(9/9)09:15盤中報31.465、續升0.21%，明日回頭確認。
+(10)⭐ADR溢價完整拆解：理論平價＝5×2,470÷31.53＝391.69(採捨入後匯率)，對市價439.00之溢價+12.08%，較9/7的9.91%擴大2.17個百分點。台股上漲+0.41%與新台幣微貶合計使溢價降至9.50%(-0.41pp)，ADR上漲+2.35%則拉升至12.08%(+2.58pp)，ADR端貢獻是壓倒性的。判讀：缺口重新回到12.08%、接近9/4的12.69%，台股今日重新具備補漲空間；⚠️反向解讀同樣成立——若台股今日不漲，代表拒絕跟隨美股，會是比回吐更負面的訊號。期間比較維持中期落後：近5日+1.23%領先大盤+0.33%(基準均為9/1)，但近1月+4.22%落後+6.51%、YTD+55.8%落後大盤+60.5%與費半+61.4%。
+(11)📅本日新聞五則(均為9/8之後發布、附來源)：①超微CFO於花旗2026 Global TMT大會表示AI市場2030年上看2兆美元、資料中心營收目標2027年達700億美元(約2026年兩倍)，AMD股價+5.90%——AMD的MI350／MI450全由台積電代工並用CoWoS，屬對先進製程與先進封裝的長約需求宣告，惟為公司自訂目標非已簽訂單(來源ts2.tech 9/8)。②艾司摩爾與台積電9/8聯合宣布推動High-NA EUV大版光罩產業轉型，2031年建12吋光罩試產線、2033年進入先進製程量產，台積電自2030年起於高量產階段導入High-NA——屬4至7年後的技術路線圖，對近期營收獲利無影響，不應讀成短期利多(來源GlobeNewswire 9/8)。③英特爾+9.05%成因為Northland上調評等至Outperform(目標價$120)、10月起PC處理器擬漲價約10%、輝達揭露持有其約299.9億美元股權、為Musk旗下Terafab計畫主要代工夥伴——漲價與缺貨反映整體晶片需求強勁(正面)，但Intel代工若取得指標客戶則為長期競爭風險，該案時程與良率均未經證實(來源Motley Fool／TradingPedia 9/8)。④輝達-2.01%，市場歸因中國AI晶片業者Mocha Thread向港交所遞交IPO保密申請、擬募資至少10億美元——短期無直接衝擊，中長期若中國自主方案成規模，其代工需求受出口管制限制未必落到台積電，列為新增觀察項(來源GuruFocus／MarketBeat 9/8)。⑤蘋果-1.17%為秋季發表會(美國時間9/9)前觀望賣壓，若確認A20採台積電N2並放量為N2稼動率佐證，惟營收貢獻要到Q4。
+(12)⚠️⚠️第一順位風險為明日(9/10)13:30的8月合併營收，這是9/7至9/8兩日上漲的全部理由。媒體引述法人估8至9月單月營收將較7月的4,675.81億元月減約3至8%(本報依該月減幅推算約當NT$4,300至4,540億；原始報導所載絕對金額本報未能核實，故不引用)。真正的檢核不是月減與否(屬季節性正常)，而是能否支撐Q3美元指引中位$45.2B所需的月均約NT$4,851億——7月已低約3.6%。同日另有美國8月PPI，9/11美國8月CPI，9/15至16 FOMC(決策台北時間9/17凌晨2:00)。
+(13)📅資料口徑與更正聲明：全程TWSE／TAIFEX／Yahoo官方端點取數(TWSE與TAIFEX一律以curl落檔再讀)；ADR收盤另以stockanalysis.com報價頁獨立核對(439.00 +10.09 (2.35%) At close: Sep 8, 2026, 4:00 PM EDT)，與Yahoo一致。技術指標依TWSE官方收盤序列(2026-01-02至2026-09-08共165個交易日)自行計算，並依例先重算9/7各項指標、與9/8日報已發布值完全一致(MA5 2,417／MA10 2,414／MA20 2,403／MA60 2,394／MA120 2,258、RSI 57.92、DIF 12.6499／DEA 9.4178／MACD柱+6.46、K 72.28／D 64.85／J 87.14、布林2,452／2,403／2,354、5日均量22,452)後才採用本日值。⚠️一項更正：前一份日報依CNBC報價頁記ADR除息US$1.114(除息日2026-09-16)，本報以stockanalysis.com股利歷史頁獨立查核得US$0.87489(記錄日9/16、發放日10/8)，兩者相差約27%；除息日兩來源一致、金額兩說並陳並維持【待官方確認】，本日嘗試連線TSMC IR官網(investor.tsmc.com)逐項核對遭HTTP 403阻擋，未能取得一手資料。⚠️另更新模板一處殘留日期：估值解讀段落硬編的「BWIBBU 9/07」已改為9/08。
+⭐綜合研判：評級維持「看多」。9/8是「續強但動能遞減、且出現第一根長上影線」的一天——漲幅自+2.07%收斂至+0.41%、外資買超自16,135張收斂至5,497張、KDJ的J值不升反降，但價量與籌碼三項門檻全數守住，趨勢並未破壞。真正改變格局的是美股：ADR+2.35%超前補漲，把溢價由9.91%重新推回12.08%，台股補漲空間回來了，這是維持看多的主要理由。立場不追高：2,505是今日的關鍵測試價、2,440(9/1前高)為多空分界。今日檢核依優先順序為(1)2,505的第二次測試——收在2,505之上為有效突破、打開至2,510與2,535；再度受阻並收在2,470之下則構成兩日雙重測試失敗，須把9/7至9/8的突破降級；(2)台股能否吃下12.08%溢價缺口的一部分，若不漲代表拒絕跟隨美股；(3)期貨端背離能否解除——未平倉已連4日減少、正價差僅+1，今日若價漲而未平倉續減甚至轉逆價差，須認定上漲缺乏期貨端資金支持。⚠️失敗條件：收在2,440之下；次要防線2,464(布林上軌)與2,460(昨日低點)。⚠️今日為TXO週三結算日，P/C比明日不可跨日比較。</t>
+        </is>
+      </c>
+      <c r="G122" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-10 日報 HTML & Excel 更新
依前一份日報自訂的降級條件，將 9/7–9/8 突破由「趨勢突破」降級為
「情緒推升」，評級自看多下修為中性偏多（收 2,465 低於 2,470、
盤中高 2,490 未能再測 2,505）。

重大更正：補上前一版遺漏的台股 2330 於 2026-09-16 除息 NT$7.00001
（TWSE 官方除權除息預告表），並據此解決 ADR 股利金額的兩來源矛盾
（NT$7.00001 × 5 ÷ 31.42 ≈ US$1.114，判定 CNBC 版正確）。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-09</t>
+          <t>報告更新日期：2026-09-10</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-09</t>
+          <t>最後更新：2026-09-10</t>
         </is>
       </c>
     </row>
@@ -7790,6 +7790,58 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" s="50" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B123" s="50" t="inlineStr">
+        <is>
+          <t>NT$2,465（9/9收）</t>
+        </is>
+      </c>
+      <c r="C123" s="57" t="inlineStr">
+        <is>
+          <t>-0.20%（9/9收）</t>
+        </is>
+      </c>
+      <c r="D123" s="50" t="inlineStr">
+        <is>
+          <t>US$435.36（9/9收）</t>
+        </is>
+      </c>
+      <c r="E123" s="50" t="inlineStr">
+        <is>
+          <t>17,799（9/9收）</t>
+        </is>
+      </c>
+      <c r="F123" s="52" t="inlineStr">
+        <is>
+          <t>報告日2026-09-10(Thu)，台股資料為2026-09-09(Wed)官方收盤；ADR、費半與全部美股個股為9/9美東收盤。⚠️本報產製時間為上午9時，台積電8月合併營收預定今日13:30公布，本報全篇不含8月營收實際數字。
+(1)⚠️⚠️本日最重要的一件事是履行前一份日報自訂的降級承諾：前報白紙黑字訂下「若再度衝高受阻並收在2,470之下，構成兩日雙重測試失敗，屆時須把9/7至9/8的突破降級為情緒行情」。9/9實際結果是收2,465(低於2,470達5點)、盤中最高僅2,490(距2,505尚差15點，連測試都沒測試成功)，條件完整成立，本報依約降級，評級自「看多」下修為「中性偏多」。⭐為何降級而不轉空，三項可驗證的理由：(a)前報同時訂下的失敗條件是「收在2,440之下」，本日收2,465、高出25點，明確未觸發；(b)五條均線全數站上且每一條仍在上彎；(c)MACD柱連3日擴張。降級處理的是「這波上漲的性質」(由趨勢突破改判為情緒推升)，失敗條件處理的是「趨勢是否反轉」，前者已成立、後者尚未。
+(2)台股2330官方收NT$2,465(-5、-0.20%、開2,480／高2,490／低2,460＝9/8當日低點、量17,799張、額NT$440.36億、65,336筆)，終結連4日收紅。⚠️型態核心證據是連2日的上影線與逐日降低的高點：9/8高2,505、收2,470(上影線35點)；9/9高2,490、收2,465(上影線25點)。最高價2,505→2,490與收盤價2,470→2,465皆逐日降低，而兩日最低價同為2,460。判讀：買方連續兩日在盤中把價格推高但都無法守住，且第二日推得比第一日更低，2,490至2,505一帶已可視為短線供給區；惟兩日最低價同為2,460且都守住，下方仍有承接，型態為收斂而非潰散。
+(3)⚠️⚠️籌碼面是本日轉弱最明確的一環：外資由連2日買超反手賣超2,559張(T86官方-2,558,862股)，終結9/7(+16,135)、9/8(+5,497)的連續買超；投信亦由買超1,205張反手賣超204張(-203,593股)；僅自營商小幅買超42張(+41,730股，自行買賣+88,900、避險-47,170)。三大法人分項加總合計賣超2,721張(官方合計欄-2,720,725股)。⭐緩解證據有二：近5日(9/3至9/9)外資合計仍淨買超19,997張(-961、+1,885、+16,135、+5,497、-2,559)；且2,559張的賣超規模在追蹤區間屬中小量(9/2曾單日賣超11,987張)、僅為9/7單日買超的15.9%。判讀：獲利了結而非撤退，但方向的轉變本身已足以支持降級。
+(4)⚠️量能腰斬，這讓「情緒行情」的判斷更站得住腳：17,799張較9/8的28,932張大減38.5%、較5日均量20,397張低12.7%，連2日站穩20,000張的條件於本日中斷。9/7量26,898張、9/8量28,932張、9/9僅17,799張，量能在兩日內腰斬，代表推升這波上漲的買盤在價格接近2,500時迅速退場而非持續進場。⚠️註：5日均量自21,867降至20,397係9/2的25,151張滾出窗口所致，但本日實際成交17,799張較前一版均量基準21,867張亦低18.6%，兩種比法結論一致——本日確實是量縮，非滾動窗口假訊號。
+(5)⭐本日有一項前報預先點名的正面發展如實兌現：收盤2,465已回到布林上軌(2,472)之下，終結連2日收在上軌之上的狀態，前報原話「若今日收回上軌之下，短線過熱即告解除，屬健康換手而非轉弱」成立。⚠️惟通道寬度自4.70%續張至5.14%，已依既定作法檢查滾動窗口：滾出的是8/12的2,415(距新中軌2,410僅5點)、滾入的是9/9的2,465(距中軌55點)，滾入值偏離遠大於滾出值，屬實質的價格分散度上升，非機械效果。
+(6)⚠️技術指標三降一升且升的那一項正在減速：RSI(14)自58.95回落至58.18(連3日上升後首度下滑，仍守50之上)。⚠️⚠️KDJ連續第2日惡化且較前一日更明顯——K自72.55回落至71.44(前一日尚為+0.27微升)、D自67.42續升至68.76，K-D差距自+5.13收斂至+2.68，金叉仍在但兩線快速靠攏；J值自82.81落至76.81(-6.00)、跌破80強勢分界。⭐前報已訂「若K跌破D形成死叉且價格同時收在2,470之下，兩項訊號合流即為突破失敗確認」——本日價格條件已成立、死叉條件尚未成立(K仍高於D達2.68)，兩項中成立一項，這正是降級而不轉空的量化依據。MACD柱自+11.27續張至+12.86(DIF 18.8646／DEA 12.4344)，惟增幅僅+1.59，相較前兩日的+6.45、+4.81收斂約七成，三日呈遞減數列。均線MA5 2,439／MA10 2,426／MA20 2,410／MA60 2,398／MA120 2,267全數站上且仍上彎，完整多頭排列自8/27起維持10個交易日；⚠️惟與MA5的距離自47點收斂至26點，前一日「間距明顯拉開」的描述在本日反轉，性質為價格向均線靠攏而非均線下彎。
+(7)⚠️期貨端未解除且惡化：CDF 202609日盤收2,471(持平、0.00%、成交6,110口、盤中高2,492／低2,465)，⭐在現貨下跌-0.20%下期貨持平，正價差自+1擴大至+6，是期貨端本日唯一正面訊號。⚠️⚠️未平倉自20,709口減至19,294口(-1,415口)，為連續第5個交易日減少(9/3 23,157、9/4 22,769、9/7 21,709、9/8 20,709、9/9 19,294)，自9/2的23,592口累計-4,298口(-18.2%)，且本日減幅為這5日最大。⭐判讀在本日有實質更新：先前是「價漲而未平倉減少」(可解讀為空單回補)，本日轉為「價跌而未平倉續減且減幅擴大」，兩種情境合看，較合理的解讀是多空雙方同步減碼離場、整個台積電期貨市場參與度在萎縮。台指期TX 202609日盤收47,187(+232、+0.49%)。⚠️⚠️TXO的P/C未平倉比自1.05降至0.96(賣權51,246口／買權53,194口、官方比率欄96.34%)，但9/9為週三結算日、未平倉雙邊各減約四成，此變化是基期重置而非部位方向改變，本報依約不做變化方向解讀；且9/11(週五)又是結算日，本週實際上沒有任何一組可供跨日比較的P/C讀數，本欄定位為「本週無有效訊號」。⭐今晨夜盤(TAIFEX標記日期2026/09/10之「盤後」列，涵蓋9/9 15:00至今晨05:00)兩者方向相反：CDF 202609收2,476(+5、+0.20%、成交1,247口)小漲，TX 202609收46,984(-194、-0.41%、成交31,951口)下跌。
+(8)⭐評價與匯率：TWSE官方BWIBBU 9/9顯示P/E 28.57x、P/B 9.94x、殖利率0.89%(9/8為28.63x／9.96x／0.89%)，財報基準維持115/2未變動，故下降100%來自股價(2,470→2,465、-0.20%)。28.57x約落5年區間第89百分位、P/B約第93百分位(本報估算)。市值約NT$63.9兆。ADR端P/E約31.8x、P/B約11.1x，係依官方值×(1+溢價11.13%)換算。⚠️匯率：新台幣9/9 16:00台北時點報31.457(採31.46)，較9/8的31.53升值0.22%。前報預告「今日09:15盤中報31.465、續升0.21%，若延續至收盤則須再次升級」——本報依約確認升值確實延續到收盤，故將匯率自「非因素」重新升級為「待觀察」；惟0.22%對毛利率影響約-9bps仍屬雜訊，升級理由是方向的連續性(9/7升0.44%、9/8貶0.03%、9/9升0.22%，三日淨升0.63%)而非單日幅度。
+(9)⚠️⚠️ADR溢價完整拆解，收斂的方式必須講清楚否則會被誤讀為利多：理論平價＝5×2,465÷31.46＝391.77(採捨入後匯率)，對市價435.36之溢價+11.13%，較9/8的12.08%收斂0.95個百分點。溢價收斂有兩種途徑——台股上漲(健康)或ADR下跌(不健康)，本日是後者。拆解：台股下跌-0.20%單獨會使溢價自12.08%擴大至12.31%(+0.23pp)；新台幣升值0.22%使平價升高、把溢價壓回12.06%(-0.25pp)；ADR下跌-0.83%則使溢價收斂至11.13%(-0.93pp)——淨效果-0.95pp之中ADR端貢獻-0.93pp，幾乎是全部。缺口是被美股「拉下來」而非被台股「追上去」，前報第二順位檢核「台股能否吃下溢價缺口」未實現，且正是前報所警示的「台股拒絕跟隨美股，會是比回吐更負面的訊號」。⭐相對強弱本日轉向：台積電-0.20%落後加權指數+0.16%(收47,183.36、+77.58)達0.36個百分點，終結連2日領先(9/7 +0.40pp、9/8 +0.88pp)，為9/3以來首度落後，且是在大盤收紅的一天落後。期間比較：近5日+3.35%領先大盤+2.21%(基準均為9/2)，近1月+4.01%落後大盤+6.69%(差距較前一日的2.29pp再擴大)，YTD+55.5%落後大盤+60.8%與費半+61.9%。
+(10)⭐⭐本日重大更正與新增(前一版遺漏)：依TWSE官方「除權除息預告表」(查詢區間2026-09-01至09-30，2330為當月79筆之一，申報基準115年第2季、每股淨值248.05、每股盈餘49.33)，台股2330將於2026-09-16(下週三、距今4個交易日)除息，每股現金股利NT$7.00001；以9/9收盤2,465計，除息參考價約2,458。本報前一版僅記載12/10那一批股利、遺漏了這一批，本日補正。⚠️讀者在比較9/16之後的股價時務必還原此約7點(約0.28%)的缺口，勿把除息誤讀為下跌；P/E與P/B屆時同步機械性下降，亦不代表評價重估。⭐⭐這同時解決了本報追蹤多日的ADR股利金額矛盾：ADR以5:1表彰，NT$7.00001×5÷匯率約31.42≈US$1.114，與CNBC報價頁所載之US$1.114/ADR完全吻合，而stockanalysis.com所載之US$0.87489無法由任何合理匯率還原——本報據此判定CNBC版本為正確、stockanalysis.com版本應為誤植，前一版的「兩說並陳」至此收斂為單一答案。⚠️惟ADR實際入帳美元金額取決於存託機構結匯當日匯率，且本報今日再次連線TSMC IR官網(investor.tsmc.com)仍回HTTP 403(Cloudflare阻擋)、未能取得一手公告，故ADR金額維持【以台股股利換算，待官方確認】。12/10為8/11董事會核准之Q2 2026股利(NT$7.0/股、基準日12/16)除息日，與9/16屬不同批次。
+(11)⭐⭐美股端本日最實質的一則且是事實而非傳聞：蘋果於美國時間9/9在Apple Park舉行「Surprise and Shine」秋季發表會，正式發表iPhone 18 Pro／Pro Max(1,199／1,299美元起)，搭載採用台積電2nm(N2)製程打造的A20 Pro晶片，官方稱效能提升最高15%或省電最高30%；同場發表首款摺疊機iPhone Duo(1,999美元、10/16開放預購)，iOS 27於9/14上市(來源CNBC／TechRadar／MacRumors現場報導)。⭐前報所訂檢核點「若確認A20採台積電2nm並放量，將是N2稼動率90至95%的直接佐證」在本日獲得確認，台積電握有蘋果旗艦晶片2nm首發供應地位。⚠️惟蘋果自身股價當日僅-0.28%(盤中一度-1%)，屬典型「賣新聞」反應——市場早已預期此事，它是中期基本面的拼圖而非當日價格催化劑，對營收的實質貢獻要到Q4才顯現。
+(12)⚠️美股9/9為連續第三日下跌(標普500收7,636.36、-0.48%；那斯達克26,253.34、-0.64%；VIX自15.72升至16.46)，媒體歸因為三項：美伊油輪議題升溫使Brent原油突破每桶101美元、財政部長Bessent宣布下次公債回購規模擬增至約60億美元使10年期公債殖利率升至4.83%(2023年10月以來新高)、市場對聯準會利率路徑重新定價。⚠️須明確標註未能證實：所查到的報導未將當日跌幅直接連結到9/10 PPI、9/11 CPI或9/15至16 FOMC，該三項僅為時序相近；另一則報導稱「交易員預期本月升息25bps機率達60%」，與一般2026年降息循環認知不符，本報未能交叉驗證，如實轉述但不採信。⭐半導體逆勢：費半收11,931.32(+0.37%、+43.45點)連4日收紅、續創本波新高。⚠️⚠️惟指數收紅但內部結構完全翻轉：9/8領漲的設備四雄本日全數收黑(科磊-3.21%為全部追蹤標的最大跌幅、艾司摩爾-2.00%、科林研發-1.43%、應用材料-0.83%)，媒體歸因為「投資人開始質疑支撐該類股今年漲幅的AI資本支出循環可持續性」(來源Yahoo Finance 9/9；⚠️該報導所載個股跌幅與9/9實際收盤不完全吻合，本報僅採其類股層級解釋，個股層面標為未查到明確歸因)；撐起指數的換成記憶體與運算——美光+2.75%($1,027.77，收復9/8跌幅並創本波新高)、超微+3.04%($521.10，連2日大漲、兩日累計+9.1%)、英特爾+1.69%($106.24)、高通+1.33%($176.40)、Amkor+1.24%($51.35)、Arm+1.03%($264.23)。台積電ADR當日-0.83%弱於費半1.20個百分點，領漲主線(記憶體)並非台積電核心業務。
+(13)⭐記憶體與HBM是本日全球半導體最明確的主線：美光+2.75%、SK海力士+3.51%(1,856,000韓元、亞洲追蹤標的最大漲幅、創本波新高)，歸因為分析師對HBM的結構性看法轉趨樂觀而非單一事件——New Street分析師Pierre Ferragu大幅調升美光目標價，主張HBM因技術複雜度高、耗用晶圓多且涉及先進封裝應享有較標準DRAM更高的評價；Susquehanna分析師Mehdi Hosseini反駁HBM跌價疑慮，指HBM3e轉HBM4可能使價格再漲逾50%(來源TheStreet／TipRanks 9/9)。⭐對台積電的傳導：HBM本身非台積電製造，但HBM4的邏輯基底晶片(base die)由台積電代工，且HBM與CoWoS為互補產能，對先進封裝定價環境有利；⚠️惟屬間接利多。⚠️美光財報公布日期本報未能查到明確來源，標為未能證實。⭐封測端兩地同步收紅：日月光+3.56%(640.00元、創本波新高、量自12,821張放大至21,514張，為量價齊揚)、Amkor+1.24%，這是前一交易日(9/8兩者方向相反)所沒有的確認。⚠️台股端其餘：華邦電-2.66%(183.00元、終結連3紅、量縮36.6%)、聯發科-1.80%(4,625元、連2日下跌、量縮至4,731張)；三星電子收平盤269,500韓元，與SK海力士的+3.51%形成明顯落差，本日全球資金主線清楚指向記憶體／HBM。⚠️輝達-0.91%($223.67)連2日下跌，本報派出的查證確認未查到獨立的公司別觸發新聞(搜尋到的相關報導經核對時間點均非9/9當日事件，已排除)，較合理判讀為隨大盤與設備類股連動；惟已連續兩個交易日弱於費半。⚠️博通-1.13%($364.38)未能守住9/8收復財報跌幅的成果，重新低於9/2的$367.24，本報9/8所記「懲罰屬情緒性而非結構性」的緩解證據在本日打了折扣。
+(14)📅資料口徑聲明：全程TWSE／TAIFEX／Yahoo官方端點取數(TWSE與TAIFEX一律以curl落檔再讀)。⚠️美股個股本日一律採Yahoo chart的meta.regularMarketPrice(時間戳2026-09-09 20:00 UTC＝美東16:00)，因日線K棒的9/9 close欄位為null；費半有完整K棒讀數且與其meta值一致，可交叉印證此取法無誤。匯率採Yahoo小時線之台北16:00讀數(TWD=X的9/9日線K棒收盤同樣為null，故小時線取法必須維持)。技術指標依TWSE官方收盤序列(2026-01-02至2026-09-09共166個交易日)自行計算，並依例先重算9/8各項指標、與9/9日報已發布值完全一致(MA5 2,423／MA10 2,421／MA20 2,407／MA60 2,397／MA120 2,263、RSI 58.95、DIF 16.4633／DEA 10.8269／MACD柱+11.27、K 72.55／D 67.42／J 82.81、布林2,464／2,407／2,350、5日均量21,867)後才採用本日值。⚠️另更新模板兩處殘留：估值解讀段落硬編的「BWIBBU 9/08」已改為9/09；9/11行事曆條目所引「目前P/E 28.63x(9/8)」已改為28.57x(9/9)。
+⭐綜合研判：評級自「看多」下修為「中性偏多」。9/9是「降級日」——不是因為跌了5點，而是因為前一份日報自訂的降級條件被完整觸發(收在2,470之下、且未能再度測試2,505)，本報依約履行，把9/7至9/8的上漲由「趨勢突破」改判為「情緒推升」。支持不轉空的三項證據明確且可驗證：失敗線2,440未破、五條均線全數站上且仍上彎、MACD柱連3日擴張。但四項轉弱訊號同樣明確：外資反手賣超、量能腰斬、KDJ的K-D收斂至2.68逼近死叉、連2日高點逐日降低。⚠️⚠️今日所有判斷都必須讓位給一個時點——13:30的8月營收，本報產製時(09:00)尚未公布。今晨台股已低開20點至2,445、09:10報2,440(-25、-1.01%、成交3,097張；加權指數46,807.08、-376.28、-0.80%)，正好落在前報所訂的失敗線上，市場帶著防禦姿態進入數字公布，這使數字的方向性影響會被放大。⚠️⚠️市場預期本身分歧為方向相反的兩說：一說法人估可突破NT$4,800億創單月新高，另一說估較7月的4,675.81億月減3至8%(約當NT$4,300至4,540億)，兩說無法同時成立、本報無法判定何者為共識——共識分歧意味無論數字落在哪裡都會有一半的參與者被意外到，波動度風險高於單純的「優於／不如預期」。真正的檢核基準是Q3美元指引中位$45.2B所需的月均約NT$4,851億，7月已低約3.6%。今日檢核依優先順序：(1)13:30的8月營收；(2)2,440這道失敗線今日能否守住收盤——若收在2,440之下，9/7至9/8的突破與四項技術指標的翻多將同時失效，須自「中性偏多」進一步下修；若營收優於預期而收復2,465之上，降級可望撤回；(3)KDJ的K-D差距僅剩2.68，今日若K再跌逾此幅度而D續升，死叉即完成，與已成立的價格條件合流。次要支撐依序為2,439(5MA)、2,410(20MA＝布林中軌)、2,398(60MA季線)；反壓為2,472(布林上軌)、2,490、2,505。⚠️同日美國公布8月PPI；9/11為美國8月CPI且為TXO結算日；9/16台股除息NT$7.00001。</t>
+        </is>
+      </c>
+      <c r="G123" s="50" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
daily: 2026-09-11 日報 HTML & Excel 更新
資料日 2026-09-10（Thu）台股收盤 + 9/10 美東收盤。

主要內容：
- 8 月合併營收 NT$5,148.1 億（+10.1% MoM、+53.3% YoY），單月首破
  NT$5,000 億、連 4 個月創歷史新高；1-8 月累計 NT$3 兆 3,868.7 億
  （+39.3% YoY）。直接讀取 pr.tsmc.com 官方原文確認。
- 台股收 2,450（-15、-0.61%）；KDJ 死叉成立（K 66.86 < D 68.13）且
  收盤低於 2,470，前報所訂「突破失敗確認」兩項條件合流，依約將立場
  自「中性偏多」下修為「中性」。
- ADR 收 428.03（-1.68%）、費半 -2.66%（終結連 4 紅、追蹤區間最大
  單日跌幅）。營收於台股收盤後公布，美股 9/10 全場已知悉該數字。

本次修正的既有錯誤：
- 52 週低點窗口過期：台股 1,065 → 1,235.00、ADR 223.70 → 257.98。
- 「ADR 同批於 9/16 除息」降級為待確認（stockanalysis.com 顯示
  ADR 除息日為 12/10），不再斷言兩地同日。
- Excel「2026展望」資本支出仍為 4 月指引 USD 52-56B，補正為
  USD 60-64B（9/2 SEMICON 上修，HTML 已於 9/2 更正）。

口徑澄清（供後續維護）：
- KDJ 的 9 日 RSV 須以最高／最低價序列計算，不可用收盤價序列；
  以高低價序列重算 9/8、9/9 兩日均完全複現已發布值。

驗證：fresh-context subagent 逐條驗收 20 項條件全數通過，並據其
回報補上 9/10 加權指數絕對值（46,940.49、-242.87）之缺漏。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSMC_股市分析報告.xlsx
+++ b/TSMC_股市分析報告.xlsx
@@ -895,7 +895,7 @@
     <row r="3" ht="30" customHeight="1" s="36">
       <c r="A3" s="41" t="inlineStr">
         <is>
-          <t>報告更新日期：2026-09-10</t>
+          <t>報告更新日期：2026-09-11</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>USD 52–56 B</t>
+          <t>USD 60-64 B</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Source: TSMC FY2025 Results</t>
+          <t>Source: 2026-09-02 SEMICON Taiwan 上修（4月法說會原指引 USD 52-56B）；HTML 日報已於 9/2 更正，本表 2026-09-11 補正</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="36" min="1" max="1"/>
@@ -3355,7 +3355,7 @@
     <row r="2" ht="22.05" customHeight="1" s="36">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>最後更新：2026-09-10</t>
+          <t>最後更新：2026-09-11</t>
         </is>
       </c>
     </row>
@@ -7842,6 +7842,62 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" s="53" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B124" s="53" t="inlineStr">
+        <is>
+          <t>NT$2,450（9/10收）</t>
+        </is>
+      </c>
+      <c r="C124" s="56" t="inlineStr">
+        <is>
+          <t>-0.61%（9/10收）</t>
+        </is>
+      </c>
+      <c r="D124" s="53" t="inlineStr">
+        <is>
+          <t>US$428.03（9/10收）</t>
+        </is>
+      </c>
+      <c r="E124" s="53" t="inlineStr">
+        <is>
+          <t>19,836（9/10收）</t>
+        </is>
+      </c>
+      <c r="F124" s="55" t="inlineStr">
+        <is>
+          <t>報告日2026-09-11(Fri)，台股資料為2026-09-10(Thu)官方收盤；ADR、費半與全部美股個股為9/10美東收盤。
+(1)⭐⭐本日最重要的基本面事實：台積電已於9/10公布8月合併營收NT$5,148.1億元(官方英文稿原文NT$514.81 billion)，月增10.1%、年增53.3%；1至8月累計NT$3兆3,868.7億元、年增39.3%(來源：台積電官網新聞稿pr.tsmc.com，發布日2026/09/10，本報直接讀取官方原文確認，非轉述媒體)。⭐⭐三項里程碑同時成立：單月營收首度突破NT$5,000億大關；連續第4個月改寫單月歷史新高(6月4,426.80億→7月4,675.81億→8月5,148.1億)；年增率自7月的+44.69%再加速至+53.3%，為本報追蹤期間最高。⭐算術自我檢核三道：4,675.81×1.101＝5,148.1(與官方MoM相符)；28,721億(1至7月)+5,148.1＝33,869.1億，與官方累計33,868.7億僅差0.4億(7月數四捨五入所致)；由YoY反推2025年8月約3,358億，量級合理。⭐對Q3指引的意義：美元指引中位$45.2B換算單季約需NT$14,553億、月均約NT$4,851億；7月4,675.81億+8月5,148.1億＝9,823.91億，已達指引中位的67.5%而時間僅過三分之二(66.7%)，9月只需約NT$4,729億(自8月月減8.1%)即可達成中位，門檻寬鬆。前一份日報列為第一順位風險的「營收兩種相反預期」由樂觀一方大勝、超出其上緣達7.3%(5,148.1 vs 4,800)，月減一說完全落空。
+(2)⚠️⚠️但技術面同日觸發前報所訂的「突破失敗確認」，本報依約下修評級：前報白紙黑字訂下「若今日K值跌破D值形成死叉，且價格同時收在2,470之下，兩項訊號合流即應視為9/7至9/8突破的失敗確認…屆時須進一步下修至中性」。9/10實際結果是兩項條件都成立：K值自71.44重挫4.58點至66.86、D值自68.76微降0.63點至68.13，K已低於D達1.27點，死叉正式成立；收盤2,450亦低於2,470達20點。本報依約將立場自「中性偏多」下修為「中性」。⚠️惟須據實指出形成方式與前報設想略有出入，不含糊帶過：前報設想「K再跌2.68點以上而D續升」，實際K跌4.58點(超過門檻)但D並未續升、反而小幅下滑0.63點。兩種路徑結論相同(死叉成立)，但D未續升代表中期均值尚未確立向下，死叉強度略弱於前報設想的情境——這正是下修至「中性」而非直接轉「偏空」的量化理由。
+(3)台股2330官方收NT$2,450(-15、-0.61%、開2,445／高2,455／低2,435、量19,836張、額NT$485.24億、85,691筆)，連2日收黑。⭐本日型態與前兩日相反且為唯一偏多證據：9/10是「探底回升」——盤中最低殺到2,435(跌破前報所訂失敗線2,440，亦跌破9/8至9/9共同低點2,460達25點)，但收盤拉回至2,450，留15點下影線、僅5點上影線，與9/8(上影線35點)、9/9(上影線25點)的「衝高受阻」方向相反，代表2,435至2,440一帶出現實質承接。⚠️兩項保留須並陳：前報失敗條件寫的是「收在2,440之下」屬收盤價條件，故字面未觸發，但盤中確實失守過，本報不隱瞞；且最高價已連續第3個交易日降低(2,505→2,490→2,455)，上方供給區壓制仍在，下影線只證明有買盤、不證明買盤能推動價格。
+(4)⚠️⚠️均線結構出現本波上漲以來第一次破口，但量級極小，兩件事須同時講清楚：收盤2,450跌破5日均線2,451，終結自8/27起連續10個交易日「五條均線全數站上」的完整多頭排列；⭐但跌破幅度僅1點(0.04%)，屬幾乎貼線的邊際穿越，與一般所稱「跌破均線支撐」意義完全不同。其餘四條均線仍明確站上：MA10(2,430)高出20點、MA20(2,410)高出40點、MA60(2,399)高出51點、MA120(2,272)高出178點。⭐更重要的是均線方向全數未變：MA5自2,439續升至2,451、MA10自2,426升至2,430、MA20持平2,410、MA60自2,398升至2,399、MA120自2,267升至2,272，五條均線無一下彎，且MA5上升速度(+12點)仍快於價格——這是「均線追上價格」而非「價格摔破均線」，兩者技術意義相反。多頭排列本身完整維持。
+(5)⚠️籌碼面連2日賣超惟規模收斂：外資9/10賣超1,944張(T86官方-1,944,284股)，較9/9的-2,559張縮小24.0%；投信賣超擴大至448張(-447,800股，前日-204張)；自營商由買轉賣97張(-97,293股，自行買賣-205,300股→-205張、避險+108,007股→+108張)。三大法人分項加總合計賣超2,489張，與官方合計欄位(-2,489,377股)換算值完全一致。⭐緩解證據：近5日(9/4至9/10)外資合計仍淨買超19,014張(+1,885、+16,135、+5,497、-2,559、-1,944)，本波9/7單日買超16,135張的主力部位尚未鬆動，連2日合計賣超4,503張僅回吐其27.9%。判讀：屬獲利了結的延續而非撤退，但連續2日方向一致已足以支持「本波買盤動能結束」的判斷。
+(6)⚠️量能回升但仍未站回均量：19,836張較9/9的17,799張回升11.4%，惟仍低於5日均量21,513張達7.8%，連2日未站回均量之上。5日均量自20,397升至21,513係9/3的14,252張滾出窗口、9/10補進19,836張所致。
+(7)⚠️技術指標：RSI(14)自58.18回落2.35點至55.83，連2日下滑且跌幅較前一日的-0.77點擴大約兩倍，仍守50之上；本波日變動依序為+2.47、+5.57、+1.03、-0.77、-2.35，「加速、減速、翻負、負向擴大」四階段已全部走完，動能轉折在本欄屬確認而非預警。⭐MACD為四項中唯一維持正值：柱狀體自+12.86收斂至+11.04(DIF 19.3343／DEA 13.8144)，終結連3日擴張——前報原話「價格只要再橫盤或小跌一至兩日，柱狀體即會轉為收斂，屆時應解讀為漲勢換檔的確認，而非新的賣出訊號」在本日如實兌現，本報維持前報所訂的解讀分寸。四日柱狀變化為+6.45、+4.81、+1.59、-1.82，遞減至翻負；惟DIF自18.86續升至19.33，收斂來自DEA(10.83→12.43→13.81)追趕而非DIF轉降，屬相對溫和的收斂型態。⚠️KDJ死叉成立(K 66.86／D 68.13／J 64.32)，K-D差距+5.13→+2.68→-1.27三日翻負；J自76.81落至64.32(-12.49，三日中最大)，距50尚有14.32點。⭐布林：收盤2,450位於上軌(2,474)與中軌(2,410)之間中上緣，連2日收在上軌之下，短線過熱持續解除；⚠️通道寬度自5.14%再張至5.27%，已依既定作法檢查滾動窗口——滾出8/13的2,400(距新中軌2,410僅10點)、滾入9/10的2,450(距中軌40點)，滾入偏離大於滾出，屬實質價格分散度上升非機械效果。
+(8)⚠️⚠️期貨端兩項同向轉弱，前報所訂「背離能否解除」連續第3日為「未解除」：(a)基差由正轉負——CDF 202609日盤收2,448(-23、-0.93%、成交7,241口、盤中高2,467／低2,443、結算價2,447)，跌幅大於現貨的-0.61%，基差自+6點翻轉為-2點逆價差。⭐意義在方向而非幅度：2點逆價差量級微不足道，但它代表期貨投資人對隔日看法自「略優於現貨」轉為「略差於現貨」，且恰發生在8月營收創新高公布的當日盤後——期貨端並未因營收利多而轉趨樂觀。(b)未平倉自19,294口減至18,850口(-444口)，連續第6個交易日減少(9/3 23,157、9/4 22,769、9/7 21,709、9/8 20,709、9/9 19,294、9/10 18,850)，自9/2的23,592口累計-4,742口(-20.1%)；⭐惟本日減幅444口為6日中最小(前5日分別為435、388、1,060、1,000、1,415)，減碼速度明顯放緩，為本欄唯一緩解證據。台指期TX 202609日盤收46,870(-308、-0.65%、成交48,692口、未平倉94,990口)。⭐三大法人台指期部位：外資淨空單83,918口(多8,264／空92,182)、投信淨多單74,483口、自營淨多單1,379口；⚠️此為大盤層級避險部位，不可直接讀為對台積電個股的看法。
+(9)⚠️TXO的P/C未平倉比0.83(賣權69,363口／買權83,906口、官方比率欄82.67%)。⚠️⚠️本週情況比平常更極端：9/9(週三)與9/11(週五)都是結算日，9/10(週四)夾在兩個結算日中間屬重建日——本週自始至終沒有任何一組具跨日可比性的P/C讀數，下一次有效比較最快要到下週一、二之間，故0.96→0.83不可讀為部位方向改變。⭐可解讀的絕對水位確實值得記錄：0.83是本報追蹤區間內買權未平倉領先賣權幅度最大的一次(買權多出14,543口、約21.0%)，結算後新建立的部位明顯偏向買權，與同日現貨下跌、美股重挫方向相反，是本日少數偏多的籌碼線索。⚠️惟三項限制份量更大：重建期基數變動劇烈(雙邊自9/9的104,440口一日回升至153,269口)、TXO為台指選擇權非個股選擇權、今日又是結算日將再次重置。本欄仍定位為「本週無有效訊號」。
+(10)⚠️⚠️美股端是本日壓力的真正來源，性質為族群與總經雙重的評價修正而非台積電個股利空：9/10美股連續第4日收黑(標普500 -0.58%收7,591.70、那斯達克-0.65%收26,081.72、道瓊-0.60%收52,064.10、VIX自16.46升至17.84)。⚠️⚠️費半-2.66%收11,614.17，終結連4日收紅，為本報追蹤區間內最大單日跌幅，跌幅遠大於大盤；此與9/9「大盤跌而費半逆勢收紅」完全相反，半導體9/9展現的相對強度一日之內全數反轉。⚠️族群內近乎全面下跌，重災區在設備與記憶體：科林研發-5.65%($298.01、跌破$300關卡)、英特爾-5.57%($100.32、幾乎跌破$100)、美光-4.90%($977.41、跌破$1,000關卡)、Arm-3.80%、Amkor-3.54%($49.53、跌破$50)、超微-3.36%($503.60)、應用材料-3.17%、科磊-3.13%、艾司摩爾-2.43%、輝達-2.37%($218.36、連3日下跌)；僅高通+0.27%收紅。⭐媒體歸因為總經因素合流：美國8月PPI年增5.4%(高於預期、前值4.8%)、布蘭特原油衝上約101美元、10年期公債殖利率升至4.94%(本報以Yahoo ^TNX核對確認，前一交易日4.84%)。⚠️油價約101美元一項僅取得單一來源描述、未附獨立可查證連結，標為待證實。
+(11)⭐⭐本日判讀的關鍵在時序而非數字，這是全篇最重要的一段：8月營收於台股收盤後公布(台北9/10下午)，換算美東時間為9/10凌晨，亦即美股9/10的整個交易時段(美東09:30至16:00)都是在已知悉「單月營收創歷史新高、首破NT$5,000億、年增53.3%」的前提下進行的——而ADR仍收$428.03(-7.33、-1.68%)。⭐這排除了「市場還沒看到數字」的解釋，只剩一種讀法：在總經壓力與5年第88百分位的評價水位下，市場對好消息的邊際反應已鈍化。⚠️惟須並陳族群背景以免過度歸因於個股：ADR跌幅小於費半0.98個百分點，屬族群回檔中的相對抗跌而非個股被單獨懲罰。ADR收盤已以stockanalysis.com獨立核對(428.03、-7.33、-1.68%、At close: Sep 10, 2026, 4:00 PM EDT、前收435.36、當日區間424.05至432.53、成交8,381,062股)，與Yahoo meta完全一致；算術自我檢核435.36-7.33＝428.03亦相符。
+(12)⭐評價：TWSE官方BWIBBU 9/10顯示P/E 28.40x、P/B 9.88x、殖利率0.90%(9/9為28.57x／9.94x／0.89%)，財報基準維持115/2未變動，故下降100%來自股價回檔(2,465→2,450、-0.61%)；算術自我檢核28.57×(1-0.0061)＝28.40完全相符。⚠️⚠️須特別說明一件易被誤讀的事：台積電8月營收雖創歷史新高，但官方P/E的分母不會因此改變——BWIBBU採115/2(Q2 2026)財報基準，月營收要到Q3財報認列後才反映，故今日的28.40x仍是舊獲利基準，營收利多尚未計入評價分母端；若Q3獲利如營收動能所示同步成長，下次財報基準切換時P/E會出現機械性下降，屆時同樣不應讀為評價重估(同8/14自115Q1換至115Q2的情形)。28.40x約落5年區間第88百分位、10年約第89百分位，P/B 9.88x約第92百分位(本報估算，非官方)。市值約NT$63.5兆。ADR端P/E約31.3x、P/B約10.9x，係依官方值×(1+溢價10.24%)換算。
+(13)⚠️匯率轉貶：新台幣9/10 16:00台北時點報31.547(採31.55)，較9/9的31.46貶值0.29%，方向與前三日升值趨勢相反，終結9/7至9/9的三日淨升0.63%。⭐前報預告「今日(9/10)09:00台北報31.454、幾乎持平，明日日報回頭確認」——本報依約確認：盤中持平並未延續，匯率自09:00的31.454一路走貶至16:00的31.547，單日貶幅0.30%，午後貶勢明顯。⭐對毛利率影響方向由不利轉為有利：0.29%貶值約+11bps，仍屬雜訊等級，但方向轉變值得記錄，且小幅改善8月營收的美元換算值與Q3美元指引達成率。本報依既定作法將匯率自「待觀察」調回「非因素」(四日淨升僅0.34%)。⚠️TWD=X的9/10日線K棒同樣缺漏，故小時線取法必須維持。
+(14)⚠️⚠️ADR溢價連2日收斂且結構較昨日更極端：理論平價＝5×2,450÷31.55＝388.27(採捨入後匯率)，對市價428.03之溢價+10.24%，較9/9的11.13%再收斂0.89個百分點。完整拆解：台股下跌-0.61%單獨會使溢價自11.13%擴大至11.81%(+0.68pp)；新台幣貶值0.29%使平價下降、再推高至12.13%(+0.32pp)；⚠️ADR下跌-1.68%則一舉壓回10.24%(-1.89pp)——淨效果-0.89pp之中，台股與匯率合計貢獻+1.00pp的擴大壓力，全數由ADR端的-1.89pp抵銷並超出。⭐連續兩日的溢價收斂都不是因為台股追上來，而是美股把ADR拉下來，且本日力道較昨日更強；本報已連2日不把溢價列為多方理由。⭐相對強弱：台積電-0.61%落後加權指數-0.51%(收46,940.49、-242.87)達0.10個百分點，連2日落後；⭐惟美股端相反——ADR -1.68%明顯抗跌於費半的-2.66%(領先0.98個百分點)，這是少見的「台股端落後、美股端領先」組合，且發生在營收創新高公布之後，顯示營收利多在美股端確實產生相對支撐，只是不足以抵銷族群整體跌勢。期間比較：近5日+2.51%小幅領先大盤+2.36%(基準均為9/3)；近1月+2.94%落後大盤+4.48%達1.54個百分點(差距較前一日的2.68pp收斂，惟成因主要為基準日自8/7前移至8/10的機械效果，非動能改善)；YTD+54.6%落後大盤+59.9%，落後費半+57.6%達3.0pp(差距較前一日的6.4pp大幅收斂，成因為費半單日重挫)。
+(15)⭐族群內兩項與大勢相反、值得記錄的例外：(a)⭐⭐蘋果9/10逆勢大漲+3.56%收$326.57，為全部追蹤標的中當日唯一大漲，且發生在全族群重挫日；一舉收復9/9發表會當日的「賣新聞」跌幅(-0.28%)並突破9/4的$319.97創本波新高。⚠️本報必須誠實標註：本次查證未能取得9/10當日的明確個股觸發新聞(如預購數據或分析師升評)，故不對漲因下定論，僅記錄價格事實。⭐對台積電的意義間接但正向：iPhone 18 Pro／Pro Max搭載採台積電2nm(N2)的A20 Pro，蘋果股價在發表會後轉強代表市場對該產品週期信心回升，而該週期正是N2稼動率(估90至95%)的主要支撐之一。(b)⭐台股端日月光+1.56%收650.00元(連2日收紅、再創本波新高)、聯發科+2.05%收4,720元(終結連2日下跌)；在台積電下跌的同一天封測與IC設計雙雙收紅，此型態已連續第2個交易日出現(9/9日月光亦逆勢+3.56%)，顯示台股半導體資金並未離開族群而是自代工龍頭轉向封測與IC設計，台積電已連2日為族群內相對弱勢股。⚠️惟其美股同業Amkor同日-3.54%，兩地封測方向相反，故9/9曾成立的「先進封裝雙市場確認」在本日不再成立。其餘台股：華邦電-1.91%(179.50元、連2日下跌)。韓股9/10小跌：SK海力士-0.16%(1,853,000韓元)、三星電子-0.19%(269,000韓元)，因韓股收盤時美股尚未開盤故未反映當晚重挫；⚠️已標明時點的盤中補充：9/11上午09:55 KST SK海力士報1,785,000韓元(-3.67%)、三星報260,000韓元(-3.35%)，為盤中即時數據非收盤值，韓股今晨正在補跌。
+(16)⭐產業消息(單一來源、未經交叉確認)：媒體報導台積電CoWoS 5.5倍光罩尺寸先進封裝已進入量產，多項AI客戶產品良率穩定在98%以上、部分達99%；並規劃2029年推出14倍光罩版本、可整合達20層HBM(來源：經濟日報)。⚠️本報未能以台積電官方公告或第二家獨立媒體交叉確認，故列為參考性資訊而非已確立事實。
+(17)⭐⭐除息事項與一處必要的降級更正：依TWSE官方「除權除息預告表」(TWT48U，本日以查詢區間2026-09-01至10-31重新確認，2330在該區間內僅此一筆)，台股2330將於2026-09-16(下週三、距今3個交易日)除息，每股現金股利NT$7.00001，日期與金額均未變動；同表載最近一次申報每股淨值248.05、每股盈餘49.33，與BWIBBU的P/B 9.88x可互相驗算(2,450÷248.05＝9.877)。⚠️除息將使股價機械性扣除約7點(約-0.29%)，P/E與P/B同步機械性下降，屆時不可讀為下跌或評價重估。⚠️⚠️本日必須修正前一版的一處過度推論：前一版寫「ADR同批於9/16除息」，但本報今日查核stockanalysis.com的TSM報價頁，其Ex-Dividend Date顯示為2026-12-10而非9/16——本報無法以手上來源確認ADR這一批的除息日，故將該敘述降級為【ADR除息日待確認】，不再斷言與台股同日。⭐金額換算部分維持前一版結論不變且仍成立：NT$7.00001×5÷匯率約31.4≈US$1.114，與CNBC報價頁一致，而stockanalysis.com的US$0.87489無法由任何合理匯率還原。⚠️台積電IR官網(investor.tsmc.com)本日再次嘗試連線仍為HTTP 403(Cloudflare阻擋)，未能取得一手公告。12/10為8/11董事會核准之Q2 2026股利(NT$7.0/股)除息日，與9/16屬不同批次。
+(18)📅資料口徑聲明：全程TWSE／TAIFEX／Yahoo官方端點取數(TWSE與TAIFEX一律以curl落檔再讀)。⚠️美股個股本日一律採Yahoo chart的meta.regularMarketPrice(時間戳2026-09-10 20:00 UTC＝美東16:00)，因日線K棒的9/10 close欄位為null；⭐費半有完整日K讀數11,614.17且與其meta值11,614.167一致，可交叉印證此取法無誤。匯率採Yahoo小時線之台北16:00讀數。技術指標依TWSE官方收盤序列(2026-01-02至2026-09-10共167個交易日)自行計算，並依例先重算9/9各項指標、與9/10日報已發布值完全一致(MA5 2,439／MA10 2,426／MA20 2,410／MA60 2,398／MA120 2,267、RSI 58.18、DIF 18.8646／DEA 12.4344／MACD柱+12.86、K 71.44／D 68.76／J 76.81、5日均量20,397)後才採用本日值。⭐本日另記錄一項口徑澄清供後續維護參考：KDJ的9日RSV須以「最高價／最低價」序列計算，不可用收盤價序列——以收盤價序列試算9/9得K 82.77／D 72.07／J 104.17與已發布值差距甚大，改用高低價序列後9/8與9/9兩日均完全複現，確認高低價為本報既定口徑。⚠️⚠️本日另補正兩處長期沿用的過期靜態欄位：52週低點因窗口前滾已失效——台股2330自1,065更正為1,235.00、ADR TSM自223.70更正為257.98(均為Yahoo meta之fiftyTwoWeekLow本日實測；stockanalysis.com同頁顯示257.75，差0.23應為盤中價與收盤價取法差異，本報採Yahoo值並標明另一讀數)。此二者並非算錯而是窗口過期未更新，屬既有靜態欄位缺口。
+⭐綜合研判：評級自「中性偏多」下修為「中性」。本日要處理一組罕見的背離——基本面交出本波最強成績單(8月營收首破NT$5,000億、+53.3% YoY、連4個月創高、Q3指引達成風險大幅降低)，價格與技術面卻同時觸發前報所訂的失敗確認(KDJ死叉＋收在2,470之下)，本報依約履行下修。⭐最關鍵的判讀在時序而非數字：營收於台股收盤後公布，美股9/10全場都在已知此數字的情況下交易，ADR仍收-1.68%、費半-2.66%——排除了「市場還沒反應」的解釋，只剩一種讀法：在總經壓力(PPI 5.4%、油價破百、殖利率4.94%)與5年第88百分位的評價水位下，市場對好消息的邊際反應已鈍化。⚠️三項偏空證據：KDJ死叉成立、收盤首度跌破MA5、外資連2日賣超；⭐三項支撐仍在：MA10以下四條均線全數站上且仍上彎、9/10留15點下影線證明2,435至2,440有承接、營收證明基本面無虞。⚠️⚠️今日盤面已先行給出答案：今晨夜盤(TAIFEX標記日期2026/09/11之「盤後」列，涵蓋9/10 15:00至今晨05:00)CDF 202609重挫32點收2,415(-1.31%、成交2,267口)、台指期TX 202609跌797點收46,072(-1.70%、成交34,522口)，兩者同向重挫且已完整反映9/10美股半導體賣壓；現貨09:19台北開2,430(低開20點)、最高2,430、最低2,415、委買2,415／委賣2,420、成交4,949張，加權指數46,213.18(-727.31、-1.55%)——現貨開盤後即向夜盤所指的2,415靠攏，夜盤預示在今晨獲得驗證。今日檢核依優先順序：(1)⚠️⚠️第一順位已自「營收數字」換成「市場對好數字的反應」，具體檢核價位為20日均線暨布林中軌2,410——今日若收在其下，回檔性質即自「向均線靠攏」升級為「跌破中軌」，須再下修至偏空；若能收復5日均線2,451，則本次死叉可視為假訊號。(2)⚠️今晚美國8月CPI，且今日同時為TXO週五結算日，兩者疊加使今日量價訊號可靠度下降；在PPI已達5.4%、油價破百、殖利率4.94%的背景下，CPI偏高將直接壓縮P/E 28.40x的評價水位。(3)⭐觀察KDJ死叉後續：J值64.32距50尚有14.32點，若J跌破50且D開始下彎(本日D為小幅下滑而非續升)，才構成中期轉弱確認。(4)⚠️台積電個股期未平倉是否止跌：已連6日減少至18,850口，惟本日減幅為6日中最小、減碼速度放緩。(5)⭐9/16(下週三、3個交易日後)台股除息NT$7.00001，屆時股價機械性扣除約7點，勿誤讀為下跌。次要支撐依序為2,435(9/10盤中低)、2,430(10MA)、2,410(20MA＝布林中軌)、2,399(60MA季線)；反壓為2,451(5MA、待收復)、2,455、2,474(布林上軌)、2,505。⚠️9/15至16 FOMC(決策台北時間9/17凌晨2:00)，本週三項總經事件時點高度集中。</t>
+        </is>
+      </c>
+      <c r="G124" s="53" t="inlineStr">
+        <is>
+          <t>Yahoo Finance / Bloomberg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:G2"/>

</xml_diff>